<commit_message>
fix: update code and rerun the code
</commit_message>
<xml_diff>
--- a/data/proteomics/membrane_size_across_compartment_Rosemary_NH4_limitation_v2.xlsx
+++ b/data/proteomics/membrane_size_across_compartment_Rosemary_NH4_limitation_v2.xlsx
@@ -538,22 +538,22 @@
         <v>175.2179951479615</v>
       </c>
       <c r="D2" t="n">
-        <v>160.0444973878097</v>
+        <v>160.0444973878101</v>
       </c>
       <c r="E2" t="n">
         <v>168.5410689658389</v>
       </c>
       <c r="F2" t="n">
-        <v>132.4694784504293</v>
+        <v>132.4694784504292</v>
       </c>
       <c r="G2" t="n">
         <v>138.9107551105769</v>
       </c>
       <c r="H2" t="n">
-        <v>194.1516392720852</v>
+        <v>194.1516392720851</v>
       </c>
       <c r="I2" t="n">
-        <v>201.8798627229507</v>
+        <v>201.8798627229512</v>
       </c>
       <c r="J2" t="n">
         <v>173.7795767292691</v>
@@ -562,31 +562,31 @@
         <v>176.5021655182092</v>
       </c>
       <c r="L2" t="n">
-        <v>188.392119752045</v>
+        <v>188.3921197520449</v>
       </c>
       <c r="M2" t="n">
-        <v>187.3070433279954</v>
+        <v>187.3070433279953</v>
       </c>
       <c r="N2" t="n">
-        <v>191.0380320703822</v>
+        <v>191.0380320703821</v>
       </c>
       <c r="O2" t="n">
-        <v>338.4823015571529</v>
+        <v>338.4823015571528</v>
       </c>
       <c r="P2" t="n">
-        <v>339.9679037431539</v>
+        <v>339.9679037431536</v>
       </c>
       <c r="Q2" t="n">
-        <v>316.4651507008169</v>
+        <v>316.465150700817</v>
       </c>
       <c r="R2" t="n">
-        <v>424.97283683609</v>
+        <v>424.9728368360899</v>
       </c>
       <c r="S2" t="n">
-        <v>452.7732087518454</v>
+        <v>452.7732087518457</v>
       </c>
       <c r="T2" t="n">
-        <v>448.8247288819235</v>
+        <v>448.824728881924</v>
       </c>
     </row>
     <row r="3">
@@ -599,7 +599,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.3708259819820348</v>
+        <v>0.3708259819820347</v>
       </c>
       <c r="D3" t="n">
         <v>0.3520361165960142</v>
@@ -626,7 +626,7 @@
         <v>0.3400807864308382</v>
       </c>
       <c r="L3" t="n">
-        <v>0.3627065316307947</v>
+        <v>0.3627065316307945</v>
       </c>
       <c r="M3" t="n">
         <v>0.3555703574112495</v>
@@ -635,13 +635,13 @@
         <v>0.3924982775995451</v>
       </c>
       <c r="O3" t="n">
-        <v>0.5003321480743244</v>
+        <v>0.5003321480743245</v>
       </c>
       <c r="P3" t="n">
         <v>0.5162502252648964</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.4992434495697613</v>
+        <v>0.4992434495697612</v>
       </c>
       <c r="R3" t="n">
         <v>0.578346559989949</v>
@@ -650,7 +650,7 @@
         <v>0.6028096168457832</v>
       </c>
       <c r="T3" t="n">
-        <v>0.5580478351504095</v>
+        <v>0.5580478351504093</v>
       </c>
     </row>
     <row r="4">
@@ -669,7 +669,7 @@
         <v>0.2601275712257239</v>
       </c>
       <c r="E4" t="n">
-        <v>0.2878897626554287</v>
+        <v>0.2878897626554286</v>
       </c>
       <c r="F4" t="n">
         <v>0.2751683226782104</v>
@@ -681,37 +681,37 @@
         <v>0.2900750027999563</v>
       </c>
       <c r="I4" t="n">
-        <v>0.4146122774205819</v>
+        <v>0.4146122774205822</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3471933041993003</v>
+        <v>0.3471933041993002</v>
       </c>
       <c r="K4" t="n">
         <v>0.3290448836663721</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3745999273268713</v>
+        <v>0.3745999273268714</v>
       </c>
       <c r="M4" t="n">
-        <v>0.4151547571207965</v>
+        <v>0.4151547571207964</v>
       </c>
       <c r="N4" t="n">
-        <v>0.4111555903524835</v>
+        <v>0.4111555903524837</v>
       </c>
       <c r="O4" t="n">
-        <v>0.6506676470786706</v>
+        <v>0.6506676470786708</v>
       </c>
       <c r="P4" t="n">
-        <v>0.6913160163047214</v>
+        <v>0.6913160163047212</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.6883910427175276</v>
+        <v>0.6883910427175277</v>
       </c>
       <c r="R4" t="n">
-        <v>0.8026681630801572</v>
+        <v>0.8026681630801574</v>
       </c>
       <c r="S4" t="n">
-        <v>0.9624695034230455</v>
+        <v>0.9624695034230457</v>
       </c>
       <c r="T4" t="n">
         <v>0.9224246385322585</v>
@@ -791,19 +791,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>104.4945795180777</v>
+        <v>104.4945795180776</v>
       </c>
       <c r="D6" t="n">
-        <v>95.81337389222566</v>
+        <v>95.8133738922256</v>
       </c>
       <c r="E6" t="n">
         <v>102.9450256576945</v>
       </c>
       <c r="F6" t="n">
-        <v>80.27718466102294</v>
+        <v>80.27718466102304</v>
       </c>
       <c r="G6" t="n">
-        <v>84.7860045561757</v>
+        <v>84.78600455617567</v>
       </c>
       <c r="H6" t="n">
         <v>114.8174438999057</v>
@@ -812,37 +812,37 @@
         <v>119.8186726907256</v>
       </c>
       <c r="J6" t="n">
-        <v>105.0651197106895</v>
+        <v>105.0651197106894</v>
       </c>
       <c r="K6" t="n">
         <v>103.9541102612538</v>
       </c>
       <c r="L6" t="n">
-        <v>107.1511386458312</v>
+        <v>107.1511386458314</v>
       </c>
       <c r="M6" t="n">
         <v>108.7628022245244</v>
       </c>
       <c r="N6" t="n">
-        <v>110.3052217624947</v>
+        <v>110.3052217624945</v>
       </c>
       <c r="O6" t="n">
-        <v>197.5002617175616</v>
+        <v>197.5002617175619</v>
       </c>
       <c r="P6" t="n">
-        <v>199.9282717881693</v>
+        <v>199.9282717881696</v>
       </c>
       <c r="Q6" t="n">
-        <v>190.4890067392386</v>
+        <v>190.4890067392384</v>
       </c>
       <c r="R6" t="n">
-        <v>263.174293165467</v>
+        <v>263.1742931654672</v>
       </c>
       <c r="S6" t="n">
-        <v>283.6896214537359</v>
+        <v>283.6896214537362</v>
       </c>
       <c r="T6" t="n">
-        <v>269.2484509264083</v>
+        <v>269.2484509264085</v>
       </c>
     </row>
     <row r="7">
@@ -858,7 +858,7 @@
         <v>227.0895431527453</v>
       </c>
       <c r="D7" t="n">
-        <v>206.7361723285035</v>
+        <v>206.7361723285034</v>
       </c>
       <c r="E7" t="n">
         <v>213.7851497908103</v>
@@ -867,46 +867,46 @@
         <v>176.2278896016975</v>
       </c>
       <c r="G7" t="n">
-        <v>186.3067644873687</v>
+        <v>186.3067644873686</v>
       </c>
       <c r="H7" t="n">
-        <v>256.1877228197559</v>
+        <v>256.187722819756</v>
       </c>
       <c r="I7" t="n">
-        <v>272.7578975486281</v>
+        <v>272.7578975486283</v>
       </c>
       <c r="J7" t="n">
-        <v>232.3532486181905</v>
+        <v>232.3532486181907</v>
       </c>
       <c r="K7" t="n">
-        <v>235.0706214611074</v>
+        <v>235.0706214611072</v>
       </c>
       <c r="L7" t="n">
-        <v>277.1407638493976</v>
+        <v>277.1407638493975</v>
       </c>
       <c r="M7" t="n">
-        <v>268.7329213330884</v>
+        <v>268.7329213330882</v>
       </c>
       <c r="N7" t="n">
-        <v>264.3676705543982</v>
+        <v>264.3676705543986</v>
       </c>
       <c r="O7" t="n">
-        <v>550.9705103015147</v>
+        <v>550.9705103015149</v>
       </c>
       <c r="P7" t="n">
         <v>550.8143144862206</v>
       </c>
       <c r="Q7" t="n">
-        <v>531.8284565095476</v>
+        <v>531.828456509548</v>
       </c>
       <c r="R7" t="n">
-        <v>759.074433036407</v>
+        <v>759.0744330364072</v>
       </c>
       <c r="S7" t="n">
-        <v>797.3983425768859</v>
+        <v>797.3983425768865</v>
       </c>
       <c r="T7" t="n">
-        <v>785.765087978192</v>
+        <v>785.7650879781916</v>
       </c>
     </row>
     <row r="8">
@@ -922,19 +922,19 @@
         <v>105.1013304776598</v>
       </c>
       <c r="D8" t="n">
-        <v>92.52612055309257</v>
+        <v>92.52612055309254</v>
       </c>
       <c r="E8" t="n">
-        <v>90.77862659703366</v>
+        <v>90.77862659703371</v>
       </c>
       <c r="F8" t="n">
-        <v>79.86886913329829</v>
+        <v>79.86886913329828</v>
       </c>
       <c r="G8" t="n">
         <v>82.45308225254723</v>
       </c>
       <c r="H8" t="n">
-        <v>124.7777434740009</v>
+        <v>124.7777434740008</v>
       </c>
       <c r="I8" t="n">
         <v>122.9903899924766</v>
@@ -943,7 +943,7 @@
         <v>107.1485899417069</v>
       </c>
       <c r="K8" t="n">
-        <v>106.7000971377189</v>
+        <v>106.700097137719</v>
       </c>
       <c r="L8" t="n">
         <v>104.1523720523613</v>
@@ -952,25 +952,25 @@
         <v>106.3532786148636</v>
       </c>
       <c r="N8" t="n">
-        <v>104.6966534357504</v>
+        <v>104.6966534357503</v>
       </c>
       <c r="O8" t="n">
         <v>202.7461011100775</v>
       </c>
       <c r="P8" t="n">
-        <v>201.4705166773789</v>
+        <v>201.470516677379</v>
       </c>
       <c r="Q8" t="n">
-        <v>197.1847244190116</v>
+        <v>197.1847244190118</v>
       </c>
       <c r="R8" t="n">
-        <v>277.9700000718029</v>
+        <v>277.9700000718026</v>
       </c>
       <c r="S8" t="n">
-        <v>308.7744288208417</v>
+        <v>308.7744288208419</v>
       </c>
       <c r="T8" t="n">
-        <v>286.234307123676</v>
+        <v>286.2343071236762</v>
       </c>
     </row>
     <row r="9">
@@ -983,10 +983,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>29.33172266429985</v>
+        <v>29.33172266429986</v>
       </c>
       <c r="D9" t="n">
-        <v>27.36723455464773</v>
+        <v>27.36723455464774</v>
       </c>
       <c r="E9" t="n">
         <v>24.98386908080797</v>
@@ -1004,10 +1004,10 @@
         <v>32.0449226823412</v>
       </c>
       <c r="J9" t="n">
-        <v>27.93061303722451</v>
+        <v>27.93061303722452</v>
       </c>
       <c r="K9" t="n">
-        <v>28.97186337142023</v>
+        <v>28.97186337142022</v>
       </c>
       <c r="L9" t="n">
         <v>25.98185544396454</v>
@@ -1016,13 +1016,13 @@
         <v>25.88520263437931</v>
       </c>
       <c r="N9" t="n">
-        <v>22.34533065527027</v>
+        <v>22.34533065527026</v>
       </c>
       <c r="O9" t="n">
         <v>51.92845623094195</v>
       </c>
       <c r="P9" t="n">
-        <v>49.64308423613164</v>
+        <v>49.64308423613163</v>
       </c>
       <c r="Q9" t="n">
         <v>55.17449330541861</v>
@@ -1031,10 +1031,10 @@
         <v>78.52670899027697</v>
       </c>
       <c r="S9" t="n">
-        <v>86.58033040432601</v>
+        <v>86.58033040432602</v>
       </c>
       <c r="T9" t="n">
-        <v>77.0120479880252</v>
+        <v>77.01204798802522</v>
       </c>
     </row>
     <row r="10">
@@ -1111,46 +1111,46 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>44.88391858779396</v>
+        <v>44.88391858779397</v>
       </c>
       <c r="D11" t="n">
         <v>39.38859037636782</v>
       </c>
       <c r="E11" t="n">
-        <v>34.16741458109772</v>
+        <v>34.16741458109771</v>
       </c>
       <c r="F11" t="n">
-        <v>30.43728128847774</v>
+        <v>30.43728128847775</v>
       </c>
       <c r="G11" t="n">
         <v>31.0882376660685</v>
       </c>
       <c r="H11" t="n">
-        <v>57.46909296549883</v>
+        <v>57.46909296549882</v>
       </c>
       <c r="I11" t="n">
         <v>49.48987799306352</v>
       </c>
       <c r="J11" t="n">
-        <v>42.47196063001724</v>
+        <v>42.47196063001721</v>
       </c>
       <c r="K11" t="n">
         <v>43.1574878017832</v>
       </c>
       <c r="L11" t="n">
-        <v>37.93758004013361</v>
+        <v>37.93758004013362</v>
       </c>
       <c r="M11" t="n">
-        <v>39.8055979145052</v>
+        <v>39.80559791450519</v>
       </c>
       <c r="N11" t="n">
-        <v>34.32068342049714</v>
+        <v>34.32068342049713</v>
       </c>
       <c r="O11" t="n">
-        <v>78.82347839509923</v>
+        <v>78.82347839509917</v>
       </c>
       <c r="P11" t="n">
-        <v>79.32295137278484</v>
+        <v>79.32295137278486</v>
       </c>
       <c r="Q11" t="n">
         <v>79.74836981076972</v>
@@ -1175,22 +1175,22 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>12.37121765109383</v>
+        <v>12.3712176510938</v>
       </c>
       <c r="D12" t="n">
-        <v>11.22209800662488</v>
+        <v>11.22209800662489</v>
       </c>
       <c r="E12" t="n">
         <v>10.99321760413046</v>
       </c>
       <c r="F12" t="n">
-        <v>10.19134887106634</v>
+        <v>10.19134887106636</v>
       </c>
       <c r="G12" t="n">
         <v>11.24906435751132</v>
       </c>
       <c r="H12" t="n">
-        <v>10.9816103740719</v>
+        <v>10.98161037407191</v>
       </c>
       <c r="I12" t="n">
         <v>16.70952615798391</v>
@@ -1205,28 +1205,28 @@
         <v>17.19123215896571</v>
       </c>
       <c r="M12" t="n">
-        <v>15.9791180294715</v>
+        <v>15.97911802947151</v>
       </c>
       <c r="N12" t="n">
         <v>17.09755670687182</v>
       </c>
       <c r="O12" t="n">
-        <v>26.60739153097735</v>
+        <v>26.60739153097733</v>
       </c>
       <c r="P12" t="n">
-        <v>27.18642336678111</v>
+        <v>27.18642336678113</v>
       </c>
       <c r="Q12" t="n">
-        <v>26.08149031429908</v>
+        <v>26.08149031429906</v>
       </c>
       <c r="R12" t="n">
-        <v>30.92416302141376</v>
+        <v>30.92416302141377</v>
       </c>
       <c r="S12" t="n">
-        <v>33.67093013591804</v>
+        <v>33.67093013591801</v>
       </c>
       <c r="T12" t="n">
-        <v>34.87168598776994</v>
+        <v>34.87168598776996</v>
       </c>
     </row>
     <row r="13">
@@ -1245,7 +1245,7 @@
         <v>1.391237317232775</v>
       </c>
       <c r="E13" t="n">
-        <v>1.432905886592719</v>
+        <v>1.432905886592718</v>
       </c>
       <c r="F13" t="n">
         <v>1.483570131170016</v>
@@ -1257,7 +1257,7 @@
         <v>1.306216968593031</v>
       </c>
       <c r="I13" t="n">
-        <v>2.609410905571942</v>
+        <v>2.609410905571941</v>
       </c>
       <c r="J13" t="n">
         <v>2.100707647950022</v>
@@ -1266,31 +1266,31 @@
         <v>2.368011853405704</v>
       </c>
       <c r="L13" t="n">
-        <v>2.733202960559168</v>
+        <v>2.733202960559169</v>
       </c>
       <c r="M13" t="n">
         <v>2.394400220074553</v>
       </c>
       <c r="N13" t="n">
-        <v>2.737326259186796</v>
+        <v>2.737326259186795</v>
       </c>
       <c r="O13" t="n">
-        <v>3.725108609580325</v>
+        <v>3.725108609580324</v>
       </c>
       <c r="P13" t="n">
         <v>3.445901137445752</v>
       </c>
       <c r="Q13" t="n">
-        <v>3.65493199032628</v>
+        <v>3.654931990326281</v>
       </c>
       <c r="R13" t="n">
-        <v>3.315162242105957</v>
+        <v>3.315162242105956</v>
       </c>
       <c r="S13" t="n">
-        <v>3.635938154208346</v>
+        <v>3.635938154208347</v>
       </c>
       <c r="T13" t="n">
-        <v>3.986433630032791</v>
+        <v>3.98643363003279</v>
       </c>
     </row>
     <row r="14">
@@ -1306,34 +1306,34 @@
         <v>8.834259072602096</v>
       </c>
       <c r="D14" t="n">
-        <v>8.706356576039489</v>
+        <v>8.706356576039491</v>
       </c>
       <c r="E14" t="n">
         <v>10.01133393430948</v>
       </c>
       <c r="F14" t="n">
-        <v>6.530599188264407</v>
+        <v>6.530599188264406</v>
       </c>
       <c r="G14" t="n">
         <v>7.555276016239143</v>
       </c>
       <c r="H14" t="n">
-        <v>9.51378560731837</v>
+        <v>9.513785607318372</v>
       </c>
       <c r="I14" t="n">
         <v>11.28547886339388</v>
       </c>
       <c r="J14" t="n">
-        <v>9.556682794319094</v>
+        <v>9.556682794319098</v>
       </c>
       <c r="K14" t="n">
-        <v>9.332337557072192</v>
+        <v>9.332337557072195</v>
       </c>
       <c r="L14" t="n">
         <v>10.29327721599667</v>
       </c>
       <c r="M14" t="n">
-        <v>9.736310523820672</v>
+        <v>9.736310523820675</v>
       </c>
       <c r="N14" t="n">
         <v>10.64477255047419</v>
@@ -1348,13 +1348,13 @@
         <v>13.04493835903978</v>
       </c>
       <c r="R14" t="n">
-        <v>15.62250490095467</v>
+        <v>15.62250490095466</v>
       </c>
       <c r="S14" t="n">
-        <v>16.78014764680845</v>
+        <v>16.78014764680844</v>
       </c>
       <c r="T14" t="n">
-        <v>17.08224206893462</v>
+        <v>17.08224206893463</v>
       </c>
     </row>
     <row r="15">
@@ -1385,7 +1385,7 @@
         <v>2.546278938749803</v>
       </c>
       <c r="I15" t="n">
-        <v>2.624838174111785</v>
+        <v>2.624838174111786</v>
       </c>
       <c r="J15" t="n">
         <v>2.266429528365788</v>
@@ -1394,7 +1394,7 @@
         <v>2.061607512407088</v>
       </c>
       <c r="L15" t="n">
-        <v>2.165748760732103</v>
+        <v>2.165748760732102</v>
       </c>
       <c r="M15" t="n">
         <v>1.990417712685602</v>
@@ -1406,7 +1406,7 @@
         <v>3.294903038112016</v>
       </c>
       <c r="P15" t="n">
-        <v>3.877453199129756</v>
+        <v>3.877453199129757</v>
       </c>
       <c r="Q15" t="n">
         <v>3.020817851880673</v>
@@ -1437,7 +1437,7 @@
         <v>1.79047701018833</v>
       </c>
       <c r="E16" t="n">
-        <v>1.675540337076725</v>
+        <v>1.675540337076726</v>
       </c>
       <c r="F16" t="n">
         <v>1.769405495628907</v>
@@ -1446,10 +1446,10 @@
         <v>1.805008251780691</v>
       </c>
       <c r="H16" t="n">
-        <v>1.393755151468504</v>
+        <v>1.393755151468505</v>
       </c>
       <c r="I16" t="n">
-        <v>2.595010764878985</v>
+        <v>2.595010764878983</v>
       </c>
       <c r="J16" t="n">
         <v>2.070685091602589</v>
@@ -1464,25 +1464,25 @@
         <v>2.626509281078438</v>
       </c>
       <c r="N16" t="n">
-        <v>2.793978906999192</v>
+        <v>2.793978906999193</v>
       </c>
       <c r="O16" t="n">
-        <v>3.906260789134768</v>
+        <v>3.906260789134767</v>
       </c>
       <c r="P16" t="n">
         <v>3.83433200290798</v>
       </c>
       <c r="Q16" t="n">
-        <v>3.761919792796915</v>
+        <v>3.761919792796914</v>
       </c>
       <c r="R16" t="n">
         <v>4.253952706653429</v>
       </c>
       <c r="S16" t="n">
-        <v>4.352405875048257</v>
+        <v>4.35240587504826</v>
       </c>
       <c r="T16" t="n">
-        <v>5.006679935035801</v>
+        <v>5.006679935035803</v>
       </c>
     </row>
     <row r="17">
@@ -1495,10 +1495,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>3.080177624420704</v>
+        <v>3.080177624420705</v>
       </c>
       <c r="D17" t="n">
-        <v>2.344927407504835</v>
+        <v>2.344927407504834</v>
       </c>
       <c r="E17" t="n">
         <v>2.474702807906972</v>
@@ -1513,19 +1513,19 @@
         <v>2.49295776067943</v>
       </c>
       <c r="I17" t="n">
-        <v>4.345404085764374</v>
+        <v>4.345404085764373</v>
       </c>
       <c r="J17" t="n">
-        <v>3.573699003903969</v>
+        <v>3.573699003903968</v>
       </c>
       <c r="K17" t="n">
-        <v>2.825545655808233</v>
+        <v>2.825545655808232</v>
       </c>
       <c r="L17" t="n">
-        <v>4.321007455276041</v>
+        <v>4.32100745527604</v>
       </c>
       <c r="M17" t="n">
-        <v>3.886444447192756</v>
+        <v>3.886444447192754</v>
       </c>
       <c r="N17" t="n">
         <v>4.277978724909394</v>
@@ -1537,16 +1537,16 @@
         <v>6.023177172559853</v>
       </c>
       <c r="Q17" t="n">
-        <v>5.554566851162716</v>
+        <v>5.554566851162718</v>
       </c>
       <c r="R17" t="n">
-        <v>6.169677931648652</v>
+        <v>6.169677931648655</v>
       </c>
       <c r="S17" t="n">
         <v>6.272894064982358</v>
       </c>
       <c r="T17" t="n">
-        <v>6.704989322128009</v>
+        <v>6.704989322128011</v>
       </c>
     </row>
     <row r="18">
@@ -1559,58 +1559,58 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2.697049978710424</v>
+        <v>2.697049978710423</v>
       </c>
       <c r="D18" t="n">
-        <v>2.367569589075473</v>
+        <v>2.367569589075471</v>
       </c>
       <c r="E18" t="n">
         <v>2.251324005595607</v>
       </c>
       <c r="F18" t="n">
-        <v>2.131324671124972</v>
+        <v>2.131324671124971</v>
       </c>
       <c r="G18" t="n">
         <v>2.354784592268257</v>
       </c>
       <c r="H18" t="n">
-        <v>2.119350125178393</v>
+        <v>2.119350125178392</v>
       </c>
       <c r="I18" t="n">
-        <v>3.484594297209453</v>
+        <v>3.484594297209451</v>
       </c>
       <c r="J18" t="n">
-        <v>2.827651824938837</v>
+        <v>2.827651824938835</v>
       </c>
       <c r="K18" t="n">
-        <v>3.247249273668731</v>
+        <v>3.247249273668733</v>
       </c>
       <c r="L18" t="n">
         <v>3.585612856636332</v>
       </c>
       <c r="M18" t="n">
-        <v>3.431604030995714</v>
+        <v>3.431604030995715</v>
       </c>
       <c r="N18" t="n">
         <v>3.538331749640751</v>
       </c>
       <c r="O18" t="n">
-        <v>5.882607456598449</v>
+        <v>5.88260745659845</v>
       </c>
       <c r="P18" t="n">
-        <v>5.949131763719676</v>
+        <v>5.949131763719678</v>
       </c>
       <c r="Q18" t="n">
-        <v>5.5952396878183</v>
+        <v>5.595239687818302</v>
       </c>
       <c r="R18" t="n">
-        <v>7.203289999042919</v>
+        <v>7.203289999042921</v>
       </c>
       <c r="S18" t="n">
-        <v>8.735446391515644</v>
+        <v>8.73544639151565</v>
       </c>
       <c r="T18" t="n">
-        <v>9.028734150007697</v>
+        <v>9.028734150007699</v>
       </c>
     </row>
     <row r="19">
@@ -1623,25 +1623,25 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.39461808147511</v>
+        <v>1.394618081475112</v>
       </c>
       <c r="D19" t="n">
         <v>1.253350678060727</v>
       </c>
       <c r="E19" t="n">
-        <v>1.282973572231973</v>
+        <v>1.282973572231972</v>
       </c>
       <c r="F19" t="n">
-        <v>1.248900046263693</v>
+        <v>1.248900046263694</v>
       </c>
       <c r="G19" t="n">
         <v>1.298498567442569</v>
       </c>
       <c r="H19" t="n">
-        <v>1.42281766388067</v>
+        <v>1.422817663880669</v>
       </c>
       <c r="I19" t="n">
-        <v>2.007546775665482</v>
+        <v>2.007546775665483</v>
       </c>
       <c r="J19" t="n">
         <v>1.754853205190291</v>
@@ -1650,7 +1650,7 @@
         <v>1.750947455166642</v>
       </c>
       <c r="L19" t="n">
-        <v>2.033171827422393</v>
+        <v>2.033171827422394</v>
       </c>
       <c r="M19" t="n">
         <v>1.965292494422673</v>
@@ -1659,22 +1659,22 @@
         <v>2.0331648319044</v>
       </c>
       <c r="O19" t="n">
-        <v>3.169463582482697</v>
+        <v>3.169463582482698</v>
       </c>
       <c r="P19" t="n">
         <v>3.224974770365973</v>
       </c>
       <c r="Q19" t="n">
-        <v>3.067936579055761</v>
+        <v>3.067936579055762</v>
       </c>
       <c r="R19" t="n">
-        <v>4.038574819956987</v>
+        <v>4.038574819956988</v>
       </c>
       <c r="S19" t="n">
-        <v>4.206550290138673</v>
+        <v>4.206550290138672</v>
       </c>
       <c r="T19" t="n">
-        <v>4.182635611530205</v>
+        <v>4.182635611530207</v>
       </c>
     </row>
     <row r="20">
@@ -1687,43 +1687,43 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4.335169502189709</v>
+        <v>4.33516950218971</v>
       </c>
       <c r="D20" t="n">
         <v>3.77073536509215</v>
       </c>
       <c r="E20" t="n">
-        <v>4.197775951766889</v>
+        <v>4.197775951766891</v>
       </c>
       <c r="F20" t="n">
         <v>3.880091227827486</v>
       </c>
       <c r="G20" t="n">
-        <v>4.205488963910328</v>
+        <v>4.205488963910329</v>
       </c>
       <c r="H20" t="n">
-        <v>5.342620371404054</v>
+        <v>5.342620371404055</v>
       </c>
       <c r="I20" t="n">
-        <v>6.275997977658265</v>
+        <v>6.275997977658262</v>
       </c>
       <c r="J20" t="n">
-        <v>5.405688715368903</v>
+        <v>5.405688715368906</v>
       </c>
       <c r="K20" t="n">
-        <v>5.517800802999912</v>
+        <v>5.517800802999911</v>
       </c>
       <c r="L20" t="n">
-        <v>6.779577136475654</v>
+        <v>6.779577136475655</v>
       </c>
       <c r="M20" t="n">
-        <v>6.822938493470521</v>
+        <v>6.822938493470524</v>
       </c>
       <c r="N20" t="n">
-        <v>6.110590743398348</v>
+        <v>6.110590743398344</v>
       </c>
       <c r="O20" t="n">
-        <v>13.27941177386085</v>
+        <v>13.27941177386086</v>
       </c>
       <c r="P20" t="n">
         <v>12.97248403445492</v>
@@ -1738,7 +1738,7 @@
         <v>14.95038329562327</v>
       </c>
       <c r="T20" t="n">
-        <v>17.12089756026327</v>
+        <v>17.12089756026326</v>
       </c>
     </row>
     <row r="21">
@@ -1815,10 +1815,10 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.5146219466097859</v>
+        <v>0.514621946609786</v>
       </c>
       <c r="D22" t="n">
-        <v>0.4638494644943264</v>
+        <v>0.4638494644943266</v>
       </c>
       <c r="E22" t="n">
         <v>0.4647205002873783</v>
@@ -1827,28 +1827,28 @@
         <v>0.4232532910037191</v>
       </c>
       <c r="G22" t="n">
-        <v>0.4508700182311752</v>
+        <v>0.4508700182311753</v>
       </c>
       <c r="H22" t="n">
         <v>0.4570617448494493</v>
       </c>
       <c r="I22" t="n">
-        <v>0.6809541129387652</v>
+        <v>0.6809541129387651</v>
       </c>
       <c r="J22" t="n">
-        <v>0.6050064616045413</v>
+        <v>0.6050064616045414</v>
       </c>
       <c r="K22" t="n">
-        <v>0.608199211606927</v>
+        <v>0.6081992116069272</v>
       </c>
       <c r="L22" t="n">
-        <v>0.7024153448399537</v>
+        <v>0.7024153448399536</v>
       </c>
       <c r="M22" t="n">
         <v>0.6831327355708822</v>
       </c>
       <c r="N22" t="n">
-        <v>0.7426155281044446</v>
+        <v>0.7426155281044445</v>
       </c>
       <c r="O22" t="n">
         <v>1.109035337770553</v>
@@ -1882,7 +1882,7 @@
         <v>22.16846366169906</v>
       </c>
       <c r="D23" t="n">
-        <v>18.03371716911288</v>
+        <v>18.03371716911289</v>
       </c>
       <c r="E23" t="n">
         <v>16.1989319814308</v>
@@ -1891,7 +1891,7 @@
         <v>13.91132598749002</v>
       </c>
       <c r="G23" t="n">
-        <v>13.28492633742168</v>
+        <v>13.28492633742167</v>
       </c>
       <c r="H23" t="n">
         <v>34.89380449301557</v>
@@ -1900,7 +1900,7 @@
         <v>27.94648952835622</v>
       </c>
       <c r="J23" t="n">
-        <v>23.30033193856781</v>
+        <v>23.3003319385678</v>
       </c>
       <c r="K23" t="n">
         <v>21.71390926757909</v>
@@ -1912,7 +1912,7 @@
         <v>21.91786035124965</v>
       </c>
       <c r="N23" t="n">
-        <v>19.95199690421991</v>
+        <v>19.95199690421992</v>
       </c>
       <c r="O23" t="n">
         <v>42.00368858747422</v>
@@ -1924,7 +1924,7 @@
         <v>40.85438593492318</v>
       </c>
       <c r="R23" t="n">
-        <v>57.45436274853692</v>
+        <v>57.45436274853693</v>
       </c>
       <c r="S23" t="n">
         <v>74.60968757876508</v>
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.0970549600016119</v>
+        <v>0.09705496000161189</v>
       </c>
       <c r="D24" t="n">
         <v>0.1000493163611742</v>
@@ -1955,10 +1955,10 @@
         <v>0.1041190861322172</v>
       </c>
       <c r="G24" t="n">
-        <v>0.09695382734747529</v>
+        <v>0.0969538273474753</v>
       </c>
       <c r="H24" t="n">
-        <v>0.1350705664009528</v>
+        <v>0.1350705664009529</v>
       </c>
       <c r="I24" t="n">
         <v>0.1843689025612976</v>
@@ -1982,7 +1982,7 @@
         <v>0.3246791236204478</v>
       </c>
       <c r="P24" t="n">
-        <v>0.3210695322001895</v>
+        <v>0.3210695322001896</v>
       </c>
       <c r="Q24" t="n">
         <v>0.3242406935439865</v>
@@ -2019,7 +2019,7 @@
         <v>1.087471494210944</v>
       </c>
       <c r="G25" t="n">
-        <v>1.182735505186204</v>
+        <v>1.182735505186205</v>
       </c>
       <c r="H25" t="n">
         <v>1.718455520972461</v>
@@ -2031,7 +2031,7 @@
         <v>1.473597603176667</v>
       </c>
       <c r="K25" t="n">
-        <v>1.558999231146299</v>
+        <v>1.558999231146298</v>
       </c>
       <c r="L25" t="n">
         <v>1.803257211624508</v>
@@ -2049,16 +2049,16 @@
         <v>3.087807269100277</v>
       </c>
       <c r="Q25" t="n">
-        <v>2.817306935382982</v>
+        <v>2.817306935382981</v>
       </c>
       <c r="R25" t="n">
-        <v>3.470960661583678</v>
+        <v>3.470960661583677</v>
       </c>
       <c r="S25" t="n">
         <v>3.571209022316342</v>
       </c>
       <c r="T25" t="n">
-        <v>3.937660405606108</v>
+        <v>3.937660405606107</v>
       </c>
     </row>
     <row r="26">
@@ -2095,7 +2095,7 @@
         <v>1.548266336633656</v>
       </c>
       <c r="K26" t="n">
-        <v>1.777768147733415</v>
+        <v>1.777768147733416</v>
       </c>
       <c r="L26" t="n">
         <v>2.056544337895579</v>
@@ -2113,7 +2113,7 @@
         <v>2.7668958712086</v>
       </c>
       <c r="Q26" t="n">
-        <v>2.76365308868008</v>
+        <v>2.763653088680079</v>
       </c>
       <c r="R26" t="n">
         <v>3.238436963249196</v>
@@ -2135,28 +2135,28 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>9.4045486148806</v>
+        <v>9.404548614880596</v>
       </c>
       <c r="D27" t="n">
-        <v>8.081672728719518</v>
+        <v>8.081672728719521</v>
       </c>
       <c r="E27" t="n">
-        <v>8.82600546099248</v>
+        <v>8.826005460992473</v>
       </c>
       <c r="F27" t="n">
-        <v>8.461035997767326</v>
+        <v>8.461035997767329</v>
       </c>
       <c r="G27" t="n">
-        <v>8.483129903838181</v>
+        <v>8.483129903838179</v>
       </c>
       <c r="H27" t="n">
-        <v>11.64739412202549</v>
+        <v>11.64739412202548</v>
       </c>
       <c r="I27" t="n">
         <v>13.82307798420801</v>
       </c>
       <c r="J27" t="n">
-        <v>11.7009042275779</v>
+        <v>11.70090422757791</v>
       </c>
       <c r="K27" t="n">
         <v>11.38292990215321</v>
@@ -2168,25 +2168,25 @@
         <v>15.1735578247713</v>
       </c>
       <c r="N27" t="n">
-        <v>15.35778525360575</v>
+        <v>15.35778525360574</v>
       </c>
       <c r="O27" t="n">
-        <v>36.04669631674181</v>
+        <v>36.04669631674182</v>
       </c>
       <c r="P27" t="n">
-        <v>38.36051604651183</v>
+        <v>38.36051604651185</v>
       </c>
       <c r="Q27" t="n">
-        <v>35.55832547782603</v>
+        <v>35.55832547782602</v>
       </c>
       <c r="R27" t="n">
-        <v>54.29853086694441</v>
+        <v>54.29853086694439</v>
       </c>
       <c r="S27" t="n">
-        <v>59.24178136349355</v>
+        <v>59.24178136349354</v>
       </c>
       <c r="T27" t="n">
-        <v>57.57534920434809</v>
+        <v>57.57534920434807</v>
       </c>
     </row>
     <row r="28">
@@ -2199,10 +2199,10 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.2966098180711586</v>
+        <v>0.2966098180711588</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2735237095728638</v>
+        <v>0.2735237095728636</v>
       </c>
       <c r="E28" t="n">
         <v>0.3179767014571709</v>
@@ -2214,40 +2214,40 @@
         <v>0.2819010151367157</v>
       </c>
       <c r="H28" t="n">
-        <v>0.2847564985576653</v>
+        <v>0.2847564985576654</v>
       </c>
       <c r="I28" t="n">
-        <v>0.3880931541475547</v>
+        <v>0.3880931541475548</v>
       </c>
       <c r="J28" t="n">
         <v>0.3325835564324551</v>
       </c>
       <c r="K28" t="n">
-        <v>0.339136010933317</v>
+        <v>0.3391360109333171</v>
       </c>
       <c r="L28" t="n">
         <v>0.3818549328205632</v>
       </c>
       <c r="M28" t="n">
-        <v>0.3916087622637228</v>
+        <v>0.3916087622637227</v>
       </c>
       <c r="N28" t="n">
         <v>0.3851934035328792</v>
       </c>
       <c r="O28" t="n">
-        <v>0.6566030779648063</v>
+        <v>0.6566030779648062</v>
       </c>
       <c r="P28" t="n">
         <v>0.618488506865019</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.6013531913225519</v>
+        <v>0.601353191322552</v>
       </c>
       <c r="R28" t="n">
-        <v>0.7095695368170816</v>
+        <v>0.7095695368170815</v>
       </c>
       <c r="S28" t="n">
-        <v>0.72383611022419</v>
+        <v>0.7238361102241901</v>
       </c>
       <c r="T28" t="n">
         <v>0.7692599133981047</v>
@@ -2266,13 +2266,13 @@
         <v>14.47655535680351</v>
       </c>
       <c r="D29" t="n">
-        <v>13.99912192870183</v>
+        <v>13.99912192870184</v>
       </c>
       <c r="E29" t="n">
         <v>14.8626514397626</v>
       </c>
       <c r="F29" t="n">
-        <v>11.67889802480416</v>
+        <v>11.67889802480415</v>
       </c>
       <c r="G29" t="n">
         <v>13.58016626048591</v>
@@ -2281,10 +2281,10 @@
         <v>11.25688282684747</v>
       </c>
       <c r="I29" t="n">
-        <v>16.07264247295188</v>
+        <v>16.07264247295189</v>
       </c>
       <c r="J29" t="n">
-        <v>13.59756969944153</v>
+        <v>13.59756969944152</v>
       </c>
       <c r="K29" t="n">
         <v>14.88343703118448</v>
@@ -2302,19 +2302,19 @@
         <v>24.25873607835889</v>
       </c>
       <c r="P29" t="n">
-        <v>24.71870188120024</v>
+        <v>24.71870188120023</v>
       </c>
       <c r="Q29" t="n">
         <v>23.55321816763551</v>
       </c>
       <c r="R29" t="n">
-        <v>27.30672319240505</v>
+        <v>27.30672319240508</v>
       </c>
       <c r="S29" t="n">
-        <v>27.95490921811762</v>
+        <v>27.95490921811761</v>
       </c>
       <c r="T29" t="n">
-        <v>30.87203135452538</v>
+        <v>30.87203135452537</v>
       </c>
     </row>
     <row r="30">
@@ -2348,7 +2348,7 @@
         <v>0.02475228135865733</v>
       </c>
       <c r="J30" t="n">
-        <v>0.02296699809063352</v>
+        <v>0.02296699809063353</v>
       </c>
       <c r="K30" t="n">
         <v>0.01986648274287118</v>
@@ -2357,10 +2357,10 @@
         <v>0.02220517251655242</v>
       </c>
       <c r="M30" t="n">
-        <v>0.02516978813192495</v>
+        <v>0.02516978813192496</v>
       </c>
       <c r="N30" t="n">
-        <v>0.02413512281717073</v>
+        <v>0.02413512281717074</v>
       </c>
       <c r="O30" t="n">
         <v>0.03954050305358028</v>
@@ -2372,7 +2372,7 @@
         <v>0.03549163257831871</v>
       </c>
       <c r="R30" t="n">
-        <v>0.05375065546140828</v>
+        <v>0.05375065546140826</v>
       </c>
       <c r="S30" t="n">
         <v>0.03593587529583502</v>
@@ -2409,7 +2409,7 @@
         <v>0.003848826448934268</v>
       </c>
       <c r="I31" t="n">
-        <v>0.004973013323210912</v>
+        <v>0.004973013323210913</v>
       </c>
       <c r="J31" t="n">
         <v>0.004464987007377502</v>
@@ -2418,13 +2418,13 @@
         <v>0.00459043738696386</v>
       </c>
       <c r="L31" t="n">
-        <v>0.005079442183379286</v>
+        <v>0.005079442183379285</v>
       </c>
       <c r="M31" t="n">
-        <v>0.005088180246803167</v>
+        <v>0.005088180246803168</v>
       </c>
       <c r="N31" t="n">
-        <v>0.005577482936193968</v>
+        <v>0.005577482936193969</v>
       </c>
       <c r="O31" t="n">
         <v>0.007651893511418113</v>
@@ -2455,7 +2455,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>19.93820832675885</v>
+        <v>19.93820832675886</v>
       </c>
       <c r="D32" t="n">
         <v>18.60115972781884</v>
@@ -2473,40 +2473,40 @@
         <v>25.25621865479846</v>
       </c>
       <c r="I32" t="n">
-        <v>24.93245450968368</v>
+        <v>24.93245450968369</v>
       </c>
       <c r="J32" t="n">
         <v>21.48656101137114</v>
       </c>
       <c r="K32" t="n">
-        <v>21.86653457998643</v>
+        <v>21.86653457998644</v>
       </c>
       <c r="L32" t="n">
-        <v>26.1346226682076</v>
+        <v>26.13462266820759</v>
       </c>
       <c r="M32" t="n">
-        <v>26.36321867281375</v>
+        <v>26.36321867281374</v>
       </c>
       <c r="N32" t="n">
         <v>24.73088385068638</v>
       </c>
       <c r="O32" t="n">
-        <v>53.2915976146195</v>
+        <v>53.29159761461949</v>
       </c>
       <c r="P32" t="n">
-        <v>50.55783057115721</v>
+        <v>50.55783057115723</v>
       </c>
       <c r="Q32" t="n">
-        <v>51.02369697691538</v>
+        <v>51.02369697691539</v>
       </c>
       <c r="R32" t="n">
-        <v>75.07397051738786</v>
+        <v>75.07397051738789</v>
       </c>
       <c r="S32" t="n">
-        <v>78.126363196377</v>
+        <v>78.12636319637694</v>
       </c>
       <c r="T32" t="n">
-        <v>74.25901315828332</v>
+        <v>74.25901315828337</v>
       </c>
     </row>
     <row r="33">
@@ -2519,13 +2519,13 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>17.68637931207861</v>
+        <v>17.68637931207862</v>
       </c>
       <c r="D33" t="n">
         <v>15.70691743160874</v>
       </c>
       <c r="E33" t="n">
-        <v>19.60435263495348</v>
+        <v>19.60435263495347</v>
       </c>
       <c r="F33" t="n">
         <v>16.60027697863732</v>
@@ -2540,13 +2540,13 @@
         <v>22.82971557122241</v>
       </c>
       <c r="J33" t="n">
-        <v>21.43984896650022</v>
+        <v>21.43984896650021</v>
       </c>
       <c r="K33" t="n">
         <v>19.98986465302142</v>
       </c>
       <c r="L33" t="n">
-        <v>18.409012450934</v>
+        <v>18.40901245093401</v>
       </c>
       <c r="M33" t="n">
         <v>19.19765185377348</v>
@@ -2555,7 +2555,7 @@
         <v>22.81341672059989</v>
       </c>
       <c r="O33" t="n">
-        <v>34.28419660999059</v>
+        <v>34.2841966099906</v>
       </c>
       <c r="P33" t="n">
         <v>35.76583284950183</v>
@@ -2564,13 +2564,13 @@
         <v>30.94050442140451</v>
       </c>
       <c r="R33" t="n">
-        <v>37.77008413281228</v>
+        <v>37.77008413281229</v>
       </c>
       <c r="S33" t="n">
         <v>37.83058400153883</v>
       </c>
       <c r="T33" t="n">
-        <v>39.01559282927751</v>
+        <v>39.01559282927752</v>
       </c>
     </row>
     <row r="34">
@@ -2586,28 +2586,28 @@
         <v>0.6398987966166346</v>
       </c>
       <c r="D34" t="n">
-        <v>0.5517763762703967</v>
+        <v>0.5517763762703968</v>
       </c>
       <c r="E34" t="n">
         <v>0.5582690650600813</v>
       </c>
       <c r="F34" t="n">
-        <v>0.4923282737418817</v>
+        <v>0.4923282737418818</v>
       </c>
       <c r="G34" t="n">
         <v>0.5244004044507818</v>
       </c>
       <c r="H34" t="n">
-        <v>0.6519480739457217</v>
+        <v>0.6519480739457216</v>
       </c>
       <c r="I34" t="n">
-        <v>0.9080652564049163</v>
+        <v>0.9080652564049164</v>
       </c>
       <c r="J34" t="n">
         <v>0.7702546375485593</v>
       </c>
       <c r="K34" t="n">
-        <v>0.7728840285905739</v>
+        <v>0.7728840285905738</v>
       </c>
       <c r="L34" t="n">
         <v>0.8898760548571358</v>
@@ -2616,7 +2616,7 @@
         <v>0.8485600622825979</v>
       </c>
       <c r="N34" t="n">
-        <v>0.8368804554497222</v>
+        <v>0.8368804554497221</v>
       </c>
       <c r="O34" t="n">
         <v>1.573818366340089</v>
@@ -2634,7 +2634,7 @@
         <v>2.183655798046823</v>
       </c>
       <c r="T34" t="n">
-        <v>2.086229208040842</v>
+        <v>2.086229208040843</v>
       </c>
     </row>
     <row r="35">
@@ -2647,10 +2647,10 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.4744506766882924</v>
+        <v>0.4744506766882923</v>
       </c>
       <c r="D35" t="n">
-        <v>0.4527354524364828</v>
+        <v>0.4527354524364829</v>
       </c>
       <c r="E35" t="n">
         <v>0.4276884542506333</v>
@@ -2659,22 +2659,22 @@
         <v>0.3947914557885837</v>
       </c>
       <c r="G35" t="n">
-        <v>0.4040374514304064</v>
+        <v>0.4040374514304065</v>
       </c>
       <c r="H35" t="n">
-        <v>0.6411577324587681</v>
+        <v>0.6411577324587679</v>
       </c>
       <c r="I35" t="n">
-        <v>0.7572241846316826</v>
+        <v>0.757224184631683</v>
       </c>
       <c r="J35" t="n">
-        <v>0.6160614310605071</v>
+        <v>0.616061431060507</v>
       </c>
       <c r="K35" t="n">
-        <v>0.6343336691637602</v>
+        <v>0.6343336691637603</v>
       </c>
       <c r="L35" t="n">
-        <v>0.7061085205936739</v>
+        <v>0.7061085205936741</v>
       </c>
       <c r="M35" t="n">
         <v>0.67793136788177</v>
@@ -2683,19 +2683,19 @@
         <v>0.6602776033856695</v>
       </c>
       <c r="O35" t="n">
-        <v>1.334863705382981</v>
+        <v>1.33486370538298</v>
       </c>
       <c r="P35" t="n">
         <v>1.344099628011233</v>
       </c>
       <c r="Q35" t="n">
-        <v>1.193097405610915</v>
+        <v>1.193097405610914</v>
       </c>
       <c r="R35" t="n">
         <v>1.419414465684149</v>
       </c>
       <c r="S35" t="n">
-        <v>1.617183317231839</v>
+        <v>1.617183317231838</v>
       </c>
       <c r="T35" t="n">
         <v>1.667507511373175</v>
@@ -2720,7 +2720,7 @@
         <v>1.060101421488198</v>
       </c>
       <c r="F36" t="n">
-        <v>0.9918783317193489</v>
+        <v>0.9918783317193488</v>
       </c>
       <c r="G36" t="n">
         <v>1.005831982981693</v>
@@ -2738,7 +2738,7 @@
         <v>1.323740422266948</v>
       </c>
       <c r="L36" t="n">
-        <v>1.498336159672434</v>
+        <v>1.498336159672435</v>
       </c>
       <c r="M36" t="n">
         <v>1.406251563128973</v>
@@ -2747,7 +2747,7 @@
         <v>1.477686988087022</v>
       </c>
       <c r="O36" t="n">
-        <v>2.504438041799733</v>
+        <v>2.504438041799734</v>
       </c>
       <c r="P36" t="n">
         <v>2.702065560424375</v>
@@ -2756,7 +2756,7 @@
         <v>2.666349493641969</v>
       </c>
       <c r="R36" t="n">
-        <v>3.054031011960829</v>
+        <v>3.05403101196083</v>
       </c>
       <c r="S36" t="n">
         <v>3.36980345429629</v>
@@ -2775,40 +2775,40 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>6.0975468137594</v>
+        <v>6.097546813759397</v>
       </c>
       <c r="D37" t="n">
-        <v>5.114140316126429</v>
+        <v>5.11414031612643</v>
       </c>
       <c r="E37" t="n">
-        <v>5.699036768997355</v>
+        <v>5.699036768997354</v>
       </c>
       <c r="F37" t="n">
         <v>4.884572606433905</v>
       </c>
       <c r="G37" t="n">
-        <v>5.202316019783635</v>
+        <v>5.202316019783631</v>
       </c>
       <c r="H37" t="n">
-        <v>7.829584069477383</v>
+        <v>7.829584069477385</v>
       </c>
       <c r="I37" t="n">
-        <v>8.87764607870011</v>
+        <v>8.877646078700108</v>
       </c>
       <c r="J37" t="n">
         <v>7.821808437450235</v>
       </c>
       <c r="K37" t="n">
-        <v>8.010174998157218</v>
+        <v>8.01017499815722</v>
       </c>
       <c r="L37" t="n">
         <v>9.004934032311967</v>
       </c>
       <c r="M37" t="n">
-        <v>8.733332666759518</v>
+        <v>8.733332666759514</v>
       </c>
       <c r="N37" t="n">
-        <v>8.676850139866698</v>
+        <v>8.676850139866703</v>
       </c>
       <c r="O37" t="n">
         <v>13.35027819563612</v>
@@ -2842,7 +2842,7 @@
         <v>0.3067922242723701</v>
       </c>
       <c r="D38" t="n">
-        <v>0.2886299712415187</v>
+        <v>0.2886299712415188</v>
       </c>
       <c r="E38" t="n">
         <v>0.3075289005296661</v>
@@ -2854,7 +2854,7 @@
         <v>0.2556200834535385</v>
       </c>
       <c r="H38" t="n">
-        <v>0.2461904830187608</v>
+        <v>0.2461904830187607</v>
       </c>
       <c r="I38" t="n">
         <v>0.3625580352376093</v>
@@ -2872,22 +2872,22 @@
         <v>0.3521634432109499</v>
       </c>
       <c r="N38" t="n">
-        <v>0.3672161387547306</v>
+        <v>0.3672161387547305</v>
       </c>
       <c r="O38" t="n">
-        <v>0.5560605283839815</v>
+        <v>0.5560605283839813</v>
       </c>
       <c r="P38" t="n">
         <v>0.5979598904923213</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.5950990026010461</v>
+        <v>0.5950990026010462</v>
       </c>
       <c r="R38" t="n">
         <v>0.7000854348229415</v>
       </c>
       <c r="S38" t="n">
-        <v>0.7025020583363109</v>
+        <v>0.7025020583363111</v>
       </c>
       <c r="T38" t="n">
         <v>0.7224778093726278</v>
@@ -2948,13 +2948,13 @@
         <v>0.2706569995989109</v>
       </c>
       <c r="R39" t="n">
-        <v>0.322706471715766</v>
+        <v>0.3227064717157661</v>
       </c>
       <c r="S39" t="n">
         <v>0.2989639581600973</v>
       </c>
       <c r="T39" t="n">
-        <v>0.3385117436309611</v>
+        <v>0.338511743630961</v>
       </c>
     </row>
     <row r="40">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.09710812149561764</v>
+        <v>0.09710812149561765</v>
       </c>
       <c r="D40" t="n">
         <v>0.07378841216035686</v>
@@ -3037,7 +3037,7 @@
         <v>0.1725111199877555</v>
       </c>
       <c r="E41" t="n">
-        <v>0.1818800407645292</v>
+        <v>0.1818800407645293</v>
       </c>
       <c r="F41" t="n">
         <v>0.1721878050353202</v>
@@ -3046,10 +3046,10 @@
         <v>0.1764086078996173</v>
       </c>
       <c r="H41" t="n">
-        <v>0.3042331661468077</v>
+        <v>0.3042331661468078</v>
       </c>
       <c r="I41" t="n">
-        <v>0.2624707868585384</v>
+        <v>0.2624707868585383</v>
       </c>
       <c r="J41" t="n">
         <v>0.2227248899821783</v>
@@ -3058,7 +3058,7 @@
         <v>0.2281883559689881</v>
       </c>
       <c r="L41" t="n">
-        <v>0.3258858758460397</v>
+        <v>0.3258858758460396</v>
       </c>
       <c r="M41" t="n">
         <v>0.2619777059145987</v>
@@ -3067,7 +3067,7 @@
         <v>0.2574253572920717</v>
       </c>
       <c r="O41" t="n">
-        <v>0.4269529431590515</v>
+        <v>0.4269529431590516</v>
       </c>
       <c r="P41" t="n">
         <v>0.4496474792223005</v>
@@ -3079,10 +3079,10 @@
         <v>0.5190737316048599</v>
       </c>
       <c r="S41" t="n">
-        <v>0.49266981765383</v>
+        <v>0.4926698176538301</v>
       </c>
       <c r="T41" t="n">
-        <v>0.5045882975581967</v>
+        <v>0.5045882975581968</v>
       </c>
     </row>
     <row r="42">
@@ -3159,40 +3159,40 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0.4714266407322931</v>
+        <v>0.471426640732293</v>
       </c>
       <c r="D43" t="n">
-        <v>0.4059216546935469</v>
+        <v>0.4059216546935468</v>
       </c>
       <c r="E43" t="n">
         <v>0.444261604002967</v>
       </c>
       <c r="F43" t="n">
-        <v>0.4067174542639535</v>
+        <v>0.4067174542639537</v>
       </c>
       <c r="G43" t="n">
-        <v>0.4522850142606717</v>
+        <v>0.4522850142606716</v>
       </c>
       <c r="H43" t="n">
-        <v>0.6343909191249647</v>
+        <v>0.6343909191249645</v>
       </c>
       <c r="I43" t="n">
         <v>0.7482193099960742</v>
       </c>
       <c r="J43" t="n">
-        <v>0.5958331305680664</v>
+        <v>0.5958331305680665</v>
       </c>
       <c r="K43" t="n">
-        <v>0.6785166683249233</v>
+        <v>0.6785166683249234</v>
       </c>
       <c r="L43" t="n">
-        <v>0.775330741583978</v>
+        <v>0.7753307415839777</v>
       </c>
       <c r="M43" t="n">
-        <v>0.7358421863239855</v>
+        <v>0.7358421863239856</v>
       </c>
       <c r="N43" t="n">
-        <v>0.7576220320898086</v>
+        <v>0.7576220320898084</v>
       </c>
       <c r="O43" t="n">
         <v>1.400432323002829</v>
@@ -3210,7 +3210,7 @@
         <v>1.750946287373406</v>
       </c>
       <c r="T43" t="n">
-        <v>1.871157889002289</v>
+        <v>1.871157889002288</v>
       </c>
     </row>
     <row r="44">
@@ -3229,13 +3229,13 @@
         <v>2.594633508041459</v>
       </c>
       <c r="E44" t="n">
-        <v>2.41172968061775</v>
+        <v>2.411729680617748</v>
       </c>
       <c r="F44" t="n">
         <v>2.391574091326178</v>
       </c>
       <c r="G44" t="n">
-        <v>2.609562577499626</v>
+        <v>2.609562577499625</v>
       </c>
       <c r="H44" t="n">
         <v>2.677117644914224</v>
@@ -3250,28 +3250,28 @@
         <v>3.583910071131089</v>
       </c>
       <c r="L44" t="n">
-        <v>4.185554924020091</v>
+        <v>4.18555492402009</v>
       </c>
       <c r="M44" t="n">
-        <v>3.925163487466426</v>
+        <v>3.925163487466424</v>
       </c>
       <c r="N44" t="n">
-        <v>4.042892391814345</v>
+        <v>4.042892391814343</v>
       </c>
       <c r="O44" t="n">
         <v>7.396388802691133</v>
       </c>
       <c r="P44" t="n">
-        <v>7.806862964356108</v>
+        <v>7.806862964356106</v>
       </c>
       <c r="Q44" t="n">
-        <v>7.558398617417602</v>
+        <v>7.558398617417603</v>
       </c>
       <c r="R44" t="n">
-        <v>8.75743615301791</v>
+        <v>8.757436153017903</v>
       </c>
       <c r="S44" t="n">
-        <v>9.836762725264924</v>
+        <v>9.83676272526492</v>
       </c>
       <c r="T44" t="n">
         <v>10.21186387658839</v>
@@ -3320,7 +3320,7 @@
         <v>0.08268256667200101</v>
       </c>
       <c r="N45" t="n">
-        <v>0.08467083455298798</v>
+        <v>0.08467083455298796</v>
       </c>
       <c r="O45" t="n">
         <v>0.1652154569972128</v>
@@ -3360,7 +3360,7 @@
         <v>0.02777653222705794</v>
       </c>
       <c r="F46" t="n">
-        <v>0.02384596323141612</v>
+        <v>0.02384596323141613</v>
       </c>
       <c r="G46" t="n">
         <v>0.02305656752295559</v>
@@ -3381,13 +3381,13 @@
         <v>0.0364376929739617</v>
       </c>
       <c r="M46" t="n">
-        <v>0.03531369372634229</v>
+        <v>0.0353136937263423</v>
       </c>
       <c r="N46" t="n">
         <v>0.03908874619543986</v>
       </c>
       <c r="O46" t="n">
-        <v>0.05484461247834844</v>
+        <v>0.05484461247834846</v>
       </c>
       <c r="P46" t="n">
         <v>0.04946406316796698</v>
@@ -3402,7 +3402,7 @@
         <v>0.04808156005787596</v>
       </c>
       <c r="T46" t="n">
-        <v>0.0607141526963925</v>
+        <v>0.06071415269639251</v>
       </c>
     </row>
     <row r="47">
@@ -3445,19 +3445,19 @@
         <v>0.167798488818556</v>
       </c>
       <c r="M47" t="n">
-        <v>0.161811391562324</v>
+        <v>0.1618113915623241</v>
       </c>
       <c r="N47" t="n">
         <v>0.1739873745788708</v>
       </c>
       <c r="O47" t="n">
-        <v>0.2363514675839616</v>
+        <v>0.2363514675839615</v>
       </c>
       <c r="P47" t="n">
-        <v>0.239473226394323</v>
+        <v>0.2394732263943229</v>
       </c>
       <c r="Q47" t="n">
-        <v>0.2383106961359086</v>
+        <v>0.2383106961359085</v>
       </c>
       <c r="R47" t="n">
         <v>0.2607051141114113</v>
@@ -3485,7 +3485,7 @@
         <v>1.538614009740354</v>
       </c>
       <c r="E48" t="n">
-        <v>1.464585610619853</v>
+        <v>1.464585610619854</v>
       </c>
       <c r="F48" t="n">
         <v>1.131158304306908</v>
@@ -3494,10 +3494,10 @@
         <v>1.409010373226669</v>
       </c>
       <c r="H48" t="n">
-        <v>1.438328062980739</v>
+        <v>1.43832806298074</v>
       </c>
       <c r="I48" t="n">
-        <v>1.93062805836466</v>
+        <v>1.930628058364659</v>
       </c>
       <c r="J48" t="n">
         <v>1.605262706341932</v>
@@ -3518,16 +3518,16 @@
         <v>3.569180612299943</v>
       </c>
       <c r="P48" t="n">
-        <v>3.777795179031264</v>
+        <v>3.777795179031263</v>
       </c>
       <c r="Q48" t="n">
-        <v>3.240435673082851</v>
+        <v>3.24043567308285</v>
       </c>
       <c r="R48" t="n">
         <v>4.387061663915111</v>
       </c>
       <c r="S48" t="n">
-        <v>5.625264225328277</v>
+        <v>5.625264225328276</v>
       </c>
       <c r="T48" t="n">
         <v>5.46888966580628</v>
@@ -3607,7 +3607,7 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0.088601724316052</v>
+        <v>0.08860172431605202</v>
       </c>
       <c r="D50" t="n">
         <v>0.07462511893453966</v>
@@ -3622,7 +3622,7 @@
         <v>0.07172424205200938</v>
       </c>
       <c r="H50" t="n">
-        <v>0.09423983597398898</v>
+        <v>0.09423983597398897</v>
       </c>
       <c r="I50" t="n">
         <v>0.1141804246804437</v>
@@ -3631,7 +3631,7 @@
         <v>0.1007247446415135</v>
       </c>
       <c r="K50" t="n">
-        <v>0.09771725670103719</v>
+        <v>0.09771725670103718</v>
       </c>
       <c r="L50" t="n">
         <v>0.1269366541588031</v>
@@ -3649,16 +3649,16 @@
         <v>0.2476153526722418</v>
       </c>
       <c r="Q50" t="n">
-        <v>0.2475292447110699</v>
+        <v>0.24752924471107</v>
       </c>
       <c r="R50" t="n">
-        <v>0.3056180042771321</v>
+        <v>0.3056180042771322</v>
       </c>
       <c r="S50" t="n">
         <v>0.3356938204301642</v>
       </c>
       <c r="T50" t="n">
-        <v>0.3253991120492345</v>
+        <v>0.3253991120492344</v>
       </c>
     </row>
     <row r="51">
@@ -3698,7 +3698,7 @@
         <v>15.04962773666824</v>
       </c>
       <c r="L51" t="n">
-        <v>21.35549863107241</v>
+        <v>21.35549863107242</v>
       </c>
       <c r="M51" t="n">
         <v>20.41376999275762</v>
@@ -3707,22 +3707,22 @@
         <v>19.13479435591571</v>
       </c>
       <c r="O51" t="n">
-        <v>50.21069115862191</v>
+        <v>50.21069115862192</v>
       </c>
       <c r="P51" t="n">
-        <v>50.22166455892092</v>
+        <v>50.22166455892091</v>
       </c>
       <c r="Q51" t="n">
-        <v>50.13837317396759</v>
+        <v>50.13837317396758</v>
       </c>
       <c r="R51" t="n">
-        <v>77.26122772373189</v>
+        <v>77.26122772373186</v>
       </c>
       <c r="S51" t="n">
-        <v>83.51987220662355</v>
+        <v>83.51987220662356</v>
       </c>
       <c r="T51" t="n">
-        <v>79.43649960610364</v>
+        <v>79.43649960610361</v>
       </c>
     </row>
     <row r="52">
@@ -3738,7 +3738,7 @@
         <v>0.2072592936204653</v>
       </c>
       <c r="D52" t="n">
-        <v>0.1889226046138226</v>
+        <v>0.1889226046138225</v>
       </c>
       <c r="E52" t="n">
         <v>0.1873915193676626</v>
@@ -3747,7 +3747,7 @@
         <v>0.1871588238984855</v>
       </c>
       <c r="G52" t="n">
-        <v>0.1992711523650431</v>
+        <v>0.1992711523650432</v>
       </c>
       <c r="H52" t="n">
         <v>0.2450922242550073</v>
@@ -3756,13 +3756,13 @@
         <v>0.3301955192627085</v>
       </c>
       <c r="J52" t="n">
-        <v>0.2838122522826748</v>
+        <v>0.2838122522826749</v>
       </c>
       <c r="K52" t="n">
         <v>0.2892103106972124</v>
       </c>
       <c r="L52" t="n">
-        <v>0.3334945218023854</v>
+        <v>0.3334945218023853</v>
       </c>
       <c r="M52" t="n">
         <v>0.3265435606084486</v>
@@ -3771,19 +3771,19 @@
         <v>0.3465252200970448</v>
       </c>
       <c r="O52" t="n">
-        <v>0.5383586329485343</v>
+        <v>0.5383586329485341</v>
       </c>
       <c r="P52" t="n">
-        <v>0.5375528631004318</v>
+        <v>0.5375528631004317</v>
       </c>
       <c r="Q52" t="n">
-        <v>0.4778548293983885</v>
+        <v>0.4778548293983886</v>
       </c>
       <c r="R52" t="n">
-        <v>0.5592223663275285</v>
+        <v>0.5592223663275284</v>
       </c>
       <c r="S52" t="n">
-        <v>0.5651631022033325</v>
+        <v>0.5651631022033324</v>
       </c>
       <c r="T52" t="n">
         <v>0.6393289829530447</v>
@@ -3802,16 +3802,16 @@
         <v>0.04237688422225861</v>
       </c>
       <c r="D53" t="n">
-        <v>0.0410082721530399</v>
+        <v>0.04100827215303991</v>
       </c>
       <c r="E53" t="n">
-        <v>0.04047991478240511</v>
+        <v>0.04047991478240512</v>
       </c>
       <c r="F53" t="n">
         <v>0.03380066366290122</v>
       </c>
       <c r="G53" t="n">
-        <v>0.03527272096626635</v>
+        <v>0.03527272096626636</v>
       </c>
       <c r="H53" t="n">
         <v>0.03724214220896253</v>
@@ -3823,13 +3823,13 @@
         <v>0.03741265908861736</v>
       </c>
       <c r="K53" t="n">
-        <v>0.03967442793739957</v>
+        <v>0.03967442793739956</v>
       </c>
       <c r="L53" t="n">
         <v>0.04477268194484697</v>
       </c>
       <c r="M53" t="n">
-        <v>0.04494895685484368</v>
+        <v>0.04494895685484367</v>
       </c>
       <c r="N53" t="n">
         <v>0.0470079201435409</v>
@@ -3841,10 +3841,10 @@
         <v>0.0706783984784168</v>
       </c>
       <c r="Q53" t="n">
-        <v>0.06363342134431832</v>
+        <v>0.06363342134431831</v>
       </c>
       <c r="R53" t="n">
-        <v>0.07107560786585659</v>
+        <v>0.07107560786585661</v>
       </c>
       <c r="S53" t="n">
         <v>0.07278457453362859</v>
@@ -3863,7 +3863,7 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>20.05955599835348</v>
+        <v>20.05955599835346</v>
       </c>
       <c r="D54" t="n">
         <v>18.21345737108491</v>
@@ -3875,7 +3875,7 @@
         <v>13.6523022805223</v>
       </c>
       <c r="G54" t="n">
-        <v>15.99289045744803</v>
+        <v>15.99289045744804</v>
       </c>
       <c r="H54" t="n">
         <v>17.95847260667807</v>
@@ -3890,31 +3890,31 @@
         <v>17.05811283337796</v>
       </c>
       <c r="L54" t="n">
-        <v>18.58251270403407</v>
+        <v>18.58251270403408</v>
       </c>
       <c r="M54" t="n">
         <v>19.07413149796638</v>
       </c>
       <c r="N54" t="n">
-        <v>19.87843876472925</v>
+        <v>19.87843876472924</v>
       </c>
       <c r="O54" t="n">
-        <v>46.85941209386324</v>
+        <v>46.85941209386321</v>
       </c>
       <c r="P54" t="n">
-        <v>42.22034522318279</v>
+        <v>42.2203452231828</v>
       </c>
       <c r="Q54" t="n">
-        <v>41.99579983189017</v>
+        <v>41.99579983189019</v>
       </c>
       <c r="R54" t="n">
-        <v>62.33204504933176</v>
+        <v>62.33204504933173</v>
       </c>
       <c r="S54" t="n">
-        <v>68.0818331262815</v>
+        <v>68.08183312628151</v>
       </c>
       <c r="T54" t="n">
-        <v>67.54040679039808</v>
+        <v>67.54040679039811</v>
       </c>
     </row>
     <row r="55">
@@ -3927,7 +3927,7 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2.436010129408095</v>
+        <v>2.436010129408096</v>
       </c>
       <c r="D55" t="n">
         <v>2.110080126989678</v>
@@ -3939,46 +3939,46 @@
         <v>2.160205859747014</v>
       </c>
       <c r="G55" t="n">
-        <v>2.313606941531642</v>
+        <v>2.313606941531643</v>
       </c>
       <c r="H55" t="n">
-        <v>3.187641228870546</v>
+        <v>3.187641228870548</v>
       </c>
       <c r="I55" t="n">
         <v>3.529625996694259</v>
       </c>
       <c r="J55" t="n">
-        <v>3.022402348416372</v>
+        <v>3.022402348416371</v>
       </c>
       <c r="K55" t="n">
-        <v>3.114295236810141</v>
+        <v>3.114295236810142</v>
       </c>
       <c r="L55" t="n">
         <v>3.300267833329399</v>
       </c>
       <c r="M55" t="n">
-        <v>3.242387635362422</v>
+        <v>3.242387635362421</v>
       </c>
       <c r="N55" t="n">
-        <v>3.222441603206716</v>
+        <v>3.222441603206717</v>
       </c>
       <c r="O55" t="n">
-        <v>5.323467152298638</v>
+        <v>5.323467152298639</v>
       </c>
       <c r="P55" t="n">
         <v>5.164562010286512</v>
       </c>
       <c r="Q55" t="n">
-        <v>5.00495213308536</v>
+        <v>5.004952133085359</v>
       </c>
       <c r="R55" t="n">
-        <v>6.287370154692155</v>
+        <v>6.287370154692156</v>
       </c>
       <c r="S55" t="n">
-        <v>6.671156152445691</v>
+        <v>6.67115615244569</v>
       </c>
       <c r="T55" t="n">
-        <v>6.586134288915915</v>
+        <v>6.586134288915916</v>
       </c>
     </row>
     <row r="56">
@@ -3991,25 +3991,25 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>9.002219528609345</v>
+        <v>9.002219528609343</v>
       </c>
       <c r="D56" t="n">
-        <v>8.001800521808399</v>
+        <v>8.001800521808397</v>
       </c>
       <c r="E56" t="n">
         <v>8.310901666166226</v>
       </c>
       <c r="F56" t="n">
-        <v>9.437856918498603</v>
+        <v>9.437856918498602</v>
       </c>
       <c r="G56" t="n">
         <v>9.872087524962</v>
       </c>
       <c r="H56" t="n">
-        <v>10.03581358518788</v>
+        <v>10.03581358518787</v>
       </c>
       <c r="I56" t="n">
-        <v>16.06705389282984</v>
+        <v>16.06705389282985</v>
       </c>
       <c r="J56" t="n">
         <v>13.5974141184299</v>
@@ -4030,7 +4030,7 @@
         <v>28.09770099886684</v>
       </c>
       <c r="P56" t="n">
-        <v>27.061580558701</v>
+        <v>27.06158055870101</v>
       </c>
       <c r="Q56" t="n">
         <v>24.16732439168008</v>
@@ -4042,7 +4042,7 @@
         <v>30.78461216488866</v>
       </c>
       <c r="T56" t="n">
-        <v>33.68994732335538</v>
+        <v>33.68994732335537</v>
       </c>
     </row>
     <row r="57">
@@ -4091,13 +4091,13 @@
         <v>0.2263504382617427</v>
       </c>
       <c r="O57" t="n">
-        <v>0.3739193495611519</v>
+        <v>0.3739193495611518</v>
       </c>
       <c r="P57" t="n">
         <v>0.3450973520570018</v>
       </c>
       <c r="Q57" t="n">
-        <v>0.3871143697981334</v>
+        <v>0.3871143697981332</v>
       </c>
       <c r="R57" t="n">
         <v>0.4228791122199831</v>
@@ -4119,10 +4119,10 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0.296847937172884</v>
+        <v>0.2968479371728841</v>
       </c>
       <c r="D58" t="n">
-        <v>0.2761931299905347</v>
+        <v>0.2761931299905348</v>
       </c>
       <c r="E58" t="n">
         <v>0.2793889979108572</v>
@@ -4143,10 +4143,10 @@
         <v>0.3114356260656577</v>
       </c>
       <c r="K58" t="n">
-        <v>0.3236855746377046</v>
+        <v>0.3236855746377045</v>
       </c>
       <c r="L58" t="n">
-        <v>0.3804854728963059</v>
+        <v>0.3804854728963058</v>
       </c>
       <c r="M58" t="n">
         <v>0.3587328305993009</v>
@@ -4155,19 +4155,19 @@
         <v>0.3984779450632038</v>
       </c>
       <c r="O58" t="n">
-        <v>0.5733265193252318</v>
+        <v>0.5733265193252319</v>
       </c>
       <c r="P58" t="n">
         <v>0.5640821584039857</v>
       </c>
       <c r="Q58" t="n">
-        <v>0.5843001414103957</v>
+        <v>0.5843001414103959</v>
       </c>
       <c r="R58" t="n">
-        <v>0.6193066921669443</v>
+        <v>0.6193066921669442</v>
       </c>
       <c r="S58" t="n">
-        <v>0.6905510298714844</v>
+        <v>0.690551029871484</v>
       </c>
       <c r="T58" t="n">
         <v>0.6905632149585152</v>
@@ -4183,7 +4183,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.3665211324782944</v>
+        <v>0.3665211324782945</v>
       </c>
       <c r="D59" t="n">
         <v>0.2616070552258732</v>
@@ -4195,7 +4195,7 @@
         <v>0.2480803905613383</v>
       </c>
       <c r="G59" t="n">
-        <v>0.3395348092814299</v>
+        <v>0.3395348092814298</v>
       </c>
       <c r="H59" t="n">
         <v>0.4708188409610112</v>
@@ -4210,31 +4210,31 @@
         <v>0.4308885404772455</v>
       </c>
       <c r="L59" t="n">
-        <v>0.5075893048054004</v>
+        <v>0.5075893048054005</v>
       </c>
       <c r="M59" t="n">
         <v>0.510434753019819</v>
       </c>
       <c r="N59" t="n">
-        <v>0.4907193142019843</v>
+        <v>0.4907193142019844</v>
       </c>
       <c r="O59" t="n">
         <v>0.7753968259582847</v>
       </c>
       <c r="P59" t="n">
-        <v>0.822912262522063</v>
+        <v>0.8229122625220627</v>
       </c>
       <c r="Q59" t="n">
-        <v>0.7637496637475516</v>
+        <v>0.7637496637475515</v>
       </c>
       <c r="R59" t="n">
         <v>1.021756852630665</v>
       </c>
       <c r="S59" t="n">
-        <v>0.8358940932905663</v>
+        <v>0.8358940932905661</v>
       </c>
       <c r="T59" t="n">
-        <v>0.9534817720727392</v>
+        <v>0.9534817720727393</v>
       </c>
     </row>
     <row r="60">
@@ -4256,37 +4256,37 @@
         <v>4.170236557246419</v>
       </c>
       <c r="F60" t="n">
-        <v>4.649035203937602</v>
+        <v>4.649035203937603</v>
       </c>
       <c r="G60" t="n">
         <v>4.493469907462325</v>
       </c>
       <c r="H60" t="n">
-        <v>5.72307323837764</v>
+        <v>5.723073238377641</v>
       </c>
       <c r="I60" t="n">
-        <v>7.696409682496403</v>
+        <v>7.696409682496405</v>
       </c>
       <c r="J60" t="n">
         <v>6.780125415666087</v>
       </c>
       <c r="K60" t="n">
-        <v>6.767072585146674</v>
+        <v>6.767072585146675</v>
       </c>
       <c r="L60" t="n">
-        <v>7.603990588882166</v>
+        <v>7.603990588882167</v>
       </c>
       <c r="M60" t="n">
         <v>7.347889275251529</v>
       </c>
       <c r="N60" t="n">
-        <v>8.062993280187831</v>
+        <v>8.062993280187833</v>
       </c>
       <c r="O60" t="n">
         <v>11.23354743482509</v>
       </c>
       <c r="P60" t="n">
-        <v>10.97800730298769</v>
+        <v>10.97800730298768</v>
       </c>
       <c r="Q60" t="n">
         <v>11.52429887559248</v>
@@ -4314,7 +4314,7 @@
         <v>0.1974613923869827</v>
       </c>
       <c r="D61" t="n">
-        <v>0.2067498450747351</v>
+        <v>0.2067498450747352</v>
       </c>
       <c r="E61" t="n">
         <v>0.1592537299886222</v>
@@ -4326,7 +4326,7 @@
         <v>0.1611237707939304</v>
       </c>
       <c r="H61" t="n">
-        <v>0.213493992460945</v>
+        <v>0.2134939924609449</v>
       </c>
       <c r="I61" t="n">
         <v>0.2680977665901244</v>
@@ -4335,7 +4335,7 @@
         <v>0.2289473495324238</v>
       </c>
       <c r="K61" t="n">
-        <v>0.203477773626796</v>
+        <v>0.2034777736267959</v>
       </c>
       <c r="L61" t="n">
         <v>0.246010848986166</v>
@@ -4347,7 +4347,7 @@
         <v>0.2430093264782666</v>
       </c>
       <c r="O61" t="n">
-        <v>0.3691221454281291</v>
+        <v>0.3691221454281292</v>
       </c>
       <c r="P61" t="n">
         <v>0.4106936260497087</v>
@@ -4356,7 +4356,7 @@
         <v>0.4121127517241336</v>
       </c>
       <c r="R61" t="n">
-        <v>0.5310232600619322</v>
+        <v>0.5310232600619323</v>
       </c>
       <c r="S61" t="n">
         <v>0.5761061180904167</v>
@@ -4399,7 +4399,7 @@
         <v>0.07419645851843938</v>
       </c>
       <c r="K62" t="n">
-        <v>0.005398043655014138</v>
+        <v>0.005398043655014137</v>
       </c>
       <c r="L62" t="n">
         <v>0.0656634102161279</v>
@@ -4411,7 +4411,7 @@
         <v>0.08612387844326093</v>
       </c>
       <c r="O62" t="n">
-        <v>0.005737491980239817</v>
+        <v>0.005737491980239818</v>
       </c>
       <c r="P62" t="n">
         <v>0.06751459582641883</v>
@@ -4420,7 +4420,7 @@
         <v>0.001975814628289631</v>
       </c>
       <c r="R62" t="n">
-        <v>0.08580228255947943</v>
+        <v>0.08580228255947944</v>
       </c>
       <c r="S62" t="n">
         <v>0.00229708657276117</v>
@@ -4442,34 +4442,34 @@
         <v>7.474025755052581</v>
       </c>
       <c r="D63" t="n">
-        <v>7.359220212472147</v>
+        <v>7.359220212472146</v>
       </c>
       <c r="E63" t="n">
         <v>7.463603077570286</v>
       </c>
       <c r="F63" t="n">
-        <v>5.116440797995488</v>
+        <v>5.116440797995489</v>
       </c>
       <c r="G63" t="n">
-        <v>6.330614555531341</v>
+        <v>6.33061455553134</v>
       </c>
       <c r="H63" t="n">
-        <v>7.399709940914338</v>
+        <v>7.399709940914341</v>
       </c>
       <c r="I63" t="n">
-        <v>7.355906746750127</v>
+        <v>7.355906746750128</v>
       </c>
       <c r="J63" t="n">
-        <v>6.666940113751791</v>
+        <v>6.666940113751793</v>
       </c>
       <c r="K63" t="n">
         <v>6.585760931303153</v>
       </c>
       <c r="L63" t="n">
-        <v>5.904347755306564</v>
+        <v>5.904347755306563</v>
       </c>
       <c r="M63" t="n">
-        <v>6.168226399682598</v>
+        <v>6.168226399682597</v>
       </c>
       <c r="N63" t="n">
         <v>7.023879547269579</v>
@@ -4481,13 +4481,13 @@
         <v>7.583220679254564</v>
       </c>
       <c r="Q63" t="n">
-        <v>6.525872006185973</v>
+        <v>6.525872006185976</v>
       </c>
       <c r="R63" t="n">
         <v>8.758523229211004</v>
       </c>
       <c r="S63" t="n">
-        <v>8.831576217316705</v>
+        <v>8.8315762173167</v>
       </c>
       <c r="T63" t="n">
         <v>7.873375497297173</v>
@@ -4506,7 +4506,7 @@
         <v>0.02371593080490814</v>
       </c>
       <c r="D64" t="n">
-        <v>0.02119374383137082</v>
+        <v>0.02119374383137081</v>
       </c>
       <c r="E64" t="n">
         <v>0.02693785174172563</v>
@@ -4524,7 +4524,7 @@
         <v>0.03868091963561889</v>
       </c>
       <c r="J64" t="n">
-        <v>0.03374692911133307</v>
+        <v>0.03374692911133308</v>
       </c>
       <c r="K64" t="n">
         <v>0.03374517860172788</v>
@@ -4539,13 +4539,13 @@
         <v>0.04246970638124706</v>
       </c>
       <c r="O64" t="n">
-        <v>0.09660918369795228</v>
+        <v>0.09660918369795229</v>
       </c>
       <c r="P64" t="n">
-        <v>0.09725104860782101</v>
+        <v>0.09725104860782102</v>
       </c>
       <c r="Q64" t="n">
-        <v>0.07683679912447719</v>
+        <v>0.07683679912447718</v>
       </c>
       <c r="R64" t="n">
         <v>0.105621725757033</v>
@@ -4576,10 +4576,10 @@
         <v>13.37936240442977</v>
       </c>
       <c r="F65" t="n">
-        <v>7.327267481926659</v>
+        <v>7.327267481926658</v>
       </c>
       <c r="G65" t="n">
-        <v>7.903251992633487</v>
+        <v>7.903251992633486</v>
       </c>
       <c r="H65" t="n">
         <v>12.56555257937037</v>
@@ -4594,7 +4594,7 @@
         <v>10.77514390013631</v>
       </c>
       <c r="L65" t="n">
-        <v>12.56411846965583</v>
+        <v>12.56411846965582</v>
       </c>
       <c r="M65" t="n">
         <v>12.02445064709249</v>
@@ -4603,22 +4603,22 @@
         <v>12.28035276699541</v>
       </c>
       <c r="O65" t="n">
-        <v>21.96548053126048</v>
+        <v>21.96548053126049</v>
       </c>
       <c r="P65" t="n">
         <v>22.28538870430981</v>
       </c>
       <c r="Q65" t="n">
-        <v>19.0441899293089</v>
+        <v>19.04418992930889</v>
       </c>
       <c r="R65" t="n">
-        <v>26.72637825991754</v>
+        <v>26.72637825991753</v>
       </c>
       <c r="S65" t="n">
-        <v>24.82385990061704</v>
+        <v>24.82385990061705</v>
       </c>
       <c r="T65" t="n">
-        <v>27.11831060220081</v>
+        <v>27.11831060220082</v>
       </c>
     </row>
     <row r="66">
@@ -4634,7 +4634,7 @@
         <v>0.5521138996539522</v>
       </c>
       <c r="D66" t="n">
-        <v>0.4811467776143714</v>
+        <v>0.4811467776143715</v>
       </c>
       <c r="E66" t="n">
         <v>0.4946621175280044</v>
@@ -4646,19 +4646,19 @@
         <v>0.4975013469952058</v>
       </c>
       <c r="H66" t="n">
-        <v>0.6712072827404821</v>
+        <v>0.671207282740482</v>
       </c>
       <c r="I66" t="n">
-        <v>0.8187225122042264</v>
+        <v>0.8187225122042263</v>
       </c>
       <c r="J66" t="n">
         <v>0.6956189370261474</v>
       </c>
       <c r="K66" t="n">
-        <v>0.6963681204728589</v>
+        <v>0.696368120472859</v>
       </c>
       <c r="L66" t="n">
-        <v>0.7551802154687061</v>
+        <v>0.7551802154687058</v>
       </c>
       <c r="M66" t="n">
         <v>0.7632263851001189</v>
@@ -4682,7 +4682,7 @@
         <v>1.558043731696295</v>
       </c>
       <c r="T66" t="n">
-        <v>1.491737739410399</v>
+        <v>1.491737739410398</v>
       </c>
     </row>
     <row r="67">
@@ -4734,7 +4734,7 @@
         <v>0.03007913890541898</v>
       </c>
       <c r="P67" t="n">
-        <v>0.03244527416312854</v>
+        <v>0.03244527416312855</v>
       </c>
       <c r="Q67" t="n">
         <v>0.02894201106568465</v>
@@ -4759,22 +4759,22 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.08860435217536049</v>
+        <v>0.0886043521753605</v>
       </c>
       <c r="D68" t="n">
-        <v>0.08338357720705422</v>
+        <v>0.08338357720705421</v>
       </c>
       <c r="E68" t="n">
         <v>0.08065678586299248</v>
       </c>
       <c r="F68" t="n">
-        <v>0.07761385131896631</v>
+        <v>0.07761385131896632</v>
       </c>
       <c r="G68" t="n">
         <v>0.07705890671204459</v>
       </c>
       <c r="H68" t="n">
-        <v>0.08908526987208798</v>
+        <v>0.08908526987208794</v>
       </c>
       <c r="I68" t="n">
         <v>0.1271922780285745</v>
@@ -4847,7 +4847,7 @@
         <v>0.2144598457362292</v>
       </c>
       <c r="K69" t="n">
-        <v>0.2027601391042351</v>
+        <v>0.202760139104235</v>
       </c>
       <c r="L69" t="n">
         <v>0.2313277859288956</v>
@@ -4859,16 +4859,16 @@
         <v>0.2299358346493484</v>
       </c>
       <c r="O69" t="n">
-        <v>0.4065884659834504</v>
+        <v>0.4065884659834503</v>
       </c>
       <c r="P69" t="n">
         <v>0.4547050420758502</v>
       </c>
       <c r="Q69" t="n">
-        <v>0.4204724715982064</v>
+        <v>0.4204724715982063</v>
       </c>
       <c r="R69" t="n">
-        <v>0.6100145977516064</v>
+        <v>0.6100145977516065</v>
       </c>
       <c r="S69" t="n">
         <v>0.6777230012673703</v>
@@ -4951,22 +4951,22 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>9.565490154526326</v>
+        <v>9.56549015452633</v>
       </c>
       <c r="D71" t="n">
-        <v>9.267283128133084</v>
+        <v>9.267283128133087</v>
       </c>
       <c r="E71" t="n">
         <v>10.94191259764819</v>
       </c>
       <c r="F71" t="n">
-        <v>7.902609448048588</v>
+        <v>7.902609448048589</v>
       </c>
       <c r="G71" t="n">
         <v>8.485819198539783</v>
       </c>
       <c r="H71" t="n">
-        <v>9.325951313710423</v>
+        <v>9.325951313710425</v>
       </c>
       <c r="I71" t="n">
         <v>12.30330279162969</v>
@@ -4993,7 +4993,7 @@
         <v>14.66952582916914</v>
       </c>
       <c r="Q71" t="n">
-        <v>14.61431866093425</v>
+        <v>14.61431866093424</v>
       </c>
       <c r="R71" t="n">
         <v>17.11880592520789</v>
@@ -5024,7 +5024,7 @@
         <v>1.675966094995908</v>
       </c>
       <c r="F72" t="n">
-        <v>1.557251233588107</v>
+        <v>1.557251233588106</v>
       </c>
       <c r="G72" t="n">
         <v>1.529452863138731</v>
@@ -5036,7 +5036,7 @@
         <v>2.454007711288746</v>
       </c>
       <c r="J72" t="n">
-        <v>2.023453764190804</v>
+        <v>2.023453764190805</v>
       </c>
       <c r="K72" t="n">
         <v>2.188914594874116</v>
@@ -5057,10 +5057,10 @@
         <v>5.377060657092476</v>
       </c>
       <c r="Q72" t="n">
-        <v>4.473685519038743</v>
+        <v>4.473685519038744</v>
       </c>
       <c r="R72" t="n">
-        <v>6.379974186720847</v>
+        <v>6.379974186720848</v>
       </c>
       <c r="S72" t="n">
         <v>5.431101620617826</v>
@@ -5079,7 +5079,7 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1.357891277061867</v>
+        <v>1.357891277061868</v>
       </c>
       <c r="D73" t="n">
         <v>1.266259381382844</v>
@@ -5091,7 +5091,7 @@
         <v>1.124091596050999</v>
       </c>
       <c r="G73" t="n">
-        <v>1.192844090757993</v>
+        <v>1.192844090757994</v>
       </c>
       <c r="H73" t="n">
         <v>1.532561732471718</v>
@@ -5100,13 +5100,13 @@
         <v>1.845931244623013</v>
       </c>
       <c r="J73" t="n">
-        <v>1.498706079619441</v>
+        <v>1.49870607961944</v>
       </c>
       <c r="K73" t="n">
         <v>1.634834905344694</v>
       </c>
       <c r="L73" t="n">
-        <v>1.875126782878658</v>
+        <v>1.875126782878659</v>
       </c>
       <c r="M73" t="n">
         <v>1.824960188839064</v>
@@ -5115,10 +5115,10 @@
         <v>1.825863106501562</v>
       </c>
       <c r="O73" t="n">
-        <v>2.703419228222107</v>
+        <v>2.703419228222108</v>
       </c>
       <c r="P73" t="n">
-        <v>2.91052028118577</v>
+        <v>2.910520281185772</v>
       </c>
       <c r="Q73" t="n">
         <v>2.601805039389385</v>
@@ -5130,7 +5130,7 @@
         <v>3.140371146369914</v>
       </c>
       <c r="T73" t="n">
-        <v>3.199083838448154</v>
+        <v>3.199083838448153</v>
       </c>
     </row>
     <row r="74">
@@ -5149,7 +5149,7 @@
         <v>1.212096825122384</v>
       </c>
       <c r="E74" t="n">
-        <v>1.269278501060561</v>
+        <v>1.269278501060562</v>
       </c>
       <c r="F74" t="n">
         <v>1.034836775534601</v>
@@ -5158,7 +5158,7 @@
         <v>1.085565508241997</v>
       </c>
       <c r="H74" t="n">
-        <v>1.846020041719575</v>
+        <v>1.846020041719576</v>
       </c>
       <c r="I74" t="n">
         <v>1.781168652879039</v>
@@ -5167,7 +5167,7 @@
         <v>1.52624738973323</v>
       </c>
       <c r="K74" t="n">
-        <v>1.439845835266314</v>
+        <v>1.439845835266313</v>
       </c>
       <c r="L74" t="n">
         <v>1.672660897899988</v>
@@ -5176,13 +5176,13 @@
         <v>1.67586973319119</v>
       </c>
       <c r="N74" t="n">
-        <v>1.759391306409165</v>
+        <v>1.759391306409166</v>
       </c>
       <c r="O74" t="n">
         <v>2.981202413708604</v>
       </c>
       <c r="P74" t="n">
-        <v>2.990116388617169</v>
+        <v>2.99011638861717</v>
       </c>
       <c r="Q74" t="n">
         <v>2.598901811319934</v>
@@ -5222,7 +5222,7 @@
         <v>0.003219639722548721</v>
       </c>
       <c r="H75" t="n">
-        <v>0.00425929002556268</v>
+        <v>0.004259290025562681</v>
       </c>
       <c r="I75" t="n">
         <v>0.004456838175412667</v>
@@ -5234,19 +5234,19 @@
         <v>0.003714001496067616</v>
       </c>
       <c r="L75" t="n">
-        <v>0.004997115966820387</v>
+        <v>0.004997115966820386</v>
       </c>
       <c r="M75" t="n">
         <v>0.003986494787456262</v>
       </c>
       <c r="N75" t="n">
-        <v>0.004476151060149609</v>
+        <v>0.004476151060149608</v>
       </c>
       <c r="O75" t="n">
         <v>0.005243158880678737</v>
       </c>
       <c r="P75" t="n">
-        <v>0.005320022576707077</v>
+        <v>0.005320022576707076</v>
       </c>
       <c r="Q75" t="n">
         <v>0.006254146581994705</v>
@@ -5274,10 +5274,10 @@
         <v>1.018561139278981</v>
       </c>
       <c r="D76" t="n">
-        <v>0.8945888726264916</v>
+        <v>0.8945888726264913</v>
       </c>
       <c r="E76" t="n">
-        <v>0.8492489187710286</v>
+        <v>0.8492489187710287</v>
       </c>
       <c r="F76" t="n">
         <v>0.8277236937358575</v>
@@ -5286,7 +5286,7 @@
         <v>0.8276867994302279</v>
       </c>
       <c r="H76" t="n">
-        <v>0.7210479262269717</v>
+        <v>0.7210479262269718</v>
       </c>
       <c r="I76" t="n">
         <v>1.311242718226439</v>
@@ -5295,7 +5295,7 @@
         <v>1.112894457142302</v>
       </c>
       <c r="K76" t="n">
-        <v>1.144149575341083</v>
+        <v>1.144149575341082</v>
       </c>
       <c r="L76" t="n">
         <v>1.28495243082631</v>
@@ -5310,7 +5310,7 @@
         <v>2.074779267803994</v>
       </c>
       <c r="P76" t="n">
-        <v>2.262791692162141</v>
+        <v>2.262791692162142</v>
       </c>
       <c r="Q76" t="n">
         <v>2.174251104365404</v>
@@ -5322,7 +5322,7 @@
         <v>2.792757634222599</v>
       </c>
       <c r="T76" t="n">
-        <v>2.905019319809835</v>
+        <v>2.905019319809834</v>
       </c>
     </row>
     <row r="77">
@@ -5368,7 +5368,7 @@
         <v>0.05605225976098067</v>
       </c>
       <c r="N77" t="n">
-        <v>0.05116264471375147</v>
+        <v>0.05116264471375146</v>
       </c>
       <c r="O77" t="n">
         <v>0.09563127485471259</v>
@@ -5466,28 +5466,28 @@
         <v>0.03567012025260805</v>
       </c>
       <c r="D79" t="n">
-        <v>0.03475503153733589</v>
+        <v>0.0347550315373359</v>
       </c>
       <c r="E79" t="n">
-        <v>0.03389489950402369</v>
+        <v>0.03389489950402368</v>
       </c>
       <c r="F79" t="n">
         <v>0.03005004086549179</v>
       </c>
       <c r="G79" t="n">
-        <v>0.03005228732961067</v>
+        <v>0.03005228732961068</v>
       </c>
       <c r="H79" t="n">
         <v>0.0224562895101448</v>
       </c>
       <c r="I79" t="n">
-        <v>0.04190916760972434</v>
+        <v>0.04190916760972435</v>
       </c>
       <c r="J79" t="n">
         <v>0.03667063681036448</v>
       </c>
       <c r="K79" t="n">
-        <v>0.03891491276865704</v>
+        <v>0.03891491276865705</v>
       </c>
       <c r="L79" t="n">
         <v>0.04371732745194583</v>
@@ -5499,7 +5499,7 @@
         <v>0.04691687729155183</v>
       </c>
       <c r="O79" t="n">
-        <v>0.06758305287676421</v>
+        <v>0.06758305287676422</v>
       </c>
       <c r="P79" t="n">
         <v>0.06734807046120025</v>
@@ -5511,7 +5511,7 @@
         <v>0.07648818052484195</v>
       </c>
       <c r="S79" t="n">
-        <v>0.07569175457430552</v>
+        <v>0.07569175457430553</v>
       </c>
       <c r="T79" t="n">
         <v>0.07746444660710337</v>
@@ -5533,10 +5533,10 @@
         <v>0.08709391164304661</v>
       </c>
       <c r="E80" t="n">
-        <v>0.08973841631731856</v>
+        <v>0.08973841631731855</v>
       </c>
       <c r="F80" t="n">
-        <v>0.09397478314432429</v>
+        <v>0.09397478314432432</v>
       </c>
       <c r="G80" t="n">
         <v>0.0960544485675292</v>
@@ -5569,7 +5569,7 @@
         <v>0.3131226425413716</v>
       </c>
       <c r="Q80" t="n">
-        <v>0.325462257089227</v>
+        <v>0.3254622570892271</v>
       </c>
       <c r="R80" t="n">
         <v>0.4324860252312683</v>
@@ -5594,31 +5594,31 @@
         <v>0.05933909815392529</v>
       </c>
       <c r="D81" t="n">
-        <v>0.0574452066550057</v>
+        <v>0.05744520665500571</v>
       </c>
       <c r="E81" t="n">
-        <v>0.05839908678499228</v>
+        <v>0.05839908678499229</v>
       </c>
       <c r="F81" t="n">
         <v>0.04240415639181689</v>
       </c>
       <c r="G81" t="n">
-        <v>0.04513619269068151</v>
+        <v>0.04513619269068152</v>
       </c>
       <c r="H81" t="n">
         <v>0.05645308277290648</v>
       </c>
       <c r="I81" t="n">
-        <v>0.05996261523613866</v>
+        <v>0.05996261523613867</v>
       </c>
       <c r="J81" t="n">
-        <v>0.05164878148660472</v>
+        <v>0.05164878148660471</v>
       </c>
       <c r="K81" t="n">
-        <v>0.05421839837363157</v>
+        <v>0.05421839837363159</v>
       </c>
       <c r="L81" t="n">
-        <v>0.05970994279377561</v>
+        <v>0.0597099427937756</v>
       </c>
       <c r="M81" t="n">
         <v>0.05935430359267566</v>
@@ -5630,10 +5630,10 @@
         <v>0.09395388926363958</v>
       </c>
       <c r="P81" t="n">
-        <v>0.09981060038399732</v>
+        <v>0.09981060038399729</v>
       </c>
       <c r="Q81" t="n">
-        <v>0.07475826716118832</v>
+        <v>0.07475826716118833</v>
       </c>
       <c r="R81" t="n">
         <v>0.1077060216576888</v>
@@ -5755,10 +5755,10 @@
         <v>2.944105917051</v>
       </c>
       <c r="O83" t="n">
-        <v>5.759718135864409</v>
+        <v>5.75971813586441</v>
       </c>
       <c r="P83" t="n">
-        <v>6.161777009505935</v>
+        <v>6.161777009505934</v>
       </c>
       <c r="Q83" t="n">
         <v>5.259860609033285</v>
@@ -5810,10 +5810,10 @@
         <v>0.4533326189723015</v>
       </c>
       <c r="L84" t="n">
-        <v>0.5749132562661738</v>
+        <v>0.574913256266174</v>
       </c>
       <c r="M84" t="n">
-        <v>0.582268809677139</v>
+        <v>0.5822688096771391</v>
       </c>
       <c r="N84" t="n">
         <v>0.5583936066807866</v>
@@ -5868,7 +5868,7 @@
         <v>1.915667841593747</v>
       </c>
       <c r="J85" t="n">
-        <v>1.523997908334917</v>
+        <v>1.523997908334916</v>
       </c>
       <c r="K85" t="n">
         <v>1.712259097160009</v>
@@ -5889,7 +5889,7 @@
         <v>2.246875413497708</v>
       </c>
       <c r="Q85" t="n">
-        <v>2.289162291748106</v>
+        <v>2.289162291748105</v>
       </c>
       <c r="R85" t="n">
         <v>2.022926259040862</v>
@@ -5950,16 +5950,16 @@
         <v>0.3224537586271389</v>
       </c>
       <c r="P86" t="n">
-        <v>0.3560990120076208</v>
+        <v>0.3560990120076207</v>
       </c>
       <c r="Q86" t="n">
         <v>0.3196776778397661</v>
       </c>
       <c r="R86" t="n">
-        <v>0.4097704078995276</v>
+        <v>0.4097704078995277</v>
       </c>
       <c r="S86" t="n">
-        <v>0.4207049694510192</v>
+        <v>0.4207049694510193</v>
       </c>
       <c r="T86" t="n">
         <v>0.4153735254923928</v>
@@ -6042,7 +6042,7 @@
         <v>2.685989962690211</v>
       </c>
       <c r="D88" t="n">
-        <v>2.538532243285527</v>
+        <v>2.538532243285528</v>
       </c>
       <c r="E88" t="n">
         <v>2.908891485579277</v>
@@ -6054,13 +6054,13 @@
         <v>2.870062409272608</v>
       </c>
       <c r="H88" t="n">
-        <v>2.383001338813015</v>
+        <v>2.383001338813016</v>
       </c>
       <c r="I88" t="n">
-        <v>3.858926552936152</v>
+        <v>3.858926552936151</v>
       </c>
       <c r="J88" t="n">
-        <v>2.841505409250778</v>
+        <v>2.841505409250779</v>
       </c>
       <c r="K88" t="n">
         <v>3.198134969623061</v>
@@ -6072,7 +6072,7 @@
         <v>3.316017731220082</v>
       </c>
       <c r="N88" t="n">
-        <v>3.885575731420615</v>
+        <v>3.885575731420614</v>
       </c>
       <c r="O88" t="n">
         <v>4.943137742464316</v>
@@ -6084,13 +6084,13 @@
         <v>4.189688856175836</v>
       </c>
       <c r="R88" t="n">
-        <v>4.065838664408863</v>
+        <v>4.065838664408862</v>
       </c>
       <c r="S88" t="n">
-        <v>3.739191187375785</v>
+        <v>3.739191187375784</v>
       </c>
       <c r="T88" t="n">
-        <v>4.751524031734837</v>
+        <v>4.751524031734838</v>
       </c>
     </row>
     <row r="89">
@@ -6188,10 +6188,10 @@
         <v>0.204772633435417</v>
       </c>
       <c r="J90" t="n">
-        <v>0.1982915449839802</v>
+        <v>0.1982915449839801</v>
       </c>
       <c r="K90" t="n">
-        <v>0.1844169951137988</v>
+        <v>0.1844169951137987</v>
       </c>
       <c r="L90" t="n">
         <v>0.2064698092696904</v>
@@ -6209,13 +6209,13 @@
         <v>0.3238144553282626</v>
       </c>
       <c r="Q90" t="n">
-        <v>0.3626541629384397</v>
+        <v>0.3626541629384398</v>
       </c>
       <c r="R90" t="n">
         <v>0.3844984330313473</v>
       </c>
       <c r="S90" t="n">
-        <v>0.4584188049090527</v>
+        <v>0.4584188049090526</v>
       </c>
       <c r="T90" t="n">
         <v>0.479816283185871</v>
@@ -6243,7 +6243,7 @@
         <v>0.008640558749067722</v>
       </c>
       <c r="G91" t="n">
-        <v>0.009866529866840737</v>
+        <v>0.009866529866840735</v>
       </c>
       <c r="H91" t="n">
         <v>0.007703465989920754</v>
@@ -6252,10 +6252,10 @@
         <v>0.01204661373765589</v>
       </c>
       <c r="J91" t="n">
-        <v>0.009981556220991632</v>
+        <v>0.00998155622099163</v>
       </c>
       <c r="K91" t="n">
-        <v>0.01051261112679136</v>
+        <v>0.01051261112679135</v>
       </c>
       <c r="L91" t="n">
         <v>0.01396941527028112</v>
@@ -6270,7 +6270,7 @@
         <v>0.01870451431533712</v>
       </c>
       <c r="P91" t="n">
-        <v>0.0209732919752489</v>
+        <v>0.02097329197524889</v>
       </c>
       <c r="Q91" t="n">
         <v>0.01834703480267892</v>
@@ -6304,7 +6304,7 @@
         <v>0.07845602979168247</v>
       </c>
       <c r="F92" t="n">
-        <v>0.07100647611221503</v>
+        <v>0.07100647611221501</v>
       </c>
       <c r="G92" t="n">
         <v>0.07898176447289912</v>
@@ -6343,7 +6343,7 @@
         <v>0.2739747504793041</v>
       </c>
       <c r="S92" t="n">
-        <v>0.2402360666983507</v>
+        <v>0.2402360666983506</v>
       </c>
       <c r="T92" t="n">
         <v>0.2733600172261935</v>
@@ -6426,7 +6426,7 @@
         <v>0.4315873573546566</v>
       </c>
       <c r="D94" t="n">
-        <v>0.4431789994843116</v>
+        <v>0.4431789994843115</v>
       </c>
       <c r="E94" t="n">
         <v>0.3954804362670933</v>
@@ -6435,7 +6435,7 @@
         <v>0.3101308455065021</v>
       </c>
       <c r="G94" t="n">
-        <v>0.3552305710103722</v>
+        <v>0.3552305710103723</v>
       </c>
       <c r="H94" t="n">
         <v>0.2354046684687308</v>
@@ -6447,10 +6447,10 @@
         <v>0.3558618120515695</v>
       </c>
       <c r="K94" t="n">
-        <v>0.3998182305580216</v>
+        <v>0.3998182305580217</v>
       </c>
       <c r="L94" t="n">
-        <v>0.4546009389174043</v>
+        <v>0.4546009389174042</v>
       </c>
       <c r="M94" t="n">
         <v>0.3934110076782731</v>
@@ -6459,19 +6459,19 @@
         <v>0.4517372060521735</v>
       </c>
       <c r="O94" t="n">
-        <v>0.6649306411617704</v>
+        <v>0.6649306411617703</v>
       </c>
       <c r="P94" t="n">
         <v>0.6484568813828581</v>
       </c>
       <c r="Q94" t="n">
-        <v>0.5562359673958449</v>
+        <v>0.5562359673958448</v>
       </c>
       <c r="R94" t="n">
-        <v>0.7322264340903724</v>
+        <v>0.7322264340903725</v>
       </c>
       <c r="S94" t="n">
-        <v>0.621781769647172</v>
+        <v>0.6217817696471721</v>
       </c>
       <c r="T94" t="n">
         <v>0.6860214198591614</v>
@@ -6493,7 +6493,7 @@
         <v>0.4533992482492632</v>
       </c>
       <c r="E95" t="n">
-        <v>0.4946000472131033</v>
+        <v>0.4946000472131032</v>
       </c>
       <c r="F95" t="n">
         <v>0.3906360062656105</v>
@@ -6517,7 +6517,7 @@
         <v>0.5638320377990615</v>
       </c>
       <c r="M95" t="n">
-        <v>0.5334785492231422</v>
+        <v>0.5334785492231423</v>
       </c>
       <c r="N95" t="n">
         <v>0.5569789107032853</v>
@@ -6532,10 +6532,10 @@
         <v>0.5961390988133128</v>
       </c>
       <c r="R95" t="n">
-        <v>0.7455975000702633</v>
+        <v>0.7455975000702634</v>
       </c>
       <c r="S95" t="n">
-        <v>0.633685337909459</v>
+        <v>0.6336853379094592</v>
       </c>
       <c r="T95" t="n">
         <v>0.6727509710144711</v>
@@ -6554,25 +6554,25 @@
         <v>0.1663504701756728</v>
       </c>
       <c r="D96" t="n">
-        <v>0.1348887318010449</v>
+        <v>0.1348887318010448</v>
       </c>
       <c r="E96" t="n">
         <v>0.1323373448024628</v>
       </c>
       <c r="F96" t="n">
-        <v>0.1350146240585984</v>
+        <v>0.1350146240585985</v>
       </c>
       <c r="G96" t="n">
-        <v>0.1517260826395599</v>
+        <v>0.1517260826395598</v>
       </c>
       <c r="H96" t="n">
-        <v>0.2222941311482099</v>
+        <v>0.2222941311482098</v>
       </c>
       <c r="I96" t="n">
         <v>0.2529899056417854</v>
       </c>
       <c r="J96" t="n">
-        <v>0.2342655673948319</v>
+        <v>0.2342655673948318</v>
       </c>
       <c r="K96" t="n">
         <v>0.2364135732087782</v>
@@ -6584,7 +6584,7 @@
         <v>0.2688384950185213</v>
       </c>
       <c r="N96" t="n">
-        <v>0.2828601122862184</v>
+        <v>0.2828601122862183</v>
       </c>
       <c r="O96" t="n">
         <v>0.5207305060998288</v>
@@ -6596,7 +6596,7 @@
         <v>0.45657478758342</v>
       </c>
       <c r="R96" t="n">
-        <v>0.5965024187343203</v>
+        <v>0.5965024187343204</v>
       </c>
       <c r="S96" t="n">
         <v>0.6045335162258804</v>
@@ -6633,7 +6633,7 @@
         <v>0.02952461267833622</v>
       </c>
       <c r="I97" t="n">
-        <v>0.04806366259892491</v>
+        <v>0.0480636625989249</v>
       </c>
       <c r="J97" t="n">
         <v>0.04176296972431984</v>
@@ -6642,7 +6642,7 @@
         <v>0.04237198931489834</v>
       </c>
       <c r="L97" t="n">
-        <v>0.05996663682789351</v>
+        <v>0.05996663682789352</v>
       </c>
       <c r="M97" t="n">
         <v>0.05482763187810819</v>
@@ -6651,7 +6651,7 @@
         <v>0.0567038137452178</v>
       </c>
       <c r="O97" t="n">
-        <v>0.09357982263230565</v>
+        <v>0.09357982263230566</v>
       </c>
       <c r="P97" t="n">
         <v>0.1130803356566493</v>
@@ -6663,7 +6663,7 @@
         <v>0.1283721371705351</v>
       </c>
       <c r="S97" t="n">
-        <v>0.1339617349782584</v>
+        <v>0.1339617349782585</v>
       </c>
       <c r="T97" t="n">
         <v>0.1371763294525771</v>
@@ -6679,31 +6679,31 @@
         </is>
       </c>
       <c r="C98" t="n">
-        <v>0.06531892543288959</v>
+        <v>0.06531892543288957</v>
       </c>
       <c r="D98" t="n">
-        <v>0.06218992575321936</v>
+        <v>0.06218992575321937</v>
       </c>
       <c r="E98" t="n">
         <v>0.05996915305060359</v>
       </c>
       <c r="F98" t="n">
-        <v>0.06559046051565239</v>
+        <v>0.0655904605156524</v>
       </c>
       <c r="G98" t="n">
         <v>0.06379327013865763</v>
       </c>
       <c r="H98" t="n">
-        <v>0.07879256798772689</v>
+        <v>0.07879256798772688</v>
       </c>
       <c r="I98" t="n">
         <v>0.1045954781126142</v>
       </c>
       <c r="J98" t="n">
-        <v>0.08387857574106962</v>
+        <v>0.08387857574106959</v>
       </c>
       <c r="K98" t="n">
-        <v>0.08982486574616701</v>
+        <v>0.08982486574616702</v>
       </c>
       <c r="L98" t="n">
         <v>0.1141302357486455</v>
@@ -6730,7 +6730,7 @@
         <v>0.2210279956493577</v>
       </c>
       <c r="T98" t="n">
-        <v>0.2400608097112796</v>
+        <v>0.2400608097112797</v>
       </c>
     </row>
     <row r="99">
@@ -6743,7 +6743,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.03924334014375773</v>
+        <v>0.03924334014375772</v>
       </c>
       <c r="D99" t="n">
         <v>0.03380927103038552</v>
@@ -6755,13 +6755,13 @@
         <v>0.04217129168419489</v>
       </c>
       <c r="G99" t="n">
-        <v>0.0440196897631256</v>
+        <v>0.04401968976312561</v>
       </c>
       <c r="H99" t="n">
-        <v>0.05254094076605902</v>
+        <v>0.05254094076605903</v>
       </c>
       <c r="I99" t="n">
-        <v>0.0747091262953315</v>
+        <v>0.07470912629533148</v>
       </c>
       <c r="J99" t="n">
         <v>0.06733240946347598</v>
@@ -6816,13 +6816,13 @@
         <v>0.10628681074612</v>
       </c>
       <c r="F100" t="n">
-        <v>0.08995811277860048</v>
+        <v>0.08995811277860047</v>
       </c>
       <c r="G100" t="n">
         <v>0.088735560711039</v>
       </c>
       <c r="H100" t="n">
-        <v>0.1104927059114956</v>
+        <v>0.1104927059114957</v>
       </c>
       <c r="I100" t="n">
         <v>0.1391802220905064</v>
@@ -6843,7 +6843,7 @@
         <v>0.1423387145656542</v>
       </c>
       <c r="O100" t="n">
-        <v>0.2211778329946829</v>
+        <v>0.2211778329946828</v>
       </c>
       <c r="P100" t="n">
         <v>0.2202221022944229</v>
@@ -6858,7 +6858,7 @@
         <v>0.2482454406371755</v>
       </c>
       <c r="T100" t="n">
-        <v>0.2777215853373122</v>
+        <v>0.2777215853373123</v>
       </c>
     </row>
     <row r="101">
@@ -6874,7 +6874,7 @@
         <v>0.1758855202626069</v>
       </c>
       <c r="D101" t="n">
-        <v>0.1680631214467079</v>
+        <v>0.1680631214467078</v>
       </c>
       <c r="E101" t="n">
         <v>0.15677393430183</v>
@@ -6892,7 +6892,7 @@
         <v>0.2290820351158967</v>
       </c>
       <c r="J101" t="n">
-        <v>0.1781750935030692</v>
+        <v>0.1781750935030691</v>
       </c>
       <c r="K101" t="n">
         <v>0.2092120902187607</v>
@@ -6919,7 +6919,7 @@
         <v>0.4274906209236122</v>
       </c>
       <c r="S101" t="n">
-        <v>0.4465436722764186</v>
+        <v>0.4465436722764185</v>
       </c>
       <c r="T101" t="n">
         <v>0.4796167721842459</v>
@@ -6944,13 +6944,13 @@
         <v>1.401041974232341</v>
       </c>
       <c r="F102" t="n">
-        <v>1.185620187774639</v>
+        <v>1.185620187774638</v>
       </c>
       <c r="G102" t="n">
         <v>1.222992513548709</v>
       </c>
       <c r="H102" t="n">
-        <v>1.626012443149114</v>
+        <v>1.626012443149115</v>
       </c>
       <c r="I102" t="n">
         <v>1.916402818928399</v>
@@ -6968,7 +6968,7 @@
         <v>1.827904071538663</v>
       </c>
       <c r="N102" t="n">
-        <v>1.820918577017731</v>
+        <v>1.82091857701773</v>
       </c>
       <c r="O102" t="n">
         <v>3.415825360980258</v>
@@ -6983,7 +6983,7 @@
         <v>4.303492288392656</v>
       </c>
       <c r="S102" t="n">
-        <v>4.156584988507411</v>
+        <v>4.156584988507412</v>
       </c>
       <c r="T102" t="n">
         <v>4.32355900024305</v>
@@ -6999,10 +6999,10 @@
         </is>
       </c>
       <c r="C103" t="n">
-        <v>0.03447032355374471</v>
+        <v>0.03447032355374469</v>
       </c>
       <c r="D103" t="n">
-        <v>0.03334313565412164</v>
+        <v>0.03334313565412165</v>
       </c>
       <c r="E103" t="n">
         <v>0.03283430285606561</v>
@@ -7011,7 +7011,7 @@
         <v>0.03293331674025694</v>
       </c>
       <c r="G103" t="n">
-        <v>0.03026795626806312</v>
+        <v>0.03026795626806313</v>
       </c>
       <c r="H103" t="n">
         <v>0.04171847545225149</v>
@@ -7023,7 +7023,7 @@
         <v>0.04176760800081346</v>
       </c>
       <c r="K103" t="n">
-        <v>0.04215617076575475</v>
+        <v>0.04215617076575474</v>
       </c>
       <c r="L103" t="n">
         <v>0.04849379615433273</v>
@@ -7032,7 +7032,7 @@
         <v>0.04965816437468151</v>
       </c>
       <c r="N103" t="n">
-        <v>0.0503209612435476</v>
+        <v>0.05032096124354761</v>
       </c>
       <c r="O103" t="n">
         <v>0.07507512349838728</v>
@@ -7047,7 +7047,7 @@
         <v>0.09691409456915476</v>
       </c>
       <c r="S103" t="n">
-        <v>0.08907585487301588</v>
+        <v>0.08907585487301589</v>
       </c>
       <c r="T103" t="n">
         <v>0.08549185195936546</v>
@@ -7063,7 +7063,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>0.09044645776645846</v>
+        <v>0.09044645776645845</v>
       </c>
       <c r="D104" t="n">
         <v>0.08713636554628902</v>
@@ -7075,16 +7075,16 @@
         <v>0.08391294348413211</v>
       </c>
       <c r="G104" t="n">
-        <v>0.0867781545249897</v>
+        <v>0.08677815452498969</v>
       </c>
       <c r="H104" t="n">
-        <v>0.07192861573448958</v>
+        <v>0.07192861573448961</v>
       </c>
       <c r="I104" t="n">
         <v>0.1166249447041498</v>
       </c>
       <c r="J104" t="n">
-        <v>0.09895297046330495</v>
+        <v>0.09895297046330494</v>
       </c>
       <c r="K104" t="n">
         <v>0.1038573560059444</v>
@@ -7102,7 +7102,7 @@
         <v>0.1809315018351128</v>
       </c>
       <c r="P104" t="n">
-        <v>0.1805709191206047</v>
+        <v>0.1805709191206046</v>
       </c>
       <c r="Q104" t="n">
         <v>0.1705255841763265</v>
@@ -7130,7 +7130,7 @@
         <v>0.1027709313058061</v>
       </c>
       <c r="D105" t="n">
-        <v>0.09393807738276125</v>
+        <v>0.09393807738276126</v>
       </c>
       <c r="E105" t="n">
         <v>0.0859809181655553</v>
@@ -7139,7 +7139,7 @@
         <v>0.08509178210180697</v>
       </c>
       <c r="G105" t="n">
-        <v>0.08899277775636995</v>
+        <v>0.08899277775636993</v>
       </c>
       <c r="H105" t="n">
         <v>0.0909614702633174</v>
@@ -7163,13 +7163,13 @@
         <v>0.1381301254992021</v>
       </c>
       <c r="O105" t="n">
-        <v>0.1981927999260763</v>
+        <v>0.1981927999260762</v>
       </c>
       <c r="P105" t="n">
         <v>0.2218884171008656</v>
       </c>
       <c r="Q105" t="n">
-        <v>0.1969765872814767</v>
+        <v>0.1969765872814766</v>
       </c>
       <c r="R105" t="n">
         <v>0.2550371984085896</v>
@@ -7197,7 +7197,7 @@
         <v>0.186493448869881</v>
       </c>
       <c r="E106" t="n">
-        <v>0.2165407554716994</v>
+        <v>0.2165407554716995</v>
       </c>
       <c r="F106" t="n">
         <v>0.1744340902489996</v>
@@ -7212,7 +7212,7 @@
         <v>0.2763567556601654</v>
       </c>
       <c r="J106" t="n">
-        <v>0.2348720174067935</v>
+        <v>0.2348720174067936</v>
       </c>
       <c r="K106" t="n">
         <v>0.2353343108108224</v>
@@ -7221,7 +7221,7 @@
         <v>0.2570087429472243</v>
       </c>
       <c r="M106" t="n">
-        <v>0.2617282182589088</v>
+        <v>0.2617282182589089</v>
       </c>
       <c r="N106" t="n">
         <v>0.2794040744160127</v>
@@ -7236,7 +7236,7 @@
         <v>0.3242386714374798</v>
       </c>
       <c r="R106" t="n">
-        <v>0.4092292769400332</v>
+        <v>0.4092292769400333</v>
       </c>
       <c r="S106" t="n">
         <v>0.4236697570150296</v>
@@ -7319,31 +7319,31 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>0.5101234225125986</v>
+        <v>0.5101234225125985</v>
       </c>
       <c r="D108" t="n">
-        <v>0.4630616644207624</v>
+        <v>0.4630616644207625</v>
       </c>
       <c r="E108" t="n">
         <v>0.4783541097144987</v>
       </c>
       <c r="F108" t="n">
-        <v>0.4454307220511723</v>
+        <v>0.4454307220511722</v>
       </c>
       <c r="G108" t="n">
-        <v>0.4655193486598915</v>
+        <v>0.4655193486598914</v>
       </c>
       <c r="H108" t="n">
-        <v>0.5454465916869446</v>
+        <v>0.5454465916869444</v>
       </c>
       <c r="I108" t="n">
-        <v>0.6746552088366982</v>
+        <v>0.6746552088366979</v>
       </c>
       <c r="J108" t="n">
-        <v>0.5943378617017551</v>
+        <v>0.5943378617017552</v>
       </c>
       <c r="K108" t="n">
-        <v>0.6000502950882363</v>
+        <v>0.6000502950882358</v>
       </c>
       <c r="L108" t="n">
         <v>0.6682684462619436</v>
@@ -7352,13 +7352,13 @@
         <v>0.65904121619942</v>
       </c>
       <c r="N108" t="n">
-        <v>0.7035790012512176</v>
+        <v>0.7035790012512179</v>
       </c>
       <c r="O108" t="n">
-        <v>1.048874403837278</v>
+        <v>1.048874403837277</v>
       </c>
       <c r="P108" t="n">
-        <v>1.121128913677394</v>
+        <v>1.121128913677393</v>
       </c>
       <c r="Q108" t="n">
         <v>1.009249860728947</v>
@@ -7370,7 +7370,7 @@
         <v>1.122373491145812</v>
       </c>
       <c r="T108" t="n">
-        <v>1.271951823513564</v>
+        <v>1.271951823513563</v>
       </c>
     </row>
     <row r="109">
@@ -7511,16 +7511,16 @@
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2.428072989809201</v>
+        <v>2.428072989809202</v>
       </c>
       <c r="D111" t="n">
-        <v>2.216055675415121</v>
+        <v>2.21605567541512</v>
       </c>
       <c r="E111" t="n">
         <v>2.306171217997635</v>
       </c>
       <c r="F111" t="n">
-        <v>1.909036602409349</v>
+        <v>1.90903660240935</v>
       </c>
       <c r="G111" t="n">
         <v>2.046169947757327</v>
@@ -7529,25 +7529,25 @@
         <v>2.5330853397156</v>
       </c>
       <c r="I111" t="n">
-        <v>2.986652300048139</v>
+        <v>2.98665230004814</v>
       </c>
       <c r="J111" t="n">
         <v>2.493604682163042</v>
       </c>
       <c r="K111" t="n">
-        <v>2.608279296657932</v>
+        <v>2.608279296657933</v>
       </c>
       <c r="L111" t="n">
         <v>2.885856698444893</v>
       </c>
       <c r="M111" t="n">
-        <v>2.743713024582892</v>
+        <v>2.743713024582891</v>
       </c>
       <c r="N111" t="n">
         <v>2.783543866216574</v>
       </c>
       <c r="O111" t="n">
-        <v>4.423906837336295</v>
+        <v>4.423906837336294</v>
       </c>
       <c r="P111" t="n">
         <v>4.353706378088149</v>
@@ -7556,7 +7556,7 @@
         <v>4.206431133111779</v>
       </c>
       <c r="R111" t="n">
-        <v>4.926163053362602</v>
+        <v>4.926163053362603</v>
       </c>
       <c r="S111" t="n">
         <v>5.34815578678483</v>
@@ -7593,7 +7593,7 @@
         <v>0.1605354300777937</v>
       </c>
       <c r="I112" t="n">
-        <v>0.2082352219279814</v>
+        <v>0.2082352219279813</v>
       </c>
       <c r="J112" t="n">
         <v>0.2008420096765616</v>
@@ -7602,13 +7602,13 @@
         <v>0.1877492120083748</v>
       </c>
       <c r="L112" t="n">
-        <v>0.2106602483431022</v>
+        <v>0.2106602483431021</v>
       </c>
       <c r="M112" t="n">
-        <v>0.2223755308085498</v>
+        <v>0.2223755308085499</v>
       </c>
       <c r="N112" t="n">
-        <v>0.2170466243168654</v>
+        <v>0.2170466243168653</v>
       </c>
       <c r="O112" t="n">
         <v>0.3581196260909452</v>
@@ -7617,13 +7617,13 @@
         <v>0.330090299681918</v>
       </c>
       <c r="Q112" t="n">
-        <v>0.3695391844189431</v>
+        <v>0.3695391844189432</v>
       </c>
       <c r="R112" t="n">
         <v>0.3921391808218673</v>
       </c>
       <c r="S112" t="n">
-        <v>0.4663618835657087</v>
+        <v>0.4663618835657086</v>
       </c>
       <c r="T112" t="n">
         <v>0.487113246050039</v>
@@ -7657,10 +7657,10 @@
         <v>0.05051499283806828</v>
       </c>
       <c r="I113" t="n">
-        <v>0.04874797363411498</v>
+        <v>0.04874797363411497</v>
       </c>
       <c r="J113" t="n">
-        <v>0.04241619021635765</v>
+        <v>0.04241619021635766</v>
       </c>
       <c r="K113" t="n">
         <v>0.04037746642106956</v>
@@ -7739,19 +7739,19 @@
         <v>0.02037772726023158</v>
       </c>
       <c r="O114" t="n">
-        <v>0.03957516619987032</v>
+        <v>0.03957516619987031</v>
       </c>
       <c r="P114" t="n">
         <v>0.0452821189075249</v>
       </c>
       <c r="Q114" t="n">
-        <v>0.04274963930216525</v>
+        <v>0.04274963930216526</v>
       </c>
       <c r="R114" t="n">
         <v>0.054784359252892</v>
       </c>
       <c r="S114" t="n">
-        <v>0.04887452673400481</v>
+        <v>0.04887452673400482</v>
       </c>
       <c r="T114" t="n">
         <v>0.04519846555700199</v>
@@ -7770,7 +7770,7 @@
         <v>0.2882826782378188</v>
       </c>
       <c r="D115" t="n">
-        <v>0.2596177988731838</v>
+        <v>0.2596177988731837</v>
       </c>
       <c r="E115" t="n">
         <v>0.2643634038236027</v>
@@ -7791,7 +7791,7 @@
         <v>0.3534028506686883</v>
       </c>
       <c r="K115" t="n">
-        <v>0.3580528216494314</v>
+        <v>0.3580528216494313</v>
       </c>
       <c r="L115" t="n">
         <v>0.4480524378048032</v>
@@ -7806,16 +7806,16 @@
         <v>0.755089749759567</v>
       </c>
       <c r="P115" t="n">
-        <v>0.7370437127873852</v>
+        <v>0.7370437127873851</v>
       </c>
       <c r="Q115" t="n">
         <v>0.754051893186615</v>
       </c>
       <c r="R115" t="n">
-        <v>0.9585364727435164</v>
+        <v>0.9585364727435163</v>
       </c>
       <c r="S115" t="n">
-        <v>0.980981670757517</v>
+        <v>0.9809816707575171</v>
       </c>
       <c r="T115" t="n">
         <v>0.9485803397136801</v>
@@ -7837,7 +7837,7 @@
         <v>0.0830215154054517</v>
       </c>
       <c r="E116" t="n">
-        <v>0.0870420491802058</v>
+        <v>0.08704204918020579</v>
       </c>
       <c r="F116" t="n">
         <v>0.07737431620378392</v>
@@ -7852,7 +7852,7 @@
         <v>0.1109691571948775</v>
       </c>
       <c r="J116" t="n">
-        <v>0.09223783201410281</v>
+        <v>0.09223783201410282</v>
       </c>
       <c r="K116" t="n">
         <v>0.09876486462459264</v>
@@ -7867,13 +7867,13 @@
         <v>0.1131739929662637</v>
       </c>
       <c r="O116" t="n">
-        <v>0.1643653690071008</v>
+        <v>0.1643653690071009</v>
       </c>
       <c r="P116" t="n">
         <v>0.1650313945374654</v>
       </c>
       <c r="Q116" t="n">
-        <v>0.1583141723984232</v>
+        <v>0.1583141723984233</v>
       </c>
       <c r="R116" t="n">
         <v>0.1729668912227956</v>
@@ -7904,7 +7904,7 @@
         <v>0.04344081938351101</v>
       </c>
       <c r="F117" t="n">
-        <v>0.04909478044309922</v>
+        <v>0.04909478044309923</v>
       </c>
       <c r="G117" t="n">
         <v>0.03831377203608224</v>
@@ -7919,16 +7919,16 @@
         <v>0.07422423305444274</v>
       </c>
       <c r="K117" t="n">
-        <v>0.08741121325958065</v>
+        <v>0.08741121325958066</v>
       </c>
       <c r="L117" t="n">
         <v>0.09519134926709452</v>
       </c>
       <c r="M117" t="n">
-        <v>0.08974562578912532</v>
+        <v>0.0897456257891253</v>
       </c>
       <c r="N117" t="n">
-        <v>0.06957787094727198</v>
+        <v>0.06957787094727197</v>
       </c>
       <c r="O117" t="n">
         <v>0.184134835247514</v>
@@ -7959,7 +7959,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>0.008082196718031924</v>
+        <v>0.008082196718031922</v>
       </c>
       <c r="D118" t="n">
         <v>0.007138246939998015</v>
@@ -7971,13 +7971,13 @@
         <v>0.007373636042053182</v>
       </c>
       <c r="G118" t="n">
-        <v>0.007062712305584419</v>
+        <v>0.007062712305584418</v>
       </c>
       <c r="H118" t="n">
-        <v>0.006937971521298142</v>
+        <v>0.006937971521298141</v>
       </c>
       <c r="I118" t="n">
-        <v>0.01214372176951727</v>
+        <v>0.01214372176951726</v>
       </c>
       <c r="J118" t="n">
         <v>0.01091425179289844</v>
@@ -7995,7 +7995,7 @@
         <v>0.01306765503662449</v>
       </c>
       <c r="O118" t="n">
-        <v>0.01981490243712676</v>
+        <v>0.01981490243712675</v>
       </c>
       <c r="P118" t="n">
         <v>0.02273034247456948</v>
@@ -8035,13 +8035,13 @@
         <v>0.3117246836364982</v>
       </c>
       <c r="G119" t="n">
-        <v>0.3285180159785941</v>
+        <v>0.3285180159785942</v>
       </c>
       <c r="H119" t="n">
         <v>0.3152239826089193</v>
       </c>
       <c r="I119" t="n">
-        <v>0.5569827412216705</v>
+        <v>0.5569827412216706</v>
       </c>
       <c r="J119" t="n">
         <v>0.4755450367882136</v>
@@ -8050,22 +8050,22 @@
         <v>0.4979740274220019</v>
       </c>
       <c r="L119" t="n">
-        <v>0.5918819885997835</v>
+        <v>0.5918819885997832</v>
       </c>
       <c r="M119" t="n">
-        <v>0.5435166559557555</v>
+        <v>0.5435166559557554</v>
       </c>
       <c r="N119" t="n">
         <v>0.6030104600436827</v>
       </c>
       <c r="O119" t="n">
-        <v>0.8847711651821888</v>
+        <v>0.8847711651821889</v>
       </c>
       <c r="P119" t="n">
         <v>0.9358240422108777</v>
       </c>
       <c r="Q119" t="n">
-        <v>0.8067208686977893</v>
+        <v>0.8067208686977895</v>
       </c>
       <c r="R119" t="n">
         <v>1.013353858934098</v>
@@ -8087,28 +8087,28 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>36.39399150982232</v>
+        <v>36.39399150982233</v>
       </c>
       <c r="D120" t="n">
-        <v>31.68529641612839</v>
+        <v>31.6852964161284</v>
       </c>
       <c r="E120" t="n">
-        <v>33.57958085110323</v>
+        <v>33.57958085110324</v>
       </c>
       <c r="F120" t="n">
         <v>31.78928049077359</v>
       </c>
       <c r="G120" t="n">
-        <v>32.17709875680912</v>
+        <v>32.17709875680911</v>
       </c>
       <c r="H120" t="n">
-        <v>46.04880265413408</v>
+        <v>46.04880265413407</v>
       </c>
       <c r="I120" t="n">
-        <v>55.72667963150799</v>
+        <v>55.72667963150796</v>
       </c>
       <c r="J120" t="n">
-        <v>46.88073909451127</v>
+        <v>46.88073909451126</v>
       </c>
       <c r="K120" t="n">
         <v>46.06991967003137</v>
@@ -8117,10 +8117,10 @@
         <v>66.86606208878894</v>
       </c>
       <c r="M120" t="n">
-        <v>64.62088792362664</v>
+        <v>64.62088792362661</v>
       </c>
       <c r="N120" t="n">
-        <v>59.94315758148487</v>
+        <v>59.94315758148488</v>
       </c>
       <c r="O120" t="n">
         <v>160.0510620993676</v>
@@ -8132,7 +8132,7 @@
         <v>148.0693184042884</v>
       </c>
       <c r="R120" t="n">
-        <v>239.3649296795553</v>
+        <v>239.3649296795552</v>
       </c>
       <c r="S120" t="n">
         <v>253.2538501704686</v>
@@ -8218,7 +8218,7 @@
         <v>0.03267713971690051</v>
       </c>
       <c r="D122" t="n">
-        <v>0.03283467127118722</v>
+        <v>0.03283467127118721</v>
       </c>
       <c r="E122" t="n">
         <v>0.03143354882417708</v>
@@ -8239,7 +8239,7 @@
         <v>0.03617448979934359</v>
       </c>
       <c r="K122" t="n">
-        <v>0.03915343791191978</v>
+        <v>0.03915343791191977</v>
       </c>
       <c r="L122" t="n">
         <v>0.04065615904214659</v>
@@ -8251,7 +8251,7 @@
         <v>0.04588618740527185</v>
       </c>
       <c r="O122" t="n">
-        <v>0.05268373050962066</v>
+        <v>0.05268373050962067</v>
       </c>
       <c r="P122" t="n">
         <v>0.05704856430363184</v>
@@ -8260,13 +8260,13 @@
         <v>0.04092794229738318</v>
       </c>
       <c r="R122" t="n">
-        <v>0.0512104812345633</v>
+        <v>0.05121048123456331</v>
       </c>
       <c r="S122" t="n">
         <v>0.04549855011416423</v>
       </c>
       <c r="T122" t="n">
-        <v>0.05580483740390497</v>
+        <v>0.05580483740390496</v>
       </c>
     </row>
     <row r="123">
@@ -8282,7 +8282,7 @@
         <v>0.9399657643332729</v>
       </c>
       <c r="D123" t="n">
-        <v>0.8700527698978928</v>
+        <v>0.8700527698978929</v>
       </c>
       <c r="E123" t="n">
         <v>0.8946711411131363</v>
@@ -8291,7 +8291,7 @@
         <v>0.7474726080203441</v>
       </c>
       <c r="G123" t="n">
-        <v>0.7737824462692394</v>
+        <v>0.7737824462692393</v>
       </c>
       <c r="H123" t="n">
         <v>0.9047812536436597</v>
@@ -8321,7 +8321,7 @@
         <v>2.151554306896785</v>
       </c>
       <c r="Q123" t="n">
-        <v>2.386687071960739</v>
+        <v>2.38668707196074</v>
       </c>
       <c r="R123" t="n">
         <v>2.720748388672598</v>
@@ -8343,16 +8343,16 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>0.6172335740725087</v>
+        <v>0.6172335740725086</v>
       </c>
       <c r="D124" t="n">
         <v>0.5288835120296254</v>
       </c>
       <c r="E124" t="n">
-        <v>0.5413122800739331</v>
+        <v>0.5413122800739332</v>
       </c>
       <c r="F124" t="n">
-        <v>0.524451519869751</v>
+        <v>0.5244515198697509</v>
       </c>
       <c r="G124" t="n">
         <v>0.5934844138698824</v>
@@ -8410,7 +8410,7 @@
         <v>1.632089249198855</v>
       </c>
       <c r="D125" t="n">
-        <v>1.503509674621542</v>
+        <v>1.503509674621543</v>
       </c>
       <c r="E125" t="n">
         <v>1.374822597700631</v>
@@ -8455,7 +8455,7 @@
         <v>3.451556662640702</v>
       </c>
       <c r="S125" t="n">
-        <v>3.666081720345591</v>
+        <v>3.666081720345592</v>
       </c>
       <c r="T125" t="n">
         <v>4.442412202303252</v>
@@ -8480,7 +8480,7 @@
         <v>0.02000814786674313</v>
       </c>
       <c r="F126" t="n">
-        <v>0.02222472790999755</v>
+        <v>0.02222472790999756</v>
       </c>
       <c r="G126" t="n">
         <v>0.02327308798891593</v>
@@ -8535,13 +8535,13 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>0.1331182976813113</v>
+        <v>0.1331182976813112</v>
       </c>
       <c r="D127" t="n">
         <v>0.1174769158937752</v>
       </c>
       <c r="E127" t="n">
-        <v>0.09986227523868142</v>
+        <v>0.09986227523868139</v>
       </c>
       <c r="F127" t="n">
         <v>0.1289563043001198</v>
@@ -8574,7 +8574,7 @@
         <v>0.4301833303193309</v>
       </c>
       <c r="P127" t="n">
-        <v>0.4379004654374032</v>
+        <v>0.4379004654374033</v>
       </c>
       <c r="Q127" t="n">
         <v>0.4891456530927932</v>
@@ -8663,16 +8663,16 @@
         </is>
       </c>
       <c r="C129" t="n">
-        <v>0.08146352898443948</v>
+        <v>0.0814635289844395</v>
       </c>
       <c r="D129" t="n">
         <v>0.06766574952355979</v>
       </c>
       <c r="E129" t="n">
-        <v>0.0680378082399042</v>
+        <v>0.06803780823990419</v>
       </c>
       <c r="F129" t="n">
-        <v>0.06161345630372916</v>
+        <v>0.06161345630372915</v>
       </c>
       <c r="G129" t="n">
         <v>0.06199284811417845</v>
@@ -8708,13 +8708,13 @@
         <v>0.1965387060236291</v>
       </c>
       <c r="R129" t="n">
-        <v>0.2520648794555279</v>
+        <v>0.252064879455528</v>
       </c>
       <c r="S129" t="n">
         <v>0.2563922259951701</v>
       </c>
       <c r="T129" t="n">
-        <v>0.2403562541919454</v>
+        <v>0.2403562541919455</v>
       </c>
     </row>
     <row r="130">
@@ -8739,7 +8739,7 @@
         <v>0.04963612267915252</v>
       </c>
       <c r="G130" t="n">
-        <v>0.0501850110011607</v>
+        <v>0.05018501100116069</v>
       </c>
       <c r="H130" t="n">
         <v>0.04899177943647669</v>
@@ -8748,7 +8748,7 @@
         <v>0.07773143027355613</v>
       </c>
       <c r="J130" t="n">
-        <v>0.066698571745861</v>
+        <v>0.06669857174586101</v>
       </c>
       <c r="K130" t="n">
         <v>0.07383714990242726</v>
@@ -8800,7 +8800,7 @@
         <v>0.1254492810893389</v>
       </c>
       <c r="F131" t="n">
-        <v>0.1240649131257954</v>
+        <v>0.1240649131257953</v>
       </c>
       <c r="G131" t="n">
         <v>0.1307136115909444</v>
@@ -8827,10 +8827,10 @@
         <v>0.2132299028777321</v>
       </c>
       <c r="O131" t="n">
-        <v>0.3364997309286672</v>
+        <v>0.3364997309286671</v>
       </c>
       <c r="P131" t="n">
-        <v>0.3315956427584689</v>
+        <v>0.3315956427584688</v>
       </c>
       <c r="Q131" t="n">
         <v>0.3342315392635242</v>
@@ -8879,7 +8879,7 @@
         <v>0.09530195386705362</v>
       </c>
       <c r="K132" t="n">
-        <v>0.09868430853697009</v>
+        <v>0.09868430853697011</v>
       </c>
       <c r="L132" t="n">
         <v>0.1153296513295421</v>
@@ -8925,7 +8925,7 @@
         <v>0.9242428050988843</v>
       </c>
       <c r="E133" t="n">
-        <v>1.098011482255052</v>
+        <v>1.098011482255053</v>
       </c>
       <c r="F133" t="n">
         <v>1.19648764895406</v>
@@ -8940,7 +8940,7 @@
         <v>2.038134390304134</v>
       </c>
       <c r="J133" t="n">
-        <v>1.765012107327488</v>
+        <v>1.765012107327487</v>
       </c>
       <c r="K133" t="n">
         <v>1.704248274815274</v>
@@ -8958,13 +8958,13 @@
         <v>4.972578129277611</v>
       </c>
       <c r="P133" t="n">
-        <v>4.696528261225937</v>
+        <v>4.696528261225936</v>
       </c>
       <c r="Q133" t="n">
         <v>4.648363209790867</v>
       </c>
       <c r="R133" t="n">
-        <v>6.918524389962566</v>
+        <v>6.918524389962565</v>
       </c>
       <c r="S133" t="n">
         <v>7.004429082625482</v>
@@ -9019,7 +9019,7 @@
         <v>0.004536615683405752</v>
       </c>
       <c r="O134" t="n">
-        <v>0.004000648607851965</v>
+        <v>0.004000648607851964</v>
       </c>
       <c r="P134" t="n">
         <v>0.00588903872533335</v>
@@ -9047,7 +9047,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>0.03548847653947745</v>
+        <v>0.03548847653947744</v>
       </c>
       <c r="D135" t="n">
         <v>0.03354701671517744</v>
@@ -9062,7 +9062,7 @@
         <v>0.02459151769600704</v>
       </c>
       <c r="H135" t="n">
-        <v>0.02383153798852696</v>
+        <v>0.02383153798852695</v>
       </c>
       <c r="I135" t="n">
         <v>0.03311827583658793</v>
@@ -9086,16 +9086,16 @@
         <v>0.07073018304569616</v>
       </c>
       <c r="P135" t="n">
-        <v>0.07489858299237577</v>
+        <v>0.07489858299237576</v>
       </c>
       <c r="Q135" t="n">
         <v>0.07529819277237361</v>
       </c>
       <c r="R135" t="n">
-        <v>0.09120238656550907</v>
+        <v>0.09120238656550905</v>
       </c>
       <c r="S135" t="n">
-        <v>0.09123032222020941</v>
+        <v>0.09123032222020939</v>
       </c>
       <c r="T135" t="n">
         <v>0.09785536894197602</v>
@@ -9226,7 +9226,7 @@
         <v>0.05595093132880288</v>
       </c>
       <c r="T137" t="n">
-        <v>0.0579540795021263</v>
+        <v>0.05795407950212631</v>
       </c>
     </row>
     <row r="138">
@@ -9239,13 +9239,13 @@
         </is>
       </c>
       <c r="C138" t="n">
-        <v>0.0126749423972466</v>
+        <v>0.01267494239724661</v>
       </c>
       <c r="D138" t="n">
         <v>0.01208350221848329</v>
       </c>
       <c r="E138" t="n">
-        <v>0.008234922781882596</v>
+        <v>0.008234922781882594</v>
       </c>
       <c r="F138" t="n">
         <v>0.01200460420857307</v>
@@ -9257,10 +9257,10 @@
         <v>0.01151467317435301</v>
       </c>
       <c r="I138" t="n">
-        <v>0.01854040489564003</v>
+        <v>0.01854040489564004</v>
       </c>
       <c r="J138" t="n">
-        <v>0.01369760695128815</v>
+        <v>0.01369760695128816</v>
       </c>
       <c r="K138" t="n">
         <v>0.01577380745401011</v>
@@ -9275,7 +9275,7 @@
         <v>0.01751248503811286</v>
       </c>
       <c r="O138" t="n">
-        <v>0.02887553248198015</v>
+        <v>0.02887553248198016</v>
       </c>
       <c r="P138" t="n">
         <v>0.01840053132977065</v>
@@ -9345,7 +9345,7 @@
         <v>0.01898963170037687</v>
       </c>
       <c r="Q139" t="n">
-        <v>0.02940148822047754</v>
+        <v>0.02940148822047755</v>
       </c>
       <c r="R139" t="n">
         <v>0.01936684133885338</v>

</xml_diff>

<commit_message>
fix: add some datasets to analyse the effect of single proteins
</commit_message>
<xml_diff>
--- a/data/proteomics/membrane_size_across_compartment_Rosemary_NH4_limitation_v2.xlsx
+++ b/data/proteomics/membrane_size_across_compartment_Rosemary_NH4_limitation_v2.xlsx
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>175.2179951479612</v>
+        <v>175.2179951479614</v>
       </c>
       <c r="D2" t="n">
-        <v>160.04449738781</v>
+        <v>160.0444973878102</v>
       </c>
       <c r="E2" t="n">
         <v>168.5410689658385</v>
@@ -547,46 +547,46 @@
         <v>132.4694784504293</v>
       </c>
       <c r="G2" t="n">
-        <v>138.9107551105768</v>
+        <v>138.9107551105769</v>
       </c>
       <c r="H2" t="n">
-        <v>194.1516392720854</v>
+        <v>194.1516392720852</v>
       </c>
       <c r="I2" t="n">
-        <v>201.8798627229509</v>
+        <v>201.8798627229507</v>
       </c>
       <c r="J2" t="n">
-        <v>173.779576729269</v>
+        <v>173.7795767292694</v>
       </c>
       <c r="K2" t="n">
-        <v>176.5021655182091</v>
+        <v>176.5021655182089</v>
       </c>
       <c r="L2" t="n">
-        <v>188.392119752045</v>
+        <v>188.3921197520449</v>
       </c>
       <c r="M2" t="n">
-        <v>187.3070433279951</v>
+        <v>187.3070433279956</v>
       </c>
       <c r="N2" t="n">
-        <v>191.0380320703823</v>
+        <v>191.0380320703821</v>
       </c>
       <c r="O2" t="n">
-        <v>338.4823015571528</v>
+        <v>338.4823015571529</v>
       </c>
       <c r="P2" t="n">
-        <v>339.9679037431537</v>
+        <v>339.967903743154</v>
       </c>
       <c r="Q2" t="n">
-        <v>316.4651507008166</v>
+        <v>316.4651507008168</v>
       </c>
       <c r="R2" t="n">
-        <v>424.9728368360895</v>
+        <v>424.9728368360898</v>
       </c>
       <c r="S2" t="n">
-        <v>452.7732087518456</v>
+        <v>452.7732087518451</v>
       </c>
       <c r="T2" t="n">
-        <v>448.8247288819242</v>
+        <v>448.824728881924</v>
       </c>
     </row>
     <row r="3">
@@ -617,7 +617,7 @@
         <v>0.2667038225776687</v>
       </c>
       <c r="I3" t="n">
-        <v>0.3708542998708331</v>
+        <v>0.3708542998708332</v>
       </c>
       <c r="J3" t="n">
         <v>0.3063499146037666</v>
@@ -635,19 +635,19 @@
         <v>0.392498277599545</v>
       </c>
       <c r="O3" t="n">
-        <v>0.5003321480743245</v>
+        <v>0.5003321480743244</v>
       </c>
       <c r="P3" t="n">
         <v>0.5162502252648964</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.4992434495697613</v>
+        <v>0.4992434495697612</v>
       </c>
       <c r="R3" t="n">
-        <v>0.5783465599899491</v>
+        <v>0.578346559989949</v>
       </c>
       <c r="S3" t="n">
-        <v>0.6028096168457832</v>
+        <v>0.6028096168457833</v>
       </c>
       <c r="T3" t="n">
         <v>0.5580478351504095</v>
@@ -672,49 +672,49 @@
         <v>0.2878897626554286</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2751683226782105</v>
+        <v>0.2751683226782103</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2832108840463513</v>
+        <v>0.2832108840463514</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2900750027999564</v>
+        <v>0.2900750027999565</v>
       </c>
       <c r="I4" t="n">
-        <v>0.4146122774205823</v>
+        <v>0.4146122774205822</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3471933041993002</v>
+        <v>0.3471933041993003</v>
       </c>
       <c r="K4" t="n">
         <v>0.3290448836663721</v>
       </c>
       <c r="L4" t="n">
-        <v>0.3745999273268713</v>
+        <v>0.3745999273268714</v>
       </c>
       <c r="M4" t="n">
-        <v>0.4151547571207965</v>
+        <v>0.4151547571207964</v>
       </c>
       <c r="N4" t="n">
-        <v>0.4111555903524837</v>
+        <v>0.4111555903524836</v>
       </c>
       <c r="O4" t="n">
-        <v>0.6506676470786708</v>
+        <v>0.6506676470786709</v>
       </c>
       <c r="P4" t="n">
-        <v>0.6913160163047213</v>
+        <v>0.6913160163047212</v>
       </c>
       <c r="Q4" t="n">
         <v>0.6883910427175277</v>
       </c>
       <c r="R4" t="n">
-        <v>0.8026681630801576</v>
+        <v>0.8026681630801573</v>
       </c>
       <c r="S4" t="n">
-        <v>0.9624695034230457</v>
+        <v>0.9624695034230458</v>
       </c>
       <c r="T4" t="n">
-        <v>0.9224246385322585</v>
+        <v>0.9224246385322586</v>
       </c>
     </row>
     <row r="5">
@@ -791,25 +791,25 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>104.4945795180776</v>
+        <v>104.4945795180777</v>
       </c>
       <c r="D6" t="n">
-        <v>95.81337389222554</v>
+        <v>95.8133738922256</v>
       </c>
       <c r="E6" t="n">
-        <v>102.9450256576945</v>
+        <v>102.9450256576946</v>
       </c>
       <c r="F6" t="n">
-        <v>80.27718466102306</v>
+        <v>80.27718466102307</v>
       </c>
       <c r="G6" t="n">
-        <v>84.78600455617556</v>
+        <v>84.78600455617574</v>
       </c>
       <c r="H6" t="n">
-        <v>114.8174438999057</v>
+        <v>114.8174438999058</v>
       </c>
       <c r="I6" t="n">
-        <v>119.8186726907256</v>
+        <v>119.8186726907255</v>
       </c>
       <c r="J6" t="n">
         <v>105.0651197106895</v>
@@ -821,28 +821,28 @@
         <v>107.1511386458312</v>
       </c>
       <c r="M6" t="n">
-        <v>108.7628022245246</v>
+        <v>108.7628022245243</v>
       </c>
       <c r="N6" t="n">
-        <v>110.3052217624947</v>
+        <v>110.3052217624944</v>
       </c>
       <c r="O6" t="n">
-        <v>197.5002617175618</v>
+        <v>197.5002617175619</v>
       </c>
       <c r="P6" t="n">
         <v>199.9282717881694</v>
       </c>
       <c r="Q6" t="n">
-        <v>190.4890067392382</v>
+        <v>190.4890067392384</v>
       </c>
       <c r="R6" t="n">
-        <v>263.1742931654671</v>
+        <v>263.1742931654668</v>
       </c>
       <c r="S6" t="n">
-        <v>283.6896214537357</v>
+        <v>283.6896214537362</v>
       </c>
       <c r="T6" t="n">
-        <v>269.2484509264086</v>
+        <v>269.2484509264085</v>
       </c>
     </row>
     <row r="7">
@@ -855,58 +855,58 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>227.0895431527452</v>
+        <v>227.0895431527453</v>
       </c>
       <c r="D7" t="n">
-        <v>206.7361723285037</v>
+        <v>206.7361723285038</v>
       </c>
       <c r="E7" t="n">
         <v>213.7851497908101</v>
       </c>
       <c r="F7" t="n">
-        <v>176.2278896016975</v>
+        <v>176.2278896016976</v>
       </c>
       <c r="G7" t="n">
-        <v>186.306764487369</v>
+        <v>186.3067644873685</v>
       </c>
       <c r="H7" t="n">
-        <v>256.1877228197558</v>
+        <v>256.187722819756</v>
       </c>
       <c r="I7" t="n">
         <v>272.7578975486283</v>
       </c>
       <c r="J7" t="n">
-        <v>232.3532486181908</v>
+        <v>232.3532486181905</v>
       </c>
       <c r="K7" t="n">
-        <v>235.0706214611079</v>
+        <v>235.0706214611074</v>
       </c>
       <c r="L7" t="n">
-        <v>277.1407638493976</v>
+        <v>277.1407638493971</v>
       </c>
       <c r="M7" t="n">
-        <v>268.7329213330881</v>
+        <v>268.7329213330884</v>
       </c>
       <c r="N7" t="n">
-        <v>264.3676705543982</v>
+        <v>264.3676705543981</v>
       </c>
       <c r="O7" t="n">
-        <v>550.9705103015161</v>
+        <v>550.9705103015149</v>
       </c>
       <c r="P7" t="n">
-        <v>550.8143144862202</v>
+        <v>550.81431448622</v>
       </c>
       <c r="Q7" t="n">
-        <v>531.8284565095477</v>
+        <v>531.8284565095471</v>
       </c>
       <c r="R7" t="n">
-        <v>759.0744330364062</v>
+        <v>759.0744330364066</v>
       </c>
       <c r="S7" t="n">
         <v>797.3983425768849</v>
       </c>
       <c r="T7" t="n">
-        <v>785.7650879781918</v>
+        <v>785.7650879781927</v>
       </c>
     </row>
     <row r="8">
@@ -922,22 +922,22 @@
         <v>105.1013304776598</v>
       </c>
       <c r="D8" t="n">
-        <v>92.52612055309261</v>
+        <v>92.52612055309257</v>
       </c>
       <c r="E8" t="n">
-        <v>90.77862659703369</v>
+        <v>90.77862659703368</v>
       </c>
       <c r="F8" t="n">
-        <v>79.86886913329826</v>
+        <v>79.86886913329828</v>
       </c>
       <c r="G8" t="n">
-        <v>82.45308225254722</v>
+        <v>82.45308225254726</v>
       </c>
       <c r="H8" t="n">
         <v>124.7777434740009</v>
       </c>
       <c r="I8" t="n">
-        <v>122.9903899924766</v>
+        <v>122.9903899924765</v>
       </c>
       <c r="J8" t="n">
         <v>107.148589941707</v>
@@ -946,7 +946,7 @@
         <v>106.7000971377189</v>
       </c>
       <c r="L8" t="n">
-        <v>104.1523720523613</v>
+        <v>104.1523720523612</v>
       </c>
       <c r="M8" t="n">
         <v>106.3532786148637</v>
@@ -964,13 +964,13 @@
         <v>197.1847244190117</v>
       </c>
       <c r="R8" t="n">
-        <v>277.9700000718029</v>
+        <v>277.970000071803</v>
       </c>
       <c r="S8" t="n">
-        <v>308.7744288208421</v>
+        <v>308.774428820842</v>
       </c>
       <c r="T8" t="n">
-        <v>286.234307123676</v>
+        <v>286.2343071236759</v>
       </c>
     </row>
     <row r="9">
@@ -986,13 +986,13 @@
         <v>29.33172266429985</v>
       </c>
       <c r="D9" t="n">
-        <v>27.36723455464773</v>
+        <v>27.36723455464774</v>
       </c>
       <c r="E9" t="n">
         <v>24.98386908080797</v>
       </c>
       <c r="F9" t="n">
-        <v>21.94003474662141</v>
+        <v>21.9400347466214</v>
       </c>
       <c r="G9" t="n">
         <v>23.26167918693907</v>
@@ -1007,10 +1007,10 @@
         <v>27.93061303722451</v>
       </c>
       <c r="K9" t="n">
-        <v>28.97186337142022</v>
+        <v>28.97186337142023</v>
       </c>
       <c r="L9" t="n">
-        <v>25.98185544396455</v>
+        <v>25.98185544396454</v>
       </c>
       <c r="M9" t="n">
         <v>25.88520263437931</v>
@@ -1019,16 +1019,16 @@
         <v>22.34533065527027</v>
       </c>
       <c r="O9" t="n">
-        <v>51.92845623094193</v>
+        <v>51.92845623094195</v>
       </c>
       <c r="P9" t="n">
-        <v>49.64308423613163</v>
+        <v>49.64308423613162</v>
       </c>
       <c r="Q9" t="n">
         <v>55.17449330541861</v>
       </c>
       <c r="R9" t="n">
-        <v>78.52670899027697</v>
+        <v>78.52670899027696</v>
       </c>
       <c r="S9" t="n">
         <v>86.58033040432602</v>
@@ -1111,13 +1111,13 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>44.88391858779397</v>
+        <v>44.88391858779398</v>
       </c>
       <c r="D11" t="n">
         <v>39.38859037636782</v>
       </c>
       <c r="E11" t="n">
-        <v>34.16741458109771</v>
+        <v>34.16741458109772</v>
       </c>
       <c r="F11" t="n">
         <v>30.43728128847774</v>
@@ -1126,10 +1126,10 @@
         <v>31.0882376660685</v>
       </c>
       <c r="H11" t="n">
-        <v>57.46909296549881</v>
+        <v>57.4690929654988</v>
       </c>
       <c r="I11" t="n">
-        <v>49.48987799306352</v>
+        <v>49.48987799306351</v>
       </c>
       <c r="J11" t="n">
         <v>42.47196063001724</v>
@@ -1138,19 +1138,19 @@
         <v>43.1574878017832</v>
       </c>
       <c r="L11" t="n">
-        <v>37.93758004013362</v>
+        <v>37.93758004013361</v>
       </c>
       <c r="M11" t="n">
         <v>39.80559791450519</v>
       </c>
       <c r="N11" t="n">
-        <v>34.32068342049715</v>
+        <v>34.32068342049713</v>
       </c>
       <c r="O11" t="n">
-        <v>78.8234783950992</v>
+        <v>78.82347839509923</v>
       </c>
       <c r="P11" t="n">
-        <v>79.32295137278489</v>
+        <v>79.32295137278486</v>
       </c>
       <c r="Q11" t="n">
         <v>79.74836981076972</v>
@@ -1178,55 +1178,55 @@
         <v>12.37121765109381</v>
       </c>
       <c r="D12" t="n">
-        <v>11.22209800662489</v>
+        <v>11.22209800662488</v>
       </c>
       <c r="E12" t="n">
-        <v>10.99321760413047</v>
+        <v>10.99321760413045</v>
       </c>
       <c r="F12" t="n">
         <v>10.19134887106635</v>
       </c>
       <c r="G12" t="n">
-        <v>11.24906435751132</v>
+        <v>11.24906435751133</v>
       </c>
       <c r="H12" t="n">
-        <v>10.9816103740719</v>
+        <v>10.98161037407191</v>
       </c>
       <c r="I12" t="n">
         <v>16.70952615798391</v>
       </c>
       <c r="J12" t="n">
-        <v>14.11412453167335</v>
+        <v>14.11412453167334</v>
       </c>
       <c r="K12" t="n">
-        <v>15.01617979942495</v>
+        <v>15.01617979942496</v>
       </c>
       <c r="L12" t="n">
-        <v>17.19123215896571</v>
+        <v>17.19123215896572</v>
       </c>
       <c r="M12" t="n">
-        <v>15.9791180294715</v>
+        <v>15.97911802947151</v>
       </c>
       <c r="N12" t="n">
-        <v>17.09755670687184</v>
+        <v>17.09755670687181</v>
       </c>
       <c r="O12" t="n">
-        <v>26.60739153097735</v>
+        <v>26.60739153097736</v>
       </c>
       <c r="P12" t="n">
         <v>27.18642336678111</v>
       </c>
       <c r="Q12" t="n">
-        <v>26.08149031429907</v>
+        <v>26.08149031429904</v>
       </c>
       <c r="R12" t="n">
         <v>30.92416302141378</v>
       </c>
       <c r="S12" t="n">
-        <v>33.670930135918</v>
+        <v>33.67093013591801</v>
       </c>
       <c r="T12" t="n">
-        <v>34.87168598776994</v>
+        <v>34.87168598776996</v>
       </c>
     </row>
     <row r="13">
@@ -1266,7 +1266,7 @@
         <v>2.368011853405704</v>
       </c>
       <c r="L13" t="n">
-        <v>2.733202960559168</v>
+        <v>2.733202960559169</v>
       </c>
       <c r="M13" t="n">
         <v>2.394400220074553</v>
@@ -1284,7 +1284,7 @@
         <v>3.65493199032628</v>
       </c>
       <c r="R13" t="n">
-        <v>3.315162242105957</v>
+        <v>3.315162242105956</v>
       </c>
       <c r="S13" t="n">
         <v>3.635938154208346</v>
@@ -1303,10 +1303,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>8.834259072602094</v>
+        <v>8.834259072602102</v>
       </c>
       <c r="D14" t="n">
-        <v>8.706356576039497</v>
+        <v>8.706356576039495</v>
       </c>
       <c r="E14" t="n">
         <v>10.01133393430948</v>
@@ -1324,16 +1324,16 @@
         <v>11.28547886339388</v>
       </c>
       <c r="J14" t="n">
-        <v>9.556682794319096</v>
+        <v>9.556682794319098</v>
       </c>
       <c r="K14" t="n">
-        <v>9.332337557072192</v>
+        <v>9.332337557072194</v>
       </c>
       <c r="L14" t="n">
-        <v>10.29327721599667</v>
+        <v>10.29327721599668</v>
       </c>
       <c r="M14" t="n">
-        <v>9.736310523820674</v>
+        <v>9.736310523820675</v>
       </c>
       <c r="N14" t="n">
         <v>10.64477255047419</v>
@@ -1348,10 +1348,10 @@
         <v>13.04493835903978</v>
       </c>
       <c r="R14" t="n">
-        <v>15.62250490095467</v>
+        <v>15.62250490095466</v>
       </c>
       <c r="S14" t="n">
-        <v>16.78014764680845</v>
+        <v>16.78014764680844</v>
       </c>
       <c r="T14" t="n">
         <v>17.08224206893462</v>
@@ -1403,10 +1403,10 @@
         <v>2.219151633555639</v>
       </c>
       <c r="O15" t="n">
-        <v>3.294903038112017</v>
+        <v>3.294903038112016</v>
       </c>
       <c r="P15" t="n">
-        <v>3.877453199129756</v>
+        <v>3.877453199129755</v>
       </c>
       <c r="Q15" t="n">
         <v>3.020817851880673</v>
@@ -1449,13 +1449,13 @@
         <v>1.393755151468504</v>
       </c>
       <c r="I16" t="n">
-        <v>2.595010764878984</v>
+        <v>2.595010764878983</v>
       </c>
       <c r="J16" t="n">
         <v>2.070685091602589</v>
       </c>
       <c r="K16" t="n">
-        <v>2.30192145067995</v>
+        <v>2.301921450679949</v>
       </c>
       <c r="L16" t="n">
         <v>2.732038197793636</v>
@@ -1464,22 +1464,22 @@
         <v>2.626509281078438</v>
       </c>
       <c r="N16" t="n">
-        <v>2.793978906999192</v>
+        <v>2.793978906999193</v>
       </c>
       <c r="O16" t="n">
-        <v>3.906260789134769</v>
+        <v>3.906260789134767</v>
       </c>
       <c r="P16" t="n">
-        <v>3.83433200290798</v>
+        <v>3.834332002907979</v>
       </c>
       <c r="Q16" t="n">
-        <v>3.761919792796914</v>
+        <v>3.761919792796915</v>
       </c>
       <c r="R16" t="n">
         <v>4.253952706653428</v>
       </c>
       <c r="S16" t="n">
-        <v>4.352405875048258</v>
+        <v>4.352405875048257</v>
       </c>
       <c r="T16" t="n">
         <v>5.006679935035802</v>
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.996263537016854</v>
+        <v>1.996263537016853</v>
       </c>
       <c r="D17" t="n">
         <v>1.425017628890765</v>
@@ -1516,22 +1516,22 @@
         <v>2.495493276890576</v>
       </c>
       <c r="J17" t="n">
-        <v>2.103548345066471</v>
+        <v>2.10354834506647</v>
       </c>
       <c r="K17" t="n">
         <v>1.174927839986757</v>
       </c>
       <c r="L17" t="n">
-        <v>2.435216793887697</v>
+        <v>2.435216793887699</v>
       </c>
       <c r="M17" t="n">
-        <v>2.308095913657295</v>
+        <v>2.308095913657294</v>
       </c>
       <c r="N17" t="n">
         <v>2.353700718791571</v>
       </c>
       <c r="O17" t="n">
-        <v>1.567587789605546</v>
+        <v>1.567587789605545</v>
       </c>
       <c r="P17" t="n">
         <v>3.896234683650011</v>
@@ -1543,7 +1543,7 @@
         <v>4.294364506259151</v>
       </c>
       <c r="S17" t="n">
-        <v>4.504509553137038</v>
+        <v>4.504509553137041</v>
       </c>
       <c r="T17" t="n">
         <v>4.433210842194038</v>
@@ -1562,37 +1562,37 @@
         <v>2.697049978710424</v>
       </c>
       <c r="D18" t="n">
-        <v>2.367569589075472</v>
+        <v>2.367569589075471</v>
       </c>
       <c r="E18" t="n">
-        <v>2.251324005595606</v>
+        <v>2.251324005595607</v>
       </c>
       <c r="F18" t="n">
-        <v>2.131324671124972</v>
+        <v>2.131324671124971</v>
       </c>
       <c r="G18" t="n">
-        <v>2.354784592268258</v>
+        <v>2.354784592268257</v>
       </c>
       <c r="H18" t="n">
         <v>2.119350125178393</v>
       </c>
       <c r="I18" t="n">
-        <v>3.484594297209451</v>
+        <v>3.484594297209453</v>
       </c>
       <c r="J18" t="n">
-        <v>2.827651824938837</v>
+        <v>2.827651824938835</v>
       </c>
       <c r="K18" t="n">
         <v>3.247249273668732</v>
       </c>
       <c r="L18" t="n">
-        <v>3.585612856636331</v>
+        <v>3.585612856636333</v>
       </c>
       <c r="M18" t="n">
-        <v>3.431604030995715</v>
+        <v>3.431604030995716</v>
       </c>
       <c r="N18" t="n">
-        <v>3.538331749640752</v>
+        <v>3.538331749640751</v>
       </c>
       <c r="O18" t="n">
         <v>5.88260745659845</v>
@@ -1601,13 +1601,13 @@
         <v>5.949131763719677</v>
       </c>
       <c r="Q18" t="n">
-        <v>5.5952396878183</v>
+        <v>5.595239687818301</v>
       </c>
       <c r="R18" t="n">
-        <v>7.203289999042917</v>
+        <v>7.203289999042921</v>
       </c>
       <c r="S18" t="n">
-        <v>8.735446391515651</v>
+        <v>8.735446391515648</v>
       </c>
       <c r="T18" t="n">
         <v>9.028734150007701</v>
@@ -1623,58 +1623,58 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.394618081475112</v>
+        <v>1.394618081475111</v>
       </c>
       <c r="D19" t="n">
-        <v>1.253350678060727</v>
+        <v>1.253350678060726</v>
       </c>
       <c r="E19" t="n">
-        <v>1.282973572231972</v>
+        <v>1.282973572231973</v>
       </c>
       <c r="F19" t="n">
-        <v>1.248900046263695</v>
+        <v>1.248900046263694</v>
       </c>
       <c r="G19" t="n">
-        <v>1.29849856744257</v>
+        <v>1.298498567442569</v>
       </c>
       <c r="H19" t="n">
-        <v>1.42281766388067</v>
+        <v>1.422817663880669</v>
       </c>
       <c r="I19" t="n">
-        <v>2.007546775665482</v>
+        <v>2.007546775665483</v>
       </c>
       <c r="J19" t="n">
         <v>1.754853205190291</v>
       </c>
       <c r="K19" t="n">
-        <v>1.750947455166641</v>
+        <v>1.750947455166642</v>
       </c>
       <c r="L19" t="n">
-        <v>2.033171827422393</v>
+        <v>2.033171827422394</v>
       </c>
       <c r="M19" t="n">
-        <v>1.965292494422673</v>
+        <v>1.965292494422672</v>
       </c>
       <c r="N19" t="n">
-        <v>2.0331648319044</v>
+        <v>2.033164831904401</v>
       </c>
       <c r="O19" t="n">
         <v>3.169463582482697</v>
       </c>
       <c r="P19" t="n">
-        <v>3.224974770365974</v>
+        <v>3.224974770365975</v>
       </c>
       <c r="Q19" t="n">
-        <v>3.067936579055762</v>
+        <v>3.067936579055761</v>
       </c>
       <c r="R19" t="n">
-        <v>4.03857481995699</v>
+        <v>4.038574819956989</v>
       </c>
       <c r="S19" t="n">
         <v>4.206550290138672</v>
       </c>
       <c r="T19" t="n">
-        <v>4.182635611530208</v>
+        <v>4.182635611530206</v>
       </c>
     </row>
     <row r="20">
@@ -1687,16 +1687,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4.335169502189709</v>
+        <v>4.335169502189708</v>
       </c>
       <c r="D20" t="n">
-        <v>3.77073536509215</v>
+        <v>3.770735365092149</v>
       </c>
       <c r="E20" t="n">
-        <v>4.197775951766891</v>
+        <v>4.197775951766889</v>
       </c>
       <c r="F20" t="n">
-        <v>3.880091227827486</v>
+        <v>3.880091227827488</v>
       </c>
       <c r="G20" t="n">
         <v>4.205488963910327</v>
@@ -1705,25 +1705,25 @@
         <v>5.342620371404053</v>
       </c>
       <c r="I20" t="n">
-        <v>6.275997977658263</v>
+        <v>6.275997977658262</v>
       </c>
       <c r="J20" t="n">
-        <v>5.405688715368904</v>
+        <v>5.405688715368906</v>
       </c>
       <c r="K20" t="n">
-        <v>5.517800802999911</v>
+        <v>5.517800802999912</v>
       </c>
       <c r="L20" t="n">
-        <v>6.779577136475652</v>
+        <v>6.779577136475653</v>
       </c>
       <c r="M20" t="n">
-        <v>6.822938493470521</v>
+        <v>6.822938493470525</v>
       </c>
       <c r="N20" t="n">
-        <v>6.110590743398344</v>
+        <v>6.110590743398343</v>
       </c>
       <c r="O20" t="n">
-        <v>13.27941177386086</v>
+        <v>13.27941177386087</v>
       </c>
       <c r="P20" t="n">
         <v>12.97248403445492</v>
@@ -1735,7 +1735,7 @@
         <v>16.10289527677356</v>
       </c>
       <c r="S20" t="n">
-        <v>14.95038329562326</v>
+        <v>14.95038329562327</v>
       </c>
       <c r="T20" t="n">
         <v>17.12089756026327</v>
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.5146219466097859</v>
+        <v>0.514621946609786</v>
       </c>
       <c r="D22" t="n">
         <v>0.4638494644943265</v>
@@ -1830,10 +1830,10 @@
         <v>0.4508700182311753</v>
       </c>
       <c r="H22" t="n">
-        <v>0.4570617448494493</v>
+        <v>0.4570617448494494</v>
       </c>
       <c r="I22" t="n">
-        <v>0.6809541129387652</v>
+        <v>0.6809541129387651</v>
       </c>
       <c r="J22" t="n">
         <v>0.6050064616045413</v>
@@ -1842,7 +1842,7 @@
         <v>0.6081992116069271</v>
       </c>
       <c r="L22" t="n">
-        <v>0.7024153448399537</v>
+        <v>0.7024153448399539</v>
       </c>
       <c r="M22" t="n">
         <v>0.6831327355708822</v>
@@ -1860,7 +1860,7 @@
         <v>1.053665962554217</v>
       </c>
       <c r="R22" t="n">
-        <v>1.370383244301234</v>
+        <v>1.370383244301235</v>
       </c>
       <c r="S22" t="n">
         <v>1.378030835205638</v>
@@ -1882,13 +1882,13 @@
         <v>22.16846366169906</v>
       </c>
       <c r="D23" t="n">
-        <v>18.03371716911288</v>
+        <v>18.03371716911289</v>
       </c>
       <c r="E23" t="n">
-        <v>16.19893198143081</v>
+        <v>16.1989319814308</v>
       </c>
       <c r="F23" t="n">
-        <v>13.91132598749003</v>
+        <v>13.91132598749002</v>
       </c>
       <c r="G23" t="n">
         <v>13.28492633742167</v>
@@ -1897,10 +1897,10 @@
         <v>34.89380449301557</v>
       </c>
       <c r="I23" t="n">
-        <v>27.94648952835623</v>
+        <v>27.94648952835622</v>
       </c>
       <c r="J23" t="n">
-        <v>23.3003319385678</v>
+        <v>23.30033193856781</v>
       </c>
       <c r="K23" t="n">
         <v>21.71390926757909</v>
@@ -1915,22 +1915,22 @@
         <v>19.95199690421991</v>
       </c>
       <c r="O23" t="n">
-        <v>42.00368858747422</v>
+        <v>42.0036885874742</v>
       </c>
       <c r="P23" t="n">
         <v>43.51516009209706</v>
       </c>
       <c r="Q23" t="n">
-        <v>40.85438593492317</v>
+        <v>40.85438593492318</v>
       </c>
       <c r="R23" t="n">
-        <v>57.45436274853692</v>
+        <v>57.45436274853693</v>
       </c>
       <c r="S23" t="n">
-        <v>74.60968757876508</v>
+        <v>74.60968757876509</v>
       </c>
       <c r="T23" t="n">
-        <v>61.97072864975438</v>
+        <v>61.97072864975439</v>
       </c>
     </row>
     <row r="24">
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.0970549600016119</v>
+        <v>0.09705496000161189</v>
       </c>
       <c r="D24" t="n">
         <v>0.1000493163611742</v>
@@ -1955,7 +1955,7 @@
         <v>0.1041190861322172</v>
       </c>
       <c r="G24" t="n">
-        <v>0.0969538273474753</v>
+        <v>0.09695382734747529</v>
       </c>
       <c r="H24" t="n">
         <v>0.1350705664009529</v>
@@ -1979,10 +1979,10 @@
         <v>0.1718320453756577</v>
       </c>
       <c r="O24" t="n">
-        <v>0.3246791236204478</v>
+        <v>0.3246791236204479</v>
       </c>
       <c r="P24" t="n">
-        <v>0.3210695322001895</v>
+        <v>0.3210695322001896</v>
       </c>
       <c r="Q24" t="n">
         <v>0.3242406935439865</v>
@@ -2043,13 +2043,13 @@
         <v>1.780468192537126</v>
       </c>
       <c r="O25" t="n">
-        <v>3.103087807084307</v>
+        <v>3.103087807084308</v>
       </c>
       <c r="P25" t="n">
         <v>3.087807269100277</v>
       </c>
       <c r="Q25" t="n">
-        <v>2.817306935382981</v>
+        <v>2.817306935382982</v>
       </c>
       <c r="R25" t="n">
         <v>3.470960661583677</v>
@@ -2101,13 +2101,13 @@
         <v>2.056544337895579</v>
       </c>
       <c r="M26" t="n">
-        <v>1.904726755139886</v>
+        <v>1.904726755139885</v>
       </c>
       <c r="N26" t="n">
         <v>2.004021483978576</v>
       </c>
       <c r="O26" t="n">
-        <v>2.872239639466172</v>
+        <v>2.872239639466171</v>
       </c>
       <c r="P26" t="n">
         <v>2.766895871208599</v>
@@ -2119,7 +2119,7 @@
         <v>3.238436963249196</v>
       </c>
       <c r="S26" t="n">
-        <v>3.451649865653488</v>
+        <v>3.451649865653489</v>
       </c>
       <c r="T26" t="n">
         <v>3.984225577084572</v>
@@ -2135,13 +2135,13 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>9.404548614880595</v>
+        <v>9.404548614880596</v>
       </c>
       <c r="D27" t="n">
-        <v>8.08167272871952</v>
+        <v>8.081672728719516</v>
       </c>
       <c r="E27" t="n">
-        <v>8.826005460992478</v>
+        <v>8.826005460992477</v>
       </c>
       <c r="F27" t="n">
         <v>8.461035997767327</v>
@@ -2150,13 +2150,13 @@
         <v>8.483129903838181</v>
       </c>
       <c r="H27" t="n">
-        <v>11.64739412202548</v>
+        <v>11.64739412202549</v>
       </c>
       <c r="I27" t="n">
         <v>13.82307798420801</v>
       </c>
       <c r="J27" t="n">
-        <v>11.70090422757791</v>
+        <v>11.7009042275779</v>
       </c>
       <c r="K27" t="n">
         <v>11.38292990215321</v>
@@ -2174,19 +2174,19 @@
         <v>36.04669631674182</v>
       </c>
       <c r="P27" t="n">
-        <v>38.36051604651185</v>
+        <v>38.36051604651183</v>
       </c>
       <c r="Q27" t="n">
-        <v>35.55832547782604</v>
+        <v>35.55832547782603</v>
       </c>
       <c r="R27" t="n">
-        <v>54.29853086694438</v>
+        <v>54.2985308669444</v>
       </c>
       <c r="S27" t="n">
-        <v>59.24178136349355</v>
+        <v>59.24178136349357</v>
       </c>
       <c r="T27" t="n">
-        <v>57.5753492043481</v>
+        <v>57.57534920434811</v>
       </c>
     </row>
     <row r="28">
@@ -2199,7 +2199,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.2966098180711588</v>
+        <v>0.2966098180711587</v>
       </c>
       <c r="D28" t="n">
         <v>0.2735237095728636</v>
@@ -2208,19 +2208,19 @@
         <v>0.3179767014571709</v>
       </c>
       <c r="F28" t="n">
-        <v>0.2737142751873577</v>
+        <v>0.2737142751873576</v>
       </c>
       <c r="G28" t="n">
         <v>0.2819010151367157</v>
       </c>
       <c r="H28" t="n">
-        <v>0.2847564985576654</v>
+        <v>0.2847564985576653</v>
       </c>
       <c r="I28" t="n">
         <v>0.3880931541475547</v>
       </c>
       <c r="J28" t="n">
-        <v>0.332583556432455</v>
+        <v>0.3325835564324551</v>
       </c>
       <c r="K28" t="n">
         <v>0.339136010933317</v>
@@ -2235,19 +2235,19 @@
         <v>0.3851934035328792</v>
       </c>
       <c r="O28" t="n">
-        <v>0.6566030779648064</v>
+        <v>0.6566030779648065</v>
       </c>
       <c r="P28" t="n">
-        <v>0.6184885068650192</v>
+        <v>0.6184885068650191</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.6013531913225518</v>
+        <v>0.601353191322552</v>
       </c>
       <c r="R28" t="n">
         <v>0.7095695368170815</v>
       </c>
       <c r="S28" t="n">
-        <v>0.72383611022419</v>
+        <v>0.7238361102241899</v>
       </c>
       <c r="T28" t="n">
         <v>0.7692599133981047</v>
@@ -2278,16 +2278,16 @@
         <v>13.58016626048591</v>
       </c>
       <c r="H29" t="n">
-        <v>11.25688282684747</v>
+        <v>11.25688282684746</v>
       </c>
       <c r="I29" t="n">
         <v>16.07264247295188</v>
       </c>
       <c r="J29" t="n">
-        <v>13.59756969944153</v>
+        <v>13.59756969944152</v>
       </c>
       <c r="K29" t="n">
-        <v>14.88343703118447</v>
+        <v>14.88343703118448</v>
       </c>
       <c r="L29" t="n">
         <v>16.56965801981578</v>
@@ -2296,25 +2296,25 @@
         <v>15.58310716611139</v>
       </c>
       <c r="N29" t="n">
-        <v>16.85428648851559</v>
+        <v>16.8542864885156</v>
       </c>
       <c r="O29" t="n">
-        <v>24.25873607835888</v>
+        <v>24.2587360783589</v>
       </c>
       <c r="P29" t="n">
         <v>24.71870188120023</v>
       </c>
       <c r="Q29" t="n">
-        <v>23.55321816763553</v>
+        <v>23.55321816763552</v>
       </c>
       <c r="R29" t="n">
-        <v>27.30672319240507</v>
+        <v>27.30672319240506</v>
       </c>
       <c r="S29" t="n">
-        <v>27.95490921811761</v>
+        <v>27.95490921811762</v>
       </c>
       <c r="T29" t="n">
-        <v>30.87203135452536</v>
+        <v>30.87203135452537</v>
       </c>
     </row>
     <row r="30">
@@ -2333,7 +2333,7 @@
         <v>0.02072222810167829</v>
       </c>
       <c r="E30" t="n">
-        <v>0.02320293886576925</v>
+        <v>0.02320293886576924</v>
       </c>
       <c r="F30" t="n">
         <v>0.01831735455400737</v>
@@ -2348,7 +2348,7 @@
         <v>0.02475228135865733</v>
       </c>
       <c r="J30" t="n">
-        <v>0.02296699809063352</v>
+        <v>0.02296699809063353</v>
       </c>
       <c r="K30" t="n">
         <v>0.01986648274287118</v>
@@ -2357,13 +2357,13 @@
         <v>0.02220517251655242</v>
       </c>
       <c r="M30" t="n">
-        <v>0.02516978813192495</v>
+        <v>0.02516978813192496</v>
       </c>
       <c r="N30" t="n">
         <v>0.02413512281717074</v>
       </c>
       <c r="O30" t="n">
-        <v>0.03954050305358027</v>
+        <v>0.03954050305358028</v>
       </c>
       <c r="P30" t="n">
         <v>0.04147805068852546</v>
@@ -2372,7 +2372,7 @@
         <v>0.03549163257831871</v>
       </c>
       <c r="R30" t="n">
-        <v>0.05375065546140827</v>
+        <v>0.05375065546140826</v>
       </c>
       <c r="S30" t="n">
         <v>0.03593587529583502</v>
@@ -2464,22 +2464,22 @@
         <v>24.53759922338814</v>
       </c>
       <c r="F32" t="n">
-        <v>16.48422927123905</v>
+        <v>16.48422927123904</v>
       </c>
       <c r="G32" t="n">
-        <v>17.4686910856083</v>
+        <v>17.46869108560829</v>
       </c>
       <c r="H32" t="n">
-        <v>25.25621865479845</v>
+        <v>25.25621865479847</v>
       </c>
       <c r="I32" t="n">
-        <v>24.93245450968369</v>
+        <v>24.93245450968368</v>
       </c>
       <c r="J32" t="n">
-        <v>21.48656101137113</v>
+        <v>21.48656101137114</v>
       </c>
       <c r="K32" t="n">
-        <v>21.86653457998644</v>
+        <v>21.86653457998643</v>
       </c>
       <c r="L32" t="n">
         <v>26.13462266820759</v>
@@ -2488,25 +2488,25 @@
         <v>26.36321867281373</v>
       </c>
       <c r="N32" t="n">
-        <v>24.73088385068638</v>
+        <v>24.73088385068639</v>
       </c>
       <c r="O32" t="n">
-        <v>53.29159761461952</v>
+        <v>53.2915976146195</v>
       </c>
       <c r="P32" t="n">
         <v>50.55783057115722</v>
       </c>
       <c r="Q32" t="n">
-        <v>51.02369697691538</v>
+        <v>51.0236969769154</v>
       </c>
       <c r="R32" t="n">
-        <v>75.07397051738789</v>
+        <v>75.07397051738791</v>
       </c>
       <c r="S32" t="n">
-        <v>78.126363196377</v>
+        <v>78.12636319637697</v>
       </c>
       <c r="T32" t="n">
-        <v>74.2590131582833</v>
+        <v>74.25901315828335</v>
       </c>
     </row>
     <row r="33">
@@ -2519,16 +2519,16 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>17.68637931207861</v>
+        <v>17.68637931207862</v>
       </c>
       <c r="D33" t="n">
         <v>15.70691743160874</v>
       </c>
       <c r="E33" t="n">
-        <v>19.60435263495348</v>
+        <v>19.60435263495347</v>
       </c>
       <c r="F33" t="n">
-        <v>16.60027697863732</v>
+        <v>16.60027697863731</v>
       </c>
       <c r="G33" t="n">
         <v>17.20854420664552</v>
@@ -2540,10 +2540,10 @@
         <v>22.82971557122241</v>
       </c>
       <c r="J33" t="n">
-        <v>21.43984896650021</v>
+        <v>21.43984896650022</v>
       </c>
       <c r="K33" t="n">
-        <v>19.98986465302143</v>
+        <v>19.98986465302142</v>
       </c>
       <c r="L33" t="n">
         <v>18.40901245093401</v>
@@ -2555,19 +2555,19 @@
         <v>22.81341672059988</v>
       </c>
       <c r="O33" t="n">
-        <v>34.28419660999059</v>
+        <v>34.28419660999061</v>
       </c>
       <c r="P33" t="n">
         <v>35.76583284950183</v>
       </c>
       <c r="Q33" t="n">
-        <v>30.9405044214045</v>
+        <v>30.94050442140451</v>
       </c>
       <c r="R33" t="n">
-        <v>37.77008413281229</v>
+        <v>37.77008413281227</v>
       </c>
       <c r="S33" t="n">
-        <v>37.83058400153881</v>
+        <v>37.83058400153884</v>
       </c>
       <c r="T33" t="n">
         <v>39.01559282927752</v>
@@ -2583,7 +2583,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0.6398987966166348</v>
+        <v>0.6398987966166346</v>
       </c>
       <c r="D34" t="n">
         <v>0.5517763762703966</v>
@@ -2598,25 +2598,25 @@
         <v>0.524400404450782</v>
       </c>
       <c r="H34" t="n">
-        <v>0.6519480739457215</v>
+        <v>0.6519480739457217</v>
       </c>
       <c r="I34" t="n">
-        <v>0.9080652564049163</v>
+        <v>0.9080652564049165</v>
       </c>
       <c r="J34" t="n">
-        <v>0.7702546375485594</v>
+        <v>0.7702546375485588</v>
       </c>
       <c r="K34" t="n">
-        <v>0.7728840285905738</v>
+        <v>0.7728840285905741</v>
       </c>
       <c r="L34" t="n">
-        <v>0.8898760548571356</v>
+        <v>0.8898760548571358</v>
       </c>
       <c r="M34" t="n">
         <v>0.8485600622825981</v>
       </c>
       <c r="N34" t="n">
-        <v>0.8368804554497221</v>
+        <v>0.8368804554497222</v>
       </c>
       <c r="O34" t="n">
         <v>1.573818366340089</v>
@@ -2647,10 +2647,10 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.4744506766882923</v>
+        <v>0.4744506766882924</v>
       </c>
       <c r="D35" t="n">
-        <v>0.4527354524364829</v>
+        <v>0.4527354524364828</v>
       </c>
       <c r="E35" t="n">
         <v>0.4276884542506333</v>
@@ -2659,19 +2659,19 @@
         <v>0.3947914557885837</v>
       </c>
       <c r="G35" t="n">
-        <v>0.4040374514304065</v>
+        <v>0.4040374514304064</v>
       </c>
       <c r="H35" t="n">
-        <v>0.6411577324587681</v>
+        <v>0.6411577324587682</v>
       </c>
       <c r="I35" t="n">
-        <v>0.7572241846316828</v>
+        <v>0.7572241846316827</v>
       </c>
       <c r="J35" t="n">
-        <v>0.6160614310605069</v>
+        <v>0.616061431060507</v>
       </c>
       <c r="K35" t="n">
-        <v>0.6343336691637603</v>
+        <v>0.6343336691637602</v>
       </c>
       <c r="L35" t="n">
         <v>0.706108520593674</v>
@@ -2680,10 +2680,10 @@
         <v>0.67793136788177</v>
       </c>
       <c r="N35" t="n">
-        <v>0.6602776033856694</v>
+        <v>0.6602776033856697</v>
       </c>
       <c r="O35" t="n">
-        <v>1.334863705382981</v>
+        <v>1.33486370538298</v>
       </c>
       <c r="P35" t="n">
         <v>1.344099628011233</v>
@@ -2698,7 +2698,7 @@
         <v>1.617183317231839</v>
       </c>
       <c r="T35" t="n">
-        <v>1.667507511373175</v>
+        <v>1.667507511373176</v>
       </c>
     </row>
     <row r="36">
@@ -2720,16 +2720,16 @@
         <v>1.060101421488198</v>
       </c>
       <c r="F36" t="n">
-        <v>0.9918783317193489</v>
+        <v>0.991878331719349</v>
       </c>
       <c r="G36" t="n">
         <v>1.005831982981693</v>
       </c>
       <c r="H36" t="n">
-        <v>0.8712875694146194</v>
+        <v>0.8712875694146192</v>
       </c>
       <c r="I36" t="n">
-        <v>1.509803313929872</v>
+        <v>1.509803313929873</v>
       </c>
       <c r="J36" t="n">
         <v>1.309335653968299</v>
@@ -2744,7 +2744,7 @@
         <v>1.406251563128973</v>
       </c>
       <c r="N36" t="n">
-        <v>1.477686988087022</v>
+        <v>1.477686988087023</v>
       </c>
       <c r="O36" t="n">
         <v>2.504438041799734</v>
@@ -2753,10 +2753,10 @@
         <v>2.702065560424375</v>
       </c>
       <c r="Q36" t="n">
-        <v>2.666349493641969</v>
+        <v>2.66634949364197</v>
       </c>
       <c r="R36" t="n">
-        <v>3.054031011960829</v>
+        <v>3.05403101196083</v>
       </c>
       <c r="S36" t="n">
         <v>3.36980345429629</v>
@@ -2775,7 +2775,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>6.097546813759397</v>
+        <v>6.097546813759399</v>
       </c>
       <c r="D37" t="n">
         <v>5.114140316126428</v>
@@ -2784,31 +2784,31 @@
         <v>5.699036768997352</v>
       </c>
       <c r="F37" t="n">
-        <v>4.884572606433907</v>
+        <v>4.884572606433904</v>
       </c>
       <c r="G37" t="n">
-        <v>5.202316019783634</v>
+        <v>5.202316019783632</v>
       </c>
       <c r="H37" t="n">
-        <v>7.829584069477383</v>
+        <v>7.829584069477384</v>
       </c>
       <c r="I37" t="n">
-        <v>8.877646078700112</v>
+        <v>8.87764607870011</v>
       </c>
       <c r="J37" t="n">
-        <v>7.821808437450236</v>
+        <v>7.821808437450237</v>
       </c>
       <c r="K37" t="n">
-        <v>8.01017499815722</v>
+        <v>8.010174998157218</v>
       </c>
       <c r="L37" t="n">
         <v>9.004934032311969</v>
       </c>
       <c r="M37" t="n">
-        <v>8.733332666759518</v>
+        <v>8.733332666759516</v>
       </c>
       <c r="N37" t="n">
-        <v>8.676850139866698</v>
+        <v>8.676850139866703</v>
       </c>
       <c r="O37" t="n">
         <v>13.35027819563612</v>
@@ -2823,10 +2823,10 @@
         <v>15.07712930581885</v>
       </c>
       <c r="S37" t="n">
-        <v>13.83875879936987</v>
+        <v>13.83875879936986</v>
       </c>
       <c r="T37" t="n">
-        <v>16.0987323626082</v>
+        <v>16.09873236260819</v>
       </c>
     </row>
     <row r="38">
@@ -2842,13 +2842,13 @@
         <v>0.3067922242723701</v>
       </c>
       <c r="D38" t="n">
-        <v>0.2886299712415187</v>
+        <v>0.2886299712415188</v>
       </c>
       <c r="E38" t="n">
         <v>0.3075289005296661</v>
       </c>
       <c r="F38" t="n">
-        <v>0.2541057001269997</v>
+        <v>0.2541057001269998</v>
       </c>
       <c r="G38" t="n">
         <v>0.2556200834535385</v>
@@ -2857,7 +2857,7 @@
         <v>0.2461904830187608</v>
       </c>
       <c r="I38" t="n">
-        <v>0.3625580352376091</v>
+        <v>0.3625580352376092</v>
       </c>
       <c r="J38" t="n">
         <v>0.3012688587454551</v>
@@ -2866,7 +2866,7 @@
         <v>0.3067471673055576</v>
       </c>
       <c r="L38" t="n">
-        <v>0.3671450306366575</v>
+        <v>0.3671450306366577</v>
       </c>
       <c r="M38" t="n">
         <v>0.3521634432109499</v>
@@ -2875,7 +2875,7 @@
         <v>0.3672161387547305</v>
       </c>
       <c r="O38" t="n">
-        <v>0.5560605283839813</v>
+        <v>0.5560605283839812</v>
       </c>
       <c r="P38" t="n">
         <v>0.5979598904923212</v>
@@ -2884,10 +2884,10 @@
         <v>0.5950990026010461</v>
       </c>
       <c r="R38" t="n">
-        <v>0.7000854348229416</v>
+        <v>0.7000854348229418</v>
       </c>
       <c r="S38" t="n">
-        <v>0.7025020583363111</v>
+        <v>0.7025020583363112</v>
       </c>
       <c r="T38" t="n">
         <v>0.7224778093726278</v>
@@ -2954,7 +2954,7 @@
         <v>0.2989639581600973</v>
       </c>
       <c r="T39" t="n">
-        <v>0.3385117436309611</v>
+        <v>0.338511743630961</v>
       </c>
     </row>
     <row r="40">
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.09710812149561764</v>
+        <v>0.09710812149561765</v>
       </c>
       <c r="D40" t="n">
         <v>0.07378841216035686</v>
@@ -3034,7 +3034,7 @@
         <v>0.2221327367623503</v>
       </c>
       <c r="D41" t="n">
-        <v>0.1725111199877555</v>
+        <v>0.1725111199877554</v>
       </c>
       <c r="E41" t="n">
         <v>0.1818800407645293</v>
@@ -3061,7 +3061,7 @@
         <v>0.3258858758460397</v>
       </c>
       <c r="M41" t="n">
-        <v>0.2619777059145986</v>
+        <v>0.2619777059145987</v>
       </c>
       <c r="N41" t="n">
         <v>0.2574253572920717</v>
@@ -3073,16 +3073,16 @@
         <v>0.4496474792223005</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.3981511220443802</v>
+        <v>0.3981511220443804</v>
       </c>
       <c r="R41" t="n">
-        <v>0.51907373160486</v>
+        <v>0.5190737316048599</v>
       </c>
       <c r="S41" t="n">
-        <v>0.4926698176538301</v>
+        <v>0.4926698176538302</v>
       </c>
       <c r="T41" t="n">
-        <v>0.5045882975581968</v>
+        <v>0.5045882975581967</v>
       </c>
     </row>
     <row r="42">
@@ -3116,7 +3116,7 @@
         <v>0.2795976787246109</v>
       </c>
       <c r="J42" t="n">
-        <v>0.2313455560769902</v>
+        <v>0.2313455560769903</v>
       </c>
       <c r="K42" t="n">
         <v>0.2370927516089911</v>
@@ -3137,10 +3137,10 @@
         <v>0.3996174953893472</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.4029380843034595</v>
+        <v>0.4029380843034596</v>
       </c>
       <c r="R42" t="n">
-        <v>0.4685313158556249</v>
+        <v>0.4685313158556248</v>
       </c>
       <c r="S42" t="n">
         <v>0.4689794849502715</v>
@@ -3165,16 +3165,16 @@
         <v>0.4059216546935467</v>
       </c>
       <c r="E43" t="n">
-        <v>0.4442616040029671</v>
+        <v>0.444261604002967</v>
       </c>
       <c r="F43" t="n">
-        <v>0.4067174542639537</v>
+        <v>0.4067174542639536</v>
       </c>
       <c r="G43" t="n">
-        <v>0.4522850142606717</v>
+        <v>0.4522850142606716</v>
       </c>
       <c r="H43" t="n">
-        <v>0.6343909191249647</v>
+        <v>0.6343909191249649</v>
       </c>
       <c r="I43" t="n">
         <v>0.7482193099960742</v>
@@ -3183,7 +3183,7 @@
         <v>0.5958331305680664</v>
       </c>
       <c r="K43" t="n">
-        <v>0.6785166683249232</v>
+        <v>0.6785166683249233</v>
       </c>
       <c r="L43" t="n">
         <v>0.7753307415839777</v>
@@ -3192,13 +3192,13 @@
         <v>0.7358421863239855</v>
       </c>
       <c r="N43" t="n">
-        <v>0.7576220320898085</v>
+        <v>0.7576220320898088</v>
       </c>
       <c r="O43" t="n">
         <v>1.400432323002829</v>
       </c>
       <c r="P43" t="n">
-        <v>1.394145542172853</v>
+        <v>1.394145542172852</v>
       </c>
       <c r="Q43" t="n">
         <v>1.441774165774629</v>
@@ -3210,7 +3210,7 @@
         <v>1.750946287373406</v>
       </c>
       <c r="T43" t="n">
-        <v>1.871157889002289</v>
+        <v>1.871157889002288</v>
       </c>
     </row>
     <row r="44">
@@ -3223,25 +3223,25 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3.024542231082156</v>
+        <v>3.024542231082155</v>
       </c>
       <c r="D44" t="n">
         <v>2.59463350804146</v>
       </c>
       <c r="E44" t="n">
-        <v>2.411729680617749</v>
+        <v>2.41172968061775</v>
       </c>
       <c r="F44" t="n">
         <v>2.391574091326178</v>
       </c>
       <c r="G44" t="n">
-        <v>2.609562577499625</v>
+        <v>2.609562577499626</v>
       </c>
       <c r="H44" t="n">
         <v>2.677117644914224</v>
       </c>
       <c r="I44" t="n">
-        <v>3.987484973550337</v>
+        <v>3.987484973550339</v>
       </c>
       <c r="J44" t="n">
         <v>3.47230724128306</v>
@@ -3253,19 +3253,19 @@
         <v>4.185554924020091</v>
       </c>
       <c r="M44" t="n">
-        <v>3.925163487466424</v>
+        <v>3.925163487466425</v>
       </c>
       <c r="N44" t="n">
-        <v>4.042892391814344</v>
+        <v>4.042892391814342</v>
       </c>
       <c r="O44" t="n">
-        <v>7.39638880269113</v>
+        <v>7.396388802691133</v>
       </c>
       <c r="P44" t="n">
-        <v>7.806862964356107</v>
+        <v>7.806862964356106</v>
       </c>
       <c r="Q44" t="n">
-        <v>7.558398617417605</v>
+        <v>7.558398617417602</v>
       </c>
       <c r="R44" t="n">
         <v>8.757436153017908</v>
@@ -3290,13 +3290,13 @@
         <v>0.06775541010962828</v>
       </c>
       <c r="D45" t="n">
-        <v>0.05768933578430235</v>
+        <v>0.05768933578430236</v>
       </c>
       <c r="E45" t="n">
         <v>0.05867967829297586</v>
       </c>
       <c r="F45" t="n">
-        <v>0.05347339224858023</v>
+        <v>0.05347339224858022</v>
       </c>
       <c r="G45" t="n">
         <v>0.05282702229007273</v>
@@ -3317,7 +3317,7 @@
         <v>0.09633633359715214</v>
       </c>
       <c r="M45" t="n">
-        <v>0.082682566672001</v>
+        <v>0.08268256667200101</v>
       </c>
       <c r="N45" t="n">
         <v>0.08467083455298798</v>
@@ -3402,7 +3402,7 @@
         <v>0.04808156005787596</v>
       </c>
       <c r="T46" t="n">
-        <v>0.06071415269639251</v>
+        <v>0.0607141526963925</v>
       </c>
     </row>
     <row r="47">
@@ -3451,10 +3451,10 @@
         <v>0.1739873745788708</v>
       </c>
       <c r="O47" t="n">
-        <v>0.2363514675839615</v>
+        <v>0.2363514675839616</v>
       </c>
       <c r="P47" t="n">
-        <v>0.2394732263943229</v>
+        <v>0.239473226394323</v>
       </c>
       <c r="Q47" t="n">
         <v>0.2383106961359085</v>
@@ -3463,10 +3463,10 @@
         <v>0.2607051141114113</v>
       </c>
       <c r="S47" t="n">
-        <v>0.296278098906221</v>
+        <v>0.2962780989062211</v>
       </c>
       <c r="T47" t="n">
-        <v>0.2941269442488873</v>
+        <v>0.2941269442488872</v>
       </c>
     </row>
     <row r="48">
@@ -3503,7 +3503,7 @@
         <v>1.605262706341932</v>
       </c>
       <c r="K48" t="n">
-        <v>1.900433259945865</v>
+        <v>1.900433259945866</v>
       </c>
       <c r="L48" t="n">
         <v>1.959481859451967</v>
@@ -3521,16 +3521,16 @@
         <v>3.777795179031263</v>
       </c>
       <c r="Q48" t="n">
-        <v>3.24043567308285</v>
+        <v>3.240435673082851</v>
       </c>
       <c r="R48" t="n">
         <v>4.387061663915111</v>
       </c>
       <c r="S48" t="n">
-        <v>5.625264225328277</v>
+        <v>5.625264225328275</v>
       </c>
       <c r="T48" t="n">
-        <v>5.46888966580628</v>
+        <v>5.468889665806282</v>
       </c>
     </row>
     <row r="49">
@@ -3607,13 +3607,13 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0.08860172431605201</v>
+        <v>0.08860172431605198</v>
       </c>
       <c r="D50" t="n">
-        <v>0.07462511893453964</v>
+        <v>0.07462511893453966</v>
       </c>
       <c r="E50" t="n">
-        <v>0.08198445385099677</v>
+        <v>0.08198445385099679</v>
       </c>
       <c r="F50" t="n">
         <v>0.06922494332878612</v>
@@ -3631,7 +3631,7 @@
         <v>0.1007247446415135</v>
       </c>
       <c r="K50" t="n">
-        <v>0.09771725670103719</v>
+        <v>0.09771725670103722</v>
       </c>
       <c r="L50" t="n">
         <v>0.1269366541588031</v>
@@ -3640,10 +3640,10 @@
         <v>0.127132903867545</v>
       </c>
       <c r="N50" t="n">
-        <v>0.120143993537056</v>
+        <v>0.1201439935370561</v>
       </c>
       <c r="O50" t="n">
-        <v>0.2378016392687133</v>
+        <v>0.2378016392687132</v>
       </c>
       <c r="P50" t="n">
         <v>0.2476153526722418</v>
@@ -3652,13 +3652,13 @@
         <v>0.2475292447110699</v>
       </c>
       <c r="R50" t="n">
-        <v>0.3056180042771321</v>
+        <v>0.3056180042771322</v>
       </c>
       <c r="S50" t="n">
         <v>0.3356938204301642</v>
       </c>
       <c r="T50" t="n">
-        <v>0.3253991120492345</v>
+        <v>0.3253991120492344</v>
       </c>
     </row>
     <row r="51">
@@ -3689,7 +3689,7 @@
         <v>13.97551201437595</v>
       </c>
       <c r="I51" t="n">
-        <v>17.96573575479981</v>
+        <v>17.9657357547998</v>
       </c>
       <c r="J51" t="n">
         <v>15.27050302327962</v>
@@ -3698,7 +3698,7 @@
         <v>15.04962773666824</v>
       </c>
       <c r="L51" t="n">
-        <v>21.35549863107241</v>
+        <v>21.35549863107242</v>
       </c>
       <c r="M51" t="n">
         <v>20.41376999275762</v>
@@ -3707,10 +3707,10 @@
         <v>19.13479435591571</v>
       </c>
       <c r="O51" t="n">
-        <v>50.21069115862193</v>
+        <v>50.21069115862192</v>
       </c>
       <c r="P51" t="n">
-        <v>50.22166455892093</v>
+        <v>50.22166455892091</v>
       </c>
       <c r="Q51" t="n">
         <v>50.13837317396758</v>
@@ -3722,7 +3722,7 @@
         <v>83.51987220662355</v>
       </c>
       <c r="T51" t="n">
-        <v>79.43649960610361</v>
+        <v>79.43649960610364</v>
       </c>
     </row>
     <row r="52">
@@ -3744,13 +3744,13 @@
         <v>0.1873915193676626</v>
       </c>
       <c r="F52" t="n">
-        <v>0.1871588238984856</v>
+        <v>0.1871588238984855</v>
       </c>
       <c r="G52" t="n">
         <v>0.1992711523650431</v>
       </c>
       <c r="H52" t="n">
-        <v>0.2450922242550073</v>
+        <v>0.2450922242550072</v>
       </c>
       <c r="I52" t="n">
         <v>0.3301955192627085</v>
@@ -3759,7 +3759,7 @@
         <v>0.2838122522826749</v>
       </c>
       <c r="K52" t="n">
-        <v>0.2892103106972125</v>
+        <v>0.2892103106972123</v>
       </c>
       <c r="L52" t="n">
         <v>0.3334945218023855</v>
@@ -3768,22 +3768,22 @@
         <v>0.3265435606084486</v>
       </c>
       <c r="N52" t="n">
-        <v>0.3465252200970447</v>
+        <v>0.3465252200970448</v>
       </c>
       <c r="O52" t="n">
-        <v>0.5383586329485341</v>
+        <v>0.5383586329485343</v>
       </c>
       <c r="P52" t="n">
-        <v>0.5375528631004318</v>
+        <v>0.5375528631004317</v>
       </c>
       <c r="Q52" t="n">
         <v>0.4778548293983886</v>
       </c>
       <c r="R52" t="n">
-        <v>0.5592223663275285</v>
+        <v>0.5592223663275284</v>
       </c>
       <c r="S52" t="n">
-        <v>0.5651631022033324</v>
+        <v>0.5651631022033325</v>
       </c>
       <c r="T52" t="n">
         <v>0.6393289829530447</v>
@@ -3805,10 +3805,10 @@
         <v>0.04100827215303991</v>
       </c>
       <c r="E53" t="n">
-        <v>0.0404799147824051</v>
+        <v>0.04047991478240511</v>
       </c>
       <c r="F53" t="n">
-        <v>0.03380066366290121</v>
+        <v>0.03380066366290122</v>
       </c>
       <c r="G53" t="n">
         <v>0.03527272096626635</v>
@@ -3817,19 +3817,19 @@
         <v>0.03724214220896253</v>
       </c>
       <c r="I53" t="n">
-        <v>0.04582945961866256</v>
+        <v>0.04582945961866257</v>
       </c>
       <c r="J53" t="n">
         <v>0.03741265908861736</v>
       </c>
       <c r="K53" t="n">
-        <v>0.03967442793739957</v>
+        <v>0.03967442793739956</v>
       </c>
       <c r="L53" t="n">
         <v>0.04477268194484697</v>
       </c>
       <c r="M53" t="n">
-        <v>0.04494895685484368</v>
+        <v>0.04494895685484367</v>
       </c>
       <c r="N53" t="n">
         <v>0.0470079201435409</v>
@@ -3838,19 +3838,19 @@
         <v>0.06515883312020487</v>
       </c>
       <c r="P53" t="n">
-        <v>0.07067839847841681</v>
+        <v>0.0706783984784168</v>
       </c>
       <c r="Q53" t="n">
-        <v>0.06363342134431831</v>
+        <v>0.06363342134431832</v>
       </c>
       <c r="R53" t="n">
         <v>0.07107560786585661</v>
       </c>
       <c r="S53" t="n">
-        <v>0.0727845745336286</v>
+        <v>0.07278457453362859</v>
       </c>
       <c r="T53" t="n">
-        <v>0.0802778951032702</v>
+        <v>0.08027789510327019</v>
       </c>
     </row>
     <row r="54">
@@ -3866,10 +3866,10 @@
         <v>20.05955599835347</v>
       </c>
       <c r="D54" t="n">
-        <v>18.21345737108491</v>
+        <v>18.21345737108492</v>
       </c>
       <c r="E54" t="n">
-        <v>18.99311284141382</v>
+        <v>18.99311284141383</v>
       </c>
       <c r="F54" t="n">
         <v>13.6523022805223</v>
@@ -3881,40 +3881,40 @@
         <v>17.95847260667808</v>
       </c>
       <c r="I54" t="n">
-        <v>20.96259668949901</v>
+        <v>20.962596689499</v>
       </c>
       <c r="J54" t="n">
         <v>17.07160064407507</v>
       </c>
       <c r="K54" t="n">
-        <v>17.05811283337797</v>
+        <v>17.05811283337796</v>
       </c>
       <c r="L54" t="n">
-        <v>18.58251270403408</v>
+        <v>18.58251270403407</v>
       </c>
       <c r="M54" t="n">
-        <v>19.07413149796639</v>
+        <v>19.07413149796638</v>
       </c>
       <c r="N54" t="n">
         <v>19.87843876472925</v>
       </c>
       <c r="O54" t="n">
-        <v>46.85941209386325</v>
+        <v>46.85941209386324</v>
       </c>
       <c r="P54" t="n">
-        <v>42.2203452231828</v>
+        <v>42.22034522318278</v>
       </c>
       <c r="Q54" t="n">
-        <v>41.99579983189018</v>
+        <v>41.99579983189019</v>
       </c>
       <c r="R54" t="n">
-        <v>62.33204504933173</v>
+        <v>62.33204504933176</v>
       </c>
       <c r="S54" t="n">
-        <v>68.08183312628151</v>
+        <v>68.08183312628148</v>
       </c>
       <c r="T54" t="n">
-        <v>67.54040679039808</v>
+        <v>67.54040679039809</v>
       </c>
     </row>
     <row r="55">
@@ -3927,22 +3927,22 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2.436010129408096</v>
+        <v>2.436010129408095</v>
       </c>
       <c r="D55" t="n">
         <v>2.110080126989678</v>
       </c>
       <c r="E55" t="n">
-        <v>2.277600249919772</v>
+        <v>2.277600249919771</v>
       </c>
       <c r="F55" t="n">
         <v>2.160205859747014</v>
       </c>
       <c r="G55" t="n">
-        <v>2.313606941531643</v>
+        <v>2.313606941531642</v>
       </c>
       <c r="H55" t="n">
-        <v>3.187641228870546</v>
+        <v>3.187641228870548</v>
       </c>
       <c r="I55" t="n">
         <v>3.529625996694259</v>
@@ -3954,7 +3954,7 @@
         <v>3.114295236810142</v>
       </c>
       <c r="L55" t="n">
-        <v>3.300267833329398</v>
+        <v>3.300267833329399</v>
       </c>
       <c r="M55" t="n">
         <v>3.242387635362422</v>
@@ -3963,13 +3963,13 @@
         <v>3.222441603206717</v>
       </c>
       <c r="O55" t="n">
-        <v>5.323467152298636</v>
+        <v>5.323467152298638</v>
       </c>
       <c r="P55" t="n">
-        <v>5.164562010286511</v>
+        <v>5.164562010286512</v>
       </c>
       <c r="Q55" t="n">
-        <v>5.004952133085361</v>
+        <v>5.00495213308536</v>
       </c>
       <c r="R55" t="n">
         <v>6.287370154692156</v>
@@ -3991,34 +3991,34 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>9.002219528609341</v>
+        <v>9.002219528609343</v>
       </c>
       <c r="D56" t="n">
-        <v>8.001800521808397</v>
+        <v>8.001800521808399</v>
       </c>
       <c r="E56" t="n">
-        <v>8.310901666166227</v>
+        <v>8.310901666166226</v>
       </c>
       <c r="F56" t="n">
-        <v>9.437856918498605</v>
+        <v>9.437856918498602</v>
       </c>
       <c r="G56" t="n">
-        <v>9.872087524962003</v>
+        <v>9.872087524962005</v>
       </c>
       <c r="H56" t="n">
         <v>10.03581358518788</v>
       </c>
       <c r="I56" t="n">
-        <v>16.06705389282985</v>
+        <v>16.06705389282984</v>
       </c>
       <c r="J56" t="n">
-        <v>13.59741411842991</v>
+        <v>13.5974141184299</v>
       </c>
       <c r="K56" t="n">
-        <v>14.54418936305818</v>
+        <v>14.54418936305817</v>
       </c>
       <c r="L56" t="n">
-        <v>17.56714647826358</v>
+        <v>17.56714647826359</v>
       </c>
       <c r="M56" t="n">
         <v>16.81914736292005</v>
@@ -4030,19 +4030,19 @@
         <v>28.09770099886684</v>
       </c>
       <c r="P56" t="n">
-        <v>27.06158055870101</v>
+        <v>27.06158055870102</v>
       </c>
       <c r="Q56" t="n">
-        <v>24.16732439168009</v>
+        <v>24.16732439168008</v>
       </c>
       <c r="R56" t="n">
-        <v>27.90142995101546</v>
+        <v>27.90142995101545</v>
       </c>
       <c r="S56" t="n">
-        <v>30.78461216488867</v>
+        <v>30.78461216488866</v>
       </c>
       <c r="T56" t="n">
-        <v>33.68994732335536</v>
+        <v>33.68994732335537</v>
       </c>
     </row>
     <row r="57">
@@ -4085,7 +4085,7 @@
         <v>0.2206493916154403</v>
       </c>
       <c r="M57" t="n">
-        <v>0.2327865465708243</v>
+        <v>0.2327865465708244</v>
       </c>
       <c r="N57" t="n">
         <v>0.2263504382617427</v>
@@ -4119,25 +4119,25 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0.2968479371728841</v>
+        <v>0.296847937172884</v>
       </c>
       <c r="D58" t="n">
-        <v>0.2761931299905348</v>
+        <v>0.2761931299905347</v>
       </c>
       <c r="E58" t="n">
         <v>0.2793889979108572</v>
       </c>
       <c r="F58" t="n">
-        <v>0.2622196916297053</v>
+        <v>0.2622196916297052</v>
       </c>
       <c r="G58" t="n">
-        <v>0.2872729529123517</v>
+        <v>0.2872729529123516</v>
       </c>
       <c r="H58" t="n">
         <v>0.2146458058583305</v>
       </c>
       <c r="I58" t="n">
-        <v>0.3730450479624073</v>
+        <v>0.3730450479624072</v>
       </c>
       <c r="J58" t="n">
         <v>0.3114356260656577</v>
@@ -4146,7 +4146,7 @@
         <v>0.3236855746377045</v>
       </c>
       <c r="L58" t="n">
-        <v>0.3804854728963058</v>
+        <v>0.3804854728963059</v>
       </c>
       <c r="M58" t="n">
         <v>0.3587328305993009</v>
@@ -4158,19 +4158,19 @@
         <v>0.5733265193252318</v>
       </c>
       <c r="P58" t="n">
-        <v>0.5640821584039858</v>
+        <v>0.5640821584039857</v>
       </c>
       <c r="Q58" t="n">
         <v>0.5843001414103959</v>
       </c>
       <c r="R58" t="n">
-        <v>0.6193066921669442</v>
+        <v>0.6193066921669443</v>
       </c>
       <c r="S58" t="n">
-        <v>0.6905510298714844</v>
+        <v>0.6905510298714843</v>
       </c>
       <c r="T58" t="n">
-        <v>0.6905632149585152</v>
+        <v>0.6905632149585151</v>
       </c>
     </row>
     <row r="59">
@@ -4183,7 +4183,7 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.3665211324782944</v>
+        <v>0.3665211324782943</v>
       </c>
       <c r="D59" t="n">
         <v>0.2616070552258732</v>
@@ -4201,10 +4201,10 @@
         <v>0.4708188409610112</v>
       </c>
       <c r="I59" t="n">
-        <v>0.494194412178551</v>
+        <v>0.4941944121785509</v>
       </c>
       <c r="J59" t="n">
-        <v>0.4742208117594475</v>
+        <v>0.4742208117594476</v>
       </c>
       <c r="K59" t="n">
         <v>0.4308885404772455</v>
@@ -4219,7 +4219,7 @@
         <v>0.4907193142019842</v>
       </c>
       <c r="O59" t="n">
-        <v>0.7753968259582847</v>
+        <v>0.7753968259582845</v>
       </c>
       <c r="P59" t="n">
         <v>0.8229122625220627</v>
@@ -4228,10 +4228,10 @@
         <v>0.7637496637475516</v>
       </c>
       <c r="R59" t="n">
-        <v>1.021756852630665</v>
+        <v>1.021756852630664</v>
       </c>
       <c r="S59" t="n">
-        <v>0.8358940932905663</v>
+        <v>0.835894093290566</v>
       </c>
       <c r="T59" t="n">
         <v>0.9534817720727391</v>
@@ -4268,13 +4268,13 @@
         <v>7.696409682496404</v>
       </c>
       <c r="J60" t="n">
-        <v>6.780125415666087</v>
+        <v>6.780125415666086</v>
       </c>
       <c r="K60" t="n">
-        <v>6.767072585146675</v>
+        <v>6.767072585146673</v>
       </c>
       <c r="L60" t="n">
-        <v>7.603990588882165</v>
+        <v>7.603990588882166</v>
       </c>
       <c r="M60" t="n">
         <v>7.347889275251528</v>
@@ -4311,13 +4311,13 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0.1974613923869828</v>
+        <v>0.1974613923869827</v>
       </c>
       <c r="D61" t="n">
-        <v>0.2067498450747352</v>
+        <v>0.2067498450747351</v>
       </c>
       <c r="E61" t="n">
-        <v>0.1592537299886222</v>
+        <v>0.1592537299886221</v>
       </c>
       <c r="F61" t="n">
         <v>0.1597263109206815</v>
@@ -4332,7 +4332,7 @@
         <v>0.2680977665901244</v>
       </c>
       <c r="J61" t="n">
-        <v>0.2289473495324237</v>
+        <v>0.2289473495324238</v>
       </c>
       <c r="K61" t="n">
         <v>0.203477773626796</v>
@@ -4341,7 +4341,7 @@
         <v>0.246010848986166</v>
       </c>
       <c r="M61" t="n">
-        <v>0.2383280794542197</v>
+        <v>0.2383280794542198</v>
       </c>
       <c r="N61" t="n">
         <v>0.2430093264782666</v>
@@ -4399,7 +4399,7 @@
         <v>0.07419645851843938</v>
       </c>
       <c r="K62" t="n">
-        <v>0.005398043655014138</v>
+        <v>0.005398043655014137</v>
       </c>
       <c r="L62" t="n">
         <v>0.0656634102161279</v>
@@ -4442,37 +4442,37 @@
         <v>7.474025755052581</v>
       </c>
       <c r="D63" t="n">
-        <v>7.359220212472146</v>
+        <v>7.359220212472145</v>
       </c>
       <c r="E63" t="n">
-        <v>7.463603077570289</v>
+        <v>7.463603077570285</v>
       </c>
       <c r="F63" t="n">
-        <v>5.116440797995487</v>
+        <v>5.116440797995491</v>
       </c>
       <c r="G63" t="n">
         <v>6.33061455553134</v>
       </c>
       <c r="H63" t="n">
-        <v>7.399709940914338</v>
+        <v>7.399709940914342</v>
       </c>
       <c r="I63" t="n">
-        <v>7.355906746750128</v>
+        <v>7.355906746750129</v>
       </c>
       <c r="J63" t="n">
-        <v>6.666940113751793</v>
+        <v>6.666940113751791</v>
       </c>
       <c r="K63" t="n">
-        <v>6.585760931303153</v>
+        <v>6.585760931303156</v>
       </c>
       <c r="L63" t="n">
-        <v>5.904347755306564</v>
+        <v>5.904347755306565</v>
       </c>
       <c r="M63" t="n">
-        <v>6.168226399682597</v>
+        <v>6.1682263996826</v>
       </c>
       <c r="N63" t="n">
-        <v>7.02387954726958</v>
+        <v>7.023879547269578</v>
       </c>
       <c r="O63" t="n">
         <v>7.576125406056336</v>
@@ -4481,13 +4481,13 @@
         <v>7.583220679254564</v>
       </c>
       <c r="Q63" t="n">
-        <v>6.525872006185975</v>
+        <v>6.525872006185976</v>
       </c>
       <c r="R63" t="n">
-        <v>8.758523229211004</v>
+        <v>8.758523229211001</v>
       </c>
       <c r="S63" t="n">
-        <v>8.831576217316707</v>
+        <v>8.831576217316705</v>
       </c>
       <c r="T63" t="n">
         <v>7.873375497297173</v>
@@ -4506,7 +4506,7 @@
         <v>0.02371593080490814</v>
       </c>
       <c r="D64" t="n">
-        <v>0.02119374383137081</v>
+        <v>0.02119374383137082</v>
       </c>
       <c r="E64" t="n">
         <v>0.02693785174172563</v>
@@ -4521,10 +4521,10 @@
         <v>0.03098704064161814</v>
       </c>
       <c r="I64" t="n">
-        <v>0.03868091963561889</v>
+        <v>0.0386809196356189</v>
       </c>
       <c r="J64" t="n">
-        <v>0.03374692911133308</v>
+        <v>0.03374692911133307</v>
       </c>
       <c r="K64" t="n">
         <v>0.03374517860172788</v>
@@ -4542,7 +4542,7 @@
         <v>0.09660918369795228</v>
       </c>
       <c r="P64" t="n">
-        <v>0.09725104860782101</v>
+        <v>0.09725104860782102</v>
       </c>
       <c r="Q64" t="n">
         <v>0.07683679912447719</v>
@@ -4554,7 +4554,7 @@
         <v>0.1258254157547768</v>
       </c>
       <c r="T64" t="n">
-        <v>0.1212508408923788</v>
+        <v>0.1212508408923787</v>
       </c>
     </row>
     <row r="65">
@@ -4579,10 +4579,10 @@
         <v>7.327267481926659</v>
       </c>
       <c r="G65" t="n">
-        <v>7.903251992633487</v>
+        <v>7.903251992633484</v>
       </c>
       <c r="H65" t="n">
-        <v>12.56555257937036</v>
+        <v>12.56555257937037</v>
       </c>
       <c r="I65" t="n">
         <v>11.95210472771455</v>
@@ -4594,7 +4594,7 @@
         <v>10.77514390013631</v>
       </c>
       <c r="L65" t="n">
-        <v>12.56411846965582</v>
+        <v>12.56411846965583</v>
       </c>
       <c r="M65" t="n">
         <v>12.02445064709249</v>
@@ -4606,10 +4606,10 @@
         <v>21.96548053126049</v>
       </c>
       <c r="P65" t="n">
-        <v>22.2853887043098</v>
+        <v>22.28538870430981</v>
       </c>
       <c r="Q65" t="n">
-        <v>19.04418992930889</v>
+        <v>19.0441899293089</v>
       </c>
       <c r="R65" t="n">
         <v>26.72637825991753</v>
@@ -4634,34 +4634,34 @@
         <v>0.5521138996539523</v>
       </c>
       <c r="D66" t="n">
-        <v>0.4811467776143714</v>
+        <v>0.4811467776143715</v>
       </c>
       <c r="E66" t="n">
-        <v>0.4946621175280044</v>
+        <v>0.4946621175280045</v>
       </c>
       <c r="F66" t="n">
-        <v>0.4553056621614987</v>
+        <v>0.4553056621614988</v>
       </c>
       <c r="G66" t="n">
         <v>0.4975013469952058</v>
       </c>
       <c r="H66" t="n">
-        <v>0.6712072827404822</v>
+        <v>0.6712072827404821</v>
       </c>
       <c r="I66" t="n">
         <v>0.8187225122042264</v>
       </c>
       <c r="J66" t="n">
-        <v>0.6956189370261473</v>
+        <v>0.6956189370261474</v>
       </c>
       <c r="K66" t="n">
         <v>0.6963681204728589</v>
       </c>
       <c r="L66" t="n">
-        <v>0.7551802154687057</v>
+        <v>0.7551802154687058</v>
       </c>
       <c r="M66" t="n">
-        <v>0.763226385100119</v>
+        <v>0.7632263851001189</v>
       </c>
       <c r="N66" t="n">
         <v>0.7570082705146345</v>
@@ -4701,7 +4701,7 @@
         <v>0.02175221901825343</v>
       </c>
       <c r="E67" t="n">
-        <v>0.02091373098466212</v>
+        <v>0.02091373098466211</v>
       </c>
       <c r="F67" t="n">
         <v>0.01867519038105681</v>
@@ -4759,19 +4759,19 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.0886043521753605</v>
+        <v>0.08860435217536049</v>
       </c>
       <c r="D68" t="n">
-        <v>0.08338357720705418</v>
+        <v>0.08338357720705421</v>
       </c>
       <c r="E68" t="n">
-        <v>0.08065678586299246</v>
+        <v>0.08065678586299248</v>
       </c>
       <c r="F68" t="n">
         <v>0.07761385131896632</v>
       </c>
       <c r="G68" t="n">
-        <v>0.0770589067120446</v>
+        <v>0.07705890671204459</v>
       </c>
       <c r="H68" t="n">
         <v>0.08908526987208795</v>
@@ -4798,7 +4798,7 @@
         <v>0.20967058173589</v>
       </c>
       <c r="P68" t="n">
-        <v>0.2030245335134442</v>
+        <v>0.2030245335134443</v>
       </c>
       <c r="Q68" t="n">
         <v>0.1926497405625261</v>
@@ -4847,7 +4847,7 @@
         <v>0.2144598457362292</v>
       </c>
       <c r="K69" t="n">
-        <v>0.2027601391042351</v>
+        <v>0.202760139104235</v>
       </c>
       <c r="L69" t="n">
         <v>0.2313277859288956</v>
@@ -4859,13 +4859,13 @@
         <v>0.2299358346493484</v>
       </c>
       <c r="O69" t="n">
-        <v>0.4065884659834503</v>
+        <v>0.4065884659834504</v>
       </c>
       <c r="P69" t="n">
         <v>0.4547050420758502</v>
       </c>
       <c r="Q69" t="n">
-        <v>0.4204724715982064</v>
+        <v>0.4204724715982063</v>
       </c>
       <c r="R69" t="n">
         <v>0.6100145977516065</v>
@@ -4951,10 +4951,10 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>9.565490154526328</v>
+        <v>9.565490154526326</v>
       </c>
       <c r="D71" t="n">
-        <v>9.267283128133085</v>
+        <v>9.267283128133087</v>
       </c>
       <c r="E71" t="n">
         <v>10.94191259764819</v>
@@ -4966,7 +4966,7 @@
         <v>8.485819198539783</v>
       </c>
       <c r="H71" t="n">
-        <v>9.325951313710426</v>
+        <v>9.325951313710425</v>
       </c>
       <c r="I71" t="n">
         <v>12.30330279162969</v>
@@ -4975,7 +4975,7 @@
         <v>10.59051285354356</v>
       </c>
       <c r="K71" t="n">
-        <v>10.50167169870799</v>
+        <v>10.501671698708</v>
       </c>
       <c r="L71" t="n">
         <v>11.47118551683275</v>
@@ -4999,7 +4999,7 @@
         <v>17.11880592520788</v>
       </c>
       <c r="S71" t="n">
-        <v>17.9386799591219</v>
+        <v>17.93867995912189</v>
       </c>
       <c r="T71" t="n">
         <v>18.34885510296303</v>
@@ -5039,7 +5039,7 @@
         <v>2.023453764190804</v>
       </c>
       <c r="K72" t="n">
-        <v>2.188914594874116</v>
+        <v>2.188914594874115</v>
       </c>
       <c r="L72" t="n">
         <v>2.659499514689071</v>
@@ -5051,13 +5051,13 @@
         <v>2.40286715698553</v>
       </c>
       <c r="O72" t="n">
-        <v>5.147166574557633</v>
+        <v>5.147166574557632</v>
       </c>
       <c r="P72" t="n">
-        <v>5.377060657092477</v>
+        <v>5.377060657092476</v>
       </c>
       <c r="Q72" t="n">
-        <v>4.473685519038742</v>
+        <v>4.473685519038743</v>
       </c>
       <c r="R72" t="n">
         <v>6.379974186720848</v>
@@ -5066,7 +5066,7 @@
         <v>5.431101620617825</v>
       </c>
       <c r="T72" t="n">
-        <v>6.941913179724765</v>
+        <v>6.941913179724764</v>
       </c>
     </row>
     <row r="73">
@@ -5085,13 +5085,13 @@
         <v>1.266259381382845</v>
       </c>
       <c r="E73" t="n">
-        <v>1.247334570870389</v>
+        <v>1.24733457087039</v>
       </c>
       <c r="F73" t="n">
         <v>1.124091596050999</v>
       </c>
       <c r="G73" t="n">
-        <v>1.192844090757994</v>
+        <v>1.192844090757993</v>
       </c>
       <c r="H73" t="n">
         <v>1.532561732471719</v>
@@ -5109,7 +5109,7 @@
         <v>1.875126782878658</v>
       </c>
       <c r="M73" t="n">
-        <v>1.824960188839065</v>
+        <v>1.824960188839064</v>
       </c>
       <c r="N73" t="n">
         <v>1.825863106501562</v>
@@ -5124,13 +5124,13 @@
         <v>2.601805039389385</v>
       </c>
       <c r="R73" t="n">
-        <v>3.159059213605379</v>
+        <v>3.159059213605377</v>
       </c>
       <c r="S73" t="n">
         <v>3.140371146369913</v>
       </c>
       <c r="T73" t="n">
-        <v>3.199083838448154</v>
+        <v>3.199083838448153</v>
       </c>
     </row>
     <row r="74">
@@ -5176,7 +5176,7 @@
         <v>1.67586973319119</v>
       </c>
       <c r="N74" t="n">
-        <v>1.759391306409165</v>
+        <v>1.759391306409166</v>
       </c>
       <c r="O74" t="n">
         <v>2.981202413708604</v>
@@ -5194,7 +5194,7 @@
         <v>3.263613274909259</v>
       </c>
       <c r="T74" t="n">
-        <v>3.633930412665087</v>
+        <v>3.633930412665086</v>
       </c>
     </row>
     <row r="75">
@@ -5216,7 +5216,7 @@
         <v>0.00352918485838404</v>
       </c>
       <c r="F75" t="n">
-        <v>0.003097117446052132</v>
+        <v>0.003097117446052133</v>
       </c>
       <c r="G75" t="n">
         <v>0.003219639722548721</v>
@@ -5234,7 +5234,7 @@
         <v>0.003714001496067616</v>
       </c>
       <c r="L75" t="n">
-        <v>0.004997115966820387</v>
+        <v>0.004997115966820386</v>
       </c>
       <c r="M75" t="n">
         <v>0.003986494787456262</v>
@@ -5246,7 +5246,7 @@
         <v>0.005243158880678737</v>
       </c>
       <c r="P75" t="n">
-        <v>0.005320022576707077</v>
+        <v>0.005320022576707076</v>
       </c>
       <c r="Q75" t="n">
         <v>0.006254146581994705</v>
@@ -5274,10 +5274,10 @@
         <v>1.018561139278981</v>
       </c>
       <c r="D76" t="n">
-        <v>0.8945888726264916</v>
+        <v>0.8945888726264914</v>
       </c>
       <c r="E76" t="n">
-        <v>0.8492489187710287</v>
+        <v>0.8492489187710286</v>
       </c>
       <c r="F76" t="n">
         <v>0.8277236937358575</v>
@@ -5295,16 +5295,16 @@
         <v>1.112894457142302</v>
       </c>
       <c r="K76" t="n">
-        <v>1.144149575341083</v>
+        <v>1.144149575341082</v>
       </c>
       <c r="L76" t="n">
-        <v>1.284952430826309</v>
+        <v>1.28495243082631</v>
       </c>
       <c r="M76" t="n">
         <v>1.179875785866946</v>
       </c>
       <c r="N76" t="n">
-        <v>1.256437534535654</v>
+        <v>1.256437534535655</v>
       </c>
       <c r="O76" t="n">
         <v>2.074779267803994</v>
@@ -5319,7 +5319,7 @@
         <v>2.555310431736634</v>
       </c>
       <c r="S76" t="n">
-        <v>2.7927576342226</v>
+        <v>2.792757634222599</v>
       </c>
       <c r="T76" t="n">
         <v>2.905019319809834</v>
@@ -5338,7 +5338,7 @@
         <v>0.02665883122237917</v>
       </c>
       <c r="D77" t="n">
-        <v>0.02675760155556802</v>
+        <v>0.02675760155556803</v>
       </c>
       <c r="E77" t="n">
         <v>0.02375496416693737</v>
@@ -5487,16 +5487,16 @@
         <v>0.03667063681036448</v>
       </c>
       <c r="K79" t="n">
-        <v>0.03891491276865705</v>
+        <v>0.03891491276865704</v>
       </c>
       <c r="L79" t="n">
-        <v>0.04371732745194583</v>
+        <v>0.04371732745194584</v>
       </c>
       <c r="M79" t="n">
-        <v>0.04117212522759247</v>
+        <v>0.04117212522759246</v>
       </c>
       <c r="N79" t="n">
-        <v>0.04691687729155184</v>
+        <v>0.04691687729155183</v>
       </c>
       <c r="O79" t="n">
         <v>0.06758305287676421</v>
@@ -5505,13 +5505,13 @@
         <v>0.06734807046120025</v>
       </c>
       <c r="Q79" t="n">
-        <v>0.06520952053710403</v>
+        <v>0.06520952053710402</v>
       </c>
       <c r="R79" t="n">
         <v>0.07648818052484195</v>
       </c>
       <c r="S79" t="n">
-        <v>0.07569175457430555</v>
+        <v>0.07569175457430552</v>
       </c>
       <c r="T79" t="n">
         <v>0.07746444660710337</v>
@@ -5536,7 +5536,7 @@
         <v>0.08973841631731855</v>
       </c>
       <c r="F80" t="n">
-        <v>0.09397478314432434</v>
+        <v>0.09397478314432432</v>
       </c>
       <c r="G80" t="n">
         <v>0.0960544485675292</v>
@@ -5569,7 +5569,7 @@
         <v>0.3131226425413716</v>
       </c>
       <c r="Q80" t="n">
-        <v>0.3254622570892271</v>
+        <v>0.325462257089227</v>
       </c>
       <c r="R80" t="n">
         <v>0.4324860252312683</v>
@@ -5594,49 +5594,49 @@
         <v>0.05933909815392528</v>
       </c>
       <c r="D81" t="n">
-        <v>0.05744520665500569</v>
+        <v>0.05744520665500571</v>
       </c>
       <c r="E81" t="n">
         <v>0.05839908678499228</v>
       </c>
       <c r="F81" t="n">
-        <v>0.0424041563918169</v>
+        <v>0.04240415639181689</v>
       </c>
       <c r="G81" t="n">
         <v>0.04513619269068152</v>
       </c>
       <c r="H81" t="n">
-        <v>0.05645308277290649</v>
+        <v>0.05645308277290648</v>
       </c>
       <c r="I81" t="n">
-        <v>0.05996261523613867</v>
+        <v>0.05996261523613866</v>
       </c>
       <c r="J81" t="n">
         <v>0.05164878148660471</v>
       </c>
       <c r="K81" t="n">
-        <v>0.05421839837363158</v>
+        <v>0.05421839837363159</v>
       </c>
       <c r="L81" t="n">
-        <v>0.05970994279377559</v>
+        <v>0.0597099427937756</v>
       </c>
       <c r="M81" t="n">
-        <v>0.05935430359267566</v>
+        <v>0.05935430359267565</v>
       </c>
       <c r="N81" t="n">
         <v>0.06510591134099562</v>
       </c>
       <c r="O81" t="n">
-        <v>0.09395388926363958</v>
+        <v>0.0939538892636396</v>
       </c>
       <c r="P81" t="n">
-        <v>0.09981060038399729</v>
+        <v>0.09981060038399728</v>
       </c>
       <c r="Q81" t="n">
-        <v>0.07475826716118832</v>
+        <v>0.07475826716118834</v>
       </c>
       <c r="R81" t="n">
-        <v>0.1077060216576887</v>
+        <v>0.1077060216576888</v>
       </c>
       <c r="S81" t="n">
         <v>0.1030255051232642</v>
@@ -5737,7 +5737,7 @@
         <v>2.295126493131328</v>
       </c>
       <c r="I83" t="n">
-        <v>2.836273562241488</v>
+        <v>2.836273562241487</v>
       </c>
       <c r="J83" t="n">
         <v>2.417174992534311</v>
@@ -5758,10 +5758,10 @@
         <v>5.75971813586441</v>
       </c>
       <c r="P83" t="n">
-        <v>6.161777009505934</v>
+        <v>6.161777009505935</v>
       </c>
       <c r="Q83" t="n">
-        <v>5.259860609033285</v>
+        <v>5.259860609033284</v>
       </c>
       <c r="R83" t="n">
         <v>6.622326851860395</v>
@@ -5770,7 +5770,7 @@
         <v>7.043896003059909</v>
       </c>
       <c r="T83" t="n">
-        <v>7.089961413254846</v>
+        <v>7.089961413254847</v>
       </c>
     </row>
     <row r="84">
@@ -5783,28 +5783,28 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>0.2770257419772108</v>
+        <v>0.2770257419772107</v>
       </c>
       <c r="D84" t="n">
         <v>0.2565259353815104</v>
       </c>
       <c r="E84" t="n">
-        <v>0.2989229648615855</v>
+        <v>0.2989229648615854</v>
       </c>
       <c r="F84" t="n">
-        <v>0.2793423110584456</v>
+        <v>0.2793423110584455</v>
       </c>
       <c r="G84" t="n">
         <v>0.3009511868359865</v>
       </c>
       <c r="H84" t="n">
-        <v>0.5183574239175386</v>
+        <v>0.5183574239175387</v>
       </c>
       <c r="I84" t="n">
-        <v>0.5324069396702634</v>
+        <v>0.5324069396702635</v>
       </c>
       <c r="J84" t="n">
-        <v>0.4822571045037669</v>
+        <v>0.4822571045037668</v>
       </c>
       <c r="K84" t="n">
         <v>0.4533326189723015</v>
@@ -5813,10 +5813,10 @@
         <v>0.5749132562661738</v>
       </c>
       <c r="M84" t="n">
-        <v>0.582268809677139</v>
+        <v>0.5822688096771389</v>
       </c>
       <c r="N84" t="n">
-        <v>0.5583936066807865</v>
+        <v>0.5583936066807866</v>
       </c>
       <c r="O84" t="n">
         <v>1.244031089143612</v>
@@ -5932,7 +5932,7 @@
         <v>0.2180784732951097</v>
       </c>
       <c r="J86" t="n">
-        <v>0.1927303369778628</v>
+        <v>0.1927303369778627</v>
       </c>
       <c r="K86" t="n">
         <v>0.1846386056041955</v>
@@ -5947,19 +5947,19 @@
         <v>0.226086820747178</v>
       </c>
       <c r="O86" t="n">
-        <v>0.322453758627139</v>
+        <v>0.3224537586271389</v>
       </c>
       <c r="P86" t="n">
-        <v>0.3560990120076208</v>
+        <v>0.3560990120076207</v>
       </c>
       <c r="Q86" t="n">
         <v>0.3196776778397661</v>
       </c>
       <c r="R86" t="n">
-        <v>0.4097704078995275</v>
+        <v>0.4097704078995276</v>
       </c>
       <c r="S86" t="n">
-        <v>0.4207049694510192</v>
+        <v>0.4207049694510193</v>
       </c>
       <c r="T86" t="n">
         <v>0.4153735254923928</v>
@@ -6045,7 +6045,7 @@
         <v>2.538532243285527</v>
       </c>
       <c r="E88" t="n">
-        <v>2.908891485579277</v>
+        <v>2.908891485579278</v>
       </c>
       <c r="F88" t="n">
         <v>2.422515020312858</v>
@@ -6054,19 +6054,19 @@
         <v>2.870062409272608</v>
       </c>
       <c r="H88" t="n">
-        <v>2.383001338813016</v>
+        <v>2.383001338813015</v>
       </c>
       <c r="I88" t="n">
-        <v>3.858926552936152</v>
+        <v>3.858926552936151</v>
       </c>
       <c r="J88" t="n">
         <v>2.841505409250779</v>
       </c>
       <c r="K88" t="n">
-        <v>3.198134969623061</v>
+        <v>3.198134969623062</v>
       </c>
       <c r="L88" t="n">
-        <v>3.504481677827541</v>
+        <v>3.50448167782754</v>
       </c>
       <c r="M88" t="n">
         <v>3.316017731220082</v>
@@ -6078,7 +6078,7 @@
         <v>4.943137742464317</v>
       </c>
       <c r="P88" t="n">
-        <v>4.685707881822316</v>
+        <v>4.685707881822317</v>
       </c>
       <c r="Q88" t="n">
         <v>4.189688856175836</v>
@@ -6087,10 +6087,10 @@
         <v>4.065838664408862</v>
       </c>
       <c r="S88" t="n">
-        <v>3.739191187375784</v>
+        <v>3.739191187375785</v>
       </c>
       <c r="T88" t="n">
-        <v>4.751524031734838</v>
+        <v>4.751524031734837</v>
       </c>
     </row>
     <row r="89">
@@ -6295,19 +6295,19 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>0.08625592042688514</v>
+        <v>0.08625592042688515</v>
       </c>
       <c r="D92" t="n">
-        <v>0.07801647536873967</v>
+        <v>0.07801647536873964</v>
       </c>
       <c r="E92" t="n">
         <v>0.07845602979168247</v>
       </c>
       <c r="F92" t="n">
-        <v>0.07100647611221501</v>
+        <v>0.07100647611221503</v>
       </c>
       <c r="G92" t="n">
-        <v>0.07898176447289912</v>
+        <v>0.0789817644728991</v>
       </c>
       <c r="H92" t="n">
         <v>0.0661880222322547</v>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>0.7712787491124983</v>
+        <v>0.7712787491124984</v>
       </c>
       <c r="D93" t="n">
         <v>0.6554054395758764</v>
@@ -6371,7 +6371,7 @@
         <v>0.5143752206739165</v>
       </c>
       <c r="G93" t="n">
-        <v>0.547505922225374</v>
+        <v>0.5475059222253742</v>
       </c>
       <c r="H93" t="n">
         <v>1.047038876766988</v>
@@ -6380,10 +6380,10 @@
         <v>0.9282720152435452</v>
       </c>
       <c r="J93" t="n">
-        <v>0.7557886439370869</v>
+        <v>0.755788643937087</v>
       </c>
       <c r="K93" t="n">
-        <v>0.7292431431132188</v>
+        <v>0.7292431431132189</v>
       </c>
       <c r="L93" t="n">
         <v>0.7961537520618309</v>
@@ -6441,25 +6441,25 @@
         <v>0.2354046684687308</v>
       </c>
       <c r="I94" t="n">
-        <v>0.4290254973591948</v>
+        <v>0.4290254973591949</v>
       </c>
       <c r="J94" t="n">
         <v>0.3558618120515695</v>
       </c>
       <c r="K94" t="n">
-        <v>0.3998182305580216</v>
+        <v>0.3998182305580217</v>
       </c>
       <c r="L94" t="n">
-        <v>0.4546009389174043</v>
+        <v>0.4546009389174042</v>
       </c>
       <c r="M94" t="n">
-        <v>0.3934110076782731</v>
+        <v>0.393411007678273</v>
       </c>
       <c r="N94" t="n">
         <v>0.4517372060521735</v>
       </c>
       <c r="O94" t="n">
-        <v>0.6649306411617701</v>
+        <v>0.6649306411617704</v>
       </c>
       <c r="P94" t="n">
         <v>0.6484568813828581</v>
@@ -6471,10 +6471,10 @@
         <v>0.7322264340903725</v>
       </c>
       <c r="S94" t="n">
-        <v>0.6217817696471721</v>
+        <v>0.621781769647172</v>
       </c>
       <c r="T94" t="n">
-        <v>0.6860214198591614</v>
+        <v>0.6860214198591617</v>
       </c>
     </row>
     <row r="95">
@@ -6523,10 +6523,10 @@
         <v>0.5569789107032853</v>
       </c>
       <c r="O95" t="n">
-        <v>0.6782095792201265</v>
+        <v>0.6782095792201264</v>
       </c>
       <c r="P95" t="n">
-        <v>0.7640684764955331</v>
+        <v>0.764068476495533</v>
       </c>
       <c r="Q95" t="n">
         <v>0.5961390988133128</v>
@@ -6538,7 +6538,7 @@
         <v>0.6336853379094591</v>
       </c>
       <c r="T95" t="n">
-        <v>0.6727509710144709</v>
+        <v>0.672750971014471</v>
       </c>
     </row>
     <row r="96">
@@ -6560,10 +6560,10 @@
         <v>0.1323373448024628</v>
       </c>
       <c r="F96" t="n">
-        <v>0.1350146240585985</v>
+        <v>0.1350146240585984</v>
       </c>
       <c r="G96" t="n">
-        <v>0.1517260826395598</v>
+        <v>0.1517260826395599</v>
       </c>
       <c r="H96" t="n">
         <v>0.2222941311482099</v>
@@ -6590,13 +6590,13 @@
         <v>0.5207305060998288</v>
       </c>
       <c r="P96" t="n">
-        <v>0.461269311143139</v>
+        <v>0.4612693111431391</v>
       </c>
       <c r="Q96" t="n">
         <v>0.45657478758342</v>
       </c>
       <c r="R96" t="n">
-        <v>0.5965024187343203</v>
+        <v>0.5965024187343202</v>
       </c>
       <c r="S96" t="n">
         <v>0.6045335162258804</v>
@@ -6627,13 +6627,13 @@
         <v>0.0304712767108469</v>
       </c>
       <c r="G97" t="n">
-        <v>0.03234292294534803</v>
+        <v>0.03234292294534802</v>
       </c>
       <c r="H97" t="n">
         <v>0.02952461267833622</v>
       </c>
       <c r="I97" t="n">
-        <v>0.0480636625989249</v>
+        <v>0.04806366259892491</v>
       </c>
       <c r="J97" t="n">
         <v>0.04176296972431984</v>
@@ -6642,7 +6642,7 @@
         <v>0.04237198931489834</v>
       </c>
       <c r="L97" t="n">
-        <v>0.05996663682789352</v>
+        <v>0.05996663682789351</v>
       </c>
       <c r="M97" t="n">
         <v>0.05482763187810819</v>
@@ -6694,16 +6694,16 @@
         <v>0.06379327013865761</v>
       </c>
       <c r="H98" t="n">
-        <v>0.07879256798772689</v>
+        <v>0.07879256798772688</v>
       </c>
       <c r="I98" t="n">
         <v>0.1045954781126142</v>
       </c>
       <c r="J98" t="n">
-        <v>0.08387857574106962</v>
+        <v>0.08387857574106961</v>
       </c>
       <c r="K98" t="n">
-        <v>0.08982486574616703</v>
+        <v>0.08982486574616702</v>
       </c>
       <c r="L98" t="n">
         <v>0.1141302357486455</v>
@@ -6712,7 +6712,7 @@
         <v>0.1101661804162813</v>
       </c>
       <c r="N98" t="n">
-        <v>0.1141678410423172</v>
+        <v>0.1141678410423171</v>
       </c>
       <c r="O98" t="n">
         <v>0.1994971335262662</v>
@@ -6721,13 +6721,13 @@
         <v>0.2110116619531146</v>
       </c>
       <c r="Q98" t="n">
-        <v>0.1906983546248198</v>
+        <v>0.1906983546248199</v>
       </c>
       <c r="R98" t="n">
-        <v>0.2374188615686211</v>
+        <v>0.2374188615686212</v>
       </c>
       <c r="S98" t="n">
-        <v>0.2210279956493578</v>
+        <v>0.2210279956493577</v>
       </c>
       <c r="T98" t="n">
         <v>0.2400608097112797</v>
@@ -6743,7 +6743,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.03924334014375773</v>
+        <v>0.03924334014375772</v>
       </c>
       <c r="D99" t="n">
         <v>0.03380927103038552</v>
@@ -6755,7 +6755,7 @@
         <v>0.04217129168419489</v>
       </c>
       <c r="G99" t="n">
-        <v>0.0440196897631256</v>
+        <v>0.04401968976312559</v>
       </c>
       <c r="H99" t="n">
         <v>0.05254094076605902</v>
@@ -6764,28 +6764,28 @@
         <v>0.0747091262953315</v>
       </c>
       <c r="J99" t="n">
-        <v>0.06733240946347598</v>
+        <v>0.067332409463476</v>
       </c>
       <c r="K99" t="n">
-        <v>0.06364515952936126</v>
+        <v>0.06364515952936124</v>
       </c>
       <c r="L99" t="n">
-        <v>0.07579122685742141</v>
+        <v>0.07579122685742143</v>
       </c>
       <c r="M99" t="n">
         <v>0.07194246703752807</v>
       </c>
       <c r="N99" t="n">
-        <v>0.07706706696222779</v>
+        <v>0.07706706696222777</v>
       </c>
       <c r="O99" t="n">
         <v>0.1325393248572746</v>
       </c>
       <c r="P99" t="n">
-        <v>0.1329179924229129</v>
+        <v>0.132917992422913</v>
       </c>
       <c r="Q99" t="n">
-        <v>0.1265788327576677</v>
+        <v>0.1265788327576678</v>
       </c>
       <c r="R99" t="n">
         <v>0.1629636241676406</v>
@@ -6843,7 +6843,7 @@
         <v>0.1423387145656542</v>
       </c>
       <c r="O100" t="n">
-        <v>0.2211778329946828</v>
+        <v>0.2211778329946829</v>
       </c>
       <c r="P100" t="n">
         <v>0.2202221022944229</v>
@@ -6858,7 +6858,7 @@
         <v>0.2482454406371755</v>
       </c>
       <c r="T100" t="n">
-        <v>0.2777215853373123</v>
+        <v>0.2777215853373122</v>
       </c>
     </row>
     <row r="101">
@@ -6889,10 +6889,10 @@
         <v>0.1311580633096534</v>
       </c>
       <c r="I101" t="n">
-        <v>0.2290820351158966</v>
+        <v>0.2290820351158967</v>
       </c>
       <c r="J101" t="n">
-        <v>0.1781750935030691</v>
+        <v>0.1781750935030692</v>
       </c>
       <c r="K101" t="n">
         <v>0.2092120902187607</v>
@@ -6919,7 +6919,7 @@
         <v>0.4274906209236122</v>
       </c>
       <c r="S101" t="n">
-        <v>0.4465436722764186</v>
+        <v>0.4465436722764185</v>
       </c>
       <c r="T101" t="n">
         <v>0.4796167721842459</v>
@@ -7008,7 +7008,7 @@
         <v>0.03283430285606561</v>
       </c>
       <c r="F103" t="n">
-        <v>0.03293331674025694</v>
+        <v>0.03293331674025695</v>
       </c>
       <c r="G103" t="n">
         <v>0.03026795626806312</v>
@@ -7035,22 +7035,22 @@
         <v>0.0503209612435476</v>
       </c>
       <c r="O103" t="n">
-        <v>0.07507512349838727</v>
+        <v>0.07507512349838728</v>
       </c>
       <c r="P103" t="n">
-        <v>0.07287907595229684</v>
+        <v>0.07287907595229685</v>
       </c>
       <c r="Q103" t="n">
-        <v>0.07541772980031555</v>
+        <v>0.07541772980031558</v>
       </c>
       <c r="R103" t="n">
-        <v>0.09691409456915476</v>
+        <v>0.09691409456915474</v>
       </c>
       <c r="S103" t="n">
         <v>0.08907585487301589</v>
       </c>
       <c r="T103" t="n">
-        <v>0.08549185195936546</v>
+        <v>0.08549185195936547</v>
       </c>
     </row>
     <row r="104">
@@ -7075,10 +7075,10 @@
         <v>0.08391294348413214</v>
       </c>
       <c r="G104" t="n">
-        <v>0.0867781545249897</v>
+        <v>0.08677815452498969</v>
       </c>
       <c r="H104" t="n">
-        <v>0.07192861573448958</v>
+        <v>0.0719286157344896</v>
       </c>
       <c r="I104" t="n">
         <v>0.1166249447041498</v>
@@ -7099,7 +7099,7 @@
         <v>0.1258960182297028</v>
       </c>
       <c r="O104" t="n">
-        <v>0.1809315018351127</v>
+        <v>0.1809315018351128</v>
       </c>
       <c r="P104" t="n">
         <v>0.1805709191206047</v>
@@ -7108,7 +7108,7 @@
         <v>0.1705255841763265</v>
       </c>
       <c r="R104" t="n">
-        <v>0.1910374347783412</v>
+        <v>0.1910374347783411</v>
       </c>
       <c r="S104" t="n">
         <v>0.1906562970796666</v>
@@ -7139,10 +7139,10 @@
         <v>0.08509178210180696</v>
       </c>
       <c r="G105" t="n">
-        <v>0.08899277775636993</v>
+        <v>0.08899277775636995</v>
       </c>
       <c r="H105" t="n">
-        <v>0.09096147026331741</v>
+        <v>0.0909614702633174</v>
       </c>
       <c r="I105" t="n">
         <v>0.1374754101796</v>
@@ -7197,7 +7197,7 @@
         <v>0.186493448869881</v>
       </c>
       <c r="E106" t="n">
-        <v>0.2165407554716994</v>
+        <v>0.2165407554716995</v>
       </c>
       <c r="F106" t="n">
         <v>0.1744340902489996</v>
@@ -7221,7 +7221,7 @@
         <v>0.2570087429472243</v>
       </c>
       <c r="M106" t="n">
-        <v>0.2617282182589088</v>
+        <v>0.2617282182589089</v>
       </c>
       <c r="N106" t="n">
         <v>0.2794040744160127</v>
@@ -7279,13 +7279,13 @@
         <v>0.07030848800768889</v>
       </c>
       <c r="K107" t="n">
-        <v>0.06896695079849764</v>
+        <v>0.06896695079849763</v>
       </c>
       <c r="L107" t="n">
         <v>0.06449414900494278</v>
       </c>
       <c r="M107" t="n">
-        <v>0.07345723056398124</v>
+        <v>0.07345723056398122</v>
       </c>
       <c r="N107" t="n">
         <v>0.0678873037541696</v>
@@ -7322,25 +7322,25 @@
         <v>0.5101234225125985</v>
       </c>
       <c r="D108" t="n">
-        <v>0.4630616644207624</v>
+        <v>0.4630616644207623</v>
       </c>
       <c r="E108" t="n">
-        <v>0.4783541097144987</v>
+        <v>0.4783541097144988</v>
       </c>
       <c r="F108" t="n">
-        <v>0.4454307220511722</v>
+        <v>0.4454307220511723</v>
       </c>
       <c r="G108" t="n">
-        <v>0.4655193486598914</v>
+        <v>0.4655193486598913</v>
       </c>
       <c r="H108" t="n">
-        <v>0.5454465916869446</v>
+        <v>0.5454465916869444</v>
       </c>
       <c r="I108" t="n">
-        <v>0.6746552088366983</v>
+        <v>0.6746552088366982</v>
       </c>
       <c r="J108" t="n">
-        <v>0.5943378617017551</v>
+        <v>0.594337861701755</v>
       </c>
       <c r="K108" t="n">
         <v>0.6000502950882362</v>
@@ -7349,7 +7349,7 @@
         <v>0.6682684462619436</v>
       </c>
       <c r="M108" t="n">
-        <v>0.6590412161994201</v>
+        <v>0.6590412161994198</v>
       </c>
       <c r="N108" t="n">
         <v>0.7035790012512178</v>
@@ -7422,7 +7422,7 @@
         <v>0.007017540010765875</v>
       </c>
       <c r="P109" t="n">
-        <v>0.006791461285416963</v>
+        <v>0.006791461285416964</v>
       </c>
       <c r="Q109" t="n">
         <v>0.006974414556841088</v>
@@ -7483,7 +7483,7 @@
         <v>0.1932500887452609</v>
       </c>
       <c r="O110" t="n">
-        <v>0.3133784444673173</v>
+        <v>0.3133784444673172</v>
       </c>
       <c r="P110" t="n">
         <v>0.3451279815988144</v>
@@ -7514,16 +7514,16 @@
         <v>2.428072989809201</v>
       </c>
       <c r="D111" t="n">
-        <v>2.216055675415121</v>
+        <v>2.21605567541512</v>
       </c>
       <c r="E111" t="n">
-        <v>2.306171217997635</v>
+        <v>2.306171217997636</v>
       </c>
       <c r="F111" t="n">
-        <v>1.90903660240935</v>
+        <v>1.909036602409349</v>
       </c>
       <c r="G111" t="n">
-        <v>2.046169947757326</v>
+        <v>2.046169947757327</v>
       </c>
       <c r="H111" t="n">
         <v>2.5330853397156</v>
@@ -7538,19 +7538,19 @@
         <v>2.608279296657933</v>
       </c>
       <c r="L111" t="n">
-        <v>2.885856698444892</v>
+        <v>2.885856698444893</v>
       </c>
       <c r="M111" t="n">
-        <v>2.743713024582892</v>
+        <v>2.743713024582891</v>
       </c>
       <c r="N111" t="n">
         <v>2.783543866216574</v>
       </c>
       <c r="O111" t="n">
-        <v>4.423906837336294</v>
+        <v>4.423906837336295</v>
       </c>
       <c r="P111" t="n">
-        <v>4.353706378088149</v>
+        <v>4.35370637808815</v>
       </c>
       <c r="Q111" t="n">
         <v>4.206431133111779</v>
@@ -7559,7 +7559,7 @@
         <v>4.926163053362603</v>
       </c>
       <c r="S111" t="n">
-        <v>5.34815578678483</v>
+        <v>5.348155786784831</v>
       </c>
       <c r="T111" t="n">
         <v>5.343083739330379</v>
@@ -7605,7 +7605,7 @@
         <v>0.2106602483431021</v>
       </c>
       <c r="M112" t="n">
-        <v>0.2223755308085498</v>
+        <v>0.2223755308085499</v>
       </c>
       <c r="N112" t="n">
         <v>0.2170466243168654</v>
@@ -7626,7 +7626,7 @@
         <v>0.4663618835657086</v>
       </c>
       <c r="T112" t="n">
-        <v>0.487113246050039</v>
+        <v>0.4871132460500389</v>
       </c>
     </row>
     <row r="113">
@@ -7660,7 +7660,7 @@
         <v>0.04874797363411498</v>
       </c>
       <c r="J113" t="n">
-        <v>0.04241619021635765</v>
+        <v>0.04241619021635766</v>
       </c>
       <c r="K113" t="n">
         <v>0.04037746642106956</v>
@@ -7678,10 +7678,10 @@
         <v>0.08287078400642736</v>
       </c>
       <c r="P113" t="n">
-        <v>0.08996835551590758</v>
+        <v>0.08996835551590757</v>
       </c>
       <c r="Q113" t="n">
-        <v>0.0898961334915731</v>
+        <v>0.08989613349157312</v>
       </c>
       <c r="R113" t="n">
         <v>0.1093438533910073</v>
@@ -7718,7 +7718,7 @@
         <v>0.01405106662459578</v>
       </c>
       <c r="H114" t="n">
-        <v>0.02317985066823312</v>
+        <v>0.02317985066823313</v>
       </c>
       <c r="I114" t="n">
         <v>0.02220003525830457</v>
@@ -7742,7 +7742,7 @@
         <v>0.03957516619987031</v>
       </c>
       <c r="P114" t="n">
-        <v>0.04528211890752491</v>
+        <v>0.0452821189075249</v>
       </c>
       <c r="Q114" t="n">
         <v>0.04274963930216526</v>
@@ -7751,10 +7751,10 @@
         <v>0.054784359252892</v>
       </c>
       <c r="S114" t="n">
-        <v>0.04887452673400481</v>
+        <v>0.04887452673400482</v>
       </c>
       <c r="T114" t="n">
-        <v>0.04519846555700199</v>
+        <v>0.04519846555700198</v>
       </c>
     </row>
     <row r="115">
@@ -7770,7 +7770,7 @@
         <v>0.2882826782378188</v>
       </c>
       <c r="D115" t="n">
-        <v>0.2596177988731838</v>
+        <v>0.2596177988731837</v>
       </c>
       <c r="E115" t="n">
         <v>0.2643634038236027</v>
@@ -7803,7 +7803,7 @@
         <v>0.4226519572721288</v>
       </c>
       <c r="O115" t="n">
-        <v>0.755089749759567</v>
+        <v>0.7550897497595671</v>
       </c>
       <c r="P115" t="n">
         <v>0.7370437127873851</v>
@@ -7831,28 +7831,28 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>0.09242939732681776</v>
+        <v>0.09242939732681775</v>
       </c>
       <c r="D116" t="n">
-        <v>0.0830215154054517</v>
+        <v>0.08302151540545169</v>
       </c>
       <c r="E116" t="n">
         <v>0.0870420491802058</v>
       </c>
       <c r="F116" t="n">
-        <v>0.07737431620378393</v>
+        <v>0.0773743162037839</v>
       </c>
       <c r="G116" t="n">
-        <v>0.08321588227671042</v>
+        <v>0.08321588227671044</v>
       </c>
       <c r="H116" t="n">
-        <v>0.08613127181832982</v>
+        <v>0.0861312718183298</v>
       </c>
       <c r="I116" t="n">
         <v>0.1109691571948775</v>
       </c>
       <c r="J116" t="n">
-        <v>0.09223783201410281</v>
+        <v>0.09223783201410282</v>
       </c>
       <c r="K116" t="n">
         <v>0.09876486462459264</v>
@@ -7861,19 +7861,19 @@
         <v>0.1049099458252576</v>
       </c>
       <c r="M116" t="n">
-        <v>0.1050776726829563</v>
+        <v>0.1050776726829564</v>
       </c>
       <c r="N116" t="n">
         <v>0.1131739929662637</v>
       </c>
       <c r="O116" t="n">
-        <v>0.1643653690071008</v>
+        <v>0.1643653690071009</v>
       </c>
       <c r="P116" t="n">
         <v>0.1650313945374654</v>
       </c>
       <c r="Q116" t="n">
-        <v>0.1583141723984233</v>
+        <v>0.1583141723984232</v>
       </c>
       <c r="R116" t="n">
         <v>0.1729668912227956</v>
@@ -7904,7 +7904,7 @@
         <v>0.04344081938351101</v>
       </c>
       <c r="F117" t="n">
-        <v>0.04909478044309923</v>
+        <v>0.04909478044309922</v>
       </c>
       <c r="G117" t="n">
         <v>0.03831377203608224</v>
@@ -7919,16 +7919,16 @@
         <v>0.07422423305444274</v>
       </c>
       <c r="K117" t="n">
-        <v>0.08741121325958066</v>
+        <v>0.08741121325958065</v>
       </c>
       <c r="L117" t="n">
         <v>0.09519134926709452</v>
       </c>
       <c r="M117" t="n">
-        <v>0.0897456257891253</v>
+        <v>0.08974562578912532</v>
       </c>
       <c r="N117" t="n">
-        <v>0.06957787094727197</v>
+        <v>0.06957787094727198</v>
       </c>
       <c r="O117" t="n">
         <v>0.184134835247514</v>
@@ -8023,7 +8023,7 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>0.2925431235820296</v>
+        <v>0.2925431235820297</v>
       </c>
       <c r="D119" t="n">
         <v>0.2459295862975192</v>
@@ -8035,7 +8035,7 @@
         <v>0.3117246836364982</v>
       </c>
       <c r="G119" t="n">
-        <v>0.3285180159785942</v>
+        <v>0.3285180159785941</v>
       </c>
       <c r="H119" t="n">
         <v>0.3152239826089193</v>
@@ -8053,13 +8053,13 @@
         <v>0.5918819885997834</v>
       </c>
       <c r="M119" t="n">
-        <v>0.5435166559557554</v>
+        <v>0.5435166559557555</v>
       </c>
       <c r="N119" t="n">
         <v>0.6030104600436829</v>
       </c>
       <c r="O119" t="n">
-        <v>0.8847711651821888</v>
+        <v>0.8847711651821889</v>
       </c>
       <c r="P119" t="n">
         <v>0.9358240422108777</v>
@@ -8090,10 +8090,10 @@
         <v>36.39399150982232</v>
       </c>
       <c r="D120" t="n">
-        <v>31.6852964161284</v>
+        <v>31.68529641612839</v>
       </c>
       <c r="E120" t="n">
-        <v>33.57958085110324</v>
+        <v>33.57958085110323</v>
       </c>
       <c r="F120" t="n">
         <v>31.78928049077359</v>
@@ -8105,19 +8105,19 @@
         <v>46.04880265413406</v>
       </c>
       <c r="I120" t="n">
-        <v>55.72667963150798</v>
+        <v>55.72667963150799</v>
       </c>
       <c r="J120" t="n">
-        <v>46.88073909451126</v>
+        <v>46.88073909451125</v>
       </c>
       <c r="K120" t="n">
-        <v>46.06991967003137</v>
+        <v>46.06991967003136</v>
       </c>
       <c r="L120" t="n">
-        <v>66.86606208878894</v>
+        <v>66.86606208878895</v>
       </c>
       <c r="M120" t="n">
-        <v>64.62088792362663</v>
+        <v>64.6208879236266</v>
       </c>
       <c r="N120" t="n">
         <v>59.94315758148488</v>
@@ -8132,7 +8132,7 @@
         <v>148.0693184042884</v>
       </c>
       <c r="R120" t="n">
-        <v>239.3649296795553</v>
+        <v>239.3649296795552</v>
       </c>
       <c r="S120" t="n">
         <v>253.2538501704686</v>
@@ -8254,7 +8254,7 @@
         <v>0.05268373050962067</v>
       </c>
       <c r="P122" t="n">
-        <v>0.05704856430363185</v>
+        <v>0.05704856430363184</v>
       </c>
       <c r="Q122" t="n">
         <v>0.04092794229738319</v>
@@ -8282,10 +8282,10 @@
         <v>0.9399657643332729</v>
       </c>
       <c r="D123" t="n">
-        <v>0.870052769897893</v>
+        <v>0.8700527698978928</v>
       </c>
       <c r="E123" t="n">
-        <v>0.8946711411131362</v>
+        <v>0.8946711411131363</v>
       </c>
       <c r="F123" t="n">
         <v>0.7474726080203441</v>
@@ -8294,7 +8294,7 @@
         <v>0.7737824462692394</v>
       </c>
       <c r="H123" t="n">
-        <v>0.9047812536436596</v>
+        <v>0.9047812536436597</v>
       </c>
       <c r="I123" t="n">
         <v>1.20360330990213</v>
@@ -8349,7 +8349,7 @@
         <v>0.5288835120296254</v>
       </c>
       <c r="E124" t="n">
-        <v>0.5413122800739332</v>
+        <v>0.5413122800739331</v>
       </c>
       <c r="F124" t="n">
         <v>0.5244515198697509</v>
@@ -8367,13 +8367,13 @@
         <v>0.6110722362148712</v>
       </c>
       <c r="K124" t="n">
-        <v>0.7190629827271918</v>
+        <v>0.7190629827271917</v>
       </c>
       <c r="L124" t="n">
         <v>0.758670705816567</v>
       </c>
       <c r="M124" t="n">
-        <v>0.7949750095406467</v>
+        <v>0.7949750095406468</v>
       </c>
       <c r="N124" t="n">
         <v>0.8005035758992184</v>
@@ -8431,7 +8431,7 @@
         <v>1.732914417703089</v>
       </c>
       <c r="K125" t="n">
-        <v>1.997007496237453</v>
+        <v>1.997007496237452</v>
       </c>
       <c r="L125" t="n">
         <v>2.241979550608346</v>
@@ -8455,10 +8455,10 @@
         <v>3.451556662640702</v>
       </c>
       <c r="S125" t="n">
-        <v>3.666081720345591</v>
+        <v>3.666081720345592</v>
       </c>
       <c r="T125" t="n">
-        <v>4.442412202303252</v>
+        <v>4.442412202303253</v>
       </c>
     </row>
     <row r="126">
@@ -8541,7 +8541,7 @@
         <v>0.1174769158937752</v>
       </c>
       <c r="E127" t="n">
-        <v>0.09986227523868141</v>
+        <v>0.09986227523868139</v>
       </c>
       <c r="F127" t="n">
         <v>0.1289563043001198</v>
@@ -8574,7 +8574,7 @@
         <v>0.4301833303193309</v>
       </c>
       <c r="P127" t="n">
-        <v>0.4379004654374033</v>
+        <v>0.4379004654374034</v>
       </c>
       <c r="Q127" t="n">
         <v>0.4891456530927932</v>
@@ -8608,7 +8608,7 @@
         <v>0.2455474380539036</v>
       </c>
       <c r="F128" t="n">
-        <v>0.2323648850570763</v>
+        <v>0.2323648850570762</v>
       </c>
       <c r="G128" t="n">
         <v>0.2507387602561719</v>
@@ -8626,7 +8626,7 @@
         <v>0.3039635694242478</v>
       </c>
       <c r="L128" t="n">
-        <v>0.3290283871870609</v>
+        <v>0.329028387187061</v>
       </c>
       <c r="M128" t="n">
         <v>0.3057712926624337</v>
@@ -8666,10 +8666,10 @@
         <v>0.08146352898443948</v>
       </c>
       <c r="D129" t="n">
-        <v>0.06766574952355979</v>
+        <v>0.06766574952355978</v>
       </c>
       <c r="E129" t="n">
-        <v>0.0680378082399042</v>
+        <v>0.06803780823990419</v>
       </c>
       <c r="F129" t="n">
         <v>0.06161345630372916</v>
@@ -8708,7 +8708,7 @@
         <v>0.1965387060236291</v>
       </c>
       <c r="R129" t="n">
-        <v>0.2520648794555279</v>
+        <v>0.252064879455528</v>
       </c>
       <c r="S129" t="n">
         <v>0.2563922259951701</v>
@@ -8739,7 +8739,7 @@
         <v>0.04963612267915252</v>
       </c>
       <c r="G130" t="n">
-        <v>0.05018501100116069</v>
+        <v>0.0501850110011607</v>
       </c>
       <c r="H130" t="n">
         <v>0.04899177943647669</v>
@@ -8757,10 +8757,10 @@
         <v>0.07093129061950607</v>
       </c>
       <c r="M130" t="n">
-        <v>0.07324323171672965</v>
+        <v>0.07324323171672967</v>
       </c>
       <c r="N130" t="n">
-        <v>0.07751611637523578</v>
+        <v>0.07751611637523577</v>
       </c>
       <c r="O130" t="n">
         <v>0.142358980203267</v>
@@ -8821,13 +8821,13 @@
         <v>0.2078554888761593</v>
       </c>
       <c r="M131" t="n">
-        <v>0.2024193901456537</v>
+        <v>0.2024193901456536</v>
       </c>
       <c r="N131" t="n">
         <v>0.2132299028777321</v>
       </c>
       <c r="O131" t="n">
-        <v>0.3364997309286671</v>
+        <v>0.3364997309286672</v>
       </c>
       <c r="P131" t="n">
         <v>0.3315956427584689</v>
@@ -8855,7 +8855,7 @@
         </is>
       </c>
       <c r="C132" t="n">
-        <v>0.08626191425146823</v>
+        <v>0.08626191425146824</v>
       </c>
       <c r="D132" t="n">
         <v>0.06897424787377004</v>
@@ -8867,7 +8867,7 @@
         <v>0.06981645244968782</v>
       </c>
       <c r="G132" t="n">
-        <v>0.07213817805808047</v>
+        <v>0.07213817805808045</v>
       </c>
       <c r="H132" t="n">
         <v>0.08460764374923067</v>
@@ -8879,7 +8879,7 @@
         <v>0.09530195386705362</v>
       </c>
       <c r="K132" t="n">
-        <v>0.09868430853697009</v>
+        <v>0.09868430853697011</v>
       </c>
       <c r="L132" t="n">
         <v>0.1153296513295421</v>
@@ -8891,10 +8891,10 @@
         <v>0.1138610377952679</v>
       </c>
       <c r="O132" t="n">
-        <v>0.1784285836989163</v>
+        <v>0.1784285836989162</v>
       </c>
       <c r="P132" t="n">
-        <v>0.1834864678085094</v>
+        <v>0.1834864678085093</v>
       </c>
       <c r="Q132" t="n">
         <v>0.184133170478274</v>
@@ -8925,7 +8925,7 @@
         <v>0.9242428050988843</v>
       </c>
       <c r="E133" t="n">
-        <v>1.098011482255052</v>
+        <v>1.098011482255053</v>
       </c>
       <c r="F133" t="n">
         <v>1.19648764895406</v>
@@ -8940,7 +8940,7 @@
         <v>2.038134390304134</v>
       </c>
       <c r="J133" t="n">
-        <v>1.765012107327488</v>
+        <v>1.765012107327487</v>
       </c>
       <c r="K133" t="n">
         <v>1.704248274815274</v>
@@ -8964,7 +8964,7 @@
         <v>4.648363209790867</v>
       </c>
       <c r="R133" t="n">
-        <v>6.918524389962566</v>
+        <v>6.918524389962565</v>
       </c>
       <c r="S133" t="n">
         <v>7.004429082625482</v>
@@ -8992,7 +8992,7 @@
         <v>0.003855378850455751</v>
       </c>
       <c r="F134" t="n">
-        <v>0.003265007207208154</v>
+        <v>0.003265007207208155</v>
       </c>
       <c r="G134" t="n">
         <v>0.003464109047324646</v>
@@ -9013,28 +9013,28 @@
         <v>0.004562543078647831</v>
       </c>
       <c r="M134" t="n">
-        <v>0.004425020456848928</v>
+        <v>0.004425020456848929</v>
       </c>
       <c r="N134" t="n">
         <v>0.004536615683405752</v>
       </c>
       <c r="O134" t="n">
-        <v>0.004000648607851965</v>
+        <v>0.004000648607851964</v>
       </c>
       <c r="P134" t="n">
         <v>0.00588903872533335</v>
       </c>
       <c r="Q134" t="n">
-        <v>0.004415197859653697</v>
+        <v>0.004415197859653696</v>
       </c>
       <c r="R134" t="n">
-        <v>0.005707098546805792</v>
+        <v>0.005707098546805793</v>
       </c>
       <c r="S134" t="n">
         <v>0.004711373892475688</v>
       </c>
       <c r="T134" t="n">
-        <v>0.006278111539059244</v>
+        <v>0.006278111539059245</v>
       </c>
     </row>
     <row r="135">
@@ -9047,7 +9047,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>0.03548847653947744</v>
+        <v>0.03548847653947745</v>
       </c>
       <c r="D135" t="n">
         <v>0.03354701671517744</v>
@@ -9062,13 +9062,13 @@
         <v>0.02459151769600704</v>
       </c>
       <c r="H135" t="n">
-        <v>0.02383153798852696</v>
+        <v>0.02383153798852695</v>
       </c>
       <c r="I135" t="n">
         <v>0.03311827583658793</v>
       </c>
       <c r="J135" t="n">
-        <v>0.0286805328324798</v>
+        <v>0.02868053283247979</v>
       </c>
       <c r="K135" t="n">
         <v>0.0286921302474362</v>
@@ -9083,19 +9083,19 @@
         <v>0.0403911500339118</v>
       </c>
       <c r="O135" t="n">
-        <v>0.07073018304569616</v>
+        <v>0.07073018304569614</v>
       </c>
       <c r="P135" t="n">
-        <v>0.07489858299237577</v>
+        <v>0.07489858299237576</v>
       </c>
       <c r="Q135" t="n">
-        <v>0.07529819277237361</v>
+        <v>0.07529819277237362</v>
       </c>
       <c r="R135" t="n">
-        <v>0.09120238656550907</v>
+        <v>0.09120238656550905</v>
       </c>
       <c r="S135" t="n">
-        <v>0.09123032222020941</v>
+        <v>0.09123032222020939</v>
       </c>
       <c r="T135" t="n">
         <v>0.09785536894197602</v>
@@ -9226,7 +9226,7 @@
         <v>0.05595093132880288</v>
       </c>
       <c r="T137" t="n">
-        <v>0.05795407950212631</v>
+        <v>0.0579540795021263</v>
       </c>
     </row>
     <row r="138">
@@ -9245,10 +9245,10 @@
         <v>0.01208350221848329</v>
       </c>
       <c r="E138" t="n">
-        <v>0.008234922781882594</v>
+        <v>0.008234922781882596</v>
       </c>
       <c r="F138" t="n">
-        <v>0.01200460420857307</v>
+        <v>0.01200460420857306</v>
       </c>
       <c r="G138" t="n">
         <v>0.01260922027339027</v>
@@ -9260,7 +9260,7 @@
         <v>0.01854040489564004</v>
       </c>
       <c r="J138" t="n">
-        <v>0.01369760695128816</v>
+        <v>0.01369760695128815</v>
       </c>
       <c r="K138" t="n">
         <v>0.01577380745401011</v>
@@ -9275,7 +9275,7 @@
         <v>0.01751248503811286</v>
       </c>
       <c r="O138" t="n">
-        <v>0.02887553248198015</v>
+        <v>0.02887553248198016</v>
       </c>
       <c r="P138" t="n">
         <v>0.01840053132977065</v>
@@ -9306,13 +9306,13 @@
         <v>0.01112961171932348</v>
       </c>
       <c r="D139" t="n">
-        <v>0.01097461440130991</v>
+        <v>0.01097461440130992</v>
       </c>
       <c r="E139" t="n">
-        <v>0.007180006235608428</v>
+        <v>0.007180006235608427</v>
       </c>
       <c r="F139" t="n">
-        <v>0.01057830314920887</v>
+        <v>0.01057830314920888</v>
       </c>
       <c r="G139" t="n">
         <v>0.01148385668877884</v>
@@ -9345,7 +9345,7 @@
         <v>0.01898963170037687</v>
       </c>
       <c r="Q139" t="n">
-        <v>0.02940148822047755</v>
+        <v>0.02940148822047754</v>
       </c>
       <c r="R139" t="n">
         <v>0.01936684133885338</v>

</xml_diff>

<commit_message>
fix: update part of scripts
</commit_message>
<xml_diff>
--- a/data/proteomics/membrane_size_across_compartment_Rosemary_NH4_limitation_v2.xlsx
+++ b/data/proteomics/membrane_size_across_compartment_Rosemary_NH4_limitation_v2.xlsx
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>175.2179951479614</v>
+        <v>175.2179951479613</v>
       </c>
       <c r="D2" t="n">
-        <v>160.0444973878102</v>
+        <v>160.0444973878098</v>
       </c>
       <c r="E2" t="n">
         <v>168.5410689658385</v>
@@ -547,34 +547,34 @@
         <v>132.4694784504293</v>
       </c>
       <c r="G2" t="n">
-        <v>138.9107551105769</v>
+        <v>138.9107551105768</v>
       </c>
       <c r="H2" t="n">
         <v>194.1516392720852</v>
       </c>
       <c r="I2" t="n">
-        <v>201.8798627229507</v>
+        <v>201.879862722951</v>
       </c>
       <c r="J2" t="n">
-        <v>173.7795767292694</v>
+        <v>173.7795767292693</v>
       </c>
       <c r="K2" t="n">
-        <v>176.5021655182089</v>
+        <v>176.5021655182091</v>
       </c>
       <c r="L2" t="n">
-        <v>188.3921197520449</v>
+        <v>188.392119752045</v>
       </c>
       <c r="M2" t="n">
-        <v>187.3070433279956</v>
+        <v>187.3070433279952</v>
       </c>
       <c r="N2" t="n">
-        <v>191.0380320703821</v>
+        <v>191.0380320703822</v>
       </c>
       <c r="O2" t="n">
-        <v>338.4823015571529</v>
+        <v>338.4823015571532</v>
       </c>
       <c r="P2" t="n">
-        <v>339.967903743154</v>
+        <v>339.9679037431537</v>
       </c>
       <c r="Q2" t="n">
         <v>316.4651507008168</v>
@@ -583,10 +583,10 @@
         <v>424.9728368360898</v>
       </c>
       <c r="S2" t="n">
-        <v>452.7732087518451</v>
+        <v>452.7732087518457</v>
       </c>
       <c r="T2" t="n">
-        <v>448.824728881924</v>
+        <v>448.8247288819236</v>
       </c>
     </row>
     <row r="3">
@@ -626,10 +626,10 @@
         <v>0.3400807864308382</v>
       </c>
       <c r="L3" t="n">
-        <v>0.3627065316307947</v>
+        <v>0.3627065316307946</v>
       </c>
       <c r="M3" t="n">
-        <v>0.3555703574112495</v>
+        <v>0.3555703574112494</v>
       </c>
       <c r="N3" t="n">
         <v>0.392498277599545</v>
@@ -641,13 +641,13 @@
         <v>0.5162502252648964</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.4992434495697612</v>
+        <v>0.4992434495697613</v>
       </c>
       <c r="R3" t="n">
         <v>0.578346559989949</v>
       </c>
       <c r="S3" t="n">
-        <v>0.6028096168457833</v>
+        <v>0.602809616845783</v>
       </c>
       <c r="T3" t="n">
         <v>0.5580478351504095</v>
@@ -663,7 +663,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.2768303852909353</v>
+        <v>0.2768303852909352</v>
       </c>
       <c r="D4" t="n">
         <v>0.2601275712257239</v>
@@ -672,19 +672,19 @@
         <v>0.2878897626554286</v>
       </c>
       <c r="F4" t="n">
-        <v>0.2751683226782103</v>
+        <v>0.2751683226782104</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2832108840463514</v>
+        <v>0.2832108840463513</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2900750027999565</v>
+        <v>0.2900750027999563</v>
       </c>
       <c r="I4" t="n">
         <v>0.4146122774205822</v>
       </c>
       <c r="J4" t="n">
-        <v>0.3471933041993003</v>
+        <v>0.3471933041993001</v>
       </c>
       <c r="K4" t="n">
         <v>0.3290448836663721</v>
@@ -693,28 +693,28 @@
         <v>0.3745999273268714</v>
       </c>
       <c r="M4" t="n">
-        <v>0.4151547571207964</v>
+        <v>0.4151547571207966</v>
       </c>
       <c r="N4" t="n">
         <v>0.4111555903524836</v>
       </c>
       <c r="O4" t="n">
-        <v>0.6506676470786709</v>
+        <v>0.6506676470786705</v>
       </c>
       <c r="P4" t="n">
-        <v>0.6913160163047212</v>
+        <v>0.6913160163047213</v>
       </c>
       <c r="Q4" t="n">
-        <v>0.6883910427175277</v>
+        <v>0.6883910427175275</v>
       </c>
       <c r="R4" t="n">
-        <v>0.8026681630801573</v>
+        <v>0.8026681630801574</v>
       </c>
       <c r="S4" t="n">
-        <v>0.9624695034230458</v>
+        <v>0.9624695034230457</v>
       </c>
       <c r="T4" t="n">
-        <v>0.9224246385322586</v>
+        <v>0.9224246385322584</v>
       </c>
     </row>
     <row r="5">
@@ -794,55 +794,55 @@
         <v>104.4945795180777</v>
       </c>
       <c r="D6" t="n">
-        <v>95.8133738922256</v>
+        <v>95.81337389222574</v>
       </c>
       <c r="E6" t="n">
-        <v>102.9450256576946</v>
+        <v>102.9450256576944</v>
       </c>
       <c r="F6" t="n">
-        <v>80.27718466102307</v>
+        <v>80.27718466102297</v>
       </c>
       <c r="G6" t="n">
-        <v>84.78600455617574</v>
+        <v>84.78600455617567</v>
       </c>
       <c r="H6" t="n">
-        <v>114.8174438999058</v>
+        <v>114.8174438999056</v>
       </c>
       <c r="I6" t="n">
-        <v>119.8186726907255</v>
+        <v>119.8186726907256</v>
       </c>
       <c r="J6" t="n">
-        <v>105.0651197106895</v>
+        <v>105.0651197106894</v>
       </c>
       <c r="K6" t="n">
         <v>103.9541102612538</v>
       </c>
       <c r="L6" t="n">
-        <v>107.1511386458312</v>
+        <v>107.1511386458313</v>
       </c>
       <c r="M6" t="n">
-        <v>108.7628022245243</v>
+        <v>108.7628022245245</v>
       </c>
       <c r="N6" t="n">
-        <v>110.3052217624944</v>
+        <v>110.3052217624946</v>
       </c>
       <c r="O6" t="n">
-        <v>197.5002617175619</v>
+        <v>197.5002617175616</v>
       </c>
       <c r="P6" t="n">
-        <v>199.9282717881694</v>
+        <v>199.9282717881698</v>
       </c>
       <c r="Q6" t="n">
-        <v>190.4890067392384</v>
+        <v>190.4890067392383</v>
       </c>
       <c r="R6" t="n">
-        <v>263.1742931654668</v>
+        <v>263.174293165467</v>
       </c>
       <c r="S6" t="n">
-        <v>283.6896214537362</v>
+        <v>283.6896214537356</v>
       </c>
       <c r="T6" t="n">
-        <v>269.2484509264085</v>
+        <v>269.2484509264082</v>
       </c>
     </row>
     <row r="7">
@@ -858,55 +858,55 @@
         <v>227.0895431527453</v>
       </c>
       <c r="D7" t="n">
-        <v>206.7361723285038</v>
+        <v>206.7361723285037</v>
       </c>
       <c r="E7" t="n">
-        <v>213.7851497908101</v>
+        <v>213.78514979081</v>
       </c>
       <c r="F7" t="n">
-        <v>176.2278896016976</v>
+        <v>176.2278896016973</v>
       </c>
       <c r="G7" t="n">
-        <v>186.3067644873685</v>
+        <v>186.3067644873686</v>
       </c>
       <c r="H7" t="n">
-        <v>256.187722819756</v>
+        <v>256.1877228197557</v>
       </c>
       <c r="I7" t="n">
-        <v>272.7578975486283</v>
+        <v>272.7578975486281</v>
       </c>
       <c r="J7" t="n">
-        <v>232.3532486181905</v>
+        <v>232.3532486181906</v>
       </c>
       <c r="K7" t="n">
-        <v>235.0706214611074</v>
+        <v>235.0706214611075</v>
       </c>
       <c r="L7" t="n">
-        <v>277.1407638493971</v>
+        <v>277.1407638493972</v>
       </c>
       <c r="M7" t="n">
-        <v>268.7329213330884</v>
+        <v>268.7329213330883</v>
       </c>
       <c r="N7" t="n">
-        <v>264.3676705543981</v>
+        <v>264.3676705543982</v>
       </c>
       <c r="O7" t="n">
         <v>550.9705103015149</v>
       </c>
       <c r="P7" t="n">
-        <v>550.81431448622</v>
+        <v>550.8143144862203</v>
       </c>
       <c r="Q7" t="n">
-        <v>531.8284565095471</v>
+        <v>531.8284565095472</v>
       </c>
       <c r="R7" t="n">
-        <v>759.0744330364066</v>
+        <v>759.0744330364084</v>
       </c>
       <c r="S7" t="n">
-        <v>797.3983425768849</v>
+        <v>797.3983425768851</v>
       </c>
       <c r="T7" t="n">
-        <v>785.7650879781927</v>
+        <v>785.7650879781916</v>
       </c>
     </row>
     <row r="8">
@@ -925,19 +925,19 @@
         <v>92.52612055309257</v>
       </c>
       <c r="E8" t="n">
-        <v>90.77862659703368</v>
+        <v>90.77862659703358</v>
       </c>
       <c r="F8" t="n">
-        <v>79.86886913329828</v>
+        <v>79.86886913329825</v>
       </c>
       <c r="G8" t="n">
-        <v>82.45308225254726</v>
+        <v>82.45308225254715</v>
       </c>
       <c r="H8" t="n">
         <v>124.7777434740009</v>
       </c>
       <c r="I8" t="n">
-        <v>122.9903899924765</v>
+        <v>122.9903899924766</v>
       </c>
       <c r="J8" t="n">
         <v>107.148589941707</v>
@@ -946,7 +946,7 @@
         <v>106.7000971377189</v>
       </c>
       <c r="L8" t="n">
-        <v>104.1523720523612</v>
+        <v>104.1523720523613</v>
       </c>
       <c r="M8" t="n">
         <v>106.3532786148637</v>
@@ -955,22 +955,22 @@
         <v>104.6966534357503</v>
       </c>
       <c r="O8" t="n">
-        <v>202.7461011100773</v>
+        <v>202.7461011100774</v>
       </c>
       <c r="P8" t="n">
-        <v>201.4705166773788</v>
+        <v>201.4705166773789</v>
       </c>
       <c r="Q8" t="n">
-        <v>197.1847244190117</v>
+        <v>197.1847244190116</v>
       </c>
       <c r="R8" t="n">
-        <v>277.970000071803</v>
+        <v>277.9700000718027</v>
       </c>
       <c r="S8" t="n">
         <v>308.774428820842</v>
       </c>
       <c r="T8" t="n">
-        <v>286.2343071236759</v>
+        <v>286.2343071236758</v>
       </c>
     </row>
     <row r="9">
@@ -986,19 +986,19 @@
         <v>29.33172266429985</v>
       </c>
       <c r="D9" t="n">
-        <v>27.36723455464774</v>
+        <v>27.36723455464773</v>
       </c>
       <c r="E9" t="n">
         <v>24.98386908080797</v>
       </c>
       <c r="F9" t="n">
-        <v>21.9400347466214</v>
+        <v>21.94003474662142</v>
       </c>
       <c r="G9" t="n">
         <v>23.26167918693907</v>
       </c>
       <c r="H9" t="n">
-        <v>33.77244137235143</v>
+        <v>33.77244137235142</v>
       </c>
       <c r="I9" t="n">
         <v>32.0449226823412</v>
@@ -1022,7 +1022,7 @@
         <v>51.92845623094195</v>
       </c>
       <c r="P9" t="n">
-        <v>49.64308423613162</v>
+        <v>49.64308423613163</v>
       </c>
       <c r="Q9" t="n">
         <v>55.17449330541861</v>
@@ -1111,19 +1111,19 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>44.88391858779398</v>
+        <v>44.88391858779397</v>
       </c>
       <c r="D11" t="n">
         <v>39.38859037636782</v>
       </c>
       <c r="E11" t="n">
-        <v>34.16741458109772</v>
+        <v>34.16741458109771</v>
       </c>
       <c r="F11" t="n">
-        <v>30.43728128847774</v>
+        <v>30.43728128847775</v>
       </c>
       <c r="G11" t="n">
-        <v>31.0882376660685</v>
+        <v>31.08823766606849</v>
       </c>
       <c r="H11" t="n">
         <v>57.4690929654988</v>
@@ -1141,7 +1141,7 @@
         <v>37.93758004013361</v>
       </c>
       <c r="M11" t="n">
-        <v>39.80559791450519</v>
+        <v>39.8055979145052</v>
       </c>
       <c r="N11" t="n">
         <v>34.32068342049713</v>
@@ -1184,28 +1184,28 @@
         <v>10.99321760413045</v>
       </c>
       <c r="F12" t="n">
-        <v>10.19134887106635</v>
+        <v>10.19134887106634</v>
       </c>
       <c r="G12" t="n">
-        <v>11.24906435751133</v>
+        <v>11.24906435751132</v>
       </c>
       <c r="H12" t="n">
-        <v>10.98161037407191</v>
+        <v>10.98161037407189</v>
       </c>
       <c r="I12" t="n">
-        <v>16.70952615798391</v>
+        <v>16.7095261579839</v>
       </c>
       <c r="J12" t="n">
         <v>14.11412453167334</v>
       </c>
       <c r="K12" t="n">
-        <v>15.01617979942496</v>
+        <v>15.01617979942495</v>
       </c>
       <c r="L12" t="n">
-        <v>17.19123215896572</v>
+        <v>17.19123215896573</v>
       </c>
       <c r="M12" t="n">
-        <v>15.97911802947151</v>
+        <v>15.9791180294715</v>
       </c>
       <c r="N12" t="n">
         <v>17.09755670687181</v>
@@ -1217,16 +1217,16 @@
         <v>27.18642336678111</v>
       </c>
       <c r="Q12" t="n">
-        <v>26.08149031429904</v>
+        <v>26.08149031429905</v>
       </c>
       <c r="R12" t="n">
-        <v>30.92416302141378</v>
+        <v>30.92416302141377</v>
       </c>
       <c r="S12" t="n">
         <v>33.67093013591801</v>
       </c>
       <c r="T12" t="n">
-        <v>34.87168598776996</v>
+        <v>34.87168598776997</v>
       </c>
     </row>
     <row r="13">
@@ -1239,13 +1239,13 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.594856480246183</v>
+        <v>1.594856480246182</v>
       </c>
       <c r="D13" t="n">
         <v>1.391237317232775</v>
       </c>
       <c r="E13" t="n">
-        <v>1.432905886592719</v>
+        <v>1.432905886592718</v>
       </c>
       <c r="F13" t="n">
         <v>1.483570131170016</v>
@@ -1257,7 +1257,7 @@
         <v>1.306216968593031</v>
       </c>
       <c r="I13" t="n">
-        <v>2.609410905571941</v>
+        <v>2.609410905571942</v>
       </c>
       <c r="J13" t="n">
         <v>2.100707647950022</v>
@@ -1275,19 +1275,19 @@
         <v>2.737326259186796</v>
       </c>
       <c r="O13" t="n">
-        <v>3.725108609580325</v>
+        <v>3.725108609580324</v>
       </c>
       <c r="P13" t="n">
         <v>3.445901137445752</v>
       </c>
       <c r="Q13" t="n">
-        <v>3.65493199032628</v>
+        <v>3.654931990326281</v>
       </c>
       <c r="R13" t="n">
-        <v>3.315162242105956</v>
+        <v>3.315162242105957</v>
       </c>
       <c r="S13" t="n">
-        <v>3.635938154208346</v>
+        <v>3.635938154208347</v>
       </c>
       <c r="T13" t="n">
         <v>3.986433630032791</v>
@@ -1303,10 +1303,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>8.834259072602102</v>
+        <v>8.834259072602103</v>
       </c>
       <c r="D14" t="n">
-        <v>8.706356576039495</v>
+        <v>8.706356576039489</v>
       </c>
       <c r="E14" t="n">
         <v>10.01133393430948</v>
@@ -1327,13 +1327,13 @@
         <v>9.556682794319098</v>
       </c>
       <c r="K14" t="n">
-        <v>9.332337557072194</v>
+        <v>9.332337557072195</v>
       </c>
       <c r="L14" t="n">
         <v>10.29327721599668</v>
       </c>
       <c r="M14" t="n">
-        <v>9.736310523820675</v>
+        <v>9.736310523820674</v>
       </c>
       <c r="N14" t="n">
         <v>10.64477255047419</v>
@@ -1348,13 +1348,13 @@
         <v>13.04493835903978</v>
       </c>
       <c r="R14" t="n">
-        <v>15.62250490095466</v>
+        <v>15.62250490095467</v>
       </c>
       <c r="S14" t="n">
         <v>16.78014764680844</v>
       </c>
       <c r="T14" t="n">
-        <v>17.08224206893462</v>
+        <v>17.08224206893463</v>
       </c>
     </row>
     <row r="15">
@@ -1388,7 +1388,7 @@
         <v>2.624838174111786</v>
       </c>
       <c r="J15" t="n">
-        <v>2.266429528365787</v>
+        <v>2.266429528365788</v>
       </c>
       <c r="K15" t="n">
         <v>2.061607512407088</v>
@@ -1409,16 +1409,16 @@
         <v>3.877453199129755</v>
       </c>
       <c r="Q15" t="n">
-        <v>3.020817851880673</v>
+        <v>3.020817851880674</v>
       </c>
       <c r="R15" t="n">
         <v>3.97830927028128</v>
       </c>
       <c r="S15" t="n">
-        <v>4.155985265138864</v>
+        <v>4.155985265138865</v>
       </c>
       <c r="T15" t="n">
-        <v>4.254430363801599</v>
+        <v>4.2544303638016</v>
       </c>
     </row>
     <row r="16">
@@ -1446,7 +1446,7 @@
         <v>1.805008251780691</v>
       </c>
       <c r="H16" t="n">
-        <v>1.393755151468504</v>
+        <v>1.393755151468505</v>
       </c>
       <c r="I16" t="n">
         <v>2.595010764878983</v>
@@ -1458,19 +1458,19 @@
         <v>2.301921450679949</v>
       </c>
       <c r="L16" t="n">
-        <v>2.732038197793636</v>
+        <v>2.732038197793635</v>
       </c>
       <c r="M16" t="n">
-        <v>2.626509281078438</v>
+        <v>2.626509281078437</v>
       </c>
       <c r="N16" t="n">
         <v>2.793978906999193</v>
       </c>
       <c r="O16" t="n">
-        <v>3.906260789134767</v>
+        <v>3.906260789134768</v>
       </c>
       <c r="P16" t="n">
-        <v>3.834332002907979</v>
+        <v>3.83433200290798</v>
       </c>
       <c r="Q16" t="n">
         <v>3.761919792796915</v>
@@ -1479,10 +1479,10 @@
         <v>4.253952706653428</v>
       </c>
       <c r="S16" t="n">
-        <v>4.352405875048257</v>
+        <v>4.352405875048256</v>
       </c>
       <c r="T16" t="n">
-        <v>5.006679935035802</v>
+        <v>5.006679935035803</v>
       </c>
     </row>
     <row r="17">
@@ -1495,7 +1495,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1.996263537016853</v>
+        <v>1.996263537016854</v>
       </c>
       <c r="D17" t="n">
         <v>1.425017628890765</v>
@@ -1507,7 +1507,7 @@
         <v>1.358581833911618</v>
       </c>
       <c r="G17" t="n">
-        <v>1.509385191841338</v>
+        <v>1.509385191841337</v>
       </c>
       <c r="H17" t="n">
         <v>1.625626647989878</v>
@@ -1522,10 +1522,10 @@
         <v>1.174927839986757</v>
       </c>
       <c r="L17" t="n">
-        <v>2.435216793887699</v>
+        <v>2.435216793887697</v>
       </c>
       <c r="M17" t="n">
-        <v>2.308095913657294</v>
+        <v>2.308095913657295</v>
       </c>
       <c r="N17" t="n">
         <v>2.353700718791571</v>
@@ -1540,13 +1540,13 @@
         <v>3.404364236056104</v>
       </c>
       <c r="R17" t="n">
-        <v>4.294364506259151</v>
+        <v>4.29436450625915</v>
       </c>
       <c r="S17" t="n">
-        <v>4.504509553137041</v>
+        <v>4.504509553137042</v>
       </c>
       <c r="T17" t="n">
-        <v>4.433210842194038</v>
+        <v>4.433210842194039</v>
       </c>
     </row>
     <row r="18">
@@ -1568,7 +1568,7 @@
         <v>2.251324005595607</v>
       </c>
       <c r="F18" t="n">
-        <v>2.131324671124971</v>
+        <v>2.131324671124972</v>
       </c>
       <c r="G18" t="n">
         <v>2.354784592268257</v>
@@ -1583,19 +1583,19 @@
         <v>2.827651824938835</v>
       </c>
       <c r="K18" t="n">
-        <v>3.247249273668732</v>
+        <v>3.247249273668733</v>
       </c>
       <c r="L18" t="n">
-        <v>3.585612856636333</v>
+        <v>3.585612856636332</v>
       </c>
       <c r="M18" t="n">
-        <v>3.431604030995716</v>
+        <v>3.431604030995715</v>
       </c>
       <c r="N18" t="n">
-        <v>3.538331749640751</v>
+        <v>3.53833174964075</v>
       </c>
       <c r="O18" t="n">
-        <v>5.88260745659845</v>
+        <v>5.882607456598449</v>
       </c>
       <c r="P18" t="n">
         <v>5.949131763719677</v>
@@ -1604,13 +1604,13 @@
         <v>5.595239687818301</v>
       </c>
       <c r="R18" t="n">
-        <v>7.203289999042921</v>
+        <v>7.203289999042922</v>
       </c>
       <c r="S18" t="n">
-        <v>8.735446391515648</v>
+        <v>8.735446391515651</v>
       </c>
       <c r="T18" t="n">
-        <v>9.028734150007701</v>
+        <v>9.028734150007699</v>
       </c>
     </row>
     <row r="19">
@@ -1623,16 +1623,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1.394618081475111</v>
+        <v>1.39461808147511</v>
       </c>
       <c r="D19" t="n">
-        <v>1.253350678060726</v>
+        <v>1.253350678060727</v>
       </c>
       <c r="E19" t="n">
         <v>1.282973572231973</v>
       </c>
       <c r="F19" t="n">
-        <v>1.248900046263694</v>
+        <v>1.248900046263693</v>
       </c>
       <c r="G19" t="n">
         <v>1.298498567442569</v>
@@ -1641,7 +1641,7 @@
         <v>1.422817663880669</v>
       </c>
       <c r="I19" t="n">
-        <v>2.007546775665483</v>
+        <v>2.007546775665482</v>
       </c>
       <c r="J19" t="n">
         <v>1.754853205190291</v>
@@ -1650,28 +1650,28 @@
         <v>1.750947455166642</v>
       </c>
       <c r="L19" t="n">
-        <v>2.033171827422394</v>
+        <v>2.033171827422393</v>
       </c>
       <c r="M19" t="n">
-        <v>1.965292494422672</v>
+        <v>1.965292494422673</v>
       </c>
       <c r="N19" t="n">
-        <v>2.033164831904401</v>
+        <v>2.0331648319044</v>
       </c>
       <c r="O19" t="n">
-        <v>3.169463582482697</v>
+        <v>3.169463582482698</v>
       </c>
       <c r="P19" t="n">
-        <v>3.224974770365975</v>
+        <v>3.224974770365971</v>
       </c>
       <c r="Q19" t="n">
         <v>3.067936579055761</v>
       </c>
       <c r="R19" t="n">
-        <v>4.038574819956989</v>
+        <v>4.038574819956988</v>
       </c>
       <c r="S19" t="n">
-        <v>4.206550290138672</v>
+        <v>4.206550290138673</v>
       </c>
       <c r="T19" t="n">
         <v>4.182635611530206</v>
@@ -1687,43 +1687,43 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4.335169502189708</v>
+        <v>4.335169502189711</v>
       </c>
       <c r="D20" t="n">
         <v>3.770735365092149</v>
       </c>
       <c r="E20" t="n">
-        <v>4.197775951766889</v>
+        <v>4.19777595176689</v>
       </c>
       <c r="F20" t="n">
-        <v>3.880091227827488</v>
+        <v>3.880091227827486</v>
       </c>
       <c r="G20" t="n">
-        <v>4.205488963910327</v>
+        <v>4.205488963910328</v>
       </c>
       <c r="H20" t="n">
         <v>5.342620371404053</v>
       </c>
       <c r="I20" t="n">
-        <v>6.275997977658262</v>
+        <v>6.275997977658263</v>
       </c>
       <c r="J20" t="n">
         <v>5.405688715368906</v>
       </c>
       <c r="K20" t="n">
-        <v>5.517800802999912</v>
+        <v>5.51780080299991</v>
       </c>
       <c r="L20" t="n">
-        <v>6.779577136475653</v>
+        <v>6.779577136475652</v>
       </c>
       <c r="M20" t="n">
-        <v>6.822938493470525</v>
+        <v>6.822938493470524</v>
       </c>
       <c r="N20" t="n">
-        <v>6.110590743398343</v>
+        <v>6.110590743398346</v>
       </c>
       <c r="O20" t="n">
-        <v>13.27941177386087</v>
+        <v>13.27941177386086</v>
       </c>
       <c r="P20" t="n">
         <v>12.97248403445492</v>
@@ -1738,7 +1738,7 @@
         <v>14.95038329562327</v>
       </c>
       <c r="T20" t="n">
-        <v>17.12089756026327</v>
+        <v>17.12089756026326</v>
       </c>
     </row>
     <row r="21">
@@ -1830,25 +1830,25 @@
         <v>0.4508700182311753</v>
       </c>
       <c r="H22" t="n">
-        <v>0.4570617448494494</v>
+        <v>0.4570617448494493</v>
       </c>
       <c r="I22" t="n">
-        <v>0.6809541129387651</v>
+        <v>0.6809541129387652</v>
       </c>
       <c r="J22" t="n">
         <v>0.6050064616045413</v>
       </c>
       <c r="K22" t="n">
-        <v>0.6081992116069271</v>
+        <v>0.6081992116069269</v>
       </c>
       <c r="L22" t="n">
-        <v>0.7024153448399539</v>
+        <v>0.7024153448399536</v>
       </c>
       <c r="M22" t="n">
-        <v>0.6831327355708822</v>
+        <v>0.6831327355708821</v>
       </c>
       <c r="N22" t="n">
-        <v>0.7426155281044444</v>
+        <v>0.7426155281044446</v>
       </c>
       <c r="O22" t="n">
         <v>1.109035337770553</v>
@@ -1897,10 +1897,10 @@
         <v>34.89380449301557</v>
       </c>
       <c r="I23" t="n">
-        <v>27.94648952835622</v>
+        <v>27.94648952835621</v>
       </c>
       <c r="J23" t="n">
-        <v>23.30033193856781</v>
+        <v>23.3003319385678</v>
       </c>
       <c r="K23" t="n">
         <v>21.71390926757909</v>
@@ -1915,7 +1915,7 @@
         <v>19.95199690421991</v>
       </c>
       <c r="O23" t="n">
-        <v>42.0036885874742</v>
+        <v>42.00368858747422</v>
       </c>
       <c r="P23" t="n">
         <v>43.51516009209706</v>
@@ -1927,10 +1927,10 @@
         <v>57.45436274853693</v>
       </c>
       <c r="S23" t="n">
-        <v>74.60968757876509</v>
+        <v>74.60968757876508</v>
       </c>
       <c r="T23" t="n">
-        <v>61.97072864975439</v>
+        <v>61.9707286497544</v>
       </c>
     </row>
     <row r="24">
@@ -1979,10 +1979,10 @@
         <v>0.1718320453756577</v>
       </c>
       <c r="O24" t="n">
-        <v>0.3246791236204479</v>
+        <v>0.3246791236204478</v>
       </c>
       <c r="P24" t="n">
-        <v>0.3210695322001896</v>
+        <v>0.3210695322001895</v>
       </c>
       <c r="Q24" t="n">
         <v>0.3242406935439865</v>
@@ -2043,19 +2043,19 @@
         <v>1.780468192537126</v>
       </c>
       <c r="O25" t="n">
-        <v>3.103087807084308</v>
+        <v>3.103087807084307</v>
       </c>
       <c r="P25" t="n">
-        <v>3.087807269100277</v>
+        <v>3.087807269100278</v>
       </c>
       <c r="Q25" t="n">
-        <v>2.817306935382982</v>
+        <v>2.817306935382981</v>
       </c>
       <c r="R25" t="n">
         <v>3.470960661583677</v>
       </c>
       <c r="S25" t="n">
-        <v>3.571209022316342</v>
+        <v>3.571209022316343</v>
       </c>
       <c r="T25" t="n">
         <v>3.937660405606108</v>
@@ -2098,16 +2098,16 @@
         <v>1.777768147733415</v>
       </c>
       <c r="L26" t="n">
-        <v>2.056544337895579</v>
+        <v>2.056544337895578</v>
       </c>
       <c r="M26" t="n">
-        <v>1.904726755139885</v>
+        <v>1.904726755139886</v>
       </c>
       <c r="N26" t="n">
         <v>2.004021483978576</v>
       </c>
       <c r="O26" t="n">
-        <v>2.872239639466171</v>
+        <v>2.872239639466172</v>
       </c>
       <c r="P26" t="n">
         <v>2.766895871208599</v>
@@ -2119,7 +2119,7 @@
         <v>3.238436963249196</v>
       </c>
       <c r="S26" t="n">
-        <v>3.451649865653489</v>
+        <v>3.45164986565349</v>
       </c>
       <c r="T26" t="n">
         <v>3.984225577084572</v>
@@ -2135,58 +2135,58 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>9.404548614880596</v>
+        <v>9.404548614880595</v>
       </c>
       <c r="D27" t="n">
-        <v>8.081672728719516</v>
+        <v>8.081672728719518</v>
       </c>
       <c r="E27" t="n">
-        <v>8.826005460992477</v>
+        <v>8.826005460992478</v>
       </c>
       <c r="F27" t="n">
-        <v>8.461035997767327</v>
+        <v>8.461035997767331</v>
       </c>
       <c r="G27" t="n">
         <v>8.483129903838181</v>
       </c>
       <c r="H27" t="n">
-        <v>11.64739412202549</v>
+        <v>11.64739412202548</v>
       </c>
       <c r="I27" t="n">
         <v>13.82307798420801</v>
       </c>
       <c r="J27" t="n">
-        <v>11.7009042275779</v>
+        <v>11.70090422757791</v>
       </c>
       <c r="K27" t="n">
         <v>11.38292990215321</v>
       </c>
       <c r="L27" t="n">
-        <v>15.83502613686162</v>
+        <v>15.83502613686161</v>
       </c>
       <c r="M27" t="n">
-        <v>15.1735578247713</v>
+        <v>15.17355782477129</v>
       </c>
       <c r="N27" t="n">
         <v>15.35778525360575</v>
       </c>
       <c r="O27" t="n">
-        <v>36.04669631674182</v>
+        <v>36.0466963167418</v>
       </c>
       <c r="P27" t="n">
-        <v>38.36051604651183</v>
+        <v>38.36051604651187</v>
       </c>
       <c r="Q27" t="n">
-        <v>35.55832547782603</v>
+        <v>35.55832547782605</v>
       </c>
       <c r="R27" t="n">
-        <v>54.2985308669444</v>
+        <v>54.29853086694441</v>
       </c>
       <c r="S27" t="n">
-        <v>59.24178136349357</v>
+        <v>59.24178136349356</v>
       </c>
       <c r="T27" t="n">
-        <v>57.57534920434811</v>
+        <v>57.57534920434809</v>
       </c>
     </row>
     <row r="28">
@@ -2202,13 +2202,13 @@
         <v>0.2966098180711587</v>
       </c>
       <c r="D28" t="n">
-        <v>0.2735237095728636</v>
+        <v>0.2735237095728637</v>
       </c>
       <c r="E28" t="n">
         <v>0.3179767014571709</v>
       </c>
       <c r="F28" t="n">
-        <v>0.2737142751873576</v>
+        <v>0.2737142751873577</v>
       </c>
       <c r="G28" t="n">
         <v>0.2819010151367157</v>
@@ -2232,16 +2232,16 @@
         <v>0.3916087622637227</v>
       </c>
       <c r="N28" t="n">
-        <v>0.3851934035328792</v>
+        <v>0.3851934035328791</v>
       </c>
       <c r="O28" t="n">
-        <v>0.6566030779648065</v>
+        <v>0.6566030779648063</v>
       </c>
       <c r="P28" t="n">
         <v>0.6184885068650191</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.601353191322552</v>
+        <v>0.6013531913225519</v>
       </c>
       <c r="R28" t="n">
         <v>0.7095695368170815</v>
@@ -2250,7 +2250,7 @@
         <v>0.7238361102241899</v>
       </c>
       <c r="T28" t="n">
-        <v>0.7692599133981047</v>
+        <v>0.7692599133981046</v>
       </c>
     </row>
     <row r="29">
@@ -2278,7 +2278,7 @@
         <v>13.58016626048591</v>
       </c>
       <c r="H29" t="n">
-        <v>11.25688282684746</v>
+        <v>11.25688282684747</v>
       </c>
       <c r="I29" t="n">
         <v>16.07264247295188</v>
@@ -2296,10 +2296,10 @@
         <v>15.58310716611139</v>
       </c>
       <c r="N29" t="n">
-        <v>16.8542864885156</v>
+        <v>16.85428648851559</v>
       </c>
       <c r="O29" t="n">
-        <v>24.2587360783589</v>
+        <v>24.25873607835889</v>
       </c>
       <c r="P29" t="n">
         <v>24.71870188120023</v>
@@ -2308,7 +2308,7 @@
         <v>23.55321816763552</v>
       </c>
       <c r="R29" t="n">
-        <v>27.30672319240506</v>
+        <v>27.30672319240507</v>
       </c>
       <c r="S29" t="n">
         <v>27.95490921811762</v>
@@ -2357,13 +2357,13 @@
         <v>0.02220517251655242</v>
       </c>
       <c r="M30" t="n">
-        <v>0.02516978813192496</v>
+        <v>0.02516978813192495</v>
       </c>
       <c r="N30" t="n">
         <v>0.02413512281717074</v>
       </c>
       <c r="O30" t="n">
-        <v>0.03954050305358028</v>
+        <v>0.03954050305358027</v>
       </c>
       <c r="P30" t="n">
         <v>0.04147805068852546</v>
@@ -2400,7 +2400,7 @@
         <v>0.004766503063254892</v>
       </c>
       <c r="F31" t="n">
-        <v>0.003732364605354747</v>
+        <v>0.003732364605354748</v>
       </c>
       <c r="G31" t="n">
         <v>0.003588195039972816</v>
@@ -2455,28 +2455,28 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>19.93820832675886</v>
+        <v>19.93820832675885</v>
       </c>
       <c r="D32" t="n">
-        <v>18.60115972781885</v>
+        <v>18.60115972781884</v>
       </c>
       <c r="E32" t="n">
         <v>24.53759922338814</v>
       </c>
       <c r="F32" t="n">
-        <v>16.48422927123904</v>
+        <v>16.48422927123906</v>
       </c>
       <c r="G32" t="n">
         <v>17.46869108560829</v>
       </c>
       <c r="H32" t="n">
-        <v>25.25621865479847</v>
+        <v>25.25621865479846</v>
       </c>
       <c r="I32" t="n">
         <v>24.93245450968368</v>
       </c>
       <c r="J32" t="n">
-        <v>21.48656101137114</v>
+        <v>21.48656101137113</v>
       </c>
       <c r="K32" t="n">
         <v>21.86653457998643</v>
@@ -2485,25 +2485,25 @@
         <v>26.13462266820759</v>
       </c>
       <c r="M32" t="n">
-        <v>26.36321867281373</v>
+        <v>26.36321867281374</v>
       </c>
       <c r="N32" t="n">
-        <v>24.73088385068639</v>
+        <v>24.73088385068638</v>
       </c>
       <c r="O32" t="n">
         <v>53.2915976146195</v>
       </c>
       <c r="P32" t="n">
-        <v>50.55783057115722</v>
+        <v>50.55783057115721</v>
       </c>
       <c r="Q32" t="n">
-        <v>51.0236969769154</v>
+        <v>51.02369697691539</v>
       </c>
       <c r="R32" t="n">
-        <v>75.07397051738791</v>
+        <v>75.07397051738788</v>
       </c>
       <c r="S32" t="n">
-        <v>78.12636319637697</v>
+        <v>78.126363196377</v>
       </c>
       <c r="T32" t="n">
         <v>74.25901315828335</v>
@@ -2525,22 +2525,22 @@
         <v>15.70691743160874</v>
       </c>
       <c r="E33" t="n">
-        <v>19.60435263495347</v>
+        <v>19.60435263495348</v>
       </c>
       <c r="F33" t="n">
-        <v>16.60027697863731</v>
+        <v>16.60027697863732</v>
       </c>
       <c r="G33" t="n">
         <v>17.20854420664552</v>
       </c>
       <c r="H33" t="n">
-        <v>20.63281995978073</v>
+        <v>20.63281995978072</v>
       </c>
       <c r="I33" t="n">
         <v>22.82971557122241</v>
       </c>
       <c r="J33" t="n">
-        <v>21.43984896650022</v>
+        <v>21.43984896650023</v>
       </c>
       <c r="K33" t="n">
         <v>19.98986465302142</v>
@@ -2549,25 +2549,25 @@
         <v>18.40901245093401</v>
       </c>
       <c r="M33" t="n">
-        <v>19.19765185377348</v>
+        <v>19.19765185377347</v>
       </c>
       <c r="N33" t="n">
-        <v>22.81341672059988</v>
+        <v>22.81341672059989</v>
       </c>
       <c r="O33" t="n">
-        <v>34.28419660999061</v>
+        <v>34.28419660999059</v>
       </c>
       <c r="P33" t="n">
-        <v>35.76583284950183</v>
+        <v>35.76583284950182</v>
       </c>
       <c r="Q33" t="n">
-        <v>30.94050442140451</v>
+        <v>30.9405044214045</v>
       </c>
       <c r="R33" t="n">
-        <v>37.77008413281227</v>
+        <v>37.77008413281228</v>
       </c>
       <c r="S33" t="n">
-        <v>37.83058400153884</v>
+        <v>37.83058400153882</v>
       </c>
       <c r="T33" t="n">
         <v>39.01559282927752</v>
@@ -2586,37 +2586,37 @@
         <v>0.6398987966166346</v>
       </c>
       <c r="D34" t="n">
-        <v>0.5517763762703966</v>
+        <v>0.5517763762703967</v>
       </c>
       <c r="E34" t="n">
-        <v>0.5582690650600814</v>
+        <v>0.5582690650600813</v>
       </c>
       <c r="F34" t="n">
-        <v>0.4923282737418818</v>
+        <v>0.4923282737418817</v>
       </c>
       <c r="G34" t="n">
         <v>0.524400404450782</v>
       </c>
       <c r="H34" t="n">
-        <v>0.6519480739457217</v>
+        <v>0.6519480739457219</v>
       </c>
       <c r="I34" t="n">
-        <v>0.9080652564049165</v>
+        <v>0.9080652564049163</v>
       </c>
       <c r="J34" t="n">
-        <v>0.7702546375485588</v>
+        <v>0.7702546375485592</v>
       </c>
       <c r="K34" t="n">
-        <v>0.7728840285905741</v>
+        <v>0.7728840285905738</v>
       </c>
       <c r="L34" t="n">
-        <v>0.8898760548571358</v>
+        <v>0.8898760548571359</v>
       </c>
       <c r="M34" t="n">
-        <v>0.8485600622825981</v>
+        <v>0.8485600622825979</v>
       </c>
       <c r="N34" t="n">
-        <v>0.8368804554497222</v>
+        <v>0.8368804554497221</v>
       </c>
       <c r="O34" t="n">
         <v>1.573818366340089</v>
@@ -2647,7 +2647,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0.4744506766882924</v>
+        <v>0.4744506766882923</v>
       </c>
       <c r="D35" t="n">
         <v>0.4527354524364828</v>
@@ -2662,19 +2662,19 @@
         <v>0.4040374514304064</v>
       </c>
       <c r="H35" t="n">
-        <v>0.6411577324587682</v>
+        <v>0.6411577324587681</v>
       </c>
       <c r="I35" t="n">
-        <v>0.7572241846316827</v>
+        <v>0.7572241846316825</v>
       </c>
       <c r="J35" t="n">
         <v>0.616061431060507</v>
       </c>
       <c r="K35" t="n">
-        <v>0.6343336691637602</v>
+        <v>0.6343336691637603</v>
       </c>
       <c r="L35" t="n">
-        <v>0.706108520593674</v>
+        <v>0.7061085205936739</v>
       </c>
       <c r="M35" t="n">
         <v>0.67793136788177</v>
@@ -2698,7 +2698,7 @@
         <v>1.617183317231839</v>
       </c>
       <c r="T35" t="n">
-        <v>1.667507511373176</v>
+        <v>1.667507511373175</v>
       </c>
     </row>
     <row r="36">
@@ -2726,10 +2726,10 @@
         <v>1.005831982981693</v>
       </c>
       <c r="H36" t="n">
-        <v>0.8712875694146192</v>
+        <v>0.8712875694146193</v>
       </c>
       <c r="I36" t="n">
-        <v>1.509803313929873</v>
+        <v>1.509803313929872</v>
       </c>
       <c r="J36" t="n">
         <v>1.309335653968299</v>
@@ -2738,25 +2738,25 @@
         <v>1.323740422266948</v>
       </c>
       <c r="L36" t="n">
-        <v>1.498336159672434</v>
+        <v>1.498336159672435</v>
       </c>
       <c r="M36" t="n">
-        <v>1.406251563128973</v>
+        <v>1.406251563128972</v>
       </c>
       <c r="N36" t="n">
-        <v>1.477686988087023</v>
+        <v>1.477686988087022</v>
       </c>
       <c r="O36" t="n">
         <v>2.504438041799734</v>
       </c>
       <c r="P36" t="n">
-        <v>2.702065560424375</v>
+        <v>2.702065560424374</v>
       </c>
       <c r="Q36" t="n">
-        <v>2.66634949364197</v>
+        <v>2.666349493641968</v>
       </c>
       <c r="R36" t="n">
-        <v>3.05403101196083</v>
+        <v>3.054031011960829</v>
       </c>
       <c r="S36" t="n">
         <v>3.36980345429629</v>
@@ -2775,37 +2775,37 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>6.097546813759399</v>
+        <v>6.097546813759396</v>
       </c>
       <c r="D37" t="n">
-        <v>5.114140316126428</v>
+        <v>5.114140316126429</v>
       </c>
       <c r="E37" t="n">
         <v>5.699036768997352</v>
       </c>
       <c r="F37" t="n">
-        <v>4.884572606433904</v>
+        <v>4.884572606433907</v>
       </c>
       <c r="G37" t="n">
-        <v>5.202316019783632</v>
+        <v>5.202316019783634</v>
       </c>
       <c r="H37" t="n">
-        <v>7.829584069477384</v>
+        <v>7.829584069477383</v>
       </c>
       <c r="I37" t="n">
-        <v>8.87764607870011</v>
+        <v>8.877646078700113</v>
       </c>
       <c r="J37" t="n">
-        <v>7.821808437450237</v>
+        <v>7.821808437450235</v>
       </c>
       <c r="K37" t="n">
-        <v>8.010174998157218</v>
+        <v>8.01017499815722</v>
       </c>
       <c r="L37" t="n">
         <v>9.004934032311969</v>
       </c>
       <c r="M37" t="n">
-        <v>8.733332666759516</v>
+        <v>8.733332666759519</v>
       </c>
       <c r="N37" t="n">
         <v>8.676850139866703</v>
@@ -2823,10 +2823,10 @@
         <v>15.07712930581885</v>
       </c>
       <c r="S37" t="n">
-        <v>13.83875879936986</v>
+        <v>13.83875879936987</v>
       </c>
       <c r="T37" t="n">
-        <v>16.09873236260819</v>
+        <v>16.0987323626082</v>
       </c>
     </row>
     <row r="38">
@@ -2848,19 +2848,19 @@
         <v>0.3075289005296661</v>
       </c>
       <c r="F38" t="n">
-        <v>0.2541057001269998</v>
+        <v>0.2541057001269997</v>
       </c>
       <c r="G38" t="n">
         <v>0.2556200834535385</v>
       </c>
       <c r="H38" t="n">
-        <v>0.2461904830187608</v>
+        <v>0.2461904830187607</v>
       </c>
       <c r="I38" t="n">
         <v>0.3625580352376092</v>
       </c>
       <c r="J38" t="n">
-        <v>0.3012688587454551</v>
+        <v>0.3012688587454552</v>
       </c>
       <c r="K38" t="n">
         <v>0.3067471673055576</v>
@@ -2875,22 +2875,22 @@
         <v>0.3672161387547305</v>
       </c>
       <c r="O38" t="n">
-        <v>0.5560605283839812</v>
+        <v>0.5560605283839815</v>
       </c>
       <c r="P38" t="n">
         <v>0.5979598904923212</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.5950990026010461</v>
+        <v>0.5950990026010462</v>
       </c>
       <c r="R38" t="n">
-        <v>0.7000854348229418</v>
+        <v>0.7000854348229416</v>
       </c>
       <c r="S38" t="n">
         <v>0.7025020583363112</v>
       </c>
       <c r="T38" t="n">
-        <v>0.7224778093726278</v>
+        <v>0.7224778093726277</v>
       </c>
     </row>
     <row r="39">
@@ -2948,7 +2948,7 @@
         <v>0.2706569995989109</v>
       </c>
       <c r="R39" t="n">
-        <v>0.3227064717157661</v>
+        <v>0.322706471715766</v>
       </c>
       <c r="S39" t="n">
         <v>0.2989639581600973</v>
@@ -2967,7 +2967,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0.09710812149561765</v>
+        <v>0.09710812149561764</v>
       </c>
       <c r="D40" t="n">
         <v>0.07378841216035686</v>
@@ -2976,7 +2976,7 @@
         <v>0.08033090647511303</v>
       </c>
       <c r="F40" t="n">
-        <v>0.07192437571553252</v>
+        <v>0.07192437571553253</v>
       </c>
       <c r="G40" t="n">
         <v>0.07691835437345299</v>
@@ -3034,13 +3034,13 @@
         <v>0.2221327367623503</v>
       </c>
       <c r="D41" t="n">
-        <v>0.1725111199877554</v>
+        <v>0.1725111199877555</v>
       </c>
       <c r="E41" t="n">
         <v>0.1818800407645293</v>
       </c>
       <c r="F41" t="n">
-        <v>0.1721878050353202</v>
+        <v>0.1721878050353203</v>
       </c>
       <c r="G41" t="n">
         <v>0.1764086078996173</v>
@@ -3070,19 +3070,19 @@
         <v>0.4269529431590516</v>
       </c>
       <c r="P41" t="n">
-        <v>0.4496474792223005</v>
+        <v>0.4496474792223004</v>
       </c>
       <c r="Q41" t="n">
-        <v>0.3981511220443804</v>
+        <v>0.3981511220443802</v>
       </c>
       <c r="R41" t="n">
-        <v>0.5190737316048599</v>
+        <v>0.51907373160486</v>
       </c>
       <c r="S41" t="n">
-        <v>0.4926698176538302</v>
+        <v>0.4926698176538301</v>
       </c>
       <c r="T41" t="n">
-        <v>0.5045882975581967</v>
+        <v>0.5045882975581968</v>
       </c>
     </row>
     <row r="42">
@@ -3116,7 +3116,7 @@
         <v>0.2795976787246109</v>
       </c>
       <c r="J42" t="n">
-        <v>0.2313455560769903</v>
+        <v>0.2313455560769902</v>
       </c>
       <c r="K42" t="n">
         <v>0.2370927516089911</v>
@@ -3137,7 +3137,7 @@
         <v>0.3996174953893472</v>
       </c>
       <c r="Q42" t="n">
-        <v>0.4029380843034596</v>
+        <v>0.4029380843034595</v>
       </c>
       <c r="R42" t="n">
         <v>0.4685313158556248</v>
@@ -3165,19 +3165,19 @@
         <v>0.4059216546935467</v>
       </c>
       <c r="E43" t="n">
-        <v>0.444261604002967</v>
+        <v>0.4442616040029671</v>
       </c>
       <c r="F43" t="n">
-        <v>0.4067174542639536</v>
+        <v>0.4067174542639537</v>
       </c>
       <c r="G43" t="n">
         <v>0.4522850142606716</v>
       </c>
       <c r="H43" t="n">
-        <v>0.6343909191249649</v>
+        <v>0.6343909191249647</v>
       </c>
       <c r="I43" t="n">
-        <v>0.7482193099960742</v>
+        <v>0.7482193099960741</v>
       </c>
       <c r="J43" t="n">
         <v>0.5958331305680664</v>
@@ -3186,19 +3186,19 @@
         <v>0.6785166683249233</v>
       </c>
       <c r="L43" t="n">
-        <v>0.7753307415839777</v>
+        <v>0.7753307415839779</v>
       </c>
       <c r="M43" t="n">
         <v>0.7358421863239855</v>
       </c>
       <c r="N43" t="n">
-        <v>0.7576220320898088</v>
+        <v>0.7576220320898085</v>
       </c>
       <c r="O43" t="n">
         <v>1.400432323002829</v>
       </c>
       <c r="P43" t="n">
-        <v>1.394145542172852</v>
+        <v>1.394145542172853</v>
       </c>
       <c r="Q43" t="n">
         <v>1.441774165774629</v>
@@ -3223,13 +3223,13 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3.024542231082155</v>
+        <v>3.024542231082156</v>
       </c>
       <c r="D44" t="n">
-        <v>2.59463350804146</v>
+        <v>2.594633508041459</v>
       </c>
       <c r="E44" t="n">
-        <v>2.41172968061775</v>
+        <v>2.411729680617749</v>
       </c>
       <c r="F44" t="n">
         <v>2.391574091326178</v>
@@ -3238,10 +3238,10 @@
         <v>2.609562577499626</v>
       </c>
       <c r="H44" t="n">
-        <v>2.677117644914224</v>
+        <v>2.677117644914225</v>
       </c>
       <c r="I44" t="n">
-        <v>3.987484973550339</v>
+        <v>3.987484973550338</v>
       </c>
       <c r="J44" t="n">
         <v>3.47230724128306</v>
@@ -3250,28 +3250,28 @@
         <v>3.583910071131089</v>
       </c>
       <c r="L44" t="n">
-        <v>4.185554924020091</v>
+        <v>4.18555492402009</v>
       </c>
       <c r="M44" t="n">
-        <v>3.925163487466425</v>
+        <v>3.925163487466424</v>
       </c>
       <c r="N44" t="n">
-        <v>4.042892391814342</v>
+        <v>4.042892391814343</v>
       </c>
       <c r="O44" t="n">
         <v>7.396388802691133</v>
       </c>
       <c r="P44" t="n">
-        <v>7.806862964356106</v>
+        <v>7.806862964356108</v>
       </c>
       <c r="Q44" t="n">
-        <v>7.558398617417602</v>
+        <v>7.558398617417603</v>
       </c>
       <c r="R44" t="n">
-        <v>8.757436153017908</v>
+        <v>8.757436153017904</v>
       </c>
       <c r="S44" t="n">
-        <v>9.836762725264927</v>
+        <v>9.836762725264926</v>
       </c>
       <c r="T44" t="n">
         <v>10.21186387658839</v>
@@ -3360,7 +3360,7 @@
         <v>0.02777653222705794</v>
       </c>
       <c r="F46" t="n">
-        <v>0.02384596323141613</v>
+        <v>0.02384596323141612</v>
       </c>
       <c r="G46" t="n">
         <v>0.02305656752295559</v>
@@ -3378,7 +3378,7 @@
         <v>0.03317865970596384</v>
       </c>
       <c r="L46" t="n">
-        <v>0.0364376929739617</v>
+        <v>0.03643769297396171</v>
       </c>
       <c r="M46" t="n">
         <v>0.0353136937263423</v>
@@ -3387,7 +3387,7 @@
         <v>0.03908874619543986</v>
       </c>
       <c r="O46" t="n">
-        <v>0.05484461247834845</v>
+        <v>0.05484461247834844</v>
       </c>
       <c r="P46" t="n">
         <v>0.04946406316796698</v>
@@ -3442,7 +3442,7 @@
         <v>0.124397015941951</v>
       </c>
       <c r="L47" t="n">
-        <v>0.1677984888185559</v>
+        <v>0.167798488818556</v>
       </c>
       <c r="M47" t="n">
         <v>0.161811391562324</v>
@@ -3460,13 +3460,13 @@
         <v>0.2383106961359085</v>
       </c>
       <c r="R47" t="n">
-        <v>0.2607051141114113</v>
+        <v>0.2607051141114112</v>
       </c>
       <c r="S47" t="n">
         <v>0.2962780989062211</v>
       </c>
       <c r="T47" t="n">
-        <v>0.2941269442488872</v>
+        <v>0.2941269442488873</v>
       </c>
     </row>
     <row r="48">
@@ -3503,7 +3503,7 @@
         <v>1.605262706341932</v>
       </c>
       <c r="K48" t="n">
-        <v>1.900433259945866</v>
+        <v>1.900433259945865</v>
       </c>
       <c r="L48" t="n">
         <v>1.959481859451967</v>
@@ -3518,19 +3518,19 @@
         <v>3.569180612299943</v>
       </c>
       <c r="P48" t="n">
-        <v>3.777795179031263</v>
+        <v>3.777795179031264</v>
       </c>
       <c r="Q48" t="n">
-        <v>3.240435673082851</v>
+        <v>3.24043567308285</v>
       </c>
       <c r="R48" t="n">
         <v>4.387061663915111</v>
       </c>
       <c r="S48" t="n">
-        <v>5.625264225328275</v>
+        <v>5.625264225328277</v>
       </c>
       <c r="T48" t="n">
-        <v>5.468889665806282</v>
+        <v>5.46888966580628</v>
       </c>
     </row>
     <row r="49">
@@ -3607,19 +3607,19 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0.08860172431605198</v>
+        <v>0.08860172431605201</v>
       </c>
       <c r="D50" t="n">
-        <v>0.07462511893453966</v>
+        <v>0.07462511893453967</v>
       </c>
       <c r="E50" t="n">
-        <v>0.08198445385099679</v>
+        <v>0.0819844538509968</v>
       </c>
       <c r="F50" t="n">
-        <v>0.06922494332878612</v>
+        <v>0.06922494332878613</v>
       </c>
       <c r="G50" t="n">
-        <v>0.07172424205200938</v>
+        <v>0.07172424205200939</v>
       </c>
       <c r="H50" t="n">
         <v>0.09423983597398897</v>
@@ -3631,7 +3631,7 @@
         <v>0.1007247446415135</v>
       </c>
       <c r="K50" t="n">
-        <v>0.09771725670103722</v>
+        <v>0.0977172567010372</v>
       </c>
       <c r="L50" t="n">
         <v>0.1269366541588031</v>
@@ -3640,7 +3640,7 @@
         <v>0.127132903867545</v>
       </c>
       <c r="N50" t="n">
-        <v>0.1201439935370561</v>
+        <v>0.120143993537056</v>
       </c>
       <c r="O50" t="n">
         <v>0.2378016392687132</v>
@@ -3683,7 +3683,7 @@
         <v>10.44642706198168</v>
       </c>
       <c r="G51" t="n">
-        <v>10.43091333113151</v>
+        <v>10.43091333113152</v>
       </c>
       <c r="H51" t="n">
         <v>13.97551201437595</v>
@@ -3701,7 +3701,7 @@
         <v>21.35549863107242</v>
       </c>
       <c r="M51" t="n">
-        <v>20.41376999275762</v>
+        <v>20.41376999275761</v>
       </c>
       <c r="N51" t="n">
         <v>19.13479435591571</v>
@@ -3713,13 +3713,13 @@
         <v>50.22166455892091</v>
       </c>
       <c r="Q51" t="n">
-        <v>50.13837317396758</v>
+        <v>50.13837317396757</v>
       </c>
       <c r="R51" t="n">
-        <v>77.26122772373186</v>
+        <v>77.26122772373185</v>
       </c>
       <c r="S51" t="n">
-        <v>83.51987220662355</v>
+        <v>83.51987220662356</v>
       </c>
       <c r="T51" t="n">
         <v>79.43649960610364</v>
@@ -3747,10 +3747,10 @@
         <v>0.1871588238984855</v>
       </c>
       <c r="G52" t="n">
-        <v>0.1992711523650431</v>
+        <v>0.1992711523650432</v>
       </c>
       <c r="H52" t="n">
-        <v>0.2450922242550072</v>
+        <v>0.2450922242550073</v>
       </c>
       <c r="I52" t="n">
         <v>0.3301955192627085</v>
@@ -3759,10 +3759,10 @@
         <v>0.2838122522826749</v>
       </c>
       <c r="K52" t="n">
-        <v>0.2892103106972123</v>
+        <v>0.2892103106972124</v>
       </c>
       <c r="L52" t="n">
-        <v>0.3334945218023855</v>
+        <v>0.3334945218023854</v>
       </c>
       <c r="M52" t="n">
         <v>0.3265435606084486</v>
@@ -3771,13 +3771,13 @@
         <v>0.3465252200970448</v>
       </c>
       <c r="O52" t="n">
-        <v>0.5383586329485343</v>
+        <v>0.5383586329485341</v>
       </c>
       <c r="P52" t="n">
-        <v>0.5375528631004317</v>
+        <v>0.5375528631004318</v>
       </c>
       <c r="Q52" t="n">
-        <v>0.4778548293983886</v>
+        <v>0.4778548293983885</v>
       </c>
       <c r="R52" t="n">
         <v>0.5592223663275284</v>
@@ -3799,13 +3799,13 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0.04237688422225861</v>
+        <v>0.04237688422225862</v>
       </c>
       <c r="D53" t="n">
         <v>0.04100827215303991</v>
       </c>
       <c r="E53" t="n">
-        <v>0.04047991478240511</v>
+        <v>0.0404799147824051</v>
       </c>
       <c r="F53" t="n">
         <v>0.03380066366290122</v>
@@ -3814,10 +3814,10 @@
         <v>0.03527272096626635</v>
       </c>
       <c r="H53" t="n">
-        <v>0.03724214220896253</v>
+        <v>0.03724214220896254</v>
       </c>
       <c r="I53" t="n">
-        <v>0.04582945961866257</v>
+        <v>0.04582945961866256</v>
       </c>
       <c r="J53" t="n">
         <v>0.03741265908861736</v>
@@ -3829,7 +3829,7 @@
         <v>0.04477268194484697</v>
       </c>
       <c r="M53" t="n">
-        <v>0.04494895685484367</v>
+        <v>0.04494895685484368</v>
       </c>
       <c r="N53" t="n">
         <v>0.0470079201435409</v>
@@ -3838,13 +3838,13 @@
         <v>0.06515883312020487</v>
       </c>
       <c r="P53" t="n">
-        <v>0.0706783984784168</v>
+        <v>0.07067839847841681</v>
       </c>
       <c r="Q53" t="n">
-        <v>0.06363342134431832</v>
+        <v>0.06363342134431831</v>
       </c>
       <c r="R53" t="n">
-        <v>0.07107560786585661</v>
+        <v>0.07107560786585662</v>
       </c>
       <c r="S53" t="n">
         <v>0.07278457453362859</v>
@@ -3866,7 +3866,7 @@
         <v>20.05955599835347</v>
       </c>
       <c r="D54" t="n">
-        <v>18.21345737108492</v>
+        <v>18.21345737108491</v>
       </c>
       <c r="E54" t="n">
         <v>18.99311284141383</v>
@@ -3881,25 +3881,25 @@
         <v>17.95847260667808</v>
       </c>
       <c r="I54" t="n">
-        <v>20.962596689499</v>
+        <v>20.96259668949901</v>
       </c>
       <c r="J54" t="n">
         <v>17.07160064407507</v>
       </c>
       <c r="K54" t="n">
-        <v>17.05811283337796</v>
+        <v>17.05811283337795</v>
       </c>
       <c r="L54" t="n">
-        <v>18.58251270403407</v>
+        <v>18.58251270403408</v>
       </c>
       <c r="M54" t="n">
         <v>19.07413149796638</v>
       </c>
       <c r="N54" t="n">
-        <v>19.87843876472925</v>
+        <v>19.87843876472924</v>
       </c>
       <c r="O54" t="n">
-        <v>46.85941209386324</v>
+        <v>46.85941209386323</v>
       </c>
       <c r="P54" t="n">
         <v>42.22034522318278</v>
@@ -3908,7 +3908,7 @@
         <v>41.99579983189019</v>
       </c>
       <c r="R54" t="n">
-        <v>62.33204504933176</v>
+        <v>62.33204504933173</v>
       </c>
       <c r="S54" t="n">
         <v>68.08183312628148</v>
@@ -3927,19 +3927,19 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2.436010129408095</v>
+        <v>2.436010129408096</v>
       </c>
       <c r="D55" t="n">
-        <v>2.110080126989678</v>
+        <v>2.110080126989677</v>
       </c>
       <c r="E55" t="n">
-        <v>2.277600249919771</v>
+        <v>2.277600249919772</v>
       </c>
       <c r="F55" t="n">
         <v>2.160205859747014</v>
       </c>
       <c r="G55" t="n">
-        <v>2.313606941531642</v>
+        <v>2.313606941531643</v>
       </c>
       <c r="H55" t="n">
         <v>3.187641228870548</v>
@@ -3948,34 +3948,34 @@
         <v>3.529625996694259</v>
       </c>
       <c r="J55" t="n">
-        <v>3.022402348416371</v>
+        <v>3.022402348416372</v>
       </c>
       <c r="K55" t="n">
-        <v>3.114295236810142</v>
+        <v>3.114295236810141</v>
       </c>
       <c r="L55" t="n">
-        <v>3.300267833329399</v>
+        <v>3.300267833329398</v>
       </c>
       <c r="M55" t="n">
         <v>3.242387635362422</v>
       </c>
       <c r="N55" t="n">
-        <v>3.222441603206717</v>
+        <v>3.222441603206716</v>
       </c>
       <c r="O55" t="n">
-        <v>5.323467152298638</v>
+        <v>5.323467152298636</v>
       </c>
       <c r="P55" t="n">
-        <v>5.164562010286512</v>
+        <v>5.164562010286514</v>
       </c>
       <c r="Q55" t="n">
-        <v>5.00495213308536</v>
+        <v>5.004952133085361</v>
       </c>
       <c r="R55" t="n">
         <v>6.287370154692156</v>
       </c>
       <c r="S55" t="n">
-        <v>6.671156152445691</v>
+        <v>6.671156152445692</v>
       </c>
       <c r="T55" t="n">
         <v>6.586134288915916</v>
@@ -3991,16 +3991,16 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>9.002219528609343</v>
+        <v>9.002219528609345</v>
       </c>
       <c r="D56" t="n">
-        <v>8.001800521808399</v>
+        <v>8.001800521808397</v>
       </c>
       <c r="E56" t="n">
-        <v>8.310901666166226</v>
+        <v>8.310901666166224</v>
       </c>
       <c r="F56" t="n">
-        <v>9.437856918498602</v>
+        <v>9.437856918498607</v>
       </c>
       <c r="G56" t="n">
         <v>9.872087524962005</v>
@@ -4018,7 +4018,7 @@
         <v>14.54418936305817</v>
       </c>
       <c r="L56" t="n">
-        <v>17.56714647826359</v>
+        <v>17.56714647826357</v>
       </c>
       <c r="M56" t="n">
         <v>16.81914736292005</v>
@@ -4027,22 +4027,22 @@
         <v>17.98478547434986</v>
       </c>
       <c r="O56" t="n">
-        <v>28.09770099886684</v>
+        <v>28.09770099886685</v>
       </c>
       <c r="P56" t="n">
-        <v>27.06158055870102</v>
+        <v>27.061580558701</v>
       </c>
       <c r="Q56" t="n">
         <v>24.16732439168008</v>
       </c>
       <c r="R56" t="n">
-        <v>27.90142995101545</v>
+        <v>27.90142995101546</v>
       </c>
       <c r="S56" t="n">
         <v>30.78461216488866</v>
       </c>
       <c r="T56" t="n">
-        <v>33.68994732335537</v>
+        <v>33.68994732335536</v>
       </c>
     </row>
     <row r="57">
@@ -4085,7 +4085,7 @@
         <v>0.2206493916154403</v>
       </c>
       <c r="M57" t="n">
-        <v>0.2327865465708244</v>
+        <v>0.2327865465708243</v>
       </c>
       <c r="N57" t="n">
         <v>0.2263504382617427</v>
@@ -4097,7 +4097,7 @@
         <v>0.3450973520570018</v>
       </c>
       <c r="Q57" t="n">
-        <v>0.3871143697981332</v>
+        <v>0.3871143697981334</v>
       </c>
       <c r="R57" t="n">
         <v>0.4228791122199831</v>
@@ -4106,7 +4106,7 @@
         <v>0.4854848696430998</v>
       </c>
       <c r="T57" t="n">
-        <v>0.5083179191588839</v>
+        <v>0.508317919158884</v>
       </c>
     </row>
     <row r="58">
@@ -4122,7 +4122,7 @@
         <v>0.296847937172884</v>
       </c>
       <c r="D58" t="n">
-        <v>0.2761931299905347</v>
+        <v>0.2761931299905348</v>
       </c>
       <c r="E58" t="n">
         <v>0.2793889979108572</v>
@@ -4131,13 +4131,13 @@
         <v>0.2622196916297052</v>
       </c>
       <c r="G58" t="n">
-        <v>0.2872729529123516</v>
+        <v>0.2872729529123517</v>
       </c>
       <c r="H58" t="n">
         <v>0.2146458058583305</v>
       </c>
       <c r="I58" t="n">
-        <v>0.3730450479624072</v>
+        <v>0.3730450479624073</v>
       </c>
       <c r="J58" t="n">
         <v>0.3114356260656577</v>
@@ -4149,7 +4149,7 @@
         <v>0.3804854728963059</v>
       </c>
       <c r="M58" t="n">
-        <v>0.3587328305993009</v>
+        <v>0.3587328305993011</v>
       </c>
       <c r="N58" t="n">
         <v>0.3984779450632039</v>
@@ -4158,10 +4158,10 @@
         <v>0.5733265193252318</v>
       </c>
       <c r="P58" t="n">
-        <v>0.5640821584039857</v>
+        <v>0.5640821584039858</v>
       </c>
       <c r="Q58" t="n">
-        <v>0.5843001414103959</v>
+        <v>0.5843001414103958</v>
       </c>
       <c r="R58" t="n">
         <v>0.6193066921669443</v>
@@ -4170,7 +4170,7 @@
         <v>0.6905510298714843</v>
       </c>
       <c r="T58" t="n">
-        <v>0.6905632149585151</v>
+        <v>0.6905632149585154</v>
       </c>
     </row>
     <row r="59">
@@ -4183,13 +4183,13 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0.3665211324782943</v>
+        <v>0.3665211324782944</v>
       </c>
       <c r="D59" t="n">
         <v>0.2616070552258732</v>
       </c>
       <c r="E59" t="n">
-        <v>0.332311477815813</v>
+        <v>0.3323114778158131</v>
       </c>
       <c r="F59" t="n">
         <v>0.2480803905613383</v>
@@ -4198,10 +4198,10 @@
         <v>0.3395348092814298</v>
       </c>
       <c r="H59" t="n">
-        <v>0.4708188409610112</v>
+        <v>0.4708188409610113</v>
       </c>
       <c r="I59" t="n">
-        <v>0.4941944121785509</v>
+        <v>0.494194412178551</v>
       </c>
       <c r="J59" t="n">
         <v>0.4742208117594476</v>
@@ -4219,19 +4219,19 @@
         <v>0.4907193142019842</v>
       </c>
       <c r="O59" t="n">
-        <v>0.7753968259582845</v>
+        <v>0.7753968259582847</v>
       </c>
       <c r="P59" t="n">
         <v>0.8229122625220627</v>
       </c>
       <c r="Q59" t="n">
-        <v>0.7637496637475516</v>
+        <v>0.7637496637475517</v>
       </c>
       <c r="R59" t="n">
-        <v>1.021756852630664</v>
+        <v>1.021756852630665</v>
       </c>
       <c r="S59" t="n">
-        <v>0.835894093290566</v>
+        <v>0.8358940932905661</v>
       </c>
       <c r="T59" t="n">
         <v>0.9534817720727391</v>
@@ -4250,7 +4250,7 @@
         <v>4.161584142186904</v>
       </c>
       <c r="D60" t="n">
-        <v>3.649819862934674</v>
+        <v>3.649819862934673</v>
       </c>
       <c r="E60" t="n">
         <v>4.170236557246419</v>
@@ -4268,13 +4268,13 @@
         <v>7.696409682496404</v>
       </c>
       <c r="J60" t="n">
-        <v>6.780125415666086</v>
+        <v>6.780125415666087</v>
       </c>
       <c r="K60" t="n">
-        <v>6.767072585146673</v>
+        <v>6.767072585146674</v>
       </c>
       <c r="L60" t="n">
-        <v>7.603990588882166</v>
+        <v>7.603990588882167</v>
       </c>
       <c r="M60" t="n">
         <v>7.347889275251528</v>
@@ -4286,7 +4286,7 @@
         <v>11.23354743482509</v>
       </c>
       <c r="P60" t="n">
-        <v>10.97800730298769</v>
+        <v>10.97800730298768</v>
       </c>
       <c r="Q60" t="n">
         <v>11.52429887559248</v>
@@ -4295,7 +4295,7 @@
         <v>13.66599580628666</v>
       </c>
       <c r="S60" t="n">
-        <v>13.97065214339741</v>
+        <v>13.9706521433974</v>
       </c>
       <c r="T60" t="n">
         <v>14.59932269287497</v>
@@ -4314,10 +4314,10 @@
         <v>0.1974613923869827</v>
       </c>
       <c r="D61" t="n">
-        <v>0.2067498450747351</v>
+        <v>0.2067498450747352</v>
       </c>
       <c r="E61" t="n">
-        <v>0.1592537299886221</v>
+        <v>0.1592537299886222</v>
       </c>
       <c r="F61" t="n">
         <v>0.1597263109206815</v>
@@ -4332,7 +4332,7 @@
         <v>0.2680977665901244</v>
       </c>
       <c r="J61" t="n">
-        <v>0.2289473495324238</v>
+        <v>0.2289473495324237</v>
       </c>
       <c r="K61" t="n">
         <v>0.203477773626796</v>
@@ -4350,7 +4350,7 @@
         <v>0.3691221454281292</v>
       </c>
       <c r="P61" t="n">
-        <v>0.4106936260497087</v>
+        <v>0.4106936260497088</v>
       </c>
       <c r="Q61" t="n">
         <v>0.4121127517241336</v>
@@ -4399,7 +4399,7 @@
         <v>0.07419645851843938</v>
       </c>
       <c r="K62" t="n">
-        <v>0.005398043655014137</v>
+        <v>0.005398043655014138</v>
       </c>
       <c r="L62" t="n">
         <v>0.0656634102161279</v>
@@ -4442,55 +4442,55 @@
         <v>7.474025755052581</v>
       </c>
       <c r="D63" t="n">
-        <v>7.359220212472145</v>
+        <v>7.359220212472147</v>
       </c>
       <c r="E63" t="n">
-        <v>7.463603077570285</v>
+        <v>7.463603077570286</v>
       </c>
       <c r="F63" t="n">
-        <v>5.116440797995491</v>
+        <v>5.116440797995489</v>
       </c>
       <c r="G63" t="n">
-        <v>6.33061455553134</v>
+        <v>6.330614555531341</v>
       </c>
       <c r="H63" t="n">
-        <v>7.399709940914342</v>
+        <v>7.399709940914338</v>
       </c>
       <c r="I63" t="n">
-        <v>7.355906746750129</v>
+        <v>7.355906746750128</v>
       </c>
       <c r="J63" t="n">
         <v>6.666940113751791</v>
       </c>
       <c r="K63" t="n">
-        <v>6.585760931303156</v>
+        <v>6.585760931303155</v>
       </c>
       <c r="L63" t="n">
-        <v>5.904347755306565</v>
+        <v>5.904347755306564</v>
       </c>
       <c r="M63" t="n">
-        <v>6.1682263996826</v>
+        <v>6.168226399682599</v>
       </c>
       <c r="N63" t="n">
-        <v>7.023879547269578</v>
+        <v>7.023879547269579</v>
       </c>
       <c r="O63" t="n">
-        <v>7.576125406056336</v>
+        <v>7.576125406056337</v>
       </c>
       <c r="P63" t="n">
         <v>7.583220679254564</v>
       </c>
       <c r="Q63" t="n">
-        <v>6.525872006185976</v>
+        <v>6.525872006185974</v>
       </c>
       <c r="R63" t="n">
-        <v>8.758523229211001</v>
+        <v>8.758523229211004</v>
       </c>
       <c r="S63" t="n">
-        <v>8.831576217316705</v>
+        <v>8.831576217316703</v>
       </c>
       <c r="T63" t="n">
-        <v>7.873375497297173</v>
+        <v>7.873375497297174</v>
       </c>
     </row>
     <row r="64">
@@ -4503,7 +4503,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0.02371593080490814</v>
+        <v>0.02371593080490813</v>
       </c>
       <c r="D64" t="n">
         <v>0.02119374383137082</v>
@@ -4521,7 +4521,7 @@
         <v>0.03098704064161814</v>
       </c>
       <c r="I64" t="n">
-        <v>0.0386809196356189</v>
+        <v>0.03868091963561889</v>
       </c>
       <c r="J64" t="n">
         <v>0.03374692911133307</v>
@@ -4554,7 +4554,7 @@
         <v>0.1258254157547768</v>
       </c>
       <c r="T64" t="n">
-        <v>0.1212508408923787</v>
+        <v>0.1212508408923788</v>
       </c>
     </row>
     <row r="65">
@@ -4579,7 +4579,7 @@
         <v>7.327267481926659</v>
       </c>
       <c r="G65" t="n">
-        <v>7.903251992633484</v>
+        <v>7.903251992633487</v>
       </c>
       <c r="H65" t="n">
         <v>12.56555257937037</v>
@@ -4609,16 +4609,16 @@
         <v>22.28538870430981</v>
       </c>
       <c r="Q65" t="n">
-        <v>19.0441899293089</v>
+        <v>19.04418992930889</v>
       </c>
       <c r="R65" t="n">
-        <v>26.72637825991753</v>
+        <v>26.72637825991754</v>
       </c>
       <c r="S65" t="n">
         <v>24.82385990061705</v>
       </c>
       <c r="T65" t="n">
-        <v>27.11831060220081</v>
+        <v>27.11831060220082</v>
       </c>
     </row>
     <row r="66">
@@ -4637,7 +4637,7 @@
         <v>0.4811467776143715</v>
       </c>
       <c r="E66" t="n">
-        <v>0.4946621175280045</v>
+        <v>0.4946621175280044</v>
       </c>
       <c r="F66" t="n">
         <v>0.4553056621614988</v>
@@ -4646,7 +4646,7 @@
         <v>0.4975013469952058</v>
       </c>
       <c r="H66" t="n">
-        <v>0.6712072827404821</v>
+        <v>0.6712072827404822</v>
       </c>
       <c r="I66" t="n">
         <v>0.8187225122042264</v>
@@ -4655,13 +4655,13 @@
         <v>0.6956189370261474</v>
       </c>
       <c r="K66" t="n">
-        <v>0.6963681204728589</v>
+        <v>0.6963681204728591</v>
       </c>
       <c r="L66" t="n">
-        <v>0.7551802154687058</v>
+        <v>0.7551802154687057</v>
       </c>
       <c r="M66" t="n">
-        <v>0.7632263851001189</v>
+        <v>0.763226385100119</v>
       </c>
       <c r="N66" t="n">
         <v>0.7570082705146345</v>
@@ -4740,7 +4740,7 @@
         <v>0.02894201106568465</v>
       </c>
       <c r="R67" t="n">
-        <v>0.0348797651381259</v>
+        <v>0.03487976513812589</v>
       </c>
       <c r="S67" t="n">
         <v>0.03304330346265144</v>
@@ -4759,16 +4759,16 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0.08860435217536049</v>
+        <v>0.0886043521753605</v>
       </c>
       <c r="D68" t="n">
-        <v>0.08338357720705421</v>
+        <v>0.08338357720705422</v>
       </c>
       <c r="E68" t="n">
-        <v>0.08065678586299248</v>
+        <v>0.08065678586299246</v>
       </c>
       <c r="F68" t="n">
-        <v>0.07761385131896632</v>
+        <v>0.07761385131896631</v>
       </c>
       <c r="G68" t="n">
         <v>0.07705890671204459</v>
@@ -4798,7 +4798,7 @@
         <v>0.20967058173589</v>
       </c>
       <c r="P68" t="n">
-        <v>0.2030245335134443</v>
+        <v>0.2030245335134442</v>
       </c>
       <c r="Q68" t="n">
         <v>0.1926497405625261</v>
@@ -4807,7 +4807,7 @@
         <v>0.2277342449158929</v>
       </c>
       <c r="S68" t="n">
-        <v>0.2340839958658352</v>
+        <v>0.2340839958658353</v>
       </c>
       <c r="T68" t="n">
         <v>0.2534092645360634</v>
@@ -4859,7 +4859,7 @@
         <v>0.2299358346493484</v>
       </c>
       <c r="O69" t="n">
-        <v>0.4065884659834504</v>
+        <v>0.4065884659834503</v>
       </c>
       <c r="P69" t="n">
         <v>0.4547050420758502</v>
@@ -4868,7 +4868,7 @@
         <v>0.4204724715982063</v>
       </c>
       <c r="R69" t="n">
-        <v>0.6100145977516065</v>
+        <v>0.6100145977516064</v>
       </c>
       <c r="S69" t="n">
         <v>0.6777230012673703</v>
@@ -4966,7 +4966,7 @@
         <v>8.485819198539783</v>
       </c>
       <c r="H71" t="n">
-        <v>9.325951313710425</v>
+        <v>9.325951313710423</v>
       </c>
       <c r="I71" t="n">
         <v>12.30330279162969</v>
@@ -4993,16 +4993,16 @@
         <v>14.66952582916914</v>
       </c>
       <c r="Q71" t="n">
-        <v>14.61431866093425</v>
+        <v>14.61431866093424</v>
       </c>
       <c r="R71" t="n">
-        <v>17.11880592520788</v>
+        <v>17.11880592520789</v>
       </c>
       <c r="S71" t="n">
         <v>17.93867995912189</v>
       </c>
       <c r="T71" t="n">
-        <v>18.34885510296303</v>
+        <v>18.34885510296304</v>
       </c>
     </row>
     <row r="72">
@@ -5039,10 +5039,10 @@
         <v>2.023453764190804</v>
       </c>
       <c r="K72" t="n">
-        <v>2.188914594874115</v>
+        <v>2.188914594874116</v>
       </c>
       <c r="L72" t="n">
-        <v>2.659499514689071</v>
+        <v>2.659499514689072</v>
       </c>
       <c r="M72" t="n">
         <v>2.419760414856627</v>
@@ -5054,7 +5054,7 @@
         <v>5.147166574557632</v>
       </c>
       <c r="P72" t="n">
-        <v>5.377060657092476</v>
+        <v>5.377060657092477</v>
       </c>
       <c r="Q72" t="n">
         <v>4.473685519038743</v>
@@ -5066,7 +5066,7 @@
         <v>5.431101620617825</v>
       </c>
       <c r="T72" t="n">
-        <v>6.941913179724764</v>
+        <v>6.941913179724765</v>
       </c>
     </row>
     <row r="73">
@@ -5094,13 +5094,13 @@
         <v>1.192844090757993</v>
       </c>
       <c r="H73" t="n">
-        <v>1.532561732471719</v>
+        <v>1.532561732471718</v>
       </c>
       <c r="I73" t="n">
-        <v>1.845931244623013</v>
+        <v>1.845931244623012</v>
       </c>
       <c r="J73" t="n">
-        <v>1.498706079619441</v>
+        <v>1.49870607961944</v>
       </c>
       <c r="K73" t="n">
         <v>1.634834905344694</v>
@@ -5115,19 +5115,19 @@
         <v>1.825863106501562</v>
       </c>
       <c r="O73" t="n">
-        <v>2.703419228222107</v>
+        <v>2.703419228222108</v>
       </c>
       <c r="P73" t="n">
-        <v>2.910520281185771</v>
+        <v>2.91052028118577</v>
       </c>
       <c r="Q73" t="n">
         <v>2.601805039389385</v>
       </c>
       <c r="R73" t="n">
-        <v>3.159059213605377</v>
+        <v>3.159059213605378</v>
       </c>
       <c r="S73" t="n">
-        <v>3.140371146369913</v>
+        <v>3.140371146369914</v>
       </c>
       <c r="T73" t="n">
         <v>3.199083838448153</v>
@@ -5146,7 +5146,7 @@
         <v>1.302261208263902</v>
       </c>
       <c r="D74" t="n">
-        <v>1.212096825122384</v>
+        <v>1.212096825122385</v>
       </c>
       <c r="E74" t="n">
         <v>1.269278501060561</v>
@@ -5158,7 +5158,7 @@
         <v>1.085565508241997</v>
       </c>
       <c r="H74" t="n">
-        <v>1.846020041719576</v>
+        <v>1.846020041719575</v>
       </c>
       <c r="I74" t="n">
         <v>1.781168652879039</v>
@@ -5176,25 +5176,25 @@
         <v>1.67586973319119</v>
       </c>
       <c r="N74" t="n">
-        <v>1.759391306409166</v>
+        <v>1.759391306409165</v>
       </c>
       <c r="O74" t="n">
-        <v>2.981202413708604</v>
+        <v>2.981202413708605</v>
       </c>
       <c r="P74" t="n">
-        <v>2.99011638861717</v>
+        <v>2.990116388617168</v>
       </c>
       <c r="Q74" t="n">
         <v>2.598901811319934</v>
       </c>
       <c r="R74" t="n">
-        <v>3.430566588778875</v>
+        <v>3.430566588778874</v>
       </c>
       <c r="S74" t="n">
-        <v>3.263613274909259</v>
+        <v>3.263613274909258</v>
       </c>
       <c r="T74" t="n">
-        <v>3.633930412665086</v>
+        <v>3.633930412665087</v>
       </c>
     </row>
     <row r="75">
@@ -5274,16 +5274,16 @@
         <v>1.018561139278981</v>
       </c>
       <c r="D76" t="n">
-        <v>0.8945888726264914</v>
+        <v>0.8945888726264916</v>
       </c>
       <c r="E76" t="n">
-        <v>0.8492489187710286</v>
+        <v>0.8492489187710288</v>
       </c>
       <c r="F76" t="n">
-        <v>0.8277236937358575</v>
+        <v>0.8277236937358576</v>
       </c>
       <c r="G76" t="n">
-        <v>0.8276867994302279</v>
+        <v>0.8276867994302278</v>
       </c>
       <c r="H76" t="n">
         <v>0.7210479262269718</v>
@@ -5304,13 +5304,13 @@
         <v>1.179875785866946</v>
       </c>
       <c r="N76" t="n">
-        <v>1.256437534535655</v>
+        <v>1.256437534535654</v>
       </c>
       <c r="O76" t="n">
         <v>2.074779267803994</v>
       </c>
       <c r="P76" t="n">
-        <v>2.262791692162141</v>
+        <v>2.262791692162142</v>
       </c>
       <c r="Q76" t="n">
         <v>2.174251104365404</v>
@@ -5368,7 +5368,7 @@
         <v>0.05605225976098067</v>
       </c>
       <c r="N77" t="n">
-        <v>0.05116264471375147</v>
+        <v>0.05116264471375146</v>
       </c>
       <c r="O77" t="n">
         <v>0.09563127485471259</v>
@@ -5463,7 +5463,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>0.03567012025260805</v>
+        <v>0.03567012025260804</v>
       </c>
       <c r="D79" t="n">
         <v>0.0347550315373359</v>
@@ -5490,7 +5490,7 @@
         <v>0.03891491276865704</v>
       </c>
       <c r="L79" t="n">
-        <v>0.04371732745194584</v>
+        <v>0.04371732745194582</v>
       </c>
       <c r="M79" t="n">
         <v>0.04117212522759246</v>
@@ -5511,10 +5511,10 @@
         <v>0.07648818052484195</v>
       </c>
       <c r="S79" t="n">
-        <v>0.07569175457430552</v>
+        <v>0.07569175457430555</v>
       </c>
       <c r="T79" t="n">
-        <v>0.07746444660710337</v>
+        <v>0.07746444660710339</v>
       </c>
     </row>
     <row r="80">
@@ -5533,13 +5533,13 @@
         <v>0.08709391164304661</v>
       </c>
       <c r="E80" t="n">
-        <v>0.08973841631731855</v>
+        <v>0.08973841631731856</v>
       </c>
       <c r="F80" t="n">
         <v>0.09397478314432432</v>
       </c>
       <c r="G80" t="n">
-        <v>0.0960544485675292</v>
+        <v>0.09605444856752922</v>
       </c>
       <c r="H80" t="n">
         <v>0.1305250556246922</v>
@@ -5600,7 +5600,7 @@
         <v>0.05839908678499228</v>
       </c>
       <c r="F81" t="n">
-        <v>0.04240415639181689</v>
+        <v>0.0424041563918169</v>
       </c>
       <c r="G81" t="n">
         <v>0.04513619269068152</v>
@@ -5609,19 +5609,19 @@
         <v>0.05645308277290648</v>
       </c>
       <c r="I81" t="n">
-        <v>0.05996261523613866</v>
+        <v>0.05996261523613867</v>
       </c>
       <c r="J81" t="n">
         <v>0.05164878148660471</v>
       </c>
       <c r="K81" t="n">
-        <v>0.05421839837363159</v>
+        <v>0.05421839837363158</v>
       </c>
       <c r="L81" t="n">
-        <v>0.0597099427937756</v>
+        <v>0.05970994279377559</v>
       </c>
       <c r="M81" t="n">
-        <v>0.05935430359267565</v>
+        <v>0.05935430359267566</v>
       </c>
       <c r="N81" t="n">
         <v>0.06510591134099562</v>
@@ -5630,10 +5630,10 @@
         <v>0.0939538892636396</v>
       </c>
       <c r="P81" t="n">
-        <v>0.09981060038399728</v>
+        <v>0.09981060038399726</v>
       </c>
       <c r="Q81" t="n">
-        <v>0.07475826716118834</v>
+        <v>0.07475826716118832</v>
       </c>
       <c r="R81" t="n">
         <v>0.1077060216576888</v>
@@ -5691,7 +5691,7 @@
         <v>0.1406300368012715</v>
       </c>
       <c r="O82" t="n">
-        <v>0.2624932424661769</v>
+        <v>0.262493242466177</v>
       </c>
       <c r="P82" t="n">
         <v>0.2965181102235944</v>
@@ -5755,13 +5755,13 @@
         <v>2.944105917051</v>
       </c>
       <c r="O83" t="n">
-        <v>5.75971813586441</v>
+        <v>5.759718135864409</v>
       </c>
       <c r="P83" t="n">
-        <v>6.161777009505935</v>
+        <v>6.161777009505934</v>
       </c>
       <c r="Q83" t="n">
-        <v>5.259860609033284</v>
+        <v>5.259860609033285</v>
       </c>
       <c r="R83" t="n">
         <v>6.622326851860395</v>
@@ -5770,7 +5770,7 @@
         <v>7.043896003059909</v>
       </c>
       <c r="T83" t="n">
-        <v>7.089961413254847</v>
+        <v>7.089961413254848</v>
       </c>
     </row>
     <row r="84">
@@ -5801,7 +5801,7 @@
         <v>0.5183574239175387</v>
       </c>
       <c r="I84" t="n">
-        <v>0.5324069396702635</v>
+        <v>0.5324069396702634</v>
       </c>
       <c r="J84" t="n">
         <v>0.4822571045037668</v>
@@ -5810,10 +5810,10 @@
         <v>0.4533326189723015</v>
       </c>
       <c r="L84" t="n">
-        <v>0.5749132562661738</v>
+        <v>0.574913256266174</v>
       </c>
       <c r="M84" t="n">
-        <v>0.5822688096771389</v>
+        <v>0.582268809677139</v>
       </c>
       <c r="N84" t="n">
         <v>0.5583936066807866</v>
@@ -5825,7 +5825,7 @@
         <v>1.207290579391694</v>
       </c>
       <c r="Q84" t="n">
-        <v>1.067176372910878</v>
+        <v>1.067176372910877</v>
       </c>
       <c r="R84" t="n">
         <v>1.350471142691147</v>
@@ -5862,7 +5862,7 @@
         <v>1.248856893688337</v>
       </c>
       <c r="H85" t="n">
-        <v>0.8977009922761626</v>
+        <v>0.8977009922761627</v>
       </c>
       <c r="I85" t="n">
         <v>1.915667841593747</v>
@@ -5883,13 +5883,13 @@
         <v>2.003314533415022</v>
       </c>
       <c r="O85" t="n">
-        <v>2.395896523025483</v>
+        <v>2.395896523025484</v>
       </c>
       <c r="P85" t="n">
-        <v>2.246875413497708</v>
+        <v>2.246875413497707</v>
       </c>
       <c r="Q85" t="n">
-        <v>2.289162291748105</v>
+        <v>2.289162291748106</v>
       </c>
       <c r="R85" t="n">
         <v>2.022926259040862</v>
@@ -5911,7 +5911,7 @@
         </is>
       </c>
       <c r="C86" t="n">
-        <v>0.15282476319892</v>
+        <v>0.1528247631989199</v>
       </c>
       <c r="D86" t="n">
         <v>0.1437978112685632</v>
@@ -5947,7 +5947,7 @@
         <v>0.226086820747178</v>
       </c>
       <c r="O86" t="n">
-        <v>0.3224537586271389</v>
+        <v>0.322453758627139</v>
       </c>
       <c r="P86" t="n">
         <v>0.3560990120076207</v>
@@ -5962,7 +5962,7 @@
         <v>0.4207049694510193</v>
       </c>
       <c r="T86" t="n">
-        <v>0.4153735254923928</v>
+        <v>0.4153735254923927</v>
       </c>
     </row>
     <row r="87">
@@ -6045,7 +6045,7 @@
         <v>2.538532243285527</v>
       </c>
       <c r="E88" t="n">
-        <v>2.908891485579278</v>
+        <v>2.908891485579277</v>
       </c>
       <c r="F88" t="n">
         <v>2.422515020312858</v>
@@ -6054,7 +6054,7 @@
         <v>2.870062409272608</v>
       </c>
       <c r="H88" t="n">
-        <v>2.383001338813015</v>
+        <v>2.383001338813016</v>
       </c>
       <c r="I88" t="n">
         <v>3.858926552936151</v>
@@ -6063,7 +6063,7 @@
         <v>2.841505409250779</v>
       </c>
       <c r="K88" t="n">
-        <v>3.198134969623062</v>
+        <v>3.198134969623061</v>
       </c>
       <c r="L88" t="n">
         <v>3.50448167782754</v>
@@ -6075,10 +6075,10 @@
         <v>3.885575731420615</v>
       </c>
       <c r="O88" t="n">
-        <v>4.943137742464317</v>
+        <v>4.943137742464316</v>
       </c>
       <c r="P88" t="n">
-        <v>4.685707881822317</v>
+        <v>4.685707881822316</v>
       </c>
       <c r="Q88" t="n">
         <v>4.189688856175836</v>
@@ -6090,7 +6090,7 @@
         <v>3.739191187375785</v>
       </c>
       <c r="T88" t="n">
-        <v>4.751524031734837</v>
+        <v>4.751524031734838</v>
       </c>
     </row>
     <row r="89">
@@ -6191,7 +6191,7 @@
         <v>0.1982915449839801</v>
       </c>
       <c r="K90" t="n">
-        <v>0.1844169951137988</v>
+        <v>0.1844169951137987</v>
       </c>
       <c r="L90" t="n">
         <v>0.2064698092696904</v>
@@ -6237,13 +6237,13 @@
         <v>0.00895872860779065</v>
       </c>
       <c r="E91" t="n">
-        <v>0.009749478190825936</v>
+        <v>0.009749478190825937</v>
       </c>
       <c r="F91" t="n">
-        <v>0.008640558749067722</v>
+        <v>0.008640558749067724</v>
       </c>
       <c r="G91" t="n">
-        <v>0.009866529866840737</v>
+        <v>0.009866529866840735</v>
       </c>
       <c r="H91" t="n">
         <v>0.007703465989920753</v>
@@ -6252,7 +6252,7 @@
         <v>0.01204661373765589</v>
       </c>
       <c r="J91" t="n">
-        <v>0.00998155622099163</v>
+        <v>0.009981556220991632</v>
       </c>
       <c r="K91" t="n">
         <v>0.01051261112679136</v>
@@ -6295,7 +6295,7 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>0.08625592042688515</v>
+        <v>0.08625592042688514</v>
       </c>
       <c r="D92" t="n">
         <v>0.07801647536873964</v>
@@ -6307,7 +6307,7 @@
         <v>0.07100647611221503</v>
       </c>
       <c r="G92" t="n">
-        <v>0.0789817644728991</v>
+        <v>0.07898176447289912</v>
       </c>
       <c r="H92" t="n">
         <v>0.0661880222322547</v>
@@ -6319,7 +6319,7 @@
         <v>0.09697468775771055</v>
       </c>
       <c r="K92" t="n">
-        <v>0.1009982068395509</v>
+        <v>0.100998206839551</v>
       </c>
       <c r="L92" t="n">
         <v>0.1249070614196443</v>
@@ -6359,7 +6359,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>0.7712787491124984</v>
+        <v>0.7712787491124983</v>
       </c>
       <c r="D93" t="n">
         <v>0.6554054395758764</v>
@@ -6368,10 +6368,10 @@
         <v>0.7348946877395629</v>
       </c>
       <c r="F93" t="n">
-        <v>0.5143752206739165</v>
+        <v>0.5143752206739164</v>
       </c>
       <c r="G93" t="n">
-        <v>0.5475059222253742</v>
+        <v>0.547505922225374</v>
       </c>
       <c r="H93" t="n">
         <v>1.047038876766988</v>
@@ -6380,13 +6380,13 @@
         <v>0.9282720152435452</v>
       </c>
       <c r="J93" t="n">
-        <v>0.755788643937087</v>
+        <v>0.7557886439370869</v>
       </c>
       <c r="K93" t="n">
-        <v>0.7292431431132189</v>
+        <v>0.7292431431132188</v>
       </c>
       <c r="L93" t="n">
-        <v>0.7961537520618309</v>
+        <v>0.796153752061831</v>
       </c>
       <c r="M93" t="n">
         <v>0.7659542689636312</v>
@@ -6401,7 +6401,7 @@
         <v>1.116509428003112</v>
       </c>
       <c r="Q93" t="n">
-        <v>0.5997736627781288</v>
+        <v>0.5997736627781289</v>
       </c>
       <c r="R93" t="n">
         <v>1.491387534136776</v>
@@ -6441,7 +6441,7 @@
         <v>0.2354046684687308</v>
       </c>
       <c r="I94" t="n">
-        <v>0.4290254973591949</v>
+        <v>0.4290254973591948</v>
       </c>
       <c r="J94" t="n">
         <v>0.3558618120515695</v>
@@ -6453,7 +6453,7 @@
         <v>0.4546009389174042</v>
       </c>
       <c r="M94" t="n">
-        <v>0.393411007678273</v>
+        <v>0.3934110076782731</v>
       </c>
       <c r="N94" t="n">
         <v>0.4517372060521735</v>
@@ -6490,7 +6490,7 @@
         <v>0.4953693692724408</v>
       </c>
       <c r="D95" t="n">
-        <v>0.4533992482492631</v>
+        <v>0.4533992482492632</v>
       </c>
       <c r="E95" t="n">
         <v>0.4946000472131031</v>
@@ -6502,7 +6502,7 @@
         <v>0.4343755437320184</v>
       </c>
       <c r="H95" t="n">
-        <v>0.5264363576669171</v>
+        <v>0.526436357666917</v>
       </c>
       <c r="I95" t="n">
         <v>0.570102900138062</v>
@@ -6520,13 +6520,13 @@
         <v>0.5334785492231423</v>
       </c>
       <c r="N95" t="n">
-        <v>0.5569789107032853</v>
+        <v>0.5569789107032852</v>
       </c>
       <c r="O95" t="n">
         <v>0.6782095792201264</v>
       </c>
       <c r="P95" t="n">
-        <v>0.764068476495533</v>
+        <v>0.7640684764955331</v>
       </c>
       <c r="Q95" t="n">
         <v>0.5961390988133128</v>
@@ -6535,7 +6535,7 @@
         <v>0.7455975000702634</v>
       </c>
       <c r="S95" t="n">
-        <v>0.6336853379094591</v>
+        <v>0.6336853379094592</v>
       </c>
       <c r="T95" t="n">
         <v>0.672750971014471</v>
@@ -6563,7 +6563,7 @@
         <v>0.1350146240585984</v>
       </c>
       <c r="G96" t="n">
-        <v>0.1517260826395599</v>
+        <v>0.1517260826395598</v>
       </c>
       <c r="H96" t="n">
         <v>0.2222941311482099</v>
@@ -6572,7 +6572,7 @@
         <v>0.2529899056417854</v>
       </c>
       <c r="J96" t="n">
-        <v>0.2342655673948319</v>
+        <v>0.2342655673948318</v>
       </c>
       <c r="K96" t="n">
         <v>0.2364135732087782</v>
@@ -6590,19 +6590,19 @@
         <v>0.5207305060998288</v>
       </c>
       <c r="P96" t="n">
-        <v>0.4612693111431391</v>
+        <v>0.461269311143139</v>
       </c>
       <c r="Q96" t="n">
         <v>0.45657478758342</v>
       </c>
       <c r="R96" t="n">
-        <v>0.5965024187343202</v>
+        <v>0.5965024187343203</v>
       </c>
       <c r="S96" t="n">
         <v>0.6045335162258804</v>
       </c>
       <c r="T96" t="n">
-        <v>0.5858840725609685</v>
+        <v>0.5858840725609684</v>
       </c>
     </row>
     <row r="97">
@@ -6627,13 +6627,13 @@
         <v>0.0304712767108469</v>
       </c>
       <c r="G97" t="n">
-        <v>0.03234292294534802</v>
+        <v>0.03234292294534803</v>
       </c>
       <c r="H97" t="n">
         <v>0.02952461267833622</v>
       </c>
       <c r="I97" t="n">
-        <v>0.04806366259892491</v>
+        <v>0.0480636625989249</v>
       </c>
       <c r="J97" t="n">
         <v>0.04176296972431984</v>
@@ -6642,7 +6642,7 @@
         <v>0.04237198931489834</v>
       </c>
       <c r="L97" t="n">
-        <v>0.05996663682789351</v>
+        <v>0.05996663682789352</v>
       </c>
       <c r="M97" t="n">
         <v>0.05482763187810819</v>
@@ -6651,7 +6651,7 @@
         <v>0.0567038137452178</v>
       </c>
       <c r="O97" t="n">
-        <v>0.09357982263230565</v>
+        <v>0.09357982263230566</v>
       </c>
       <c r="P97" t="n">
         <v>0.1130803356566493</v>
@@ -6663,7 +6663,7 @@
         <v>0.1283721371705351</v>
       </c>
       <c r="S97" t="n">
-        <v>0.1339617349782585</v>
+        <v>0.1339617349782584</v>
       </c>
       <c r="T97" t="n">
         <v>0.1371763294525771</v>
@@ -6682,7 +6682,7 @@
         <v>0.06531892543288957</v>
       </c>
       <c r="D98" t="n">
-        <v>0.06218992575321937</v>
+        <v>0.06218992575321935</v>
       </c>
       <c r="E98" t="n">
         <v>0.05996915305060359</v>
@@ -6691,19 +6691,19 @@
         <v>0.0655904605156524</v>
       </c>
       <c r="G98" t="n">
-        <v>0.06379327013865761</v>
+        <v>0.06379327013865763</v>
       </c>
       <c r="H98" t="n">
-        <v>0.07879256798772688</v>
+        <v>0.07879256798772689</v>
       </c>
       <c r="I98" t="n">
         <v>0.1045954781126142</v>
       </c>
       <c r="J98" t="n">
-        <v>0.08387857574106961</v>
+        <v>0.08387857574106963</v>
       </c>
       <c r="K98" t="n">
-        <v>0.08982486574616702</v>
+        <v>0.08982486574616703</v>
       </c>
       <c r="L98" t="n">
         <v>0.1141302357486455</v>
@@ -6718,16 +6718,16 @@
         <v>0.1994971335262662</v>
       </c>
       <c r="P98" t="n">
-        <v>0.2110116619531146</v>
+        <v>0.2110116619531147</v>
       </c>
       <c r="Q98" t="n">
-        <v>0.1906983546248199</v>
+        <v>0.1906983546248198</v>
       </c>
       <c r="R98" t="n">
-        <v>0.2374188615686212</v>
+        <v>0.2374188615686211</v>
       </c>
       <c r="S98" t="n">
-        <v>0.2210279956493577</v>
+        <v>0.2210279956493578</v>
       </c>
       <c r="T98" t="n">
         <v>0.2400608097112797</v>
@@ -6743,7 +6743,7 @@
         </is>
       </c>
       <c r="C99" t="n">
-        <v>0.03924334014375772</v>
+        <v>0.03924334014375773</v>
       </c>
       <c r="D99" t="n">
         <v>0.03380927103038552</v>
@@ -6755,7 +6755,7 @@
         <v>0.04217129168419489</v>
       </c>
       <c r="G99" t="n">
-        <v>0.04401968976312559</v>
+        <v>0.0440196897631256</v>
       </c>
       <c r="H99" t="n">
         <v>0.05254094076605902</v>
@@ -6764,10 +6764,10 @@
         <v>0.0747091262953315</v>
       </c>
       <c r="J99" t="n">
-        <v>0.067332409463476</v>
+        <v>0.06733240946347598</v>
       </c>
       <c r="K99" t="n">
-        <v>0.06364515952936124</v>
+        <v>0.06364515952936126</v>
       </c>
       <c r="L99" t="n">
         <v>0.07579122685742143</v>
@@ -6776,7 +6776,7 @@
         <v>0.07194246703752807</v>
       </c>
       <c r="N99" t="n">
-        <v>0.07706706696222777</v>
+        <v>0.07706706696222779</v>
       </c>
       <c r="O99" t="n">
         <v>0.1325393248572746</v>
@@ -6816,7 +6816,7 @@
         <v>0.10628681074612</v>
       </c>
       <c r="F100" t="n">
-        <v>0.08995811277860048</v>
+        <v>0.0899581127786005</v>
       </c>
       <c r="G100" t="n">
         <v>0.088735560711039</v>
@@ -6843,7 +6843,7 @@
         <v>0.1423387145656542</v>
       </c>
       <c r="O100" t="n">
-        <v>0.2211778329946829</v>
+        <v>0.2211778329946828</v>
       </c>
       <c r="P100" t="n">
         <v>0.2202221022944229</v>
@@ -6855,7 +6855,7 @@
         <v>0.2466078947535292</v>
       </c>
       <c r="S100" t="n">
-        <v>0.2482454406371755</v>
+        <v>0.2482454406371754</v>
       </c>
       <c r="T100" t="n">
         <v>0.2777215853373122</v>
@@ -6919,7 +6919,7 @@
         <v>0.4274906209236122</v>
       </c>
       <c r="S101" t="n">
-        <v>0.4465436722764185</v>
+        <v>0.4465436722764186</v>
       </c>
       <c r="T101" t="n">
         <v>0.4796167721842459</v>
@@ -7011,16 +7011,16 @@
         <v>0.03293331674025695</v>
       </c>
       <c r="G103" t="n">
-        <v>0.03026795626806312</v>
+        <v>0.03026795626806313</v>
       </c>
       <c r="H103" t="n">
-        <v>0.04171847545225149</v>
+        <v>0.04171847545225148</v>
       </c>
       <c r="I103" t="n">
         <v>0.04793581835401663</v>
       </c>
       <c r="J103" t="n">
-        <v>0.04176760800081346</v>
+        <v>0.04176760800081347</v>
       </c>
       <c r="K103" t="n">
         <v>0.04215617076575474</v>
@@ -7029,7 +7029,7 @@
         <v>0.04849379615433273</v>
       </c>
       <c r="M103" t="n">
-        <v>0.04965816437468151</v>
+        <v>0.04965816437468149</v>
       </c>
       <c r="N103" t="n">
         <v>0.0503209612435476</v>
@@ -7041,7 +7041,7 @@
         <v>0.07287907595229685</v>
       </c>
       <c r="Q103" t="n">
-        <v>0.07541772980031558</v>
+        <v>0.07541772980031555</v>
       </c>
       <c r="R103" t="n">
         <v>0.09691409456915474</v>
@@ -7050,7 +7050,7 @@
         <v>0.08907585487301589</v>
       </c>
       <c r="T103" t="n">
-        <v>0.08549185195936547</v>
+        <v>0.08549185195936546</v>
       </c>
     </row>
     <row r="104">
@@ -7063,7 +7063,7 @@
         </is>
       </c>
       <c r="C104" t="n">
-        <v>0.09044645776645846</v>
+        <v>0.09044645776645845</v>
       </c>
       <c r="D104" t="n">
         <v>0.08713636554628902</v>
@@ -7075,7 +7075,7 @@
         <v>0.08391294348413214</v>
       </c>
       <c r="G104" t="n">
-        <v>0.08677815452498969</v>
+        <v>0.0867781545249897</v>
       </c>
       <c r="H104" t="n">
         <v>0.0719286157344896</v>
@@ -7084,7 +7084,7 @@
         <v>0.1166249447041498</v>
       </c>
       <c r="J104" t="n">
-        <v>0.09895297046330495</v>
+        <v>0.09895297046330494</v>
       </c>
       <c r="K104" t="n">
         <v>0.1038573560059444</v>
@@ -7102,13 +7102,13 @@
         <v>0.1809315018351128</v>
       </c>
       <c r="P104" t="n">
-        <v>0.1805709191206047</v>
+        <v>0.1805709191206046</v>
       </c>
       <c r="Q104" t="n">
         <v>0.1705255841763265</v>
       </c>
       <c r="R104" t="n">
-        <v>0.1910374347783411</v>
+        <v>0.1910374347783412</v>
       </c>
       <c r="S104" t="n">
         <v>0.1906562970796666</v>
@@ -7130,19 +7130,19 @@
         <v>0.1027709313058061</v>
       </c>
       <c r="D105" t="n">
-        <v>0.09393807738276126</v>
+        <v>0.09393807738276125</v>
       </c>
       <c r="E105" t="n">
-        <v>0.0859809181655553</v>
+        <v>0.08598091816555528</v>
       </c>
       <c r="F105" t="n">
         <v>0.08509178210180696</v>
       </c>
       <c r="G105" t="n">
-        <v>0.08899277775636995</v>
+        <v>0.08899277775636993</v>
       </c>
       <c r="H105" t="n">
-        <v>0.0909614702633174</v>
+        <v>0.09096147026331741</v>
       </c>
       <c r="I105" t="n">
         <v>0.1374754101796</v>
@@ -7175,7 +7175,7 @@
         <v>0.2550371984085896</v>
       </c>
       <c r="S105" t="n">
-        <v>0.2435966559983967</v>
+        <v>0.2435966559983966</v>
       </c>
       <c r="T105" t="n">
         <v>0.23795260190567</v>
@@ -7197,7 +7197,7 @@
         <v>0.186493448869881</v>
       </c>
       <c r="E106" t="n">
-        <v>0.2165407554716995</v>
+        <v>0.2165407554716994</v>
       </c>
       <c r="F106" t="n">
         <v>0.1744340902489996</v>
@@ -7212,7 +7212,7 @@
         <v>0.2763567556601654</v>
       </c>
       <c r="J106" t="n">
-        <v>0.2348720174067936</v>
+        <v>0.2348720174067935</v>
       </c>
       <c r="K106" t="n">
         <v>0.2353343108108224</v>
@@ -7221,7 +7221,7 @@
         <v>0.2570087429472243</v>
       </c>
       <c r="M106" t="n">
-        <v>0.2617282182589089</v>
+        <v>0.2617282182589088</v>
       </c>
       <c r="N106" t="n">
         <v>0.2794040744160127</v>
@@ -7255,7 +7255,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>0.05829479483327835</v>
+        <v>0.05829479483327837</v>
       </c>
       <c r="D107" t="n">
         <v>0.04917303096118841</v>
@@ -7279,7 +7279,7 @@
         <v>0.07030848800768889</v>
       </c>
       <c r="K107" t="n">
-        <v>0.06896695079849763</v>
+        <v>0.06896695079849764</v>
       </c>
       <c r="L107" t="n">
         <v>0.06449414900494278</v>
@@ -7288,7 +7288,7 @@
         <v>0.07345723056398122</v>
       </c>
       <c r="N107" t="n">
-        <v>0.0678873037541696</v>
+        <v>0.06788730375416958</v>
       </c>
       <c r="O107" t="n">
         <v>0.1339083718702938</v>
@@ -7322,16 +7322,16 @@
         <v>0.5101234225125985</v>
       </c>
       <c r="D108" t="n">
-        <v>0.4630616644207623</v>
+        <v>0.4630616644207625</v>
       </c>
       <c r="E108" t="n">
         <v>0.4783541097144988</v>
       </c>
       <c r="F108" t="n">
-        <v>0.4454307220511723</v>
+        <v>0.4454307220511722</v>
       </c>
       <c r="G108" t="n">
-        <v>0.4655193486598913</v>
+        <v>0.4655193486598914</v>
       </c>
       <c r="H108" t="n">
         <v>0.5454465916869444</v>
@@ -7340,19 +7340,19 @@
         <v>0.6746552088366982</v>
       </c>
       <c r="J108" t="n">
-        <v>0.594337861701755</v>
+        <v>0.5943378617017551</v>
       </c>
       <c r="K108" t="n">
         <v>0.6000502950882362</v>
       </c>
       <c r="L108" t="n">
-        <v>0.6682684462619436</v>
+        <v>0.6682684462619438</v>
       </c>
       <c r="M108" t="n">
-        <v>0.6590412161994198</v>
+        <v>0.65904121619942</v>
       </c>
       <c r="N108" t="n">
-        <v>0.7035790012512178</v>
+        <v>0.7035790012512176</v>
       </c>
       <c r="O108" t="n">
         <v>1.048874403837277</v>
@@ -7370,7 +7370,7 @@
         <v>1.122373491145812</v>
       </c>
       <c r="T108" t="n">
-        <v>1.271951823513563</v>
+        <v>1.271951823513564</v>
       </c>
     </row>
     <row r="109">
@@ -7483,7 +7483,7 @@
         <v>0.1932500887452609</v>
       </c>
       <c r="O110" t="n">
-        <v>0.3133784444673172</v>
+        <v>0.3133784444673173</v>
       </c>
       <c r="P110" t="n">
         <v>0.3451279815988144</v>
@@ -7514,16 +7514,16 @@
         <v>2.428072989809201</v>
       </c>
       <c r="D111" t="n">
-        <v>2.21605567541512</v>
+        <v>2.216055675415121</v>
       </c>
       <c r="E111" t="n">
-        <v>2.306171217997636</v>
+        <v>2.306171217997635</v>
       </c>
       <c r="F111" t="n">
         <v>1.909036602409349</v>
       </c>
       <c r="G111" t="n">
-        <v>2.046169947757327</v>
+        <v>2.046169947757326</v>
       </c>
       <c r="H111" t="n">
         <v>2.5330853397156</v>
@@ -7550,7 +7550,7 @@
         <v>4.423906837336295</v>
       </c>
       <c r="P111" t="n">
-        <v>4.35370637808815</v>
+        <v>4.353706378088149</v>
       </c>
       <c r="Q111" t="n">
         <v>4.206431133111779</v>
@@ -7562,7 +7562,7 @@
         <v>5.348155786784831</v>
       </c>
       <c r="T111" t="n">
-        <v>5.343083739330379</v>
+        <v>5.34308373933038</v>
       </c>
     </row>
     <row r="112">
@@ -7605,25 +7605,25 @@
         <v>0.2106602483431021</v>
       </c>
       <c r="M112" t="n">
-        <v>0.2223755308085499</v>
+        <v>0.2223755308085498</v>
       </c>
       <c r="N112" t="n">
-        <v>0.2170466243168654</v>
+        <v>0.2170466243168653</v>
       </c>
       <c r="O112" t="n">
-        <v>0.3581196260909452</v>
+        <v>0.3581196260909453</v>
       </c>
       <c r="P112" t="n">
         <v>0.330090299681918</v>
       </c>
       <c r="Q112" t="n">
-        <v>0.3695391844189431</v>
+        <v>0.3695391844189432</v>
       </c>
       <c r="R112" t="n">
         <v>0.3921391808218673</v>
       </c>
       <c r="S112" t="n">
-        <v>0.4663618835657086</v>
+        <v>0.4663618835657087</v>
       </c>
       <c r="T112" t="n">
         <v>0.4871132460500389</v>
@@ -7639,10 +7639,10 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>0.04491887659854188</v>
+        <v>0.04491887659854187</v>
       </c>
       <c r="D113" t="n">
-        <v>0.0298296366955252</v>
+        <v>0.02982963669552521</v>
       </c>
       <c r="E113" t="n">
         <v>0.03193271867545315</v>
@@ -7660,10 +7660,10 @@
         <v>0.04874797363411498</v>
       </c>
       <c r="J113" t="n">
-        <v>0.04241619021635766</v>
+        <v>0.04241619021635765</v>
       </c>
       <c r="K113" t="n">
-        <v>0.04037746642106956</v>
+        <v>0.04037746642106957</v>
       </c>
       <c r="L113" t="n">
         <v>0.04963104701768073</v>
@@ -7718,10 +7718,10 @@
         <v>0.01405106662459578</v>
       </c>
       <c r="H114" t="n">
-        <v>0.02317985066823313</v>
+        <v>0.02317985066823312</v>
       </c>
       <c r="I114" t="n">
-        <v>0.02220003525830457</v>
+        <v>0.02220003525830456</v>
       </c>
       <c r="J114" t="n">
         <v>0.01858928597674101</v>
@@ -7751,10 +7751,10 @@
         <v>0.054784359252892</v>
       </c>
       <c r="S114" t="n">
-        <v>0.04887452673400482</v>
+        <v>0.04887452673400481</v>
       </c>
       <c r="T114" t="n">
-        <v>0.04519846555700198</v>
+        <v>0.04519846555700199</v>
       </c>
     </row>
     <row r="115">
@@ -7770,7 +7770,7 @@
         <v>0.2882826782378188</v>
       </c>
       <c r="D115" t="n">
-        <v>0.2596177988731837</v>
+        <v>0.2596177988731838</v>
       </c>
       <c r="E115" t="n">
         <v>0.2643634038236027</v>
@@ -7788,7 +7788,7 @@
         <v>0.4026607505222828</v>
       </c>
       <c r="J115" t="n">
-        <v>0.3534028506686883</v>
+        <v>0.3534028506686882</v>
       </c>
       <c r="K115" t="n">
         <v>0.3580528216494313</v>
@@ -7800,19 +7800,19 @@
         <v>0.4429762482509985</v>
       </c>
       <c r="N115" t="n">
-        <v>0.4226519572721288</v>
+        <v>0.4226519572721289</v>
       </c>
       <c r="O115" t="n">
-        <v>0.7550897497595671</v>
+        <v>0.7550897497595669</v>
       </c>
       <c r="P115" t="n">
-        <v>0.7370437127873851</v>
+        <v>0.7370437127873852</v>
       </c>
       <c r="Q115" t="n">
         <v>0.754051893186615</v>
       </c>
       <c r="R115" t="n">
-        <v>0.9585364727435163</v>
+        <v>0.9585364727435164</v>
       </c>
       <c r="S115" t="n">
         <v>0.9809816707575171</v>
@@ -7831,28 +7831,28 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>0.09242939732681775</v>
+        <v>0.09242939732681776</v>
       </c>
       <c r="D116" t="n">
-        <v>0.08302151540545169</v>
+        <v>0.0830215154054517</v>
       </c>
       <c r="E116" t="n">
         <v>0.0870420491802058</v>
       </c>
       <c r="F116" t="n">
-        <v>0.0773743162037839</v>
+        <v>0.07737431620378392</v>
       </c>
       <c r="G116" t="n">
-        <v>0.08321588227671044</v>
+        <v>0.08321588227671042</v>
       </c>
       <c r="H116" t="n">
-        <v>0.0861312718183298</v>
+        <v>0.08613127181832982</v>
       </c>
       <c r="I116" t="n">
         <v>0.1109691571948775</v>
       </c>
       <c r="J116" t="n">
-        <v>0.09223783201410282</v>
+        <v>0.09223783201410281</v>
       </c>
       <c r="K116" t="n">
         <v>0.09876486462459264</v>
@@ -7861,13 +7861,13 @@
         <v>0.1049099458252576</v>
       </c>
       <c r="M116" t="n">
-        <v>0.1050776726829564</v>
+        <v>0.1050776726829563</v>
       </c>
       <c r="N116" t="n">
         <v>0.1131739929662637</v>
       </c>
       <c r="O116" t="n">
-        <v>0.1643653690071009</v>
+        <v>0.1643653690071008</v>
       </c>
       <c r="P116" t="n">
         <v>0.1650313945374654</v>
@@ -7882,7 +7882,7 @@
         <v>0.1760549860689678</v>
       </c>
       <c r="T116" t="n">
-        <v>0.2037713736459129</v>
+        <v>0.203771373645913</v>
       </c>
     </row>
     <row r="117">
@@ -7904,7 +7904,7 @@
         <v>0.04344081938351101</v>
       </c>
       <c r="F117" t="n">
-        <v>0.04909478044309922</v>
+        <v>0.04909478044309923</v>
       </c>
       <c r="G117" t="n">
         <v>0.03831377203608224</v>
@@ -7913,22 +7913,22 @@
         <v>0.05801065755781137</v>
       </c>
       <c r="I117" t="n">
-        <v>0.1010451866933929</v>
+        <v>0.1010451866933928</v>
       </c>
       <c r="J117" t="n">
         <v>0.07422423305444274</v>
       </c>
       <c r="K117" t="n">
-        <v>0.08741121325958065</v>
+        <v>0.08741121325958066</v>
       </c>
       <c r="L117" t="n">
         <v>0.09519134926709452</v>
       </c>
       <c r="M117" t="n">
-        <v>0.08974562578912532</v>
+        <v>0.0897456257891253</v>
       </c>
       <c r="N117" t="n">
-        <v>0.06957787094727198</v>
+        <v>0.06957787094727197</v>
       </c>
       <c r="O117" t="n">
         <v>0.184134835247514</v>
@@ -7974,7 +7974,7 @@
         <v>0.007062712305584419</v>
       </c>
       <c r="H118" t="n">
-        <v>0.006937971521298141</v>
+        <v>0.006937971521298142</v>
       </c>
       <c r="I118" t="n">
         <v>0.01214372176951727</v>
@@ -8035,10 +8035,10 @@
         <v>0.3117246836364982</v>
       </c>
       <c r="G119" t="n">
-        <v>0.3285180159785941</v>
+        <v>0.3285180159785942</v>
       </c>
       <c r="H119" t="n">
-        <v>0.3152239826089193</v>
+        <v>0.3152239826089192</v>
       </c>
       <c r="I119" t="n">
         <v>0.5569827412216705</v>
@@ -8056,16 +8056,16 @@
         <v>0.5435166559557555</v>
       </c>
       <c r="N119" t="n">
-        <v>0.6030104600436829</v>
+        <v>0.6030104600436826</v>
       </c>
       <c r="O119" t="n">
-        <v>0.8847711651821889</v>
+        <v>0.884771165182189</v>
       </c>
       <c r="P119" t="n">
         <v>0.9358240422108777</v>
       </c>
       <c r="Q119" t="n">
-        <v>0.8067208686977894</v>
+        <v>0.8067208686977895</v>
       </c>
       <c r="R119" t="n">
         <v>1.013353858934098</v>
@@ -8087,10 +8087,10 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>36.39399150982232</v>
+        <v>36.39399150982233</v>
       </c>
       <c r="D120" t="n">
-        <v>31.68529641612839</v>
+        <v>31.6852964161284</v>
       </c>
       <c r="E120" t="n">
         <v>33.57958085110323</v>
@@ -8099,28 +8099,28 @@
         <v>31.78928049077359</v>
       </c>
       <c r="G120" t="n">
-        <v>32.17709875680912</v>
+        <v>32.17709875680911</v>
       </c>
       <c r="H120" t="n">
         <v>46.04880265413406</v>
       </c>
       <c r="I120" t="n">
-        <v>55.72667963150799</v>
+        <v>55.72667963150798</v>
       </c>
       <c r="J120" t="n">
-        <v>46.88073909451125</v>
+        <v>46.88073909451126</v>
       </c>
       <c r="K120" t="n">
-        <v>46.06991967003136</v>
+        <v>46.06991967003137</v>
       </c>
       <c r="L120" t="n">
-        <v>66.86606208878895</v>
+        <v>66.86606208878894</v>
       </c>
       <c r="M120" t="n">
-        <v>64.6208879236266</v>
+        <v>64.62088792362663</v>
       </c>
       <c r="N120" t="n">
-        <v>59.94315758148488</v>
+        <v>59.94315758148489</v>
       </c>
       <c r="O120" t="n">
         <v>160.0510620993676</v>
@@ -8129,10 +8129,10 @@
         <v>159.2556506418967</v>
       </c>
       <c r="Q120" t="n">
-        <v>148.0693184042884</v>
+        <v>148.0693184042883</v>
       </c>
       <c r="R120" t="n">
-        <v>239.3649296795552</v>
+        <v>239.3649296795553</v>
       </c>
       <c r="S120" t="n">
         <v>253.2538501704686</v>
@@ -8236,28 +8236,28 @@
         <v>0.03907891452627016</v>
       </c>
       <c r="J122" t="n">
-        <v>0.03617448979934359</v>
+        <v>0.03617448979934358</v>
       </c>
       <c r="K122" t="n">
         <v>0.03915343791191977</v>
       </c>
       <c r="L122" t="n">
-        <v>0.0406561590421466</v>
+        <v>0.04065615904214659</v>
       </c>
       <c r="M122" t="n">
-        <v>0.03649438428811822</v>
+        <v>0.03649438428811823</v>
       </c>
       <c r="N122" t="n">
         <v>0.04588618740527185</v>
       </c>
       <c r="O122" t="n">
-        <v>0.05268373050962067</v>
+        <v>0.05268373050962066</v>
       </c>
       <c r="P122" t="n">
         <v>0.05704856430363184</v>
       </c>
       <c r="Q122" t="n">
-        <v>0.04092794229738319</v>
+        <v>0.04092794229738318</v>
       </c>
       <c r="R122" t="n">
         <v>0.05121048123456331</v>
@@ -8282,10 +8282,10 @@
         <v>0.9399657643332729</v>
       </c>
       <c r="D123" t="n">
-        <v>0.8700527698978928</v>
+        <v>0.8700527698978929</v>
       </c>
       <c r="E123" t="n">
-        <v>0.8946711411131363</v>
+        <v>0.8946711411131362</v>
       </c>
       <c r="F123" t="n">
         <v>0.7474726080203441</v>
@@ -8294,7 +8294,7 @@
         <v>0.7737824462692394</v>
       </c>
       <c r="H123" t="n">
-        <v>0.9047812536436597</v>
+        <v>0.9047812536436596</v>
       </c>
       <c r="I123" t="n">
         <v>1.20360330990213</v>
@@ -8321,7 +8321,7 @@
         <v>2.151554306896785</v>
       </c>
       <c r="Q123" t="n">
-        <v>2.386687071960739</v>
+        <v>2.38668707196074</v>
       </c>
       <c r="R123" t="n">
         <v>2.720748388672598</v>
@@ -8355,7 +8355,7 @@
         <v>0.5244515198697509</v>
       </c>
       <c r="G124" t="n">
-        <v>0.5934844138698825</v>
+        <v>0.5934844138698824</v>
       </c>
       <c r="H124" t="n">
         <v>0.524715641976671</v>
@@ -8391,7 +8391,7 @@
         <v>1.30129941627612</v>
       </c>
       <c r="S124" t="n">
-        <v>1.273681295473753</v>
+        <v>1.273681295473754</v>
       </c>
       <c r="T124" t="n">
         <v>1.259365386249102</v>
@@ -8410,7 +8410,7 @@
         <v>1.632089249198855</v>
       </c>
       <c r="D125" t="n">
-        <v>1.503509674621543</v>
+        <v>1.503509674621542</v>
       </c>
       <c r="E125" t="n">
         <v>1.374822597700631</v>
@@ -8431,7 +8431,7 @@
         <v>1.732914417703089</v>
       </c>
       <c r="K125" t="n">
-        <v>1.997007496237452</v>
+        <v>1.997007496237453</v>
       </c>
       <c r="L125" t="n">
         <v>2.241979550608346</v>
@@ -8455,10 +8455,10 @@
         <v>3.451556662640702</v>
       </c>
       <c r="S125" t="n">
-        <v>3.666081720345592</v>
+        <v>3.666081720345591</v>
       </c>
       <c r="T125" t="n">
-        <v>4.442412202303253</v>
+        <v>4.442412202303252</v>
       </c>
     </row>
     <row r="126">
@@ -8480,7 +8480,7 @@
         <v>0.02000814786674313</v>
       </c>
       <c r="F126" t="n">
-        <v>0.02222472790999756</v>
+        <v>0.02222472790999755</v>
       </c>
       <c r="G126" t="n">
         <v>0.02327308798891593</v>
@@ -8498,7 +8498,7 @@
         <v>0.02921254809571045</v>
       </c>
       <c r="L126" t="n">
-        <v>0.03621011087554069</v>
+        <v>0.03621011087554068</v>
       </c>
       <c r="M126" t="n">
         <v>0.03608157384454446</v>
@@ -8541,7 +8541,7 @@
         <v>0.1174769158937752</v>
       </c>
       <c r="E127" t="n">
-        <v>0.09986227523868139</v>
+        <v>0.09986227523868141</v>
       </c>
       <c r="F127" t="n">
         <v>0.1289563043001198</v>
@@ -8574,7 +8574,7 @@
         <v>0.4301833303193309</v>
       </c>
       <c r="P127" t="n">
-        <v>0.4379004654374034</v>
+        <v>0.4379004654374033</v>
       </c>
       <c r="Q127" t="n">
         <v>0.4891456530927932</v>
@@ -8666,10 +8666,10 @@
         <v>0.08146352898443948</v>
       </c>
       <c r="D129" t="n">
-        <v>0.06766574952355978</v>
+        <v>0.06766574952355979</v>
       </c>
       <c r="E129" t="n">
-        <v>0.06803780823990419</v>
+        <v>0.0680378082399042</v>
       </c>
       <c r="F129" t="n">
         <v>0.06161345630372916</v>
@@ -8708,7 +8708,7 @@
         <v>0.1965387060236291</v>
       </c>
       <c r="R129" t="n">
-        <v>0.252064879455528</v>
+        <v>0.2520648794555279</v>
       </c>
       <c r="S129" t="n">
         <v>0.2563922259951701</v>
@@ -8727,7 +8727,7 @@
         </is>
       </c>
       <c r="C130" t="n">
-        <v>0.05898244268949321</v>
+        <v>0.0589824426894932</v>
       </c>
       <c r="D130" t="n">
         <v>0.05595412900178483</v>
@@ -8739,7 +8739,7 @@
         <v>0.04963612267915252</v>
       </c>
       <c r="G130" t="n">
-        <v>0.0501850110011607</v>
+        <v>0.05018501100116069</v>
       </c>
       <c r="H130" t="n">
         <v>0.04899177943647669</v>
@@ -8751,13 +8751,13 @@
         <v>0.066698571745861</v>
       </c>
       <c r="K130" t="n">
-        <v>0.07383714990242726</v>
+        <v>0.07383714990242725</v>
       </c>
       <c r="L130" t="n">
         <v>0.07093129061950607</v>
       </c>
       <c r="M130" t="n">
-        <v>0.07324323171672967</v>
+        <v>0.07324323171672965</v>
       </c>
       <c r="N130" t="n">
         <v>0.07751611637523577</v>
@@ -8800,7 +8800,7 @@
         <v>0.1254492810893389</v>
       </c>
       <c r="F131" t="n">
-        <v>0.1240649131257954</v>
+        <v>0.1240649131257953</v>
       </c>
       <c r="G131" t="n">
         <v>0.1307136115909444</v>
@@ -8827,7 +8827,7 @@
         <v>0.2132299028777321</v>
       </c>
       <c r="O131" t="n">
-        <v>0.3364997309286672</v>
+        <v>0.3364997309286671</v>
       </c>
       <c r="P131" t="n">
         <v>0.3315956427584689</v>
@@ -8867,7 +8867,7 @@
         <v>0.06981645244968782</v>
       </c>
       <c r="G132" t="n">
-        <v>0.07213817805808045</v>
+        <v>0.07213817805808047</v>
       </c>
       <c r="H132" t="n">
         <v>0.08460764374923067</v>
@@ -8925,7 +8925,7 @@
         <v>0.9242428050988843</v>
       </c>
       <c r="E133" t="n">
-        <v>1.098011482255053</v>
+        <v>1.098011482255052</v>
       </c>
       <c r="F133" t="n">
         <v>1.19648764895406</v>
@@ -8940,7 +8940,7 @@
         <v>2.038134390304134</v>
       </c>
       <c r="J133" t="n">
-        <v>1.765012107327487</v>
+        <v>1.765012107327488</v>
       </c>
       <c r="K133" t="n">
         <v>1.704248274815274</v>
@@ -8958,13 +8958,13 @@
         <v>4.972578129277611</v>
       </c>
       <c r="P133" t="n">
-        <v>4.696528261225936</v>
+        <v>4.696528261225937</v>
       </c>
       <c r="Q133" t="n">
         <v>4.648363209790867</v>
       </c>
       <c r="R133" t="n">
-        <v>6.918524389962565</v>
+        <v>6.918524389962566</v>
       </c>
       <c r="S133" t="n">
         <v>7.004429082625482</v>
@@ -8992,7 +8992,7 @@
         <v>0.003855378850455751</v>
       </c>
       <c r="F134" t="n">
-        <v>0.003265007207208155</v>
+        <v>0.003265007207208154</v>
       </c>
       <c r="G134" t="n">
         <v>0.003464109047324646</v>
@@ -9013,22 +9013,22 @@
         <v>0.004562543078647831</v>
       </c>
       <c r="M134" t="n">
-        <v>0.004425020456848929</v>
+        <v>0.004425020456848928</v>
       </c>
       <c r="N134" t="n">
         <v>0.004536615683405752</v>
       </c>
       <c r="O134" t="n">
-        <v>0.004000648607851964</v>
+        <v>0.004000648607851965</v>
       </c>
       <c r="P134" t="n">
         <v>0.00588903872533335</v>
       </c>
       <c r="Q134" t="n">
-        <v>0.004415197859653696</v>
+        <v>0.004415197859653697</v>
       </c>
       <c r="R134" t="n">
-        <v>0.005707098546805793</v>
+        <v>0.005707098546805792</v>
       </c>
       <c r="S134" t="n">
         <v>0.004711373892475688</v>
@@ -9047,7 +9047,7 @@
         </is>
       </c>
       <c r="C135" t="n">
-        <v>0.03548847653947745</v>
+        <v>0.03548847653947744</v>
       </c>
       <c r="D135" t="n">
         <v>0.03354701671517744</v>
@@ -9062,13 +9062,13 @@
         <v>0.02459151769600704</v>
       </c>
       <c r="H135" t="n">
-        <v>0.02383153798852695</v>
+        <v>0.02383153798852696</v>
       </c>
       <c r="I135" t="n">
         <v>0.03311827583658793</v>
       </c>
       <c r="J135" t="n">
-        <v>0.02868053283247979</v>
+        <v>0.0286805328324798</v>
       </c>
       <c r="K135" t="n">
         <v>0.0286921302474362</v>
@@ -9083,19 +9083,19 @@
         <v>0.0403911500339118</v>
       </c>
       <c r="O135" t="n">
-        <v>0.07073018304569614</v>
+        <v>0.07073018304569616</v>
       </c>
       <c r="P135" t="n">
-        <v>0.07489858299237576</v>
+        <v>0.07489858299237577</v>
       </c>
       <c r="Q135" t="n">
-        <v>0.07529819277237362</v>
+        <v>0.07529819277237361</v>
       </c>
       <c r="R135" t="n">
-        <v>0.09120238656550905</v>
+        <v>0.09120238656550907</v>
       </c>
       <c r="S135" t="n">
-        <v>0.09123032222020939</v>
+        <v>0.09123032222020941</v>
       </c>
       <c r="T135" t="n">
         <v>0.09785536894197602</v>
@@ -9211,7 +9211,7 @@
         <v>0.04508094035460074</v>
       </c>
       <c r="O137" t="n">
-        <v>0.06116672976681157</v>
+        <v>0.06116672976681158</v>
       </c>
       <c r="P137" t="n">
         <v>0.0628337129074041</v>
@@ -9220,13 +9220,13 @@
         <v>0.05145825336683772</v>
       </c>
       <c r="R137" t="n">
-        <v>0.05927287749060194</v>
+        <v>0.05927287749060193</v>
       </c>
       <c r="S137" t="n">
         <v>0.05595093132880288</v>
       </c>
       <c r="T137" t="n">
-        <v>0.0579540795021263</v>
+        <v>0.05795407950212631</v>
       </c>
     </row>
     <row r="138">
@@ -9245,10 +9245,10 @@
         <v>0.01208350221848329</v>
       </c>
       <c r="E138" t="n">
-        <v>0.008234922781882596</v>
+        <v>0.008234922781882594</v>
       </c>
       <c r="F138" t="n">
-        <v>0.01200460420857306</v>
+        <v>0.01200460420857307</v>
       </c>
       <c r="G138" t="n">
         <v>0.01260922027339027</v>
@@ -9275,7 +9275,7 @@
         <v>0.01751248503811286</v>
       </c>
       <c r="O138" t="n">
-        <v>0.02887553248198016</v>
+        <v>0.02887553248198015</v>
       </c>
       <c r="P138" t="n">
         <v>0.01840053132977065</v>
@@ -9351,7 +9351,7 @@
         <v>0.01936684133885338</v>
       </c>
       <c r="S139" t="n">
-        <v>0.03242587372762656</v>
+        <v>0.03242587372762655</v>
       </c>
       <c r="T139" t="n">
         <v>0.03247250829720138</v>

</xml_diff>